<commit_message>
mind erreichte normen anfang
</commit_message>
<xml_diff>
--- a/web/utilities/records_kriterien.xlsx
+++ b/web/utilities/records_kriterien.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jpgna\Documents\GitHub\Lifesaving_Baden\web\utilities\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B30D4FF-83EA-48EC-AF67-EC7B4ACCE4F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D09DCEC-8EF3-482A-98F0-B1501E0A56E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="687" firstSheet="1" activeTab="7" xr2:uid="{E1AB626B-3773-4829-92A5-28DD4DB7C8F8}"/>
   </bookViews>
@@ -185,7 +185,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="672" uniqueCount="247">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="673" uniqueCount="248">
   <si>
     <t>50m Retten</t>
   </si>
@@ -926,6 +926,9 @@
   </si>
   <si>
     <t>PK - Männlich</t>
+  </si>
+  <si>
+    <t>mind. erreichte Normen</t>
   </si>
 </sst>
 </file>
@@ -1611,13 +1614,16 @@
     <xf numFmtId="0" fontId="14" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1629,6 +1635,15 @@
     <xf numFmtId="0" fontId="14" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="10" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1637,6 +1652,27 @@
     </xf>
     <xf numFmtId="0" fontId="14" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1680,45 +1716,108 @@
     <xf numFmtId="0" fontId="17" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Prozent" xfId="1" builtinId="5"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="228">
+  <dxfs count="229">
+    <dxf>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <font>
         <color theme="4"/>
@@ -4141,99 +4240,6 @@
       </fill>
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -4248,102 +4254,102 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{2C5E83EE-6B6F-478A-9C90-A846A1A76536}" name="WR_Open4" displayName="WR_Open4" ref="A4:AW31" totalsRowShown="0" headerRowDxfId="201" headerRowBorderDxfId="200" tableBorderDxfId="199">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{2C5E83EE-6B6F-478A-9C90-A846A1A76536}" name="WR_Open4" displayName="WR_Open4" ref="A4:AW31" totalsRowShown="0" headerRowDxfId="228" headerRowBorderDxfId="227" tableBorderDxfId="226">
   <autoFilter ref="A4:AW31" xr:uid="{2C5E83EE-6B6F-478A-9C90-A846A1A76536}"/>
   <tableColumns count="49">
-    <tableColumn id="1" xr3:uid="{7C0C4105-A61A-4B8D-9129-EDC4F18765AF}" name="WR-Open" dataDxfId="198">
+    <tableColumn id="1" xr3:uid="{7C0C4105-A61A-4B8D-9129-EDC4F18765AF}" name="WR-Open" dataDxfId="225">
       <calculatedColumnFormula>A4+1</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{516F5612-F85F-413F-9012-E235F415E34B}" name="50m Retten - offen - W" dataDxfId="197"/>
-    <tableColumn id="3" xr3:uid="{BC9ACAC9-0D45-42FD-B596-D19FBE3A4D83}" name="100m Retten - offen - W" dataDxfId="196"/>
-    <tableColumn id="4" xr3:uid="{CB6DBE59-EB65-43F0-93E7-0BDC3F82832B}" name="100m Kombi - offen - W" dataDxfId="195"/>
-    <tableColumn id="5" xr3:uid="{AA603C60-6831-4C14-A8CD-0AA050DA7551}" name="100m Lifesaver - offen - W" dataDxfId="194"/>
-    <tableColumn id="6" xr3:uid="{7920F147-7717-4582-940A-2610F7D310CA}" name="200m Superlifesaver - offen - W" dataDxfId="193"/>
-    <tableColumn id="7" xr3:uid="{04E21F1D-AC8D-4A1B-9B43-59B8F7901673}" name="200m Hindernis - offen - W" dataDxfId="192"/>
-    <tableColumn id="8" xr3:uid="{40E8A083-653A-48A8-9B37-0A2D850B7829}" name="50m Retten - offen - M" dataDxfId="191"/>
-    <tableColumn id="9" xr3:uid="{863824A9-134F-4189-BB14-225AE224FC44}" name="100m Retten - offen - M" dataDxfId="190"/>
+    <tableColumn id="2" xr3:uid="{516F5612-F85F-413F-9012-E235F415E34B}" name="50m Retten - offen - W" dataDxfId="224"/>
+    <tableColumn id="3" xr3:uid="{BC9ACAC9-0D45-42FD-B596-D19FBE3A4D83}" name="100m Retten - offen - W" dataDxfId="223"/>
+    <tableColumn id="4" xr3:uid="{CB6DBE59-EB65-43F0-93E7-0BDC3F82832B}" name="100m Kombi - offen - W" dataDxfId="222"/>
+    <tableColumn id="5" xr3:uid="{AA603C60-6831-4C14-A8CD-0AA050DA7551}" name="100m Lifesaver - offen - W" dataDxfId="221"/>
+    <tableColumn id="6" xr3:uid="{7920F147-7717-4582-940A-2610F7D310CA}" name="200m Superlifesaver - offen - W" dataDxfId="220"/>
+    <tableColumn id="7" xr3:uid="{04E21F1D-AC8D-4A1B-9B43-59B8F7901673}" name="200m Hindernis - offen - W" dataDxfId="219"/>
+    <tableColumn id="8" xr3:uid="{40E8A083-653A-48A8-9B37-0A2D850B7829}" name="50m Retten - offen - M" dataDxfId="218"/>
+    <tableColumn id="9" xr3:uid="{863824A9-134F-4189-BB14-225AE224FC44}" name="100m Retten - offen - M" dataDxfId="217"/>
     <tableColumn id="10" xr3:uid="{598FC6AE-DEA2-4475-9A35-CDCB8C81496A}" name="100m Kombi - offen - M"/>
     <tableColumn id="11" xr3:uid="{9FC50B37-0D51-422E-A268-A6506D4F3854}" name="100m Lifesaver - offen - M"/>
     <tableColumn id="12" xr3:uid="{B8D2552B-5D82-442A-98F0-E47D5C5F6728}" name="200m Superlifesaver - offen - M"/>
-    <tableColumn id="13" xr3:uid="{5A5E9873-0C5F-4508-AF6B-4974E0526D84}" name="200m Hindernis - offen - M" dataDxfId="189"/>
-    <tableColumn id="14" xr3:uid="{FA907992-7FCE-4CAD-8CF2-F5BEBC9B3756}" name="50m Retten - 17/18 - W" dataDxfId="188"/>
-    <tableColumn id="15" xr3:uid="{76B63DC0-CB67-48F4-9B5A-D22902F59334}" name="100m Retten - 17/18 - W" dataDxfId="187"/>
-    <tableColumn id="16" xr3:uid="{614A2419-51B1-44C0-8469-ADBFB078B81A}" name="100m Kombi -17/18 - W" dataDxfId="186"/>
-    <tableColumn id="17" xr3:uid="{2EC953EE-367D-4524-A25E-8DE3B8168E34}" name="100m Lifesaver - 17/18 - W" dataDxfId="185"/>
-    <tableColumn id="18" xr3:uid="{25711867-9BD7-4197-9094-A21392411249}" name="200m Superlifesaver - 17/18 - W" dataDxfId="184"/>
-    <tableColumn id="19" xr3:uid="{262DB142-CFB1-45C3-9332-7273CACD1B62}" name="200m Hindernis - 17/18 - W" dataDxfId="183"/>
-    <tableColumn id="20" xr3:uid="{938BA45A-8244-4637-8A14-DF49CD91A945}" name="50m Retten - 17/18 - M" dataDxfId="182"/>
-    <tableColumn id="21" xr3:uid="{737E28D8-900F-4A98-95FE-EE7B0AFDEE90}" name="100m Retten - 17/18 - M" dataDxfId="181"/>
-    <tableColumn id="22" xr3:uid="{330BD3A8-061C-45E2-ADDB-40C2F346772F}" name="100m Kombi - 17/18 - M" dataDxfId="180"/>
-    <tableColumn id="23" xr3:uid="{0CADDE90-A167-4E1D-8D33-8624E5E1A4E2}" name="100m Lifesaver - 17/18 - M" dataDxfId="179"/>
-    <tableColumn id="24" xr3:uid="{FCF9F42C-1291-4985-9D37-B9DE2DAA5DCB}" name="200m Superlifesaver - 17/18 - M" dataDxfId="178"/>
-    <tableColumn id="25" xr3:uid="{4E5397B2-F924-4F48-AE69-AF6D650AF88D}" name="200m Hindernis - 17/18 - M" dataDxfId="177"/>
-    <tableColumn id="26" xr3:uid="{0A78315A-BFDC-43EE-A66F-48B301F66508}" name="50m Retten - 15/16 - W" dataDxfId="176"/>
-    <tableColumn id="27" xr3:uid="{D3FCF8BD-6C76-450D-80C0-CC0519A79731}" name="100m Retten - 15/16 - W" dataDxfId="175"/>
-    <tableColumn id="28" xr3:uid="{6BE7937E-D62D-47CD-95DE-1730304B0DF3}" name="100m Kombi - 15/16 - W" dataDxfId="174"/>
-    <tableColumn id="29" xr3:uid="{098BA5BE-5AF6-4187-89B6-534498F24C51}" name="100m Lifesaver -  15/16 - W" dataDxfId="173"/>
-    <tableColumn id="30" xr3:uid="{2A6822CF-143C-4BF7-A440-5777527BE512}" name="200m Superlifesaver -  15/16 - W" dataDxfId="172"/>
-    <tableColumn id="31" xr3:uid="{541C7145-CDEA-4E4E-9E7A-A4F05BA6C3E5}" name="200m Hindernis -  15/16 - W" dataDxfId="171"/>
-    <tableColumn id="32" xr3:uid="{342C4488-8C61-42E6-87A9-C75BD8EB7452}" name="50m Retten - 15/16 - M" dataDxfId="170"/>
-    <tableColumn id="33" xr3:uid="{857B1D46-7D20-47F7-AB9B-732D50346E32}" name="100m Retten - 15/16 - M" dataDxfId="169"/>
-    <tableColumn id="34" xr3:uid="{4C8A2EB4-804B-45F1-A768-9A6958957F8B}" name="100m Kombi -15/16 - M" dataDxfId="168"/>
-    <tableColumn id="35" xr3:uid="{26C75B4F-21EC-4EB0-A9A9-54BC80140672}" name="100m Lifesaver - 15/16 - M" dataDxfId="167"/>
-    <tableColumn id="36" xr3:uid="{DBBB2A23-1A06-429A-A5D1-A547EF5EC16F}" name="200m Superlifesaver - 15/16 - M" dataDxfId="166"/>
-    <tableColumn id="37" xr3:uid="{84061231-CAE5-427A-87F5-6DDBA99F77D2}" name="200m Hindernis - 15/16 - M" dataDxfId="165"/>
-    <tableColumn id="38" xr3:uid="{878CCA80-A742-4B3C-90C9-E93BB814201B}" name="50m Retten - 13/14 - W" dataDxfId="164"/>
-    <tableColumn id="39" xr3:uid="{A1F57102-61CF-4784-8DE2-0B8F32D5D699}" name="50m Retten mit Flossen - 13/14 - W" dataDxfId="163"/>
-    <tableColumn id="40" xr3:uid="{0F6BAF78-3D79-42A9-9FED-E6D0E335A920}" name="100m Hindernis - 13/14 - W" dataDxfId="162"/>
-    <tableColumn id="41" xr3:uid="{EB748A68-E10D-4D76-B315-8FDB3AC33C8D}" name="50m Retten - 13/14 - M" dataDxfId="161"/>
-    <tableColumn id="42" xr3:uid="{C7B04167-6430-40F0-9A0F-D0D0BE2F9C77}" name="50m Retten mit Flossen - 13/14 - M" dataDxfId="160"/>
-    <tableColumn id="43" xr3:uid="{48704BB7-A853-445A-8CDC-8D8F86C2B66A}" name="100m Hindernis - 13/14 - M" dataDxfId="159"/>
-    <tableColumn id="44" xr3:uid="{9605FE9A-F41C-4A5F-A59C-B7A9D45C460F}" name="50m Flossen - 12 - W" dataDxfId="158"/>
-    <tableColumn id="45" xr3:uid="{4C9DBF61-35B1-4BC2-8272-526E0AFAAFFB}" name="50m komb. Schwimmen - 12 - W" dataDxfId="157"/>
-    <tableColumn id="46" xr3:uid="{CF433C95-C272-48F9-98CD-7E3C8DBB6F2C}" name="50m Hindernis - 12 - W" dataDxfId="156"/>
-    <tableColumn id="47" xr3:uid="{FADB7411-DB43-4B14-B9E8-D74CA1BA18B8}" name="50m Flossen - 12 - M" dataDxfId="155"/>
-    <tableColumn id="48" xr3:uid="{02936F84-1D82-48AC-8D7C-6D2954D68A06}" name="50m komb. Schwimmen - 12 - M" dataDxfId="154"/>
-    <tableColumn id="49" xr3:uid="{7FD9BD11-0597-4E07-8DA5-DB53384197F5}" name="50m Hindernis - 12 - M" dataDxfId="153"/>
+    <tableColumn id="13" xr3:uid="{5A5E9873-0C5F-4508-AF6B-4974E0526D84}" name="200m Hindernis - offen - M" dataDxfId="216"/>
+    <tableColumn id="14" xr3:uid="{FA907992-7FCE-4CAD-8CF2-F5BEBC9B3756}" name="50m Retten - 17/18 - W" dataDxfId="215"/>
+    <tableColumn id="15" xr3:uid="{76B63DC0-CB67-48F4-9B5A-D22902F59334}" name="100m Retten - 17/18 - W" dataDxfId="214"/>
+    <tableColumn id="16" xr3:uid="{614A2419-51B1-44C0-8469-ADBFB078B81A}" name="100m Kombi -17/18 - W" dataDxfId="213"/>
+    <tableColumn id="17" xr3:uid="{2EC953EE-367D-4524-A25E-8DE3B8168E34}" name="100m Lifesaver - 17/18 - W" dataDxfId="212"/>
+    <tableColumn id="18" xr3:uid="{25711867-9BD7-4197-9094-A21392411249}" name="200m Superlifesaver - 17/18 - W" dataDxfId="211"/>
+    <tableColumn id="19" xr3:uid="{262DB142-CFB1-45C3-9332-7273CACD1B62}" name="200m Hindernis - 17/18 - W" dataDxfId="210"/>
+    <tableColumn id="20" xr3:uid="{938BA45A-8244-4637-8A14-DF49CD91A945}" name="50m Retten - 17/18 - M" dataDxfId="209"/>
+    <tableColumn id="21" xr3:uid="{737E28D8-900F-4A98-95FE-EE7B0AFDEE90}" name="100m Retten - 17/18 - M" dataDxfId="208"/>
+    <tableColumn id="22" xr3:uid="{330BD3A8-061C-45E2-ADDB-40C2F346772F}" name="100m Kombi - 17/18 - M" dataDxfId="207"/>
+    <tableColumn id="23" xr3:uid="{0CADDE90-A167-4E1D-8D33-8624E5E1A4E2}" name="100m Lifesaver - 17/18 - M" dataDxfId="206"/>
+    <tableColumn id="24" xr3:uid="{FCF9F42C-1291-4985-9D37-B9DE2DAA5DCB}" name="200m Superlifesaver - 17/18 - M" dataDxfId="205"/>
+    <tableColumn id="25" xr3:uid="{4E5397B2-F924-4F48-AE69-AF6D650AF88D}" name="200m Hindernis - 17/18 - M" dataDxfId="204"/>
+    <tableColumn id="26" xr3:uid="{0A78315A-BFDC-43EE-A66F-48B301F66508}" name="50m Retten - 15/16 - W" dataDxfId="203"/>
+    <tableColumn id="27" xr3:uid="{D3FCF8BD-6C76-450D-80C0-CC0519A79731}" name="100m Retten - 15/16 - W" dataDxfId="202"/>
+    <tableColumn id="28" xr3:uid="{6BE7937E-D62D-47CD-95DE-1730304B0DF3}" name="100m Kombi - 15/16 - W" dataDxfId="201"/>
+    <tableColumn id="29" xr3:uid="{098BA5BE-5AF6-4187-89B6-534498F24C51}" name="100m Lifesaver -  15/16 - W" dataDxfId="200"/>
+    <tableColumn id="30" xr3:uid="{2A6822CF-143C-4BF7-A440-5777527BE512}" name="200m Superlifesaver -  15/16 - W" dataDxfId="199"/>
+    <tableColumn id="31" xr3:uid="{541C7145-CDEA-4E4E-9E7A-A4F05BA6C3E5}" name="200m Hindernis -  15/16 - W" dataDxfId="198"/>
+    <tableColumn id="32" xr3:uid="{342C4488-8C61-42E6-87A9-C75BD8EB7452}" name="50m Retten - 15/16 - M" dataDxfId="197"/>
+    <tableColumn id="33" xr3:uid="{857B1D46-7D20-47F7-AB9B-732D50346E32}" name="100m Retten - 15/16 - M" dataDxfId="196"/>
+    <tableColumn id="34" xr3:uid="{4C8A2EB4-804B-45F1-A768-9A6958957F8B}" name="100m Kombi -15/16 - M" dataDxfId="195"/>
+    <tableColumn id="35" xr3:uid="{26C75B4F-21EC-4EB0-A9A9-54BC80140672}" name="100m Lifesaver - 15/16 - M" dataDxfId="194"/>
+    <tableColumn id="36" xr3:uid="{DBBB2A23-1A06-429A-A5D1-A547EF5EC16F}" name="200m Superlifesaver - 15/16 - M" dataDxfId="193"/>
+    <tableColumn id="37" xr3:uid="{84061231-CAE5-427A-87F5-6DDBA99F77D2}" name="200m Hindernis - 15/16 - M" dataDxfId="192"/>
+    <tableColumn id="38" xr3:uid="{878CCA80-A742-4B3C-90C9-E93BB814201B}" name="50m Retten - 13/14 - W" dataDxfId="191"/>
+    <tableColumn id="39" xr3:uid="{A1F57102-61CF-4784-8DE2-0B8F32D5D699}" name="50m Retten mit Flossen - 13/14 - W" dataDxfId="190"/>
+    <tableColumn id="40" xr3:uid="{0F6BAF78-3D79-42A9-9FED-E6D0E335A920}" name="100m Hindernis - 13/14 - W" dataDxfId="189"/>
+    <tableColumn id="41" xr3:uid="{EB748A68-E10D-4D76-B315-8FDB3AC33C8D}" name="50m Retten - 13/14 - M" dataDxfId="188"/>
+    <tableColumn id="42" xr3:uid="{C7B04167-6430-40F0-9A0F-D0D0BE2F9C77}" name="50m Retten mit Flossen - 13/14 - M" dataDxfId="187"/>
+    <tableColumn id="43" xr3:uid="{48704BB7-A853-445A-8CDC-8D8F86C2B66A}" name="100m Hindernis - 13/14 - M" dataDxfId="186"/>
+    <tableColumn id="44" xr3:uid="{9605FE9A-F41C-4A5F-A59C-B7A9D45C460F}" name="50m Flossen - 12 - W" dataDxfId="185"/>
+    <tableColumn id="45" xr3:uid="{4C9DBF61-35B1-4BC2-8272-526E0AFAAFFB}" name="50m komb. Schwimmen - 12 - W" dataDxfId="184"/>
+    <tableColumn id="46" xr3:uid="{CF433C95-C272-48F9-98CD-7E3C8DBB6F2C}" name="50m Hindernis - 12 - W" dataDxfId="183"/>
+    <tableColumn id="47" xr3:uid="{FADB7411-DB43-4B14-B9E8-D74CA1BA18B8}" name="50m Flossen - 12 - M" dataDxfId="182"/>
+    <tableColumn id="48" xr3:uid="{02936F84-1D82-48AC-8D7C-6D2954D68A06}" name="50m komb. Schwimmen - 12 - M" dataDxfId="181"/>
+    <tableColumn id="49" xr3:uid="{7FD9BD11-0597-4E07-8DA5-DB53384197F5}" name="50m Hindernis - 12 - M" dataDxfId="180"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{4234D44E-A2BE-4790-B589-1A8CC19B714E}" name="WR_Youth" displayName="WR_Youth" ref="A4:M32" totalsRowShown="0" headerRowDxfId="152" dataDxfId="150" headerRowBorderDxfId="151" tableBorderDxfId="149">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{4234D44E-A2BE-4790-B589-1A8CC19B714E}" name="WR_Youth" displayName="WR_Youth" ref="A4:M32" totalsRowShown="0" headerRowDxfId="179" dataDxfId="177" headerRowBorderDxfId="178" tableBorderDxfId="176">
   <autoFilter ref="A4:M32" xr:uid="{4234D44E-A2BE-4790-B589-1A8CC19B714E}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{848E691A-41B0-42DD-B122-FB6DF43CB3EF}" name="WR-Youth" dataDxfId="148"/>
-    <tableColumn id="2" xr3:uid="{2FE43F18-485B-46A9-8946-FBC5FDAE5A8E}" name="50m Retten" dataDxfId="147"/>
-    <tableColumn id="3" xr3:uid="{CA5C3ABF-02E6-442B-868B-95B293B231D3}" name="100m Retten" dataDxfId="146"/>
-    <tableColumn id="4" xr3:uid="{7A6BBA52-2145-464D-8C04-B2CCFC1A90DC}" name="100m Kombi" dataDxfId="145"/>
-    <tableColumn id="5" xr3:uid="{21F420C9-E788-49EE-88F6-E37963ED31CF}" name="100m Lifesaver" dataDxfId="144"/>
-    <tableColumn id="6" xr3:uid="{CB87B7CD-8A9C-4775-A4D7-4D267F43FD1A}" name="200m Superlifesaver" dataDxfId="143"/>
-    <tableColumn id="7" xr3:uid="{2DC7F290-B564-4851-85AE-D211DA701B32}" name="200m Hindernis" dataDxfId="142"/>
-    <tableColumn id="8" xr3:uid="{8112783D-8796-4D6A-8414-AC675D745697}" name="50m Retten2" dataDxfId="141"/>
-    <tableColumn id="9" xr3:uid="{4E818CD4-8725-495D-9D1D-1AFCED9181F5}" name="100m Retten2" dataDxfId="140"/>
-    <tableColumn id="10" xr3:uid="{28C05A91-E302-40A9-B50A-ECF997F129FC}" name="100m Kombi2" dataDxfId="139"/>
-    <tableColumn id="11" xr3:uid="{D56FB9F2-45BF-4EC9-A84C-8A5FB59F2F05}" name="100m Lifesaver2" dataDxfId="138"/>
-    <tableColumn id="12" xr3:uid="{540169C0-2A40-4794-A872-F7DF8A887BF2}" name="200m Superlifesaver2" dataDxfId="137"/>
-    <tableColumn id="13" xr3:uid="{D104CB67-B55A-4C81-87E5-0AC758DD22A4}" name="200m Hindernis2" dataDxfId="136"/>
+    <tableColumn id="1" xr3:uid="{848E691A-41B0-42DD-B122-FB6DF43CB3EF}" name="WR-Youth" dataDxfId="175"/>
+    <tableColumn id="2" xr3:uid="{2FE43F18-485B-46A9-8946-FBC5FDAE5A8E}" name="50m Retten" dataDxfId="174"/>
+    <tableColumn id="3" xr3:uid="{CA5C3ABF-02E6-442B-868B-95B293B231D3}" name="100m Retten" dataDxfId="173"/>
+    <tableColumn id="4" xr3:uid="{7A6BBA52-2145-464D-8C04-B2CCFC1A90DC}" name="100m Kombi" dataDxfId="172"/>
+    <tableColumn id="5" xr3:uid="{21F420C9-E788-49EE-88F6-E37963ED31CF}" name="100m Lifesaver" dataDxfId="171"/>
+    <tableColumn id="6" xr3:uid="{CB87B7CD-8A9C-4775-A4D7-4D267F43FD1A}" name="200m Superlifesaver" dataDxfId="170"/>
+    <tableColumn id="7" xr3:uid="{2DC7F290-B564-4851-85AE-D211DA701B32}" name="200m Hindernis" dataDxfId="169"/>
+    <tableColumn id="8" xr3:uid="{8112783D-8796-4D6A-8414-AC675D745697}" name="50m Retten2" dataDxfId="168"/>
+    <tableColumn id="9" xr3:uid="{4E818CD4-8725-495D-9D1D-1AFCED9181F5}" name="100m Retten2" dataDxfId="167"/>
+    <tableColumn id="10" xr3:uid="{28C05A91-E302-40A9-B50A-ECF997F129FC}" name="100m Kombi2" dataDxfId="166"/>
+    <tableColumn id="11" xr3:uid="{D56FB9F2-45BF-4EC9-A84C-8A5FB59F2F05}" name="100m Lifesaver2" dataDxfId="165"/>
+    <tableColumn id="12" xr3:uid="{540169C0-2A40-4794-A872-F7DF8A887BF2}" name="200m Superlifesaver2" dataDxfId="164"/>
+    <tableColumn id="13" xr3:uid="{D104CB67-B55A-4C81-87E5-0AC758DD22A4}" name="200m Hindernis2" dataDxfId="163"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E2D2F97B-7645-4066-8AB3-F35CF6E035EB}" name="WR_Open" displayName="WR_Open" ref="A4:M32" totalsRowShown="0" headerRowDxfId="135" headerRowBorderDxfId="134" tableBorderDxfId="133">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E2D2F97B-7645-4066-8AB3-F35CF6E035EB}" name="WR_Open" displayName="WR_Open" ref="A4:M32" totalsRowShown="0" headerRowDxfId="162" headerRowBorderDxfId="161" tableBorderDxfId="160">
   <autoFilter ref="A4:M32" xr:uid="{E2D2F97B-7645-4066-8AB3-F35CF6E035EB}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{AE73402B-B27E-4B29-8DCF-30B7FC1855EF}" name="WR-Open" dataDxfId="132">
+    <tableColumn id="1" xr3:uid="{AE73402B-B27E-4B29-8DCF-30B7FC1855EF}" name="WR-Open" dataDxfId="159">
       <calculatedColumnFormula>A4+1</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{EA3EAC1F-184E-4A28-B3E3-08DE12F138EF}" name="50m Retten" dataDxfId="131"/>
-    <tableColumn id="3" xr3:uid="{E0305A3F-6087-4F8C-8B64-153E1ACAA32E}" name="100m Retten" dataDxfId="130"/>
-    <tableColumn id="4" xr3:uid="{F0B7AC37-315E-49AA-855C-7955D2B43A76}" name="100m Kombi" dataDxfId="129"/>
-    <tableColumn id="5" xr3:uid="{B5E690AB-DB7D-4864-8916-89D2A68C4128}" name="100m Lifesaver" dataDxfId="128"/>
-    <tableColumn id="6" xr3:uid="{D89BAF4D-36AE-4C73-9320-9C5736F02F8A}" name="200m Superlifesaver" dataDxfId="127"/>
-    <tableColumn id="7" xr3:uid="{58AE7517-1A90-459F-A7D2-B95265D217E7}" name="200m Hindernis" dataDxfId="126"/>
-    <tableColumn id="8" xr3:uid="{13A189FB-E897-4A1F-A001-525F61E9CFFF}" name="50m Retten2" dataDxfId="125"/>
-    <tableColumn id="9" xr3:uid="{36418AC5-46B8-400F-BD2E-D329CF4F92CD}" name="100m Retten2" dataDxfId="124"/>
+    <tableColumn id="2" xr3:uid="{EA3EAC1F-184E-4A28-B3E3-08DE12F138EF}" name="50m Retten" dataDxfId="158"/>
+    <tableColumn id="3" xr3:uid="{E0305A3F-6087-4F8C-8B64-153E1ACAA32E}" name="100m Retten" dataDxfId="157"/>
+    <tableColumn id="4" xr3:uid="{F0B7AC37-315E-49AA-855C-7955D2B43A76}" name="100m Kombi" dataDxfId="156"/>
+    <tableColumn id="5" xr3:uid="{B5E690AB-DB7D-4864-8916-89D2A68C4128}" name="100m Lifesaver" dataDxfId="155"/>
+    <tableColumn id="6" xr3:uid="{D89BAF4D-36AE-4C73-9320-9C5736F02F8A}" name="200m Superlifesaver" dataDxfId="154"/>
+    <tableColumn id="7" xr3:uid="{58AE7517-1A90-459F-A7D2-B95265D217E7}" name="200m Hindernis" dataDxfId="153"/>
+    <tableColumn id="8" xr3:uid="{13A189FB-E897-4A1F-A001-525F61E9CFFF}" name="50m Retten2" dataDxfId="152"/>
+    <tableColumn id="9" xr3:uid="{36418AC5-46B8-400F-BD2E-D329CF4F92CD}" name="100m Retten2" dataDxfId="151"/>
     <tableColumn id="10" xr3:uid="{06A35C2D-7313-472B-BC1F-4F2FB1D14782}" name="100m Kombi2"/>
     <tableColumn id="11" xr3:uid="{89966D0D-9131-4245-A7BE-1A7384D5ADA0}" name="100m Lifesaver2"/>
     <tableColumn id="12" xr3:uid="{D9D6CF56-869C-4DDE-9886-572D4E523A8F}" name="200m Superlifesaver2"/>
@@ -4354,7 +4360,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{CF3D303A-A04B-42DD-A44E-CEB6CECB77A4}" name="DP_konfig" displayName="DP_konfig" ref="A1:U3" totalsRowShown="0" headerRowDxfId="123" dataDxfId="122">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{CF3D303A-A04B-42DD-A44E-CEB6CECB77A4}" name="DP_konfig" displayName="DP_konfig" ref="A1:U3" totalsRowShown="0" headerRowDxfId="150" dataDxfId="149">
   <autoFilter ref="A1:U3" xr:uid="{CF3D303A-A04B-42DD-A44E-CEB6CECB77A4}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -4379,64 +4385,64 @@
     <filterColumn colId="20" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="21">
-    <tableColumn id="1" xr3:uid="{58D628F0-061E-4A82-8362-CDB37A2E7C60}" name="Tabellen Name" dataDxfId="121"/>
-    <tableColumn id="2" xr3:uid="{2F302F6C-F8AF-4FDE-AB08-6F30F9671015}" name="Geschlecht" dataDxfId="120"/>
-    <tableColumn id="3" xr3:uid="{4D91FBF9-386D-43DD-90D0-B49823FDB629}" name="Mindest alter" dataDxfId="119"/>
-    <tableColumn id="4" xr3:uid="{4126AAC6-AF2F-446C-B4EA-D86ACFD9FAC2}" name="Maximales Alter" dataDxfId="118"/>
-    <tableColumn id="5" xr3:uid="{8A10890A-A299-4B09-AC72-0E9AE9238AF3}" name="Qualizeitraum anfang" dataDxfId="117"/>
-    <tableColumn id="6" xr3:uid="{FBCD1C13-FC82-429B-8DE1-0C5A455FDAB8}" name="Qualizeitraum Ende" dataDxfId="116"/>
-    <tableColumn id="7" xr3:uid="{1DCCAC9B-BC46-468E-A3CE-57576C2FF11D}" name="Letzter Wettkampf am" dataDxfId="115"/>
-    <tableColumn id="8" xr3:uid="{9A6E47EE-ABD8-4A1E-87D3-9D286E4C124F}" name="Wertung" dataDxfId="114"/>
-    <tableColumn id="9" xr3:uid="{09E848D2-ED17-49C7-9775-CBF17D20DFC0}" name="Landesverband" dataDxfId="113"/>
-    <tableColumn id="10" xr3:uid="{70ABB713-23F6-4FCF-920E-3CB0CD451446}" name="OMS" dataDxfId="112"/>
-    <tableColumn id="11" xr3:uid="{9C108A1C-E6AB-4C13-9C1D-0FA8944A39A3}" name="Pool-Länge" dataDxfId="111"/>
-    <tableColumn id="12" xr3:uid="{087948DD-430D-48F1-906D-4F4EF4B46053}" name="Regelwerk" dataDxfId="110"/>
-    <tableColumn id="13" xr3:uid="{BF42D9C0-F77D-4971-A67E-32B0246C72C3}" name="Referenz" dataDxfId="109"/>
-    <tableColumn id="19" xr3:uid="{AFFB84E8-B398-4E99-805B-9A247071A040}" name="Referenz Jahr" dataDxfId="108"/>
-    <tableColumn id="20" xr3:uid="{0A59A474-DFBB-4437-8EFF-70284AFD9934}" name="Mindest Punktzahl" dataDxfId="107"/>
-    <tableColumn id="21" xr3:uid="{198BD231-EEF3-43C9-AD9B-39B4B7E9B337}" name="Mindest Disziplinen" dataDxfId="106"/>
-    <tableColumn id="14" xr3:uid="{443CD4F6-A2B2-480B-BB35-DCEEBC531727}" name="3-Kampf Regel" dataDxfId="105"/>
-    <tableColumn id="15" xr3:uid="{70116160-7666-42B1-92AC-FAC2620E6A60}" name="Anzahl Nominierte" dataDxfId="104"/>
-    <tableColumn id="16" xr3:uid="{0EFD0A46-D12B-4AB0-907C-08E5D9F282E0}" name="Anzahl Nachrücker" dataDxfId="103"/>
-    <tableColumn id="17" xr3:uid="{AA5430A0-8ED8-40E8-B7F8-DA25E4E8790F}" name="Seiten Anzahl" dataDxfId="102"/>
-    <tableColumn id="18" xr3:uid="{16F699D9-2741-43F3-AD5F-826A568EFEAC}" name="Absagen" dataDxfId="101"/>
+    <tableColumn id="1" xr3:uid="{58D628F0-061E-4A82-8362-CDB37A2E7C60}" name="Tabellen Name" dataDxfId="148"/>
+    <tableColumn id="2" xr3:uid="{2F302F6C-F8AF-4FDE-AB08-6F30F9671015}" name="Geschlecht" dataDxfId="147"/>
+    <tableColumn id="3" xr3:uid="{4D91FBF9-386D-43DD-90D0-B49823FDB629}" name="Mindest alter" dataDxfId="146"/>
+    <tableColumn id="4" xr3:uid="{4126AAC6-AF2F-446C-B4EA-D86ACFD9FAC2}" name="Maximales Alter" dataDxfId="145"/>
+    <tableColumn id="5" xr3:uid="{8A10890A-A299-4B09-AC72-0E9AE9238AF3}" name="Qualizeitraum anfang" dataDxfId="144"/>
+    <tableColumn id="6" xr3:uid="{FBCD1C13-FC82-429B-8DE1-0C5A455FDAB8}" name="Qualizeitraum Ende" dataDxfId="143"/>
+    <tableColumn id="7" xr3:uid="{1DCCAC9B-BC46-468E-A3CE-57576C2FF11D}" name="Letzter Wettkampf am" dataDxfId="142"/>
+    <tableColumn id="8" xr3:uid="{9A6E47EE-ABD8-4A1E-87D3-9D286E4C124F}" name="Wertung" dataDxfId="141"/>
+    <tableColumn id="9" xr3:uid="{09E848D2-ED17-49C7-9775-CBF17D20DFC0}" name="Landesverband" dataDxfId="140"/>
+    <tableColumn id="10" xr3:uid="{70ABB713-23F6-4FCF-920E-3CB0CD451446}" name="OMS" dataDxfId="139"/>
+    <tableColumn id="11" xr3:uid="{9C108A1C-E6AB-4C13-9C1D-0FA8944A39A3}" name="Pool-Länge" dataDxfId="138"/>
+    <tableColumn id="12" xr3:uid="{087948DD-430D-48F1-906D-4F4EF4B46053}" name="Regelwerk" dataDxfId="137"/>
+    <tableColumn id="13" xr3:uid="{BF42D9C0-F77D-4971-A67E-32B0246C72C3}" name="Referenz" dataDxfId="136"/>
+    <tableColumn id="19" xr3:uid="{AFFB84E8-B398-4E99-805B-9A247071A040}" name="Referenz Jahr" dataDxfId="135"/>
+    <tableColumn id="20" xr3:uid="{0A59A474-DFBB-4437-8EFF-70284AFD9934}" name="Mindest Punktzahl" dataDxfId="134"/>
+    <tableColumn id="21" xr3:uid="{198BD231-EEF3-43C9-AD9B-39B4B7E9B337}" name="Mindest Disziplinen" dataDxfId="133"/>
+    <tableColumn id="14" xr3:uid="{443CD4F6-A2B2-480B-BB35-DCEEBC531727}" name="3-Kampf Regel" dataDxfId="132"/>
+    <tableColumn id="15" xr3:uid="{70116160-7666-42B1-92AC-FAC2620E6A60}" name="Anzahl Nominierte" dataDxfId="131"/>
+    <tableColumn id="16" xr3:uid="{0EFD0A46-D12B-4AB0-907C-08E5D9F282E0}" name="Anzahl Nachrücker" dataDxfId="130"/>
+    <tableColumn id="17" xr3:uid="{AA5430A0-8ED8-40E8-B7F8-DA25E4E8790F}" name="Seiten Anzahl" dataDxfId="129"/>
+    <tableColumn id="18" xr3:uid="{16F699D9-2741-43F3-AD5F-826A568EFEAC}" name="Absagen" dataDxfId="128"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{CDBF6724-48A1-41AB-94B5-CC35C54BB15C}" name="BP_konfig" displayName="BP_konfig" ref="A1:U7" totalsRowShown="0" headerRowDxfId="100" dataDxfId="99">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{CDBF6724-48A1-41AB-94B5-CC35C54BB15C}" name="BP_konfig" displayName="BP_konfig" ref="A1:U7" totalsRowShown="0" headerRowDxfId="127" dataDxfId="126">
   <autoFilter ref="A1:U7" xr:uid="{CDBF6724-48A1-41AB-94B5-CC35C54BB15C}"/>
   <tableColumns count="21">
-    <tableColumn id="1" xr3:uid="{E1FB3D0C-B874-4874-BACC-6872CF171957}" name="Tabellen Name" dataDxfId="98"/>
-    <tableColumn id="2" xr3:uid="{FFDD2777-2097-450C-B020-F133CF643855}" name="Geschlecht" dataDxfId="97"/>
-    <tableColumn id="3" xr3:uid="{8CF52BE2-8020-48BD-A36D-63F13A1878DE}" name="Mindest alter" dataDxfId="96"/>
-    <tableColumn id="4" xr3:uid="{FD3A030F-CD97-4B6F-8E8C-BC2E67D79F1D}" name="Maximales Alter" dataDxfId="95"/>
-    <tableColumn id="5" xr3:uid="{3E22B645-D77C-4509-B031-9914FCB91599}" name="Qualizeitraum anfang" dataDxfId="94"/>
-    <tableColumn id="6" xr3:uid="{AE299324-3C1C-4063-ADF9-54555A161734}" name="Qualizeitraum Ende" dataDxfId="93"/>
-    <tableColumn id="7" xr3:uid="{DCC178B3-11FC-4C53-BBC6-C2FDA2C89857}" name="Letzter Wettkampf am" dataDxfId="92"/>
-    <tableColumn id="8" xr3:uid="{2811DB01-60A5-4BE4-B6F9-A806398A602A}" name="Wertung" dataDxfId="91"/>
-    <tableColumn id="9" xr3:uid="{0C16DAFE-847D-4E9E-9604-3A7D9FE924D0}" name="Landesverband" dataDxfId="90"/>
-    <tableColumn id="10" xr3:uid="{7A8A4101-A553-4BD5-9116-9AA5876B9401}" name="OMS" dataDxfId="89"/>
-    <tableColumn id="11" xr3:uid="{9807C9BD-6499-45F6-ACE0-4D13D64EF675}" name="Pool-Länge" dataDxfId="88"/>
-    <tableColumn id="12" xr3:uid="{13D336DD-650F-4F2C-836F-361CA1528F6D}" name="Regelwerk" dataDxfId="87"/>
-    <tableColumn id="13" xr3:uid="{66660E2D-ADF2-4FB5-8A13-004F826EE908}" name="Referenz" dataDxfId="86"/>
-    <tableColumn id="19" xr3:uid="{D72EDF8B-ECC3-4FF7-ABE6-B60BCE4A5E26}" name="Referenz Jahr" dataDxfId="85"/>
-    <tableColumn id="20" xr3:uid="{7B18E667-70F7-4BC1-AB1B-21C019F2AA89}" name="Mindest Punktzahl" dataDxfId="84"/>
-    <tableColumn id="21" xr3:uid="{FC185946-681B-42A6-AB1A-FC1EABB668C5}" name="Mindest Disziplinen" dataDxfId="83"/>
-    <tableColumn id="14" xr3:uid="{6A2676FD-2EC7-4C41-A35E-A1597A38F932}" name="3-Kampf Regel" dataDxfId="82"/>
-    <tableColumn id="15" xr3:uid="{718E0917-4F83-4A2B-832F-EBB16D5E21BF}" name="Anzahl Nominierte" dataDxfId="81"/>
-    <tableColumn id="16" xr3:uid="{5C66A461-D647-4E00-A81C-FD7AD44D7CC2}" name="Anzahl Nachrücker" dataDxfId="80"/>
-    <tableColumn id="17" xr3:uid="{D434BDEC-293B-4B4E-A5E9-479438960A03}" name="Seiten Anzahl" dataDxfId="79"/>
-    <tableColumn id="18" xr3:uid="{80908229-9247-473F-81C0-9C9D4C12FF06}" name="Absagen" dataDxfId="78"/>
+    <tableColumn id="1" xr3:uid="{E1FB3D0C-B874-4874-BACC-6872CF171957}" name="Tabellen Name" dataDxfId="125"/>
+    <tableColumn id="2" xr3:uid="{FFDD2777-2097-450C-B020-F133CF643855}" name="Geschlecht" dataDxfId="124"/>
+    <tableColumn id="3" xr3:uid="{8CF52BE2-8020-48BD-A36D-63F13A1878DE}" name="Mindest alter" dataDxfId="123"/>
+    <tableColumn id="4" xr3:uid="{FD3A030F-CD97-4B6F-8E8C-BC2E67D79F1D}" name="Maximales Alter" dataDxfId="122"/>
+    <tableColumn id="5" xr3:uid="{3E22B645-D77C-4509-B031-9914FCB91599}" name="Qualizeitraum anfang" dataDxfId="121"/>
+    <tableColumn id="6" xr3:uid="{AE299324-3C1C-4063-ADF9-54555A161734}" name="Qualizeitraum Ende" dataDxfId="120"/>
+    <tableColumn id="7" xr3:uid="{DCC178B3-11FC-4C53-BBC6-C2FDA2C89857}" name="Letzter Wettkampf am" dataDxfId="119"/>
+    <tableColumn id="8" xr3:uid="{2811DB01-60A5-4BE4-B6F9-A806398A602A}" name="Wertung" dataDxfId="118"/>
+    <tableColumn id="9" xr3:uid="{0C16DAFE-847D-4E9E-9604-3A7D9FE924D0}" name="Landesverband" dataDxfId="117"/>
+    <tableColumn id="10" xr3:uid="{7A8A4101-A553-4BD5-9116-9AA5876B9401}" name="OMS" dataDxfId="116"/>
+    <tableColumn id="11" xr3:uid="{9807C9BD-6499-45F6-ACE0-4D13D64EF675}" name="Pool-Länge" dataDxfId="115"/>
+    <tableColumn id="12" xr3:uid="{13D336DD-650F-4F2C-836F-361CA1528F6D}" name="Regelwerk" dataDxfId="114"/>
+    <tableColumn id="13" xr3:uid="{66660E2D-ADF2-4FB5-8A13-004F826EE908}" name="Referenz" dataDxfId="113"/>
+    <tableColumn id="19" xr3:uid="{D72EDF8B-ECC3-4FF7-ABE6-B60BCE4A5E26}" name="Referenz Jahr" dataDxfId="112"/>
+    <tableColumn id="20" xr3:uid="{7B18E667-70F7-4BC1-AB1B-21C019F2AA89}" name="Mindest Punktzahl" dataDxfId="111"/>
+    <tableColumn id="21" xr3:uid="{FC185946-681B-42A6-AB1A-FC1EABB668C5}" name="Mindest Disziplinen" dataDxfId="110"/>
+    <tableColumn id="14" xr3:uid="{6A2676FD-2EC7-4C41-A35E-A1597A38F932}" name="3-Kampf Regel" dataDxfId="109"/>
+    <tableColumn id="15" xr3:uid="{718E0917-4F83-4A2B-832F-EBB16D5E21BF}" name="Anzahl Nominierte" dataDxfId="108"/>
+    <tableColumn id="16" xr3:uid="{5C66A461-D647-4E00-A81C-FD7AD44D7CC2}" name="Anzahl Nachrücker" dataDxfId="107"/>
+    <tableColumn id="17" xr3:uid="{D434BDEC-293B-4B4E-A5E9-479438960A03}" name="Seiten Anzahl" dataDxfId="106"/>
+    <tableColumn id="18" xr3:uid="{80908229-9247-473F-81C0-9C9D4C12FF06}" name="Absagen" dataDxfId="105"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{16F87202-5A6A-4E2F-B973-3CE7EC2566C1}" name="DEM_konfig" displayName="DEM_konfig" ref="A1:X7" totalsRowShown="0" headerRowDxfId="77" dataDxfId="76">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{16F87202-5A6A-4E2F-B973-3CE7EC2566C1}" name="DEM_konfig" displayName="DEM_konfig" ref="A1:X7" totalsRowShown="0" headerRowDxfId="104" dataDxfId="103">
   <autoFilter ref="A1:X7" xr:uid="{16F87202-5A6A-4E2F-B973-3CE7EC2566C1}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -4464,37 +4470,37 @@
     <filterColumn colId="23" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="24">
-    <tableColumn id="1" xr3:uid="{4847B567-64E1-4AC3-8C4B-EFCF3F00CC6C}" name="Tabellen Name" dataDxfId="75"/>
-    <tableColumn id="2" xr3:uid="{6346FF3B-B334-4CD8-8B23-F2347E29C536}" name="Geschlecht" dataDxfId="74"/>
-    <tableColumn id="3" xr3:uid="{E793B48A-BC8A-439F-8AAF-6FD08104A619}" name="Mindest Alter" dataDxfId="73"/>
-    <tableColumn id="4" xr3:uid="{01A62C29-2F75-4107-A431-F69230BCCD0C}" name="Maximales Alter" dataDxfId="72"/>
-    <tableColumn id="5" xr3:uid="{B7E4DE90-7856-4A0C-9063-61414D7F227C}" name="Qualizeitraum anfang" dataDxfId="71"/>
-    <tableColumn id="6" xr3:uid="{B00F7CD1-82CB-42B9-A396-89F79EF419CA}" name="Qualizeitraum Ende" dataDxfId="70"/>
-    <tableColumn id="7" xr3:uid="{9E50DDE5-12E3-4BCB-801C-FBABCE309F0E}" name="Letzter Wettkampf am" dataDxfId="69"/>
-    <tableColumn id="8" xr3:uid="{57E68247-0FF2-48D8-8ACD-AB057E576A21}" name="Landesverband" dataDxfId="68"/>
-    <tableColumn id="9" xr3:uid="{EBAA439D-F69A-4C2A-8193-9AE08F1E57B8}" name="OMS" dataDxfId="67"/>
-    <tableColumn id="10" xr3:uid="{BBD11E7F-3DDF-428A-B005-4A40E6FA78DC}" name="Pool-Länge" dataDxfId="66"/>
-    <tableColumn id="11" xr3:uid="{6AE38DCA-A084-4F3D-A6A4-4E76E3E2CBC6}" name="Regelwerk" dataDxfId="65"/>
-    <tableColumn id="12" xr3:uid="{7F7470AD-5502-4CEE-BB4C-44BA308E61D7}" name="Seiten Anzahl" dataDxfId="64"/>
-    <tableColumn id="13" xr3:uid="{F416CBFA-4C9D-45CD-9BA7-E4BC57A08BC2}" name="PZ1 - 50m Retten" dataDxfId="63"/>
-    <tableColumn id="14" xr3:uid="{7117DBCA-0DA7-462C-84FE-0DC7E33B124C}" name="PZ1 - 100m Retten" dataDxfId="62"/>
-    <tableColumn id="15" xr3:uid="{E8630E91-DC30-4822-9E53-6D65487C3670}" name="PZ1 - 100m Kombi" dataDxfId="61"/>
-    <tableColumn id="16" xr3:uid="{4B3AA225-E042-430F-8259-D176887B4528}" name="PZ1 - 100m Lifesaver" dataDxfId="60"/>
-    <tableColumn id="17" xr3:uid="{798674BD-98CE-4531-BDFF-6AB06253AD7C}" name="PZ1 - 200m Super-Lifesaver" dataDxfId="59"/>
-    <tableColumn id="18" xr3:uid="{8809BB71-D58B-4E8B-A442-D0EB9A65A25D}" name="PZ1 - 200m Hindernis" dataDxfId="58"/>
-    <tableColumn id="19" xr3:uid="{93DCF463-806B-4117-B4E3-1FFAE976B37C}" name="PZ2 - 50m Retten" dataDxfId="57"/>
-    <tableColumn id="20" xr3:uid="{A514C961-559E-462F-B143-BA30974C0129}" name="PZ2 - 100m Retten" dataDxfId="56"/>
-    <tableColumn id="21" xr3:uid="{F1CF6143-45FE-498D-93D6-36F26D2F3C0B}" name="PZ2 - 100m Kombi" dataDxfId="55"/>
-    <tableColumn id="22" xr3:uid="{E90962FC-C214-467F-841F-40DF60E41456}" name="PZ2 - 100m Lifesaver" dataDxfId="54"/>
-    <tableColumn id="23" xr3:uid="{7FBC6334-C4C8-4B38-9F59-30ED95A44379}" name="PZ2 - 200m Super-Lifesaver" dataDxfId="53"/>
-    <tableColumn id="24" xr3:uid="{231BFF86-8F3A-4BA1-B25E-28175D9EDFA9}" name="PZ2 - 200m Hindernis" dataDxfId="52"/>
+    <tableColumn id="1" xr3:uid="{4847B567-64E1-4AC3-8C4B-EFCF3F00CC6C}" name="Tabellen Name" dataDxfId="102"/>
+    <tableColumn id="2" xr3:uid="{6346FF3B-B334-4CD8-8B23-F2347E29C536}" name="Geschlecht" dataDxfId="101"/>
+    <tableColumn id="3" xr3:uid="{E793B48A-BC8A-439F-8AAF-6FD08104A619}" name="Mindest Alter" dataDxfId="100"/>
+    <tableColumn id="4" xr3:uid="{01A62C29-2F75-4107-A431-F69230BCCD0C}" name="Maximales Alter" dataDxfId="99"/>
+    <tableColumn id="5" xr3:uid="{B7E4DE90-7856-4A0C-9063-61414D7F227C}" name="Qualizeitraum anfang" dataDxfId="98"/>
+    <tableColumn id="6" xr3:uid="{B00F7CD1-82CB-42B9-A396-89F79EF419CA}" name="Qualizeitraum Ende" dataDxfId="97"/>
+    <tableColumn id="7" xr3:uid="{9E50DDE5-12E3-4BCB-801C-FBABCE309F0E}" name="Letzter Wettkampf am" dataDxfId="96"/>
+    <tableColumn id="8" xr3:uid="{57E68247-0FF2-48D8-8ACD-AB057E576A21}" name="Landesverband" dataDxfId="95"/>
+    <tableColumn id="9" xr3:uid="{EBAA439D-F69A-4C2A-8193-9AE08F1E57B8}" name="OMS" dataDxfId="94"/>
+    <tableColumn id="10" xr3:uid="{BBD11E7F-3DDF-428A-B005-4A40E6FA78DC}" name="Pool-Länge" dataDxfId="93"/>
+    <tableColumn id="11" xr3:uid="{6AE38DCA-A084-4F3D-A6A4-4E76E3E2CBC6}" name="Regelwerk" dataDxfId="92"/>
+    <tableColumn id="12" xr3:uid="{7F7470AD-5502-4CEE-BB4C-44BA308E61D7}" name="Seiten Anzahl" dataDxfId="91"/>
+    <tableColumn id="13" xr3:uid="{F416CBFA-4C9D-45CD-9BA7-E4BC57A08BC2}" name="PZ1 - 50m Retten" dataDxfId="90"/>
+    <tableColumn id="14" xr3:uid="{7117DBCA-0DA7-462C-84FE-0DC7E33B124C}" name="PZ1 - 100m Retten" dataDxfId="89"/>
+    <tableColumn id="15" xr3:uid="{E8630E91-DC30-4822-9E53-6D65487C3670}" name="PZ1 - 100m Kombi" dataDxfId="88"/>
+    <tableColumn id="16" xr3:uid="{4B3AA225-E042-430F-8259-D176887B4528}" name="PZ1 - 100m Lifesaver" dataDxfId="87"/>
+    <tableColumn id="17" xr3:uid="{798674BD-98CE-4531-BDFF-6AB06253AD7C}" name="PZ1 - 200m Super-Lifesaver" dataDxfId="86"/>
+    <tableColumn id="18" xr3:uid="{8809BB71-D58B-4E8B-A442-D0EB9A65A25D}" name="PZ1 - 200m Hindernis" dataDxfId="85"/>
+    <tableColumn id="19" xr3:uid="{93DCF463-806B-4117-B4E3-1FFAE976B37C}" name="PZ2 - 50m Retten" dataDxfId="84"/>
+    <tableColumn id="20" xr3:uid="{A514C961-559E-462F-B143-BA30974C0129}" name="PZ2 - 100m Retten" dataDxfId="83"/>
+    <tableColumn id="21" xr3:uid="{F1CF6143-45FE-498D-93D6-36F26D2F3C0B}" name="PZ2 - 100m Kombi" dataDxfId="82"/>
+    <tableColumn id="22" xr3:uid="{E90962FC-C214-467F-841F-40DF60E41456}" name="PZ2 - 100m Lifesaver" dataDxfId="81"/>
+    <tableColumn id="23" xr3:uid="{7FBC6334-C4C8-4B38-9F59-30ED95A44379}" name="PZ2 - 200m Super-Lifesaver" dataDxfId="80"/>
+    <tableColumn id="24" xr3:uid="{231BFF86-8F3A-4BA1-B25E-28175D9EDFA9}" name="PZ2 - 200m Hindernis" dataDxfId="79"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D7CDEF11-F813-469D-9DE0-678961AB7005}" name="JRP_konfig" displayName="JRP_konfig" ref="A1:X3" totalsRowShown="0" headerRowDxfId="51" dataDxfId="50">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D7CDEF11-F813-469D-9DE0-678961AB7005}" name="JRP_konfig" displayName="JRP_konfig" ref="A1:X3" totalsRowShown="0" headerRowDxfId="78" dataDxfId="77">
   <autoFilter ref="A1:X3" xr:uid="{D7CDEF11-F813-469D-9DE0-678961AB7005}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -4522,63 +4528,64 @@
     <filterColumn colId="23" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="24">
-    <tableColumn id="1" xr3:uid="{021DA6E1-2C93-4474-9720-B6F016186D61}" name="Tabellen Name" dataDxfId="49"/>
-    <tableColumn id="2" xr3:uid="{733C1722-A9C9-4830-A9E2-FE62E96BCD98}" name="Geschlecht" dataDxfId="48"/>
-    <tableColumn id="3" xr3:uid="{80C0BF46-0E43-4947-BF86-B808C324772A}" name="Mindest Alter" dataDxfId="47"/>
-    <tableColumn id="4" xr3:uid="{DBA2A923-EEB7-43F9-A1A3-E78624448FB9}" name="Maximales Alter" dataDxfId="46"/>
-    <tableColumn id="5" xr3:uid="{3FDEE18A-328D-45AE-907D-69A916A93345}" name="Qualizeitraum anfang" dataDxfId="45"/>
-    <tableColumn id="6" xr3:uid="{BE002D7F-575F-4B60-9251-C71D93F59045}" name="Qualizeitraum Ende" dataDxfId="44"/>
-    <tableColumn id="7" xr3:uid="{208ABD57-DE4B-41D6-B9FC-93F2D8966E8D}" name="Letzter Wettkampf am" dataDxfId="43"/>
-    <tableColumn id="8" xr3:uid="{30C9697C-6550-4996-ADDB-7FEE5325B794}" name="Landesverband" dataDxfId="42"/>
-    <tableColumn id="9" xr3:uid="{ED2DAB77-EF46-4D8B-B8E4-90412E32E277}" name="OMS" dataDxfId="41"/>
-    <tableColumn id="10" xr3:uid="{AD534940-A91B-4A6E-9606-E3F3E517D401}" name="Pool-Länge" dataDxfId="40"/>
-    <tableColumn id="11" xr3:uid="{11F9D5D5-72FE-42CA-8624-01D513B4140F}" name="Regelwerk" dataDxfId="39"/>
-    <tableColumn id="12" xr3:uid="{3907872B-5438-4FBF-A045-3EF9EAACFC47}" name="Seiten Anzahl" dataDxfId="38"/>
-    <tableColumn id="13" xr3:uid="{FC821324-3638-40C0-BA1E-069B44E23C7A}" name="PZ1 - 50m Retten" dataDxfId="37"/>
-    <tableColumn id="14" xr3:uid="{70529619-443E-40D3-88C1-3E0F00BB2A50}" name="PZ1 - 100m Retten" dataDxfId="36"/>
-    <tableColumn id="15" xr3:uid="{EFA92FD2-C23F-42B3-83DC-5036513F19AF}" name="PZ1 - 100m Kombi" dataDxfId="35"/>
-    <tableColumn id="16" xr3:uid="{03309E52-8CF3-4E90-9EE6-A818901C3B32}" name="PZ1 - 100m Lifesaver" dataDxfId="34"/>
-    <tableColumn id="17" xr3:uid="{00B22013-AA11-4C17-9250-22060AE4B0A8}" name="PZ1 - 200m Super-Lifesaver" dataDxfId="33"/>
-    <tableColumn id="18" xr3:uid="{7E3508A9-0422-4561-A23E-53E613259B24}" name="PZ1 - 200m Hindernis" dataDxfId="32"/>
-    <tableColumn id="19" xr3:uid="{5CEA435F-F34B-4D8D-88D0-F5EBFF18B713}" name="PZ2 - 50m Retten" dataDxfId="31"/>
-    <tableColumn id="20" xr3:uid="{8585BE62-F7C4-4D5D-B287-052B43B08610}" name="PZ2 - 100m Retten" dataDxfId="30"/>
-    <tableColumn id="21" xr3:uid="{D981758B-ADAD-4E36-B787-0B0FDA808CA2}" name="PZ2 - 100m Kombi" dataDxfId="29"/>
-    <tableColumn id="22" xr3:uid="{1D4970A8-D22F-4962-934C-AEA295ED687A}" name="PZ2 - 100m Lifesaver" dataDxfId="28"/>
-    <tableColumn id="23" xr3:uid="{BE394430-C58F-4690-9615-44475E5AF9F8}" name="PZ2 - 200m Super-Lifesaver" dataDxfId="27"/>
-    <tableColumn id="24" xr3:uid="{A7036B1A-99CE-4F7C-AAB8-12E8B2696202}" name="PZ2 - 200m Hindernis" dataDxfId="26"/>
+    <tableColumn id="1" xr3:uid="{021DA6E1-2C93-4474-9720-B6F016186D61}" name="Tabellen Name" dataDxfId="76"/>
+    <tableColumn id="2" xr3:uid="{733C1722-A9C9-4830-A9E2-FE62E96BCD98}" name="Geschlecht" dataDxfId="75"/>
+    <tableColumn id="3" xr3:uid="{80C0BF46-0E43-4947-BF86-B808C324772A}" name="Mindest Alter" dataDxfId="74"/>
+    <tableColumn id="4" xr3:uid="{DBA2A923-EEB7-43F9-A1A3-E78624448FB9}" name="Maximales Alter" dataDxfId="73"/>
+    <tableColumn id="5" xr3:uid="{3FDEE18A-328D-45AE-907D-69A916A93345}" name="Qualizeitraum anfang" dataDxfId="72"/>
+    <tableColumn id="6" xr3:uid="{BE002D7F-575F-4B60-9251-C71D93F59045}" name="Qualizeitraum Ende" dataDxfId="71"/>
+    <tableColumn id="7" xr3:uid="{208ABD57-DE4B-41D6-B9FC-93F2D8966E8D}" name="Letzter Wettkampf am" dataDxfId="70"/>
+    <tableColumn id="8" xr3:uid="{30C9697C-6550-4996-ADDB-7FEE5325B794}" name="Landesverband" dataDxfId="69"/>
+    <tableColumn id="9" xr3:uid="{ED2DAB77-EF46-4D8B-B8E4-90412E32E277}" name="OMS" dataDxfId="68"/>
+    <tableColumn id="10" xr3:uid="{AD534940-A91B-4A6E-9606-E3F3E517D401}" name="Pool-Länge" dataDxfId="67"/>
+    <tableColumn id="11" xr3:uid="{11F9D5D5-72FE-42CA-8624-01D513B4140F}" name="Regelwerk" dataDxfId="66"/>
+    <tableColumn id="12" xr3:uid="{3907872B-5438-4FBF-A045-3EF9EAACFC47}" name="Seiten Anzahl" dataDxfId="65"/>
+    <tableColumn id="13" xr3:uid="{FC821324-3638-40C0-BA1E-069B44E23C7A}" name="PZ1 - 50m Retten" dataDxfId="64"/>
+    <tableColumn id="14" xr3:uid="{70529619-443E-40D3-88C1-3E0F00BB2A50}" name="PZ1 - 100m Retten" dataDxfId="63"/>
+    <tableColumn id="15" xr3:uid="{EFA92FD2-C23F-42B3-83DC-5036513F19AF}" name="PZ1 - 100m Kombi" dataDxfId="62"/>
+    <tableColumn id="16" xr3:uid="{03309E52-8CF3-4E90-9EE6-A818901C3B32}" name="PZ1 - 100m Lifesaver" dataDxfId="61"/>
+    <tableColumn id="17" xr3:uid="{00B22013-AA11-4C17-9250-22060AE4B0A8}" name="PZ1 - 200m Super-Lifesaver" dataDxfId="60"/>
+    <tableColumn id="18" xr3:uid="{7E3508A9-0422-4561-A23E-53E613259B24}" name="PZ1 - 200m Hindernis" dataDxfId="59"/>
+    <tableColumn id="19" xr3:uid="{5CEA435F-F34B-4D8D-88D0-F5EBFF18B713}" name="PZ2 - 50m Retten" dataDxfId="58"/>
+    <tableColumn id="20" xr3:uid="{8585BE62-F7C4-4D5D-B287-052B43B08610}" name="PZ2 - 100m Retten" dataDxfId="57"/>
+    <tableColumn id="21" xr3:uid="{D981758B-ADAD-4E36-B787-0B0FDA808CA2}" name="PZ2 - 100m Kombi" dataDxfId="56"/>
+    <tableColumn id="22" xr3:uid="{1D4970A8-D22F-4962-934C-AEA295ED687A}" name="PZ2 - 100m Lifesaver" dataDxfId="55"/>
+    <tableColumn id="23" xr3:uid="{BE394430-C58F-4690-9615-44475E5AF9F8}" name="PZ2 - 200m Super-Lifesaver" dataDxfId="54"/>
+    <tableColumn id="24" xr3:uid="{A7036B1A-99CE-4F7C-AAB8-12E8B2696202}" name="PZ2 - 200m Hindernis" dataDxfId="53"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{FED162EE-531E-453F-8C25-562B59ECE709}" name="LK_konfig" displayName="LK_konfig" ref="A1:X37" totalsRowShown="0" headerRowDxfId="227" dataDxfId="226">
-  <autoFilter ref="A1:X37" xr:uid="{FED162EE-531E-453F-8C25-562B59ECE709}"/>
-  <tableColumns count="24">
-    <tableColumn id="1" xr3:uid="{F985A4F0-6B8C-47C6-816F-1A31A4973EB2}" name="Tabellen Name" dataDxfId="225"/>
-    <tableColumn id="2" xr3:uid="{5E5AD859-71A2-4E8E-B434-431A89C05C57}" name="Geschlecht" dataDxfId="224"/>
-    <tableColumn id="3" xr3:uid="{85BB892C-E151-404B-8974-FC5199E0909C}" name="Mindest Alter" dataDxfId="223"/>
-    <tableColumn id="4" xr3:uid="{790F6CF9-E475-4082-AE03-D30EDE22FB61}" name="Maximales Alter" dataDxfId="222"/>
-    <tableColumn id="5" xr3:uid="{FD4B0E6E-9B64-4731-A50F-D3CE3A4ED3FC}" name="Qualizeitraum anfang" dataDxfId="221"/>
-    <tableColumn id="6" xr3:uid="{5E84CAD2-C403-49B9-BB06-D56EC5784C8C}" name="Qualizeitraum Ende" dataDxfId="220"/>
-    <tableColumn id="7" xr3:uid="{6323F8E2-5DA4-4E5B-9C35-1E8C219ADECF}" name="Letzter Wettkampf am" dataDxfId="219"/>
-    <tableColumn id="8" xr3:uid="{D2845930-152E-432F-92A0-E7F7A3EE1FF0}" name="Landesverband" dataDxfId="218"/>
-    <tableColumn id="9" xr3:uid="{87046373-5CCD-41EC-B34C-C753E71FD26C}" name="OMS" dataDxfId="217"/>
-    <tableColumn id="10" xr3:uid="{A685FE01-F23C-4533-B399-857F5A1F6C37}" name="Pool-Länge" dataDxfId="216"/>
-    <tableColumn id="11" xr3:uid="{11E0A508-0C9D-4CB6-952E-7FAC5D05BDCD}" name="Regelwerk" dataDxfId="215"/>
-    <tableColumn id="12" xr3:uid="{F220BD5F-C3B5-4935-996A-BFCDF9F392D9}" name="Seiten Anzahl" dataDxfId="214"/>
-    <tableColumn id="13" xr3:uid="{A0A5E62D-9354-426D-9A08-13E43F36F55B}" name="PZ1 - 50m Retten" dataDxfId="213"/>
-    <tableColumn id="14" xr3:uid="{5D70F54C-57E9-45E2-BC99-0DBB0422383E}" name="PZ1 - 100m Retten" dataDxfId="212"/>
-    <tableColumn id="15" xr3:uid="{1C0CF5DB-156E-4813-A8BA-9EA29A40ABF3}" name="PZ1 - 100m Kombi" dataDxfId="211"/>
-    <tableColumn id="16" xr3:uid="{691CD4E1-13D9-4455-A2D1-14C9BC41A0EA}" name="PZ1 - 100m Lifesaver" dataDxfId="210"/>
-    <tableColumn id="17" xr3:uid="{CE1BA235-770B-4FA4-B327-187675DDA6B8}" name="PZ1 - 200m Super-Lifesaver" dataDxfId="209"/>
-    <tableColumn id="18" xr3:uid="{A326EF87-5FF5-4042-85D3-7806FEED4CFA}" name="PZ1 - 200m Hindernis" dataDxfId="208"/>
-    <tableColumn id="19" xr3:uid="{ABA5540C-4356-4D68-8579-E660F9FD6EA8}" name="PZ2 - 50m Retten" dataDxfId="207"/>
-    <tableColumn id="20" xr3:uid="{62E98437-16C9-4433-8683-E3C8A1B80E76}" name="PZ2 - 100m Retten" dataDxfId="206"/>
-    <tableColumn id="21" xr3:uid="{ED4E9448-4073-4B27-A491-5385DED08F83}" name="PZ2 - 100m Kombi" dataDxfId="205"/>
-    <tableColumn id="22" xr3:uid="{53F3DC0A-267B-434A-BD8A-320943916288}" name="PZ2 - 100m Lifesaver" dataDxfId="204"/>
-    <tableColumn id="23" xr3:uid="{1586F43C-8AD2-4942-A098-687AF0A028AC}" name="PZ2 - 200m Super-Lifesaver" dataDxfId="203"/>
-    <tableColumn id="24" xr3:uid="{98AA496B-EB58-437E-91F5-800894DDD85F}" name="PZ2 - 200m Hindernis" dataDxfId="202"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{FED162EE-531E-453F-8C25-562B59ECE709}" name="LK_konfig" displayName="LK_konfig" ref="A1:Y37" totalsRowShown="0" headerRowDxfId="26" dataDxfId="25">
+  <autoFilter ref="A1:Y37" xr:uid="{FED162EE-531E-453F-8C25-562B59ECE709}"/>
+  <tableColumns count="25">
+    <tableColumn id="1" xr3:uid="{F985A4F0-6B8C-47C6-816F-1A31A4973EB2}" name="Tabellen Name" dataDxfId="24"/>
+    <tableColumn id="2" xr3:uid="{5E5AD859-71A2-4E8E-B434-431A89C05C57}" name="Geschlecht" dataDxfId="23"/>
+    <tableColumn id="3" xr3:uid="{85BB892C-E151-404B-8974-FC5199E0909C}" name="Mindest Alter" dataDxfId="22"/>
+    <tableColumn id="4" xr3:uid="{790F6CF9-E475-4082-AE03-D30EDE22FB61}" name="Maximales Alter" dataDxfId="21"/>
+    <tableColumn id="5" xr3:uid="{FD4B0E6E-9B64-4731-A50F-D3CE3A4ED3FC}" name="Qualizeitraum anfang" dataDxfId="20"/>
+    <tableColumn id="6" xr3:uid="{5E84CAD2-C403-49B9-BB06-D56EC5784C8C}" name="Qualizeitraum Ende" dataDxfId="19"/>
+    <tableColumn id="7" xr3:uid="{6323F8E2-5DA4-4E5B-9C35-1E8C219ADECF}" name="Letzter Wettkampf am" dataDxfId="18"/>
+    <tableColumn id="8" xr3:uid="{D2845930-152E-432F-92A0-E7F7A3EE1FF0}" name="Landesverband" dataDxfId="17"/>
+    <tableColumn id="9" xr3:uid="{87046373-5CCD-41EC-B34C-C753E71FD26C}" name="OMS" dataDxfId="16"/>
+    <tableColumn id="10" xr3:uid="{A685FE01-F23C-4533-B399-857F5A1F6C37}" name="Pool-Länge" dataDxfId="15"/>
+    <tableColumn id="11" xr3:uid="{11E0A508-0C9D-4CB6-952E-7FAC5D05BDCD}" name="Regelwerk" dataDxfId="14"/>
+    <tableColumn id="12" xr3:uid="{F220BD5F-C3B5-4935-996A-BFCDF9F392D9}" name="Seiten Anzahl" dataDxfId="13"/>
+    <tableColumn id="25" xr3:uid="{7CDE58FE-A5B8-4329-9F48-3913AEBA21FC}" name="mind. erreichte Normen" dataDxfId="12"/>
+    <tableColumn id="13" xr3:uid="{A0A5E62D-9354-426D-9A08-13E43F36F55B}" name="PZ1 - 50m Retten" dataDxfId="11"/>
+    <tableColumn id="14" xr3:uid="{5D70F54C-57E9-45E2-BC99-0DBB0422383E}" name="PZ1 - 100m Retten" dataDxfId="10"/>
+    <tableColumn id="15" xr3:uid="{1C0CF5DB-156E-4813-A8BA-9EA29A40ABF3}" name="PZ1 - 100m Kombi" dataDxfId="9"/>
+    <tableColumn id="16" xr3:uid="{691CD4E1-13D9-4455-A2D1-14C9BC41A0EA}" name="PZ1 - 100m Lifesaver" dataDxfId="8"/>
+    <tableColumn id="17" xr3:uid="{CE1BA235-770B-4FA4-B327-187675DDA6B8}" name="PZ1 - 200m Super-Lifesaver" dataDxfId="7"/>
+    <tableColumn id="18" xr3:uid="{A326EF87-5FF5-4042-85D3-7806FEED4CFA}" name="PZ1 - 200m Hindernis" dataDxfId="6"/>
+    <tableColumn id="19" xr3:uid="{ABA5540C-4356-4D68-8579-E660F9FD6EA8}" name="PZ2 - 50m Retten" dataDxfId="5"/>
+    <tableColumn id="20" xr3:uid="{62E98437-16C9-4433-8683-E3C8A1B80E76}" name="PZ2 - 100m Retten" dataDxfId="4"/>
+    <tableColumn id="21" xr3:uid="{ED4E9448-4073-4B27-A491-5385DED08F83}" name="PZ2 - 100m Kombi" dataDxfId="3"/>
+    <tableColumn id="22" xr3:uid="{53F3DC0A-267B-434A-BD8A-320943916288}" name="PZ2 - 100m Lifesaver" dataDxfId="2"/>
+    <tableColumn id="23" xr3:uid="{1586F43C-8AD2-4942-A098-687AF0A028AC}" name="PZ2 - 200m Super-Lifesaver" dataDxfId="1"/>
+    <tableColumn id="24" xr3:uid="{98AA496B-EB58-437E-91F5-800894DDD85F}" name="PZ2 - 200m Hindernis" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4588,12 +4595,12 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{888CE7BE-8313-44C0-AE38-83992EABD44D}" name="LK_Kalender" displayName="LK_Kalender" ref="A1:H8" totalsRowShown="0">
   <autoFilter ref="A1:H8" xr:uid="{888CE7BE-8313-44C0-AE38-83992EABD44D}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{B26B9E90-F378-41EF-B35E-CE240017E4BE}" name="datum von" dataDxfId="25"/>
+    <tableColumn id="1" xr3:uid="{B26B9E90-F378-41EF-B35E-CE240017E4BE}" name="datum von" dataDxfId="52"/>
     <tableColumn id="2" xr3:uid="{38211212-0A92-428C-895C-E4CA68F52818}" name="datum bis"/>
-    <tableColumn id="3" xr3:uid="{66E541C6-0A5E-4B2D-9B89-5E52F449A4A6}" name="uhrzeit von" dataDxfId="24"/>
-    <tableColumn id="4" xr3:uid="{D93C06A2-29AD-4073-8E3C-A685B4474CC8}" name="uhrzeit bis" dataDxfId="23"/>
-    <tableColumn id="5" xr3:uid="{C5C3979C-B528-44E8-A5A6-36F020A6034F}" name="titel" dataDxfId="22"/>
-    <tableColumn id="6" xr3:uid="{9DC09E1D-44FD-40ED-9EBE-86A8E61C38B2}" name="meta" dataDxfId="21"/>
+    <tableColumn id="3" xr3:uid="{66E541C6-0A5E-4B2D-9B89-5E52F449A4A6}" name="uhrzeit von" dataDxfId="51"/>
+    <tableColumn id="4" xr3:uid="{D93C06A2-29AD-4073-8E3C-A685B4474CC8}" name="uhrzeit bis" dataDxfId="50"/>
+    <tableColumn id="5" xr3:uid="{C5C3979C-B528-44E8-A5A6-36F020A6034F}" name="titel" dataDxfId="49"/>
+    <tableColumn id="6" xr3:uid="{9DC09E1D-44FD-40ED-9EBE-86A8E61C38B2}" name="meta" dataDxfId="48"/>
     <tableColumn id="7" xr3:uid="{E7E62A34-7A76-4361-937D-F4DE76E6E7CC}" name="ort"/>
     <tableColumn id="8" xr3:uid="{84F02734-FC16-406B-ACCA-0CCDF547D94C}" name="kader"/>
   </tableColumns>
@@ -8535,52 +8542,52 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B5:G31">
-    <cfRule type="expression" dxfId="20" priority="15">
+    <cfRule type="expression" dxfId="47" priority="15">
       <formula>B5&lt;&gt;B4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H5:M31">
-    <cfRule type="expression" dxfId="19" priority="14">
+    <cfRule type="expression" dxfId="46" priority="14">
       <formula>H5&lt;&gt;H4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N5:S31">
-    <cfRule type="expression" dxfId="18" priority="13">
+    <cfRule type="expression" dxfId="45" priority="13">
       <formula>N5&lt;&gt;N4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="T5:Y31">
-    <cfRule type="expression" dxfId="17" priority="12">
+    <cfRule type="expression" dxfId="44" priority="12">
       <formula>T5&lt;&gt;T4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z5:AE31">
-    <cfRule type="expression" dxfId="16" priority="9">
+    <cfRule type="expression" dxfId="43" priority="9">
       <formula>Z5&lt;&gt;Z4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AF5:AK31">
-    <cfRule type="expression" dxfId="15" priority="8">
+    <cfRule type="expression" dxfId="42" priority="8">
       <formula>AF5&lt;&gt;AF4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AL5:AN31">
-    <cfRule type="expression" dxfId="14" priority="6">
+    <cfRule type="expression" dxfId="41" priority="6">
       <formula>AL5&lt;&gt;AL4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AO5:AQ31">
-    <cfRule type="expression" dxfId="13" priority="5">
+    <cfRule type="expression" dxfId="40" priority="5">
       <formula>AO5&lt;&gt;AO4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AR5:AT31">
-    <cfRule type="expression" dxfId="12" priority="2">
+    <cfRule type="expression" dxfId="39" priority="2">
       <formula>AR5&lt;&gt;AR4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AU5:AW31">
-    <cfRule type="expression" dxfId="11" priority="1">
+    <cfRule type="expression" dxfId="38" priority="1">
       <formula>AU5&lt;&gt;AU4</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8802,7 +8809,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:H8">
-    <cfRule type="expression" dxfId="0" priority="1">
+    <cfRule type="expression" dxfId="27" priority="1">
       <formula>$A2&lt;TODAY()</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9808,22 +9815,22 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B6:G6">
-    <cfRule type="expression" dxfId="10" priority="20">
+    <cfRule type="expression" dxfId="37" priority="20">
       <formula>B6&lt;&gt;B4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7:G32">
-    <cfRule type="expression" dxfId="9" priority="1">
+    <cfRule type="expression" dxfId="36" priority="1">
       <formula>B7&lt;&gt;B6</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H6:M6">
-    <cfRule type="expression" dxfId="8" priority="22">
+    <cfRule type="expression" dxfId="35" priority="22">
       <formula>H6&lt;&gt;H4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H7:M32">
-    <cfRule type="expression" dxfId="7" priority="2">
+    <cfRule type="expression" dxfId="34" priority="2">
       <formula>H7&lt;&gt;H6</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11154,22 +11161,22 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B6:G6">
-    <cfRule type="expression" dxfId="6" priority="19">
+    <cfRule type="expression" dxfId="33" priority="19">
       <formula>B6&lt;&gt;B4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7:G32">
-    <cfRule type="expression" dxfId="5" priority="2">
+    <cfRule type="expression" dxfId="32" priority="2">
       <formula>B7&lt;&gt;B6</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H6:M6">
-    <cfRule type="expression" dxfId="4" priority="20">
+    <cfRule type="expression" dxfId="31" priority="20">
       <formula>H6&lt;&gt;H4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H7:M32">
-    <cfRule type="expression" dxfId="3" priority="1">
+    <cfRule type="expression" dxfId="30" priority="1">
       <formula>H7&lt;&gt;H6</formula>
     </cfRule>
   </conditionalFormatting>
@@ -12664,7 +12671,7 @@
   <sheetPr>
     <tabColor theme="5" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="A1:X37"/>
+  <dimension ref="A1:Y37"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="17.3984375" bestFit="1" customWidth="1"/>
@@ -12679,21 +12686,22 @@
     <col min="10" max="10" width="11.86328125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="11.3984375" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="13.73046875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="16.3984375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="17.3984375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="17.1328125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="19.3984375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="24.86328125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="19.86328125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="16.3984375" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.3984375" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="17.1328125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="19.3984375" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="24.86328125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="19.86328125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="24.19921875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="16.3984375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="17.3984375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="17.1328125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="19.3984375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="24.86328125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="19.86328125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="16.3984375" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="17.3984375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="17.1328125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="19.3984375" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="24.86328125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="19.86328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A1" s="25" t="s">
         <v>127</v>
       </c>
@@ -12731,43 +12739,46 @@
         <v>142</v>
       </c>
       <c r="M1" s="25" t="s">
+        <v>247</v>
+      </c>
+      <c r="N1" s="25" t="s">
         <v>166</v>
       </c>
-      <c r="N1" s="25" t="s">
+      <c r="O1" s="25" t="s">
         <v>167</v>
       </c>
-      <c r="O1" s="25" t="s">
+      <c r="P1" s="25" t="s">
         <v>168</v>
       </c>
-      <c r="P1" s="25" t="s">
+      <c r="Q1" s="25" t="s">
         <v>171</v>
       </c>
-      <c r="Q1" s="25" t="s">
+      <c r="R1" s="25" t="s">
         <v>170</v>
       </c>
-      <c r="R1" s="25" t="s">
+      <c r="S1" s="25" t="s">
         <v>169</v>
       </c>
-      <c r="S1" s="25" t="s">
+      <c r="T1" s="25" t="s">
         <v>172</v>
       </c>
-      <c r="T1" s="25" t="s">
+      <c r="U1" s="25" t="s">
         <v>173</v>
       </c>
-      <c r="U1" s="25" t="s">
+      <c r="V1" s="25" t="s">
         <v>174</v>
       </c>
-      <c r="V1" s="25" t="s">
+      <c r="W1" s="25" t="s">
         <v>175</v>
       </c>
-      <c r="W1" s="25" t="s">
+      <c r="X1" s="25" t="s">
         <v>176</v>
       </c>
-      <c r="X1" s="25" t="s">
+      <c r="Y1" s="25" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A2" s="25" t="s">
         <v>241</v>
       </c>
@@ -12800,38 +12811,41 @@
       <c r="L2" s="25">
         <v>10</v>
       </c>
-      <c r="M2" s="28">
+      <c r="M2" s="25">
+        <v>2</v>
+      </c>
+      <c r="N2" s="28">
         <f>'NK-LK Transf.'!BQ12</f>
         <v>5.3782870370370367E-4</v>
       </c>
-      <c r="N2" s="28">
+      <c r="O2" s="28">
         <f>'NK-LK Transf.'!BQ14</f>
         <v>8.139814814814815E-4</v>
       </c>
-      <c r="O2" s="28">
+      <c r="P2" s="28">
         <f>'NK-LK Transf.'!BQ13</f>
         <v>1.1029722222222222E-3</v>
       </c>
-      <c r="P2" s="28">
+      <c r="Q2" s="28">
         <f>'NK-LK Transf.'!BQ15</f>
         <v>9.026180555555556E-4</v>
       </c>
-      <c r="Q2" s="28">
+      <c r="R2" s="28">
         <f>'NK-LK Transf.'!BQ17</f>
         <v>2.1334236111111111E-3</v>
       </c>
-      <c r="R2" s="28">
+      <c r="S2" s="28">
         <f>'NK-LK Transf.'!BQ16</f>
         <v>1.9327962962962964E-3</v>
       </c>
-      <c r="S2" s="28"/>
       <c r="T2" s="28"/>
       <c r="U2" s="28"/>
       <c r="V2" s="28"/>
       <c r="W2" s="28"/>
       <c r="X2" s="28"/>
+      <c r="Y2" s="28"/>
     </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A3" s="25" t="s">
         <v>241</v>
       </c>
@@ -12864,38 +12878,41 @@
       <c r="L3" s="25">
         <v>10</v>
       </c>
-      <c r="M3" s="28">
+      <c r="M3" s="25">
+        <v>2</v>
+      </c>
+      <c r="N3" s="28">
         <f>'NK-LK Transf.'!BP12</f>
         <v>5.5107638888888893E-4</v>
       </c>
-      <c r="N3" s="28">
+      <c r="O3" s="28">
         <f>'NK-LK Transf.'!BP14</f>
         <v>8.3037037037037031E-4</v>
       </c>
-      <c r="O3" s="28">
+      <c r="P3" s="28">
         <f>'NK-LK Transf.'!BP13</f>
         <v>1.1436712962962963E-3</v>
       </c>
-      <c r="P3" s="28">
+      <c r="Q3" s="28">
         <f>'NK-LK Transf.'!BP15</f>
         <v>9.2269444444444452E-4</v>
       </c>
-      <c r="Q3" s="28">
+      <c r="R3" s="28">
         <f>'NK-LK Transf.'!BP17</f>
         <v>2.1813611111111113E-3</v>
       </c>
-      <c r="R3" s="28">
+      <c r="S3" s="28">
         <f>'NK-LK Transf.'!BP16</f>
         <v>1.9621597222222223E-3</v>
       </c>
-      <c r="S3" s="28"/>
       <c r="T3" s="28"/>
       <c r="U3" s="28"/>
       <c r="V3" s="28"/>
       <c r="W3" s="28"/>
       <c r="X3" s="28"/>
+      <c r="Y3" s="28"/>
     </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A4" s="25" t="s">
         <v>241</v>
       </c>
@@ -12928,38 +12945,41 @@
       <c r="L4" s="25">
         <v>10</v>
       </c>
-      <c r="M4" s="28">
+      <c r="M4" s="25">
+        <v>2</v>
+      </c>
+      <c r="N4" s="28">
         <f>'NK-LK Transf.'!BO12</f>
         <v>5.6332031250000002E-4</v>
       </c>
-      <c r="N4" s="28">
+      <c r="O4" s="28">
         <f>'NK-LK Transf.'!BO14</f>
         <v>8.4539351851851854E-4</v>
       </c>
-      <c r="O4" s="28">
+      <c r="P4" s="28">
         <f>'NK-LK Transf.'!BO13</f>
         <v>1.1842337962962965E-3</v>
       </c>
-      <c r="P4" s="28">
+      <c r="Q4" s="28">
         <f>'NK-LK Transf.'!BO15</f>
         <v>9.4126851851851858E-4</v>
       </c>
-      <c r="Q4" s="28">
+      <c r="R4" s="28">
         <f>'NK-LK Transf.'!BO17</f>
         <v>2.2291620370370373E-3</v>
       </c>
-      <c r="R4" s="28">
+      <c r="S4" s="28">
         <f>'NK-LK Transf.'!BO16</f>
         <v>1.9916597222222219E-3</v>
       </c>
-      <c r="S4" s="28"/>
       <c r="T4" s="28"/>
       <c r="U4" s="28"/>
       <c r="V4" s="28"/>
       <c r="W4" s="28"/>
       <c r="X4" s="28"/>
+      <c r="Y4" s="28"/>
     </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A5" s="25" t="s">
         <v>233</v>
       </c>
@@ -12992,38 +13012,41 @@
       <c r="L5" s="25">
         <v>10</v>
       </c>
-      <c r="M5" s="28">
+      <c r="M5" s="25">
+        <v>2</v>
+      </c>
+      <c r="N5" s="28">
         <f>'NK-LK Transf.'!BE12</f>
         <v>4.4791666666666667E-4</v>
       </c>
-      <c r="N5" s="28">
+      <c r="O5" s="28">
         <f>'NK-LK Transf.'!BE14</f>
         <v>7.0736111111111108E-4</v>
       </c>
-      <c r="O5" s="28">
+      <c r="P5" s="28">
         <f>'NK-LK Transf.'!BE13</f>
         <v>9.6125000000000019E-4</v>
       </c>
-      <c r="P5" s="28">
+      <c r="Q5" s="28">
         <f>'NK-LK Transf.'!BE15</f>
         <v>8.018055555555555E-4</v>
       </c>
-      <c r="Q5" s="28">
+      <c r="R5" s="28">
         <f>'NK-LK Transf.'!BE17</f>
         <v>1.9945833333333335E-3</v>
       </c>
-      <c r="R5" s="28">
+      <c r="S5" s="28">
         <f>'NK-LK Transf.'!BE16</f>
         <v>1.8218055555555552E-3</v>
       </c>
-      <c r="S5" s="28"/>
       <c r="T5" s="28"/>
       <c r="U5" s="28"/>
       <c r="V5" s="28"/>
       <c r="W5" s="28"/>
       <c r="X5" s="28"/>
+      <c r="Y5" s="28"/>
     </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A6" s="25" t="s">
         <v>233</v>
       </c>
@@ -13056,38 +13079,41 @@
       <c r="L6" s="25">
         <v>10</v>
       </c>
-      <c r="M6" s="28">
+      <c r="M6" s="25">
+        <v>2</v>
+      </c>
+      <c r="N6" s="28">
         <f>'NK-LK Transf.'!BD12</f>
         <v>4.6194444444444446E-4</v>
       </c>
-      <c r="N6" s="28">
+      <c r="O6" s="28">
         <f>'NK-LK Transf.'!BD14</f>
         <v>7.2763888888888889E-4</v>
       </c>
-      <c r="O6" s="28">
+      <c r="P6" s="28">
         <f>'NK-LK Transf.'!BD13</f>
         <v>1E-3</v>
       </c>
-      <c r="P6" s="28">
+      <c r="Q6" s="28">
         <f>'NK-LK Transf.'!BD15</f>
         <v>8.3263888888888895E-4</v>
       </c>
-      <c r="Q6" s="28">
+      <c r="R6" s="28">
         <f>'NK-LK Transf.'!BD17</f>
         <v>2.0587499999999998E-3</v>
       </c>
-      <c r="R6" s="28">
+      <c r="S6" s="28">
         <f>'NK-LK Transf.'!BD16</f>
         <v>1.8773611111111109E-3</v>
       </c>
-      <c r="S6" s="28"/>
       <c r="T6" s="28"/>
       <c r="U6" s="28"/>
       <c r="V6" s="28"/>
       <c r="W6" s="28"/>
       <c r="X6" s="28"/>
+      <c r="Y6" s="28"/>
     </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A7" s="25" t="s">
         <v>233</v>
       </c>
@@ -13120,38 +13146,41 @@
       <c r="L7" s="25">
         <v>10</v>
       </c>
-      <c r="M7" s="28">
+      <c r="M7" s="25">
+        <v>2</v>
+      </c>
+      <c r="N7" s="28">
         <f>'NK-LK Transf.'!BC12</f>
         <v>4.7138888888888881E-4</v>
       </c>
-      <c r="N7" s="28">
+      <c r="O7" s="28">
         <f>'NK-LK Transf.'!BC14</f>
         <v>7.415277777777778E-4</v>
       </c>
-      <c r="O7" s="28">
+      <c r="P7" s="28">
         <f>'NK-LK Transf.'!BC13</f>
         <v>1.0176388888888889E-3</v>
       </c>
-      <c r="P7" s="28">
+      <c r="Q7" s="28">
         <f>'NK-LK Transf.'!BC15</f>
         <v>8.5375000000000002E-4</v>
       </c>
-      <c r="Q7" s="28">
+      <c r="R7" s="28">
         <f>'NK-LK Transf.'!BC17</f>
         <v>2.1025000000000002E-3</v>
       </c>
-      <c r="R7" s="28">
+      <c r="S7" s="28">
         <f>'NK-LK Transf.'!BC16</f>
         <v>1.9152777777777779E-3</v>
       </c>
-      <c r="S7" s="28"/>
       <c r="T7" s="28"/>
       <c r="U7" s="28"/>
       <c r="V7" s="28"/>
       <c r="W7" s="28"/>
       <c r="X7" s="28"/>
+      <c r="Y7" s="28"/>
     </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A8" s="25" t="s">
         <v>240</v>
       </c>
@@ -13184,38 +13213,41 @@
       <c r="L8" s="25">
         <v>10</v>
       </c>
-      <c r="M8" s="28">
+      <c r="M8" s="25">
+        <v>2</v>
+      </c>
+      <c r="N8" s="28">
         <f>'NK-LK Transf.'!BV12</f>
         <v>4.7436458333333331E-4</v>
       </c>
-      <c r="N8" s="28">
+      <c r="O8" s="28">
         <f>'NK-LK Transf.'!BV14</f>
         <v>7.3382291666666669E-4</v>
       </c>
-      <c r="O8" s="28">
+      <c r="P8" s="28">
         <f>'NK-LK Transf.'!BV13</f>
         <v>9.7080208333333328E-4</v>
       </c>
-      <c r="P8" s="28">
+      <c r="Q8" s="28">
         <f>'NK-LK Transf.'!BV15</f>
         <v>8.0545833333333326E-4</v>
       </c>
-      <c r="Q8" s="28">
+      <c r="R8" s="28">
         <f>'NK-LK Transf.'!BV17</f>
         <v>1.9667916666666666E-3</v>
       </c>
-      <c r="R8" s="28">
+      <c r="S8" s="28">
         <f>'NK-LK Transf.'!BV16</f>
         <v>1.8239270833333334E-3</v>
       </c>
-      <c r="S8" s="28"/>
       <c r="T8" s="28"/>
       <c r="U8" s="28"/>
       <c r="V8" s="28"/>
       <c r="W8" s="28"/>
       <c r="X8" s="28"/>
+      <c r="Y8" s="28"/>
     </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A9" s="25" t="s">
         <v>240</v>
       </c>
@@ -13248,38 +13280,41 @@
       <c r="L9" s="25">
         <v>10</v>
       </c>
-      <c r="M9" s="28">
+      <c r="M9" s="25">
+        <v>2</v>
+      </c>
+      <c r="N9" s="28">
         <f>'NK-LK Transf.'!BU12</f>
         <v>4.9196875E-4</v>
       </c>
-      <c r="N9" s="28">
+      <c r="O9" s="28">
         <f>'NK-LK Transf.'!BU14</f>
         <v>7.5576041666666662E-4</v>
       </c>
-      <c r="O9" s="28">
+      <c r="P9" s="28">
         <f>'NK-LK Transf.'!BU13</f>
         <v>1.0057395833333333E-3</v>
       </c>
-      <c r="P9" s="28">
+      <c r="Q9" s="28">
         <f>'NK-LK Transf.'!BU15</f>
         <v>8.3227083333333341E-4</v>
       </c>
-      <c r="Q9" s="28">
+      <c r="R9" s="28">
         <f>'NK-LK Transf.'!BU17</f>
         <v>2.0094479166666668E-3</v>
       </c>
-      <c r="R9" s="28">
+      <c r="S9" s="28">
         <f>'NK-LK Transf.'!BU16</f>
         <v>1.8506041666666666E-3</v>
       </c>
-      <c r="S9" s="28"/>
       <c r="T9" s="28"/>
       <c r="U9" s="28"/>
       <c r="V9" s="28"/>
       <c r="W9" s="28"/>
       <c r="X9" s="28"/>
+      <c r="Y9" s="28"/>
     </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A10" s="25" t="s">
         <v>240</v>
       </c>
@@ -13312,38 +13347,41 @@
       <c r="L10" s="25">
         <v>10</v>
       </c>
-      <c r="M10" s="28">
+      <c r="M10" s="25">
+        <v>2</v>
+      </c>
+      <c r="N10" s="28">
         <f>'NK-LK Transf.'!BT12</f>
         <v>5.1593750000000001E-4</v>
       </c>
-      <c r="N10" s="28">
+      <c r="O10" s="28">
         <f>'NK-LK Transf.'!BT14</f>
         <v>7.8582291666666677E-4</v>
       </c>
-      <c r="O10" s="28">
+      <c r="P10" s="28">
         <f>'NK-LK Transf.'!BT13</f>
         <v>1.0534062499999999E-3</v>
       </c>
-      <c r="P10" s="28">
+      <c r="Q10" s="28">
         <f>'NK-LK Transf.'!BT15</f>
         <v>8.6883333333333322E-4</v>
       </c>
-      <c r="Q10" s="28">
+      <c r="R10" s="28">
         <f>'NK-LK Transf.'!BT17</f>
         <v>2.0678124999999998E-3</v>
       </c>
-      <c r="R10" s="28">
+      <c r="S10" s="28">
         <f>'NK-LK Transf.'!BT16</f>
         <v>1.887166666666667E-3</v>
       </c>
-      <c r="S10" s="28"/>
       <c r="T10" s="28"/>
       <c r="U10" s="28"/>
       <c r="V10" s="28"/>
       <c r="W10" s="28"/>
       <c r="X10" s="28"/>
+      <c r="Y10" s="28"/>
     </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A11" s="25" t="s">
         <v>239</v>
       </c>
@@ -13376,38 +13414,41 @@
       <c r="L11" s="25">
         <v>10</v>
       </c>
-      <c r="M11" s="28">
+      <c r="M11" s="25">
+        <v>2</v>
+      </c>
+      <c r="N11" s="28">
         <f>'NK-LK Transf.'!BJ12</f>
         <v>3.9324537037037041E-4</v>
       </c>
-      <c r="N11" s="28">
+      <c r="O11" s="28">
         <f>'NK-LK Transf.'!BJ14</f>
         <v>6.2564814814814818E-4</v>
       </c>
-      <c r="O11" s="28">
+      <c r="P11" s="28">
         <f>'NK-LK Transf.'!BJ13</f>
         <v>8.3428703703703703E-4</v>
       </c>
-      <c r="P11" s="28">
+      <c r="Q11" s="28">
         <f>'NK-LK Transf.'!BJ15</f>
         <v>6.8807870370370366E-4</v>
       </c>
-      <c r="Q11" s="28">
+      <c r="R11" s="28">
         <f>'NK-LK Transf.'!BJ17</f>
         <v>1.7890046296296298E-3</v>
       </c>
-      <c r="R11" s="28">
+      <c r="S11" s="28">
         <f>'NK-LK Transf.'!BJ16</f>
         <v>1.6026527777777777E-3</v>
       </c>
-      <c r="S11" s="28"/>
       <c r="T11" s="28"/>
       <c r="U11" s="28"/>
       <c r="V11" s="28"/>
       <c r="W11" s="28"/>
       <c r="X11" s="28"/>
+      <c r="Y11" s="28"/>
     </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A12" s="25" t="s">
         <v>239</v>
       </c>
@@ -13440,38 +13481,41 @@
       <c r="L12" s="25">
         <v>10</v>
       </c>
-      <c r="M12" s="28">
+      <c r="M12" s="25">
+        <v>2</v>
+      </c>
+      <c r="N12" s="28">
         <f>'NK-LK Transf.'!BI12</f>
         <v>4.0693981481481478E-4</v>
       </c>
-      <c r="N12" s="28">
+      <c r="O12" s="28">
         <f>'NK-LK Transf.'!BI14</f>
         <v>6.4565277777777776E-4</v>
       </c>
-      <c r="O12" s="28">
+      <c r="P12" s="28">
         <f>'NK-LK Transf.'!BI13</f>
         <v>8.6691203703703691E-4</v>
       </c>
-      <c r="P12" s="28">
+      <c r="Q12" s="28">
         <f>'NK-LK Transf.'!BI15</f>
         <v>7.1788425925925915E-4</v>
       </c>
-      <c r="Q12" s="28">
+      <c r="R12" s="28">
         <f>'NK-LK Transf.'!BI17</f>
         <v>1.845125E-3</v>
       </c>
-      <c r="R12" s="28">
+      <c r="S12" s="28">
         <f>'NK-LK Transf.'!BI16</f>
         <v>1.6571620370370373E-3</v>
       </c>
-      <c r="S12" s="28"/>
       <c r="T12" s="28"/>
       <c r="U12" s="28"/>
       <c r="V12" s="28"/>
       <c r="W12" s="28"/>
       <c r="X12" s="28"/>
+      <c r="Y12" s="28"/>
     </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A13" s="25" t="s">
         <v>239</v>
       </c>
@@ -13504,38 +13548,41 @@
       <c r="L13" s="25">
         <v>10</v>
       </c>
-      <c r="M13" s="28">
+      <c r="M13" s="25">
+        <v>2</v>
+      </c>
+      <c r="N13" s="28">
         <f>'NK-LK Transf.'!BH12</f>
         <v>4.1888888888888889E-4</v>
       </c>
-      <c r="N13" s="28">
+      <c r="O13" s="28">
         <f>'NK-LK Transf.'!BH14</f>
         <v>6.6324074074074072E-4</v>
       </c>
-      <c r="O13" s="28">
+      <c r="P13" s="28">
         <f>'NK-LK Transf.'!BH13</f>
         <v>8.9537500000000001E-4</v>
       </c>
-      <c r="P13" s="28">
+      <c r="Q13" s="28">
         <f>'NK-LK Transf.'!BH15</f>
         <v>7.439305555555554E-4</v>
       </c>
-      <c r="Q13" s="28">
+      <c r="R13" s="28">
         <f>'NK-LK Transf.'!BH17</f>
         <v>1.8632500000000001E-3</v>
       </c>
-      <c r="R13" s="28">
+      <c r="S13" s="28">
         <f>'NK-LK Transf.'!BH16</f>
         <v>1.7049583333333333E-3</v>
       </c>
-      <c r="S13" s="28"/>
       <c r="T13" s="28"/>
       <c r="U13" s="28"/>
       <c r="V13" s="28"/>
       <c r="W13" s="28"/>
       <c r="X13" s="28"/>
+      <c r="Y13" s="28"/>
     </row>
-    <row r="14" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A14" s="25" t="s">
         <v>222</v>
       </c>
@@ -13568,38 +13615,41 @@
       <c r="L14" s="25">
         <v>10</v>
       </c>
-      <c r="M14" s="28">
+      <c r="M14" s="25">
+        <v>1</v>
+      </c>
+      <c r="N14" s="28">
         <f>'NK-LK Transf.'!Q12</f>
         <v>4.5578703703703704E-4</v>
       </c>
-      <c r="N14" s="28">
+      <c r="O14" s="28">
         <f>'NK-LK Transf.'!Q14</f>
         <v>6.8981481481481487E-4</v>
       </c>
-      <c r="O14" s="28">
+      <c r="P14" s="28">
         <f>'NK-LK Transf.'!Q13</f>
         <v>9.3472222222222231E-4</v>
       </c>
-      <c r="P14" s="28">
+      <c r="Q14" s="28">
         <f>'NK-LK Transf.'!Q15</f>
         <v>7.6493055555555559E-4</v>
       </c>
-      <c r="Q14" s="28">
+      <c r="R14" s="28">
         <f>'NK-LK Transf.'!Q17</f>
         <v>1.8079861111111111E-3</v>
       </c>
-      <c r="R14" s="28">
+      <c r="S14" s="28">
         <f>'NK-LK Transf.'!Q16</f>
         <v>1.637962962962963E-3</v>
       </c>
-      <c r="S14" s="28"/>
       <c r="T14" s="28"/>
       <c r="U14" s="28"/>
       <c r="V14" s="28"/>
       <c r="W14" s="28"/>
       <c r="X14" s="28"/>
+      <c r="Y14" s="28"/>
     </row>
-    <row r="15" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A15" s="25" t="s">
         <v>222</v>
       </c>
@@ -13632,38 +13682,41 @@
       <c r="L15" s="25">
         <v>10</v>
       </c>
-      <c r="M15" s="28">
+      <c r="M15" s="25">
+        <v>1</v>
+      </c>
+      <c r="N15" s="28">
         <f>'NK-LK Transf.'!P12</f>
         <v>4.6701388888888888E-4</v>
       </c>
-      <c r="N15" s="28">
+      <c r="O15" s="28">
         <f>'NK-LK Transf.'!P14</f>
         <v>7.0370370370370367E-4</v>
       </c>
-      <c r="O15" s="28">
+      <c r="P15" s="28">
         <f>'NK-LK Transf.'!P13</f>
         <v>9.6921296296296295E-4</v>
       </c>
-      <c r="P15" s="28">
+      <c r="Q15" s="28">
         <f>'NK-LK Transf.'!P15</f>
         <v>7.8194444444444448E-4</v>
       </c>
-      <c r="Q15" s="28">
+      <c r="R15" s="28">
         <f>'NK-LK Transf.'!P17</f>
         <v>1.8486111111111112E-3</v>
       </c>
-      <c r="R15" s="28">
+      <c r="S15" s="28">
         <f>'NK-LK Transf.'!P16</f>
         <v>1.6628472222222225E-3</v>
       </c>
-      <c r="S15" s="28"/>
       <c r="T15" s="28"/>
       <c r="U15" s="28"/>
       <c r="V15" s="28"/>
       <c r="W15" s="28"/>
       <c r="X15" s="28"/>
+      <c r="Y15" s="28"/>
     </row>
-    <row r="16" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A16" s="25" t="s">
         <v>222</v>
       </c>
@@ -13696,38 +13749,41 @@
       <c r="L16" s="25">
         <v>10</v>
       </c>
-      <c r="M16" s="28">
+      <c r="M16" s="25">
+        <v>1</v>
+      </c>
+      <c r="N16" s="28">
         <f>'NK-LK Transf.'!O12</f>
         <v>4.7743055555555554E-4</v>
       </c>
-      <c r="N16" s="28">
+      <c r="O16" s="28">
         <f>'NK-LK Transf.'!O14</f>
         <v>7.1643518518518519E-4</v>
       </c>
-      <c r="O16" s="28">
+      <c r="P16" s="28">
         <f>'NK-LK Transf.'!O13</f>
         <v>1.0035879629629631E-3</v>
       </c>
-      <c r="P16" s="28">
+      <c r="Q16" s="28">
         <f>'NK-LK Transf.'!O15</f>
         <v>7.9768518518518524E-4</v>
       </c>
-      <c r="Q16" s="28">
+      <c r="R16" s="28">
         <f>'NK-LK Transf.'!O17</f>
         <v>1.8891203703703704E-3</v>
       </c>
-      <c r="R16" s="28">
+      <c r="S16" s="28">
         <f>'NK-LK Transf.'!O16</f>
         <v>1.6878472222222221E-3</v>
       </c>
-      <c r="S16" s="28"/>
       <c r="T16" s="28"/>
       <c r="U16" s="28"/>
       <c r="V16" s="28"/>
       <c r="W16" s="28"/>
       <c r="X16" s="28"/>
+      <c r="Y16" s="28"/>
     </row>
-    <row r="17" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A17" s="25" t="s">
         <v>220</v>
       </c>
@@ -13760,38 +13816,41 @@
       <c r="L17" s="25">
         <v>10</v>
       </c>
-      <c r="M17" s="28">
+      <c r="M17" s="25">
+        <v>1</v>
+      </c>
+      <c r="N17" s="28">
         <f>'NK-LK Transf.'!E12</f>
         <v>3.7326388888888891E-4</v>
       </c>
-      <c r="N17" s="28">
+      <c r="O17" s="28">
         <f>'NK-LK Transf.'!E14</f>
         <v>5.894675925925926E-4</v>
       </c>
-      <c r="O17" s="28">
+      <c r="P17" s="28">
         <f>'NK-LK Transf.'!E13</f>
         <v>8.0104166666666681E-4</v>
       </c>
-      <c r="P17" s="28">
+      <c r="Q17" s="28">
         <f>'NK-LK Transf.'!E15</f>
         <v>6.6817129629629626E-4</v>
       </c>
-      <c r="Q17" s="28">
+      <c r="R17" s="28">
         <f>'NK-LK Transf.'!E17</f>
         <v>1.662152777777778E-3</v>
       </c>
-      <c r="R17" s="28">
+      <c r="S17" s="28">
         <f>'NK-LK Transf.'!E16</f>
         <v>1.5181712962962961E-3</v>
       </c>
-      <c r="S17" s="28"/>
       <c r="T17" s="28"/>
       <c r="U17" s="28"/>
       <c r="V17" s="28"/>
       <c r="W17" s="28"/>
       <c r="X17" s="28"/>
+      <c r="Y17" s="28"/>
     </row>
-    <row r="18" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A18" s="25" t="s">
         <v>220</v>
       </c>
@@ -13824,38 +13883,41 @@
       <c r="L18" s="25">
         <v>10</v>
       </c>
-      <c r="M18" s="28">
+      <c r="M18" s="25">
+        <v>1</v>
+      </c>
+      <c r="N18" s="28">
         <f>'NK-LK Transf.'!D12</f>
         <v>3.8495370370370371E-4</v>
       </c>
-      <c r="N18" s="28">
+      <c r="O18" s="28">
         <f>'NK-LK Transf.'!D14</f>
         <v>6.0636574074074076E-4</v>
       </c>
-      <c r="O18" s="28">
+      <c r="P18" s="28">
         <f>'NK-LK Transf.'!D13</f>
         <v>8.3333333333333339E-4</v>
       </c>
-      <c r="P18" s="28">
+      <c r="Q18" s="28">
         <f>'NK-LK Transf.'!D15</f>
         <v>6.9386574074074077E-4</v>
       </c>
-      <c r="Q18" s="28">
+      <c r="R18" s="28">
         <f>'NK-LK Transf.'!D17</f>
         <v>1.7156249999999999E-3</v>
       </c>
-      <c r="R18" s="28">
+      <c r="S18" s="28">
         <f>'NK-LK Transf.'!D16</f>
         <v>1.5644675925925923E-3</v>
       </c>
-      <c r="S18" s="28"/>
       <c r="T18" s="28"/>
       <c r="U18" s="28"/>
       <c r="V18" s="28"/>
       <c r="W18" s="28"/>
       <c r="X18" s="28"/>
+      <c r="Y18" s="28"/>
     </row>
-    <row r="19" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A19" s="25" t="s">
         <v>220</v>
       </c>
@@ -13888,38 +13950,41 @@
       <c r="L19" s="25">
         <v>10</v>
       </c>
-      <c r="M19" s="28">
+      <c r="M19" s="25">
+        <v>1</v>
+      </c>
+      <c r="N19" s="28">
         <f>'NK-LK Transf.'!C12</f>
         <v>3.9282407407407403E-4</v>
       </c>
-      <c r="N19" s="28">
+      <c r="O19" s="28">
         <f>'NK-LK Transf.'!C14</f>
         <v>6.1793981481481487E-4</v>
       </c>
-      <c r="O19" s="28">
+      <c r="P19" s="28">
         <f>'NK-LK Transf.'!C13</f>
         <v>8.4803240740740737E-4</v>
       </c>
-      <c r="P19" s="28">
+      <c r="Q19" s="28">
         <f>'NK-LK Transf.'!C15</f>
         <v>7.1145833333333337E-4</v>
       </c>
-      <c r="Q19" s="28">
+      <c r="R19" s="28">
         <f>'NK-LK Transf.'!C17</f>
         <v>1.7520833333333334E-3</v>
       </c>
-      <c r="R19" s="28">
+      <c r="S19" s="28">
         <f>'NK-LK Transf.'!C16</f>
         <v>1.5960648148148149E-3</v>
       </c>
-      <c r="S19" s="28"/>
       <c r="T19" s="28"/>
       <c r="U19" s="28"/>
       <c r="V19" s="28"/>
       <c r="W19" s="28"/>
       <c r="X19" s="28"/>
+      <c r="Y19" s="28"/>
     </row>
-    <row r="20" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A20" s="25" t="s">
         <v>243</v>
       </c>
@@ -13952,38 +14017,41 @@
       <c r="L20" s="25">
         <v>10</v>
       </c>
-      <c r="M20" s="28">
+      <c r="M20" s="25">
+        <v>1</v>
+      </c>
+      <c r="N20" s="28">
         <f>'NK-LK Transf.'!V12</f>
         <v>4.054398148148148E-4</v>
       </c>
-      <c r="N20" s="28">
+      <c r="O20" s="28">
         <f>'NK-LK Transf.'!V14</f>
         <v>6.2719907407407407E-4</v>
       </c>
-      <c r="O20" s="28">
+      <c r="P20" s="28">
         <f>'NK-LK Transf.'!V13</f>
         <v>8.2974537037037034E-4</v>
       </c>
-      <c r="P20" s="28">
+      <c r="Q20" s="28">
         <f>'NK-LK Transf.'!V15</f>
         <v>6.8842592592592588E-4</v>
       </c>
-      <c r="Q20" s="28">
+      <c r="R20" s="28">
         <f>'NK-LK Transf.'!V17</f>
         <v>1.6810185185185185E-3</v>
       </c>
-      <c r="R20" s="28">
+      <c r="S20" s="28">
         <f>'NK-LK Transf.'!V16</f>
         <v>1.558912037037037E-3</v>
       </c>
-      <c r="S20" s="28"/>
       <c r="T20" s="28"/>
       <c r="U20" s="28"/>
       <c r="V20" s="28"/>
       <c r="W20" s="28"/>
       <c r="X20" s="28"/>
+      <c r="Y20" s="28"/>
     </row>
-    <row r="21" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A21" s="25" t="s">
         <v>243</v>
       </c>
@@ -14016,38 +14084,41 @@
       <c r="L21" s="25">
         <v>10</v>
       </c>
-      <c r="M21" s="28">
+      <c r="M21" s="25">
+        <v>1</v>
+      </c>
+      <c r="N21" s="28">
         <f>'NK-LK Transf.'!U12</f>
         <v>4.2048611111111111E-4</v>
       </c>
-      <c r="N21" s="28">
+      <c r="O21" s="28">
         <f>'NK-LK Transf.'!U14</f>
         <v>6.4594907407407407E-4</v>
       </c>
-      <c r="O21" s="28">
+      <c r="P21" s="28">
         <f>'NK-LK Transf.'!U13</f>
         <v>8.5960648148148148E-4</v>
       </c>
-      <c r="P21" s="28">
+      <c r="Q21" s="28">
         <f>'NK-LK Transf.'!U15</f>
         <v>7.1134259259259263E-4</v>
       </c>
-      <c r="Q21" s="28">
+      <c r="R21" s="28">
         <f>'NK-LK Transf.'!U17</f>
         <v>1.7174768518518518E-3</v>
       </c>
-      <c r="R21" s="28">
+      <c r="S21" s="28">
         <f>'NK-LK Transf.'!U16</f>
         <v>1.5817129629629629E-3</v>
       </c>
-      <c r="S21" s="28"/>
       <c r="T21" s="28"/>
       <c r="U21" s="28"/>
       <c r="V21" s="28"/>
       <c r="W21" s="28"/>
       <c r="X21" s="28"/>
+      <c r="Y21" s="28"/>
     </row>
-    <row r="22" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A22" s="25" t="s">
         <v>243</v>
       </c>
@@ -14080,38 +14151,41 @@
       <c r="L22" s="25">
         <v>10</v>
       </c>
-      <c r="M22" s="28">
+      <c r="M22" s="25">
+        <v>1</v>
+      </c>
+      <c r="N22" s="28">
         <f>'NK-LK Transf.'!T12</f>
         <v>4.4097222222222226E-4</v>
       </c>
-      <c r="N22" s="28">
+      <c r="O22" s="28">
         <f>'NK-LK Transf.'!T14</f>
         <v>6.7164351851851857E-4</v>
       </c>
-      <c r="O22" s="28">
+      <c r="P22" s="28">
         <f>'NK-LK Transf.'!T13</f>
         <v>9.0034722222222209E-4</v>
       </c>
-      <c r="P22" s="28">
+      <c r="Q22" s="28">
         <f>'NK-LK Transf.'!T15</f>
         <v>7.4259259259259254E-4</v>
       </c>
-      <c r="Q22" s="28">
+      <c r="R22" s="28">
         <f>'NK-LK Transf.'!T17</f>
         <v>1.767361111111111E-3</v>
       </c>
-      <c r="R22" s="28">
+      <c r="S22" s="28">
         <f>'NK-LK Transf.'!T16</f>
         <v>1.6129629629629632E-3</v>
       </c>
-      <c r="S22" s="28"/>
       <c r="T22" s="28"/>
       <c r="U22" s="28"/>
       <c r="V22" s="28"/>
       <c r="W22" s="28"/>
       <c r="X22" s="28"/>
+      <c r="Y22" s="28"/>
     </row>
-    <row r="23" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A23" s="25" t="s">
         <v>243</v>
       </c>
@@ -14144,38 +14218,41 @@
       <c r="L23" s="25">
         <v>10</v>
       </c>
-      <c r="M23" s="28">
+      <c r="M23" s="25">
+        <v>1</v>
+      </c>
+      <c r="N23" s="28">
         <f>'NK-LK Transf.'!S12</f>
         <v>4.5138888888888887E-4</v>
       </c>
-      <c r="N23" s="28">
+      <c r="O23" s="28">
         <f>'NK-LK Transf.'!S14</f>
         <v>6.8449074074074072E-4</v>
       </c>
-      <c r="O23" s="28">
+      <c r="P23" s="28">
         <f>'NK-LK Transf.'!S13</f>
         <v>9.2094907407407403E-4</v>
       </c>
-      <c r="P23" s="28">
+      <c r="Q23" s="28">
         <f>'NK-LK Transf.'!S15</f>
         <v>7.583333333333333E-4</v>
       </c>
-      <c r="Q23" s="28">
+      <c r="R23" s="28">
         <f>'NK-LK Transf.'!S17</f>
         <v>1.7916666666666669E-3</v>
       </c>
-      <c r="R23" s="28">
+      <c r="S23" s="28">
         <f>'NK-LK Transf.'!S16</f>
         <v>1.6278935185185185E-3</v>
       </c>
-      <c r="S23" s="28"/>
       <c r="T23" s="28"/>
       <c r="U23" s="28"/>
       <c r="V23" s="28"/>
       <c r="W23" s="28"/>
       <c r="X23" s="28"/>
+      <c r="Y23" s="28"/>
     </row>
-    <row r="24" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A24" s="25" t="s">
         <v>243</v>
       </c>
@@ -14208,38 +14285,41 @@
       <c r="L24" s="25">
         <v>10</v>
       </c>
-      <c r="M24" s="28">
+      <c r="M24" s="25">
+        <v>1</v>
+      </c>
+      <c r="N24" s="28">
         <f>'NK-LK Transf.'!R12</f>
         <v>4.586805555555556E-4</v>
       </c>
-      <c r="N24" s="28">
+      <c r="O24" s="28">
         <f>'NK-LK Transf.'!R14</f>
         <v>6.9837962962962963E-4</v>
       </c>
-      <c r="O24" s="28">
+      <c r="P24" s="28">
         <f>'NK-LK Transf.'!R13</f>
         <v>9.4340277777777782E-4</v>
       </c>
-      <c r="P24" s="28">
+      <c r="Q24" s="28">
         <f>'NK-LK Transf.'!R15</f>
         <v>7.7534722222222219E-4</v>
       </c>
-      <c r="Q24" s="28">
+      <c r="R24" s="28">
         <f>'NK-LK Transf.'!R17</f>
         <v>1.8180555555555554E-3</v>
       </c>
-      <c r="R24" s="28">
+      <c r="S24" s="28">
         <f>'NK-LK Transf.'!R16</f>
         <v>1.644212962962963E-3</v>
       </c>
-      <c r="S24" s="28"/>
       <c r="T24" s="28"/>
       <c r="U24" s="28"/>
       <c r="V24" s="28"/>
       <c r="W24" s="28"/>
       <c r="X24" s="28"/>
+      <c r="Y24" s="28"/>
     </row>
-    <row r="25" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A25" s="25" t="s">
         <v>244</v>
       </c>
@@ -14272,38 +14352,41 @@
       <c r="L25" s="25">
         <v>10</v>
       </c>
-      <c r="M25" s="28">
+      <c r="M25" s="25">
+        <v>1</v>
+      </c>
+      <c r="N25" s="28">
         <f>'NK-LK Transf.'!J12</f>
         <v>3.3900462962962964E-4</v>
       </c>
-      <c r="N25" s="28">
+      <c r="O25" s="28">
         <f>'NK-LK Transf.'!J14</f>
         <v>5.3935185185185184E-4</v>
       </c>
-      <c r="O25" s="28">
+      <c r="P25" s="28">
         <f>'NK-LK Transf.'!J13</f>
         <v>7.1921296296296295E-4</v>
       </c>
-      <c r="P25" s="28">
+      <c r="Q25" s="28">
         <f>'NK-LK Transf.'!J15</f>
         <v>5.9317129629629629E-4</v>
       </c>
-      <c r="Q25" s="28">
+      <c r="R25" s="28">
         <f>'NK-LK Transf.'!J17</f>
         <v>1.5422453703703705E-3</v>
       </c>
-      <c r="R25" s="28">
+      <c r="S25" s="28">
         <f>'NK-LK Transf.'!J16</f>
         <v>1.3815972222222222E-3</v>
       </c>
-      <c r="S25" s="28"/>
       <c r="T25" s="28"/>
       <c r="U25" s="28"/>
       <c r="V25" s="28"/>
       <c r="W25" s="28"/>
       <c r="X25" s="28"/>
+      <c r="Y25" s="28"/>
     </row>
-    <row r="26" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A26" s="25" t="s">
         <v>244</v>
       </c>
@@ -14336,38 +14419,41 @@
       <c r="L26" s="25">
         <v>10</v>
       </c>
-      <c r="M26" s="28">
+      <c r="M26" s="25">
+        <v>1</v>
+      </c>
+      <c r="N26" s="28">
         <f>'NK-LK Transf.'!I12</f>
         <v>3.5081018518518518E-4</v>
       </c>
-      <c r="N26" s="28">
+      <c r="O26" s="28">
         <f>'NK-LK Transf.'!I14</f>
         <v>5.5659722222222222E-4</v>
       </c>
-      <c r="O26" s="28">
+      <c r="P26" s="28">
         <f>'NK-LK Transf.'!I13</f>
         <v>7.4733796296296289E-4</v>
       </c>
-      <c r="P26" s="28">
+      <c r="Q26" s="28">
         <f>'NK-LK Transf.'!I15</f>
         <v>6.1886574074074068E-4</v>
       </c>
-      <c r="Q26" s="28">
+      <c r="R26" s="28">
         <f>'NK-LK Transf.'!I17</f>
         <v>1.590625E-3</v>
       </c>
-      <c r="R26" s="28">
+      <c r="S26" s="28">
         <f>'NK-LK Transf.'!I16</f>
         <v>1.4285879629629631E-3</v>
       </c>
-      <c r="S26" s="28"/>
       <c r="T26" s="28"/>
       <c r="U26" s="28"/>
       <c r="V26" s="28"/>
       <c r="W26" s="28"/>
       <c r="X26" s="28"/>
+      <c r="Y26" s="28"/>
     </row>
-    <row r="27" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A27" s="25" t="s">
         <v>244</v>
       </c>
@@ -14400,38 +14486,41 @@
       <c r="L27" s="25">
         <v>10</v>
       </c>
-      <c r="M27" s="28">
+      <c r="M27" s="25">
+        <v>1</v>
+      </c>
+      <c r="N27" s="28">
         <f>'NK-LK Transf.'!H12</f>
         <v>3.6111111111111109E-4</v>
       </c>
-      <c r="N27" s="28">
+      <c r="O27" s="28">
         <f>'NK-LK Transf.'!H14</f>
         <v>5.7175925925925927E-4</v>
       </c>
-      <c r="O27" s="28">
+      <c r="P27" s="28">
         <f>'NK-LK Transf.'!H13</f>
         <v>7.7187499999999999E-4</v>
       </c>
-      <c r="P27" s="28">
+      <c r="Q27" s="28">
         <f>'NK-LK Transf.'!H15</f>
         <v>6.4131944444444436E-4</v>
       </c>
-      <c r="Q27" s="28">
+      <c r="R27" s="28">
         <f>'NK-LK Transf.'!H17</f>
         <v>1.60625E-3</v>
       </c>
-      <c r="R27" s="28">
+      <c r="S27" s="28">
         <f>'NK-LK Transf.'!H16</f>
         <v>1.4697916666666666E-3</v>
       </c>
-      <c r="S27" s="28"/>
       <c r="T27" s="28"/>
       <c r="U27" s="28"/>
       <c r="V27" s="28"/>
       <c r="W27" s="28"/>
       <c r="X27" s="28"/>
+      <c r="Y27" s="28"/>
     </row>
-    <row r="28" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A28" s="25" t="s">
         <v>244</v>
       </c>
@@ -14464,38 +14553,41 @@
       <c r="L28" s="25">
         <v>10</v>
       </c>
-      <c r="M28" s="28">
+      <c r="M28" s="25">
+        <v>1</v>
+      </c>
+      <c r="N28" s="28">
         <f>'NK-LK Transf.'!G12</f>
         <v>3.6747685185185185E-4</v>
       </c>
-      <c r="N28" s="28">
+      <c r="O28" s="28">
         <f>'NK-LK Transf.'!G14</f>
         <v>5.8101851851851858E-4</v>
       </c>
-      <c r="O28" s="28">
+      <c r="P28" s="28">
         <f>'NK-LK Transf.'!G13</f>
         <v>7.8715277777777779E-4</v>
       </c>
-      <c r="P28" s="28">
+      <c r="Q28" s="28">
         <f>'NK-LK Transf.'!G15</f>
         <v>6.5532407407407401E-4</v>
       </c>
-      <c r="Q28" s="28">
+      <c r="R28" s="28">
         <f>'NK-LK Transf.'!G17</f>
         <v>1.6241898148148146E-3</v>
       </c>
-      <c r="R28" s="28">
+      <c r="S28" s="28">
         <f>'NK-LK Transf.'!G16</f>
         <v>1.4950231481481481E-3</v>
       </c>
-      <c r="S28" s="28"/>
       <c r="T28" s="28"/>
       <c r="U28" s="28"/>
       <c r="V28" s="28"/>
       <c r="W28" s="28"/>
       <c r="X28" s="28"/>
+      <c r="Y28" s="28"/>
     </row>
-    <row r="29" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A29" s="25" t="s">
         <v>244</v>
       </c>
@@ -14528,38 +14620,41 @@
       <c r="L29" s="25">
         <v>10</v>
       </c>
-      <c r="M29" s="28">
+      <c r="M29" s="25">
+        <v>1</v>
+      </c>
+      <c r="N29" s="28">
         <f>'NK-LK Transf.'!F12</f>
         <v>3.7430555555555562E-4</v>
       </c>
-      <c r="N29" s="28">
+      <c r="O29" s="28">
         <f>'NK-LK Transf.'!F14</f>
         <v>5.9097222222222222E-4</v>
       </c>
-      <c r="O29" s="28">
+      <c r="P29" s="28">
         <f>'NK-LK Transf.'!F13</f>
         <v>8.0358796296296309E-4</v>
       </c>
-      <c r="P29" s="28">
+      <c r="Q29" s="28">
         <f>'NK-LK Transf.'!F15</f>
         <v>6.7048611111111107E-4</v>
       </c>
-      <c r="Q29" s="28">
+      <c r="R29" s="28">
         <f>'NK-LK Transf.'!F17</f>
         <v>1.6435185185185185E-3</v>
       </c>
-      <c r="R29" s="28">
+      <c r="S29" s="28">
         <f>'NK-LK Transf.'!F16</f>
         <v>1.522337962962963E-3</v>
       </c>
-      <c r="S29" s="28"/>
       <c r="T29" s="28"/>
       <c r="U29" s="28"/>
       <c r="V29" s="28"/>
       <c r="W29" s="28"/>
       <c r="X29" s="28"/>
+      <c r="Y29" s="28"/>
     </row>
-    <row r="30" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A30" s="25" t="s">
         <v>245</v>
       </c>
@@ -14592,38 +14687,41 @@
       <c r="L30" s="25">
         <v>10</v>
       </c>
-      <c r="M30" s="28">
+      <c r="M30" s="25">
+        <v>1</v>
+      </c>
+      <c r="N30" s="28">
         <f>'NK-LK Transf.'!Z12</f>
         <v>4.0069444444444441E-4</v>
       </c>
-      <c r="N30" s="28">
+      <c r="O30" s="28">
         <f>'NK-LK Transf.'!Z14</f>
         <v>6.2129629629629633E-4</v>
       </c>
-      <c r="O30" s="28">
+      <c r="P30" s="28">
         <f>'NK-LK Transf.'!Z13</f>
         <v>8.2037037037037029E-4</v>
       </c>
-      <c r="P30" s="28">
+      <c r="Q30" s="28">
         <f>'NK-LK Transf.'!Z15</f>
         <v>6.8125E-4</v>
       </c>
-      <c r="Q30" s="28">
+      <c r="R30" s="28">
         <f>'NK-LK Transf.'!Z17</f>
         <v>1.6695601851851852E-3</v>
       </c>
-      <c r="R30" s="28">
+      <c r="S30" s="28">
         <f>'NK-LK Transf.'!Z16</f>
         <v>1.5517361111111109E-3</v>
       </c>
-      <c r="S30" s="28"/>
       <c r="T30" s="28"/>
       <c r="U30" s="28"/>
       <c r="V30" s="28"/>
       <c r="W30" s="28"/>
       <c r="X30" s="28"/>
+      <c r="Y30" s="28"/>
     </row>
-    <row r="31" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A31" s="25" t="s">
         <v>245</v>
       </c>
@@ -14656,38 +14754,41 @@
       <c r="L31" s="25">
         <v>10</v>
       </c>
-      <c r="M31" s="28">
+      <c r="M31" s="25">
+        <v>1</v>
+      </c>
+      <c r="N31" s="28">
         <f>'NK-LK Transf.'!Y12</f>
         <v>4.0381944444444444E-4</v>
       </c>
-      <c r="N31" s="28">
+      <c r="O31" s="28">
         <f>'NK-LK Transf.'!Y14</f>
         <v>6.2523148148148149E-4</v>
       </c>
-      <c r="O31" s="28">
+      <c r="P31" s="28">
         <f>'NK-LK Transf.'!Y13</f>
         <v>8.2662037037037036E-4</v>
       </c>
-      <c r="P31" s="28">
+      <c r="Q31" s="28">
         <f>'NK-LK Transf.'!Y15</f>
         <v>6.8611111111111108E-4</v>
       </c>
-      <c r="Q31" s="28">
+      <c r="R31" s="28">
         <f>'NK-LK Transf.'!Y17</f>
         <v>1.677199074074074E-3</v>
       </c>
-      <c r="R31" s="28">
+      <c r="S31" s="28">
         <f>'NK-LK Transf.'!Y16</f>
         <v>1.5564814814814814E-3</v>
       </c>
-      <c r="S31" s="28"/>
       <c r="T31" s="28"/>
       <c r="U31" s="28"/>
       <c r="V31" s="28"/>
       <c r="W31" s="28"/>
       <c r="X31" s="28"/>
+      <c r="Y31" s="28"/>
     </row>
-    <row r="32" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A32" s="25" t="s">
         <v>245</v>
       </c>
@@ -14720,38 +14821,41 @@
       <c r="L32" s="25">
         <v>10</v>
       </c>
-      <c r="M32" s="28">
+      <c r="M32" s="25">
+        <v>1</v>
+      </c>
+      <c r="N32" s="28">
         <f>'NK-LK Transf.'!X12</f>
         <v>4.1331018518518518E-4</v>
       </c>
-      <c r="N32" s="28">
+      <c r="O32" s="28">
         <f>'NK-LK Transf.'!X14</f>
         <v>6.3703703703703698E-4</v>
       </c>
-      <c r="O32" s="28">
+      <c r="P32" s="28">
         <f>'NK-LK Transf.'!X13</f>
         <v>8.4548611111111109E-4</v>
       </c>
-      <c r="P32" s="28">
+      <c r="Q32" s="28">
         <f>'NK-LK Transf.'!X15</f>
         <v>7.0046296296296295E-4</v>
       </c>
-      <c r="Q32" s="28">
+      <c r="R32" s="28">
         <f>'NK-LK Transf.'!X17</f>
         <v>1.7002314814814816E-3</v>
       </c>
-      <c r="R32" s="28">
+      <c r="S32" s="28">
         <f>'NK-LK Transf.'!X16</f>
         <v>1.570949074074074E-3</v>
       </c>
-      <c r="S32" s="28"/>
       <c r="T32" s="28"/>
       <c r="U32" s="28"/>
       <c r="V32" s="28"/>
       <c r="W32" s="28"/>
       <c r="X32" s="28"/>
+      <c r="Y32" s="28"/>
     </row>
-    <row r="33" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A33" s="25" t="s">
         <v>245</v>
       </c>
@@ -14784,38 +14888,41 @@
       <c r="L33" s="25">
         <v>10</v>
       </c>
-      <c r="M33" s="28">
+      <c r="M33" s="25">
+        <v>1</v>
+      </c>
+      <c r="N33" s="28">
         <f>'NK-LK Transf.'!W12</f>
         <v>4.2118055555555555E-4</v>
       </c>
-      <c r="N33" s="28">
+      <c r="O33" s="28">
         <f>'NK-LK Transf.'!W14</f>
         <v>6.4699074074074073E-4</v>
       </c>
-      <c r="O33" s="28">
+      <c r="P33" s="28">
         <f>'NK-LK Transf.'!W13</f>
         <v>8.6111111111111121E-4</v>
       </c>
-      <c r="P33" s="28">
+      <c r="Q33" s="28">
         <f>'NK-LK Transf.'!W15</f>
         <v>7.1250000000000003E-4</v>
       </c>
-      <c r="Q33" s="28">
+      <c r="R33" s="28">
         <f>'NK-LK Transf.'!W17</f>
         <v>1.7194444444444444E-3</v>
       </c>
-      <c r="R33" s="28">
+      <c r="S33" s="28">
         <f>'NK-LK Transf.'!W16</f>
         <v>1.5829861111111112E-3</v>
       </c>
-      <c r="S33" s="28"/>
       <c r="T33" s="28"/>
       <c r="U33" s="28"/>
       <c r="V33" s="28"/>
       <c r="W33" s="28"/>
       <c r="X33" s="28"/>
+      <c r="Y33" s="28"/>
     </row>
-    <row r="34" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A34" s="25" t="s">
         <v>246</v>
       </c>
@@ -14848,38 +14955,41 @@
       <c r="L34" s="25">
         <v>10</v>
       </c>
-      <c r="M34" s="28">
+      <c r="M34" s="25">
+        <v>1</v>
+      </c>
+      <c r="N34" s="28">
         <f>'NK-LK Transf.'!N12</f>
         <v>3.359953703703704E-4</v>
       </c>
-      <c r="N34" s="28">
+      <c r="O34" s="28">
         <f>'NK-LK Transf.'!N14</f>
         <v>5.3506944444444446E-4</v>
       </c>
-      <c r="O34" s="28">
+      <c r="P34" s="28">
         <f>'NK-LK Transf.'!N13</f>
         <v>7.1215277777777781E-4</v>
       </c>
-      <c r="P34" s="28">
+      <c r="Q34" s="28">
         <f>'NK-LK Transf.'!N15</f>
         <v>5.8680555555555558E-4</v>
       </c>
-      <c r="Q34" s="28">
+      <c r="R34" s="28">
         <f>'NK-LK Transf.'!N17</f>
         <v>1.4912037037037038E-3</v>
       </c>
-      <c r="R34" s="28">
+      <c r="S34" s="28">
         <f>'NK-LK Transf.'!N16</f>
         <v>1.3697916666666665E-3</v>
       </c>
-      <c r="S34" s="28"/>
       <c r="T34" s="28"/>
       <c r="U34" s="28"/>
       <c r="V34" s="28"/>
       <c r="W34" s="28"/>
       <c r="X34" s="28"/>
+      <c r="Y34" s="28"/>
     </row>
-    <row r="35" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A35" s="25" t="s">
         <v>246</v>
       </c>
@@ -14912,38 +15022,41 @@
       <c r="L35" s="25">
         <v>10</v>
       </c>
-      <c r="M35" s="28">
+      <c r="M35" s="25">
+        <v>1</v>
+      </c>
+      <c r="N35" s="28">
         <f>'NK-LK Transf.'!M12</f>
         <v>3.3796296296296298E-4</v>
       </c>
-      <c r="N35" s="28">
+      <c r="O35" s="28">
         <f>'NK-LK Transf.'!M14</f>
         <v>5.3796296296296296E-4</v>
       </c>
-      <c r="O35" s="28">
+      <c r="P35" s="28">
         <f>'NK-LK Transf.'!M13</f>
         <v>7.1678240740740741E-4</v>
       </c>
-      <c r="P35" s="28">
+      <c r="Q35" s="28">
         <f>'NK-LK Transf.'!M15</f>
         <v>5.9108796296296296E-4</v>
       </c>
-      <c r="Q35" s="28">
+      <c r="R35" s="28">
         <f>'NK-LK Transf.'!M17</f>
         <v>1.5002314814814815E-3</v>
       </c>
-      <c r="R35" s="28">
+      <c r="S35" s="28">
         <f>'NK-LK Transf.'!M16</f>
         <v>1.377662037037037E-3</v>
       </c>
-      <c r="S35" s="28"/>
       <c r="T35" s="28"/>
       <c r="U35" s="28"/>
       <c r="V35" s="28"/>
       <c r="W35" s="28"/>
       <c r="X35" s="28"/>
+      <c r="Y35" s="28"/>
     </row>
-    <row r="36" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A36" s="25" t="s">
         <v>246</v>
       </c>
@@ -14976,38 +15089,41 @@
       <c r="L36" s="25">
         <v>10</v>
       </c>
-      <c r="M36" s="28">
+      <c r="M36" s="25">
+        <v>1</v>
+      </c>
+      <c r="N36" s="28">
         <f>'NK-LK Transf.'!L12</f>
         <v>3.4386574074074077E-4</v>
       </c>
-      <c r="N36" s="28">
+      <c r="O36" s="28">
         <f>'NK-LK Transf.'!L14</f>
         <v>5.4652777777777772E-4</v>
       </c>
-      <c r="O36" s="28">
+      <c r="P36" s="28">
         <f>'NK-LK Transf.'!L13</f>
         <v>7.309027777777778E-4</v>
       </c>
-      <c r="P36" s="28">
+      <c r="Q36" s="28">
         <f>'NK-LK Transf.'!L15</f>
         <v>6.0393518518518522E-4</v>
       </c>
-      <c r="Q36" s="28">
+      <c r="R36" s="28">
         <f>'NK-LK Transf.'!L17</f>
         <v>1.5273148148148149E-3</v>
       </c>
-      <c r="R36" s="28">
+      <c r="S36" s="28">
         <f>'NK-LK Transf.'!L16</f>
         <v>1.4011574074074074E-3</v>
       </c>
-      <c r="S36" s="28"/>
       <c r="T36" s="28"/>
       <c r="U36" s="28"/>
       <c r="V36" s="28"/>
       <c r="W36" s="28"/>
       <c r="X36" s="28"/>
+      <c r="Y36" s="28"/>
     </row>
-    <row r="37" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A37" s="25" t="s">
         <v>246</v>
       </c>
@@ -15040,36 +15156,39 @@
       <c r="L37" s="25">
         <v>10</v>
       </c>
-      <c r="M37" s="28">
+      <c r="M37" s="25">
+        <v>1</v>
+      </c>
+      <c r="N37" s="28">
         <f>'NK-LK Transf.'!K12</f>
         <v>3.488425925925926E-4</v>
       </c>
-      <c r="N37" s="28">
+      <c r="O37" s="28">
         <f>'NK-LK Transf.'!K14</f>
         <v>5.5381944444444445E-4</v>
       </c>
-      <c r="O37" s="28">
+      <c r="P37" s="28">
         <f>'NK-LK Transf.'!K13</f>
         <v>7.4259259259259254E-4</v>
       </c>
-      <c r="P37" s="28">
+      <c r="Q37" s="28">
         <f>'NK-LK Transf.'!K15</f>
         <v>6.145833333333333E-4</v>
       </c>
-      <c r="Q37" s="28">
+      <c r="R37" s="28">
         <f>'NK-LK Transf.'!K17</f>
         <v>1.5498842592592593E-3</v>
       </c>
-      <c r="R37" s="28">
+      <c r="S37" s="28">
         <f>'NK-LK Transf.'!K16</f>
         <v>1.4207175925925926E-3</v>
       </c>
-      <c r="S37" s="28"/>
       <c r="T37" s="28"/>
       <c r="U37" s="28"/>
       <c r="V37" s="28"/>
       <c r="W37" s="28"/>
       <c r="X37" s="28"/>
+      <c r="Y37" s="28"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
@@ -15096,133 +15215,133 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:78" s="40" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="106">
+      <c r="A1" s="125">
         <v>2025</v>
       </c>
       <c r="B1" s="45" t="str">
         <f ca="1">CONCATENATE("in: ",YEAR(TODAY())-1," für: ", YEAR(TODAY()))</f>
         <v>in: 2025 für: 2026</v>
       </c>
-      <c r="C1" s="107" t="s">
+      <c r="C1" s="106" t="s">
         <v>220</v>
       </c>
-      <c r="D1" s="107"/>
-      <c r="E1" s="108"/>
-      <c r="F1" s="109" t="s">
+      <c r="D1" s="106"/>
+      <c r="E1" s="107"/>
+      <c r="F1" s="110" t="s">
         <v>221</v>
       </c>
-      <c r="G1" s="110"/>
-      <c r="H1" s="110"/>
-      <c r="I1" s="110"/>
-      <c r="J1" s="111"/>
-      <c r="K1" s="112" t="s">
+      <c r="G1" s="111"/>
+      <c r="H1" s="111"/>
+      <c r="I1" s="111"/>
+      <c r="J1" s="112"/>
+      <c r="K1" s="116" t="s">
         <v>225</v>
       </c>
-      <c r="L1" s="113"/>
-      <c r="M1" s="113"/>
-      <c r="N1" s="114"/>
-      <c r="O1" s="132" t="s">
+      <c r="L1" s="117"/>
+      <c r="M1" s="117"/>
+      <c r="N1" s="118"/>
+      <c r="O1" s="108" t="s">
         <v>222</v>
       </c>
-      <c r="P1" s="132"/>
-      <c r="Q1" s="133"/>
-      <c r="R1" s="134" t="s">
+      <c r="P1" s="108"/>
+      <c r="Q1" s="109"/>
+      <c r="R1" s="122" t="s">
         <v>223</v>
       </c>
-      <c r="S1" s="135"/>
-      <c r="T1" s="135"/>
-      <c r="U1" s="135"/>
-      <c r="V1" s="136"/>
-      <c r="W1" s="137" t="s">
+      <c r="S1" s="123"/>
+      <c r="T1" s="123"/>
+      <c r="U1" s="123"/>
+      <c r="V1" s="124"/>
+      <c r="W1" s="119" t="s">
         <v>226</v>
       </c>
-      <c r="X1" s="138"/>
-      <c r="Y1" s="138"/>
-      <c r="Z1" s="139"/>
+      <c r="X1" s="120"/>
+      <c r="Y1" s="120"/>
+      <c r="Z1" s="121"/>
       <c r="AA1"/>
       <c r="AB1" s="45" t="str">
         <f ca="1">CONCATENATE("in: ",YEAR(TODAY())-1," für: ", YEAR(TODAY()))</f>
         <v>in: 2025 für: 2026</v>
       </c>
-      <c r="AC1" s="115" t="s">
+      <c r="AC1" s="126" t="s">
         <v>227</v>
       </c>
-      <c r="AD1" s="115"/>
-      <c r="AE1" s="116"/>
-      <c r="AF1" s="117" t="s">
+      <c r="AD1" s="126"/>
+      <c r="AE1" s="127"/>
+      <c r="AF1" s="128" t="s">
         <v>228</v>
       </c>
-      <c r="AG1" s="118"/>
-      <c r="AH1" s="118"/>
-      <c r="AI1" s="118"/>
-      <c r="AJ1" s="119"/>
-      <c r="AK1" s="120" t="s">
+      <c r="AG1" s="129"/>
+      <c r="AH1" s="129"/>
+      <c r="AI1" s="129"/>
+      <c r="AJ1" s="130"/>
+      <c r="AK1" s="131" t="s">
         <v>229</v>
       </c>
-      <c r="AL1" s="121"/>
-      <c r="AM1" s="121"/>
-      <c r="AN1" s="122"/>
-      <c r="AO1" s="123" t="s">
+      <c r="AL1" s="132"/>
+      <c r="AM1" s="132"/>
+      <c r="AN1" s="133"/>
+      <c r="AO1" s="134" t="s">
         <v>230</v>
       </c>
-      <c r="AP1" s="124"/>
-      <c r="AQ1" s="125"/>
-      <c r="AR1" s="126" t="s">
+      <c r="AP1" s="135"/>
+      <c r="AQ1" s="136"/>
+      <c r="AR1" s="137" t="s">
         <v>231</v>
       </c>
-      <c r="AS1" s="127"/>
-      <c r="AT1" s="127"/>
-      <c r="AU1" s="127"/>
-      <c r="AV1" s="128"/>
-      <c r="AW1" s="129" t="s">
+      <c r="AS1" s="138"/>
+      <c r="AT1" s="138"/>
+      <c r="AU1" s="138"/>
+      <c r="AV1" s="139"/>
+      <c r="AW1" s="113" t="s">
         <v>232</v>
       </c>
-      <c r="AX1" s="130"/>
-      <c r="AY1" s="130"/>
-      <c r="AZ1" s="131"/>
+      <c r="AX1" s="114"/>
+      <c r="AY1" s="114"/>
+      <c r="AZ1" s="115"/>
       <c r="BB1" s="45" t="str">
         <f ca="1">CONCATENATE("in: ",YEAR(TODAY())-1," für: ", YEAR(TODAY()))</f>
         <v>in: 2025 für: 2026</v>
       </c>
-      <c r="BC1" s="107" t="s">
+      <c r="BC1" s="106" t="s">
         <v>233</v>
       </c>
-      <c r="BD1" s="107"/>
-      <c r="BE1" s="108"/>
-      <c r="BF1" s="109" t="s">
+      <c r="BD1" s="106"/>
+      <c r="BE1" s="107"/>
+      <c r="BF1" s="110" t="s">
         <v>234</v>
       </c>
-      <c r="BG1" s="110"/>
-      <c r="BH1" s="110"/>
-      <c r="BI1" s="110"/>
-      <c r="BJ1" s="111"/>
-      <c r="BK1" s="112" t="s">
+      <c r="BG1" s="111"/>
+      <c r="BH1" s="111"/>
+      <c r="BI1" s="111"/>
+      <c r="BJ1" s="112"/>
+      <c r="BK1" s="116" t="s">
         <v>235</v>
       </c>
-      <c r="BL1" s="113"/>
-      <c r="BM1" s="113"/>
-      <c r="BN1" s="114"/>
-      <c r="BO1" s="132" t="s">
+      <c r="BL1" s="117"/>
+      <c r="BM1" s="117"/>
+      <c r="BN1" s="118"/>
+      <c r="BO1" s="108" t="s">
         <v>241</v>
       </c>
-      <c r="BP1" s="132"/>
-      <c r="BQ1" s="133"/>
-      <c r="BR1" s="134" t="s">
+      <c r="BP1" s="108"/>
+      <c r="BQ1" s="109"/>
+      <c r="BR1" s="122" t="s">
         <v>242</v>
       </c>
-      <c r="BS1" s="135"/>
-      <c r="BT1" s="135"/>
-      <c r="BU1" s="135"/>
-      <c r="BV1" s="136"/>
-      <c r="BW1" s="137" t="s">
+      <c r="BS1" s="123"/>
+      <c r="BT1" s="123"/>
+      <c r="BU1" s="123"/>
+      <c r="BV1" s="124"/>
+      <c r="BW1" s="119" t="s">
         <v>236</v>
       </c>
-      <c r="BX1" s="138"/>
-      <c r="BY1" s="138"/>
-      <c r="BZ1" s="139"/>
+      <c r="BX1" s="120"/>
+      <c r="BY1" s="120"/>
+      <c r="BZ1" s="121"/>
     </row>
     <row r="2" spans="1:78" s="94" customFormat="1" ht="21.4" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="106"/>
+      <c r="A2" s="125"/>
       <c r="B2" s="46" t="s">
         <v>224</v>
       </c>
@@ -15523,7 +15642,7 @@
       </c>
     </row>
     <row r="3" spans="1:78" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A3" s="106"/>
+      <c r="A3" s="125"/>
       <c r="B3" s="47" t="s">
         <v>0</v>
       </c>
@@ -15776,7 +15895,7 @@
       </c>
     </row>
     <row r="4" spans="1:78" x14ac:dyDescent="0.45">
-      <c r="A4" s="106"/>
+      <c r="A4" s="125"/>
       <c r="B4" s="47" t="s">
         <v>185</v>
       </c>
@@ -16028,7 +16147,7 @@
       </c>
     </row>
     <row r="5" spans="1:78" x14ac:dyDescent="0.45">
-      <c r="A5" s="106"/>
+      <c r="A5" s="125"/>
       <c r="B5" s="47" t="s">
         <v>186</v>
       </c>
@@ -16280,7 +16399,7 @@
       </c>
     </row>
     <row r="6" spans="1:78" x14ac:dyDescent="0.45">
-      <c r="A6" s="106"/>
+      <c r="A6" s="125"/>
       <c r="B6" s="47" t="s">
         <v>187</v>
       </c>
@@ -16532,7 +16651,7 @@
       </c>
     </row>
     <row r="7" spans="1:78" x14ac:dyDescent="0.45">
-      <c r="A7" s="106"/>
+      <c r="A7" s="125"/>
       <c r="B7" s="47" t="s">
         <v>188</v>
       </c>
@@ -16784,7 +16903,7 @@
       </c>
     </row>
     <row r="8" spans="1:78" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A8" s="106"/>
+      <c r="A8" s="125"/>
       <c r="B8" s="50" t="s">
         <v>4</v>
       </c>
@@ -17037,132 +17156,132 @@
     </row>
     <row r="9" spans="1:78" ht="14.65" thickTop="1" x14ac:dyDescent="0.45"/>
     <row r="10" spans="1:78" ht="18" x14ac:dyDescent="0.45">
-      <c r="A10" s="106">
+      <c r="A10" s="125">
         <v>2026</v>
       </c>
       <c r="B10" s="45" t="str">
         <f ca="1">CONCATENATE("in: ",YEAR(TODAY())," für: ", YEAR(TODAY())+1)</f>
         <v>in: 2026 für: 2027</v>
       </c>
-      <c r="C10" s="107" t="s">
+      <c r="C10" s="106" t="s">
         <v>220</v>
       </c>
-      <c r="D10" s="107"/>
-      <c r="E10" s="108"/>
-      <c r="F10" s="109" t="s">
+      <c r="D10" s="106"/>
+      <c r="E10" s="107"/>
+      <c r="F10" s="110" t="s">
         <v>221</v>
       </c>
-      <c r="G10" s="110"/>
-      <c r="H10" s="110"/>
-      <c r="I10" s="110"/>
-      <c r="J10" s="111"/>
-      <c r="K10" s="112" t="s">
+      <c r="G10" s="111"/>
+      <c r="H10" s="111"/>
+      <c r="I10" s="111"/>
+      <c r="J10" s="112"/>
+      <c r="K10" s="116" t="s">
         <v>225</v>
       </c>
-      <c r="L10" s="113"/>
-      <c r="M10" s="113"/>
-      <c r="N10" s="114"/>
-      <c r="O10" s="132" t="s">
+      <c r="L10" s="117"/>
+      <c r="M10" s="117"/>
+      <c r="N10" s="118"/>
+      <c r="O10" s="108" t="s">
         <v>222</v>
       </c>
-      <c r="P10" s="132"/>
-      <c r="Q10" s="133"/>
-      <c r="R10" s="134" t="s">
+      <c r="P10" s="108"/>
+      <c r="Q10" s="109"/>
+      <c r="R10" s="122" t="s">
         <v>223</v>
       </c>
-      <c r="S10" s="135"/>
-      <c r="T10" s="135"/>
-      <c r="U10" s="135"/>
-      <c r="V10" s="136"/>
-      <c r="W10" s="137" t="s">
+      <c r="S10" s="123"/>
+      <c r="T10" s="123"/>
+      <c r="U10" s="123"/>
+      <c r="V10" s="124"/>
+      <c r="W10" s="119" t="s">
         <v>226</v>
       </c>
-      <c r="X10" s="138"/>
-      <c r="Y10" s="138"/>
-      <c r="Z10" s="139"/>
+      <c r="X10" s="120"/>
+      <c r="Y10" s="120"/>
+      <c r="Z10" s="121"/>
       <c r="AB10" s="45" t="str">
         <f ca="1">CONCATENATE("in: ",YEAR(TODAY())," für: ", YEAR(TODAY())+1)</f>
         <v>in: 2026 für: 2027</v>
       </c>
-      <c r="AC10" s="115" t="s">
+      <c r="AC10" s="126" t="s">
         <v>227</v>
       </c>
-      <c r="AD10" s="115"/>
-      <c r="AE10" s="116"/>
-      <c r="AF10" s="117" t="s">
+      <c r="AD10" s="126"/>
+      <c r="AE10" s="127"/>
+      <c r="AF10" s="128" t="s">
         <v>228</v>
       </c>
-      <c r="AG10" s="118"/>
-      <c r="AH10" s="118"/>
-      <c r="AI10" s="118"/>
-      <c r="AJ10" s="119"/>
-      <c r="AK10" s="120" t="s">
+      <c r="AG10" s="129"/>
+      <c r="AH10" s="129"/>
+      <c r="AI10" s="129"/>
+      <c r="AJ10" s="130"/>
+      <c r="AK10" s="131" t="s">
         <v>229</v>
       </c>
-      <c r="AL10" s="121"/>
-      <c r="AM10" s="121"/>
-      <c r="AN10" s="122"/>
-      <c r="AO10" s="123" t="s">
+      <c r="AL10" s="132"/>
+      <c r="AM10" s="132"/>
+      <c r="AN10" s="133"/>
+      <c r="AO10" s="134" t="s">
         <v>230</v>
       </c>
-      <c r="AP10" s="124"/>
-      <c r="AQ10" s="125"/>
-      <c r="AR10" s="126" t="s">
+      <c r="AP10" s="135"/>
+      <c r="AQ10" s="136"/>
+      <c r="AR10" s="137" t="s">
         <v>231</v>
       </c>
-      <c r="AS10" s="127"/>
-      <c r="AT10" s="127"/>
-      <c r="AU10" s="127"/>
-      <c r="AV10" s="128"/>
-      <c r="AW10" s="129" t="s">
+      <c r="AS10" s="138"/>
+      <c r="AT10" s="138"/>
+      <c r="AU10" s="138"/>
+      <c r="AV10" s="139"/>
+      <c r="AW10" s="113" t="s">
         <v>232</v>
       </c>
-      <c r="AX10" s="130"/>
-      <c r="AY10" s="130"/>
-      <c r="AZ10" s="131"/>
+      <c r="AX10" s="114"/>
+      <c r="AY10" s="114"/>
+      <c r="AZ10" s="115"/>
       <c r="BB10" s="45" t="str">
         <f ca="1">CONCATENATE("in: ",YEAR(TODAY())," für: ", YEAR(TODAY())+1)</f>
         <v>in: 2026 für: 2027</v>
       </c>
-      <c r="BC10" s="107" t="s">
+      <c r="BC10" s="106" t="s">
         <v>233</v>
       </c>
-      <c r="BD10" s="107"/>
-      <c r="BE10" s="108"/>
-      <c r="BF10" s="109" t="s">
+      <c r="BD10" s="106"/>
+      <c r="BE10" s="107"/>
+      <c r="BF10" s="110" t="s">
         <v>234</v>
       </c>
-      <c r="BG10" s="110"/>
-      <c r="BH10" s="110"/>
-      <c r="BI10" s="110"/>
-      <c r="BJ10" s="111"/>
-      <c r="BK10" s="112" t="s">
+      <c r="BG10" s="111"/>
+      <c r="BH10" s="111"/>
+      <c r="BI10" s="111"/>
+      <c r="BJ10" s="112"/>
+      <c r="BK10" s="116" t="s">
         <v>235</v>
       </c>
-      <c r="BL10" s="113"/>
-      <c r="BM10" s="113"/>
-      <c r="BN10" s="114"/>
-      <c r="BO10" s="132" t="s">
+      <c r="BL10" s="117"/>
+      <c r="BM10" s="117"/>
+      <c r="BN10" s="118"/>
+      <c r="BO10" s="108" t="s">
         <v>241</v>
       </c>
-      <c r="BP10" s="132"/>
-      <c r="BQ10" s="133"/>
-      <c r="BR10" s="134" t="s">
+      <c r="BP10" s="108"/>
+      <c r="BQ10" s="109"/>
+      <c r="BR10" s="122" t="s">
         <v>242</v>
       </c>
-      <c r="BS10" s="135"/>
-      <c r="BT10" s="135"/>
-      <c r="BU10" s="135"/>
-      <c r="BV10" s="136"/>
-      <c r="BW10" s="137" t="s">
+      <c r="BS10" s="123"/>
+      <c r="BT10" s="123"/>
+      <c r="BU10" s="123"/>
+      <c r="BV10" s="124"/>
+      <c r="BW10" s="119" t="s">
         <v>236</v>
       </c>
-      <c r="BX10" s="138"/>
-      <c r="BY10" s="138"/>
-      <c r="BZ10" s="139"/>
+      <c r="BX10" s="120"/>
+      <c r="BY10" s="120"/>
+      <c r="BZ10" s="121"/>
     </row>
     <row r="11" spans="1:78" ht="21.4" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A11" s="106"/>
+      <c r="A11" s="125"/>
       <c r="B11" s="46" t="s">
         <v>224</v>
       </c>
@@ -17463,7 +17582,7 @@
       </c>
     </row>
     <row r="12" spans="1:78" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A12" s="106"/>
+      <c r="A12" s="125"/>
       <c r="B12" s="47" t="s">
         <v>0</v>
       </c>
@@ -17715,7 +17834,7 @@
       </c>
     </row>
     <row r="13" spans="1:78" x14ac:dyDescent="0.45">
-      <c r="A13" s="106"/>
+      <c r="A13" s="125"/>
       <c r="B13" s="47" t="s">
         <v>185</v>
       </c>
@@ -17967,7 +18086,7 @@
       </c>
     </row>
     <row r="14" spans="1:78" x14ac:dyDescent="0.45">
-      <c r="A14" s="106"/>
+      <c r="A14" s="125"/>
       <c r="B14" s="47" t="s">
         <v>186</v>
       </c>
@@ -18219,7 +18338,7 @@
       </c>
     </row>
     <row r="15" spans="1:78" x14ac:dyDescent="0.45">
-      <c r="A15" s="106"/>
+      <c r="A15" s="125"/>
       <c r="B15" s="47" t="s">
         <v>187</v>
       </c>
@@ -18471,7 +18590,7 @@
       </c>
     </row>
     <row r="16" spans="1:78" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A16" s="106"/>
+      <c r="A16" s="125"/>
       <c r="B16" s="47" t="s">
         <v>188</v>
       </c>
@@ -18723,7 +18842,7 @@
       </c>
     </row>
     <row r="17" spans="1:78" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A17" s="106"/>
+      <c r="A17" s="125"/>
       <c r="B17" s="50" t="s">
         <v>4</v>
       </c>
@@ -19190,28 +19309,6 @@
     </row>
   </sheetData>
   <mergeCells count="38">
-    <mergeCell ref="C10:E10"/>
-    <mergeCell ref="O10:Q10"/>
-    <mergeCell ref="C1:E1"/>
-    <mergeCell ref="O1:Q1"/>
-    <mergeCell ref="F10:J10"/>
-    <mergeCell ref="AW10:AZ10"/>
-    <mergeCell ref="K10:N10"/>
-    <mergeCell ref="W10:Z10"/>
-    <mergeCell ref="F1:J1"/>
-    <mergeCell ref="K1:N1"/>
-    <mergeCell ref="R1:V1"/>
-    <mergeCell ref="W1:Z1"/>
-    <mergeCell ref="R10:V10"/>
-    <mergeCell ref="BO10:BQ10"/>
-    <mergeCell ref="BR10:BV10"/>
-    <mergeCell ref="BW10:BZ10"/>
-    <mergeCell ref="BC1:BE1"/>
-    <mergeCell ref="BF1:BJ1"/>
-    <mergeCell ref="BK1:BN1"/>
-    <mergeCell ref="BO1:BQ1"/>
-    <mergeCell ref="BR1:BV1"/>
-    <mergeCell ref="BW1:BZ1"/>
     <mergeCell ref="A1:A8"/>
     <mergeCell ref="A10:A17"/>
     <mergeCell ref="BC10:BE10"/>
@@ -19228,14 +19325,36 @@
     <mergeCell ref="AK10:AN10"/>
     <mergeCell ref="AO10:AQ10"/>
     <mergeCell ref="AR10:AV10"/>
+    <mergeCell ref="BO10:BQ10"/>
+    <mergeCell ref="BR10:BV10"/>
+    <mergeCell ref="BW10:BZ10"/>
+    <mergeCell ref="BC1:BE1"/>
+    <mergeCell ref="BF1:BJ1"/>
+    <mergeCell ref="BK1:BN1"/>
+    <mergeCell ref="BO1:BQ1"/>
+    <mergeCell ref="BR1:BV1"/>
+    <mergeCell ref="BW1:BZ1"/>
+    <mergeCell ref="AW10:AZ10"/>
+    <mergeCell ref="K10:N10"/>
+    <mergeCell ref="W10:Z10"/>
+    <mergeCell ref="F1:J1"/>
+    <mergeCell ref="K1:N1"/>
+    <mergeCell ref="R1:V1"/>
+    <mergeCell ref="W1:Z1"/>
+    <mergeCell ref="R10:V10"/>
+    <mergeCell ref="C10:E10"/>
+    <mergeCell ref="O10:Q10"/>
+    <mergeCell ref="C1:E1"/>
+    <mergeCell ref="O1:Q1"/>
+    <mergeCell ref="F10:J10"/>
   </mergeCells>
   <conditionalFormatting sqref="AC3:AZ8">
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="29" priority="1" operator="equal">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AC12:AZ17">
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="28" priority="2" operator="equal">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
icon Lupe und 50m Bahn für BK
</commit_message>
<xml_diff>
--- a/web/utilities/records_kriterien.xlsx
+++ b/web/utilities/records_kriterien.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jpgna\Documents\GitHub\Lifesaving_Baden\web\utilities\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D09DCEC-8EF3-482A-98F0-B1501E0A56E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3EF3FC4-98F1-4B17-964A-463DF977B517}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="687" firstSheet="1" activeTab="7" xr2:uid="{E1AB626B-3773-4829-92A5-28DD4DB7C8F8}"/>
   </bookViews>
@@ -1614,16 +1614,13 @@
     <xf numFmtId="0" fontId="14" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1635,15 +1632,6 @@
     <xf numFmtId="0" fontId="14" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="10" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1652,27 +1640,6 @@
     </xf>
     <xf numFmtId="0" fontId="14" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1716,108 +1683,45 @@
     <xf numFmtId="0" fontId="17" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Prozent" xfId="1" builtinId="5"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="229">
-    <dxf>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
     <dxf>
       <font>
         <color theme="4"/>
@@ -4240,6 +4144,102 @@
       </fill>
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -4254,102 +4254,102 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{2C5E83EE-6B6F-478A-9C90-A846A1A76536}" name="WR_Open4" displayName="WR_Open4" ref="A4:AW31" totalsRowShown="0" headerRowDxfId="228" headerRowBorderDxfId="227" tableBorderDxfId="226">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{2C5E83EE-6B6F-478A-9C90-A846A1A76536}" name="WR_Open4" displayName="WR_Open4" ref="A4:AW31" totalsRowShown="0" headerRowDxfId="201" headerRowBorderDxfId="200" tableBorderDxfId="199">
   <autoFilter ref="A4:AW31" xr:uid="{2C5E83EE-6B6F-478A-9C90-A846A1A76536}"/>
   <tableColumns count="49">
-    <tableColumn id="1" xr3:uid="{7C0C4105-A61A-4B8D-9129-EDC4F18765AF}" name="WR-Open" dataDxfId="225">
+    <tableColumn id="1" xr3:uid="{7C0C4105-A61A-4B8D-9129-EDC4F18765AF}" name="WR-Open" dataDxfId="198">
       <calculatedColumnFormula>A4+1</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{516F5612-F85F-413F-9012-E235F415E34B}" name="50m Retten - offen - W" dataDxfId="224"/>
-    <tableColumn id="3" xr3:uid="{BC9ACAC9-0D45-42FD-B596-D19FBE3A4D83}" name="100m Retten - offen - W" dataDxfId="223"/>
-    <tableColumn id="4" xr3:uid="{CB6DBE59-EB65-43F0-93E7-0BDC3F82832B}" name="100m Kombi - offen - W" dataDxfId="222"/>
-    <tableColumn id="5" xr3:uid="{AA603C60-6831-4C14-A8CD-0AA050DA7551}" name="100m Lifesaver - offen - W" dataDxfId="221"/>
-    <tableColumn id="6" xr3:uid="{7920F147-7717-4582-940A-2610F7D310CA}" name="200m Superlifesaver - offen - W" dataDxfId="220"/>
-    <tableColumn id="7" xr3:uid="{04E21F1D-AC8D-4A1B-9B43-59B8F7901673}" name="200m Hindernis - offen - W" dataDxfId="219"/>
-    <tableColumn id="8" xr3:uid="{40E8A083-653A-48A8-9B37-0A2D850B7829}" name="50m Retten - offen - M" dataDxfId="218"/>
-    <tableColumn id="9" xr3:uid="{863824A9-134F-4189-BB14-225AE224FC44}" name="100m Retten - offen - M" dataDxfId="217"/>
+    <tableColumn id="2" xr3:uid="{516F5612-F85F-413F-9012-E235F415E34B}" name="50m Retten - offen - W" dataDxfId="197"/>
+    <tableColumn id="3" xr3:uid="{BC9ACAC9-0D45-42FD-B596-D19FBE3A4D83}" name="100m Retten - offen - W" dataDxfId="196"/>
+    <tableColumn id="4" xr3:uid="{CB6DBE59-EB65-43F0-93E7-0BDC3F82832B}" name="100m Kombi - offen - W" dataDxfId="195"/>
+    <tableColumn id="5" xr3:uid="{AA603C60-6831-4C14-A8CD-0AA050DA7551}" name="100m Lifesaver - offen - W" dataDxfId="194"/>
+    <tableColumn id="6" xr3:uid="{7920F147-7717-4582-940A-2610F7D310CA}" name="200m Superlifesaver - offen - W" dataDxfId="193"/>
+    <tableColumn id="7" xr3:uid="{04E21F1D-AC8D-4A1B-9B43-59B8F7901673}" name="200m Hindernis - offen - W" dataDxfId="192"/>
+    <tableColumn id="8" xr3:uid="{40E8A083-653A-48A8-9B37-0A2D850B7829}" name="50m Retten - offen - M" dataDxfId="191"/>
+    <tableColumn id="9" xr3:uid="{863824A9-134F-4189-BB14-225AE224FC44}" name="100m Retten - offen - M" dataDxfId="190"/>
     <tableColumn id="10" xr3:uid="{598FC6AE-DEA2-4475-9A35-CDCB8C81496A}" name="100m Kombi - offen - M"/>
     <tableColumn id="11" xr3:uid="{9FC50B37-0D51-422E-A268-A6506D4F3854}" name="100m Lifesaver - offen - M"/>
     <tableColumn id="12" xr3:uid="{B8D2552B-5D82-442A-98F0-E47D5C5F6728}" name="200m Superlifesaver - offen - M"/>
-    <tableColumn id="13" xr3:uid="{5A5E9873-0C5F-4508-AF6B-4974E0526D84}" name="200m Hindernis - offen - M" dataDxfId="216"/>
-    <tableColumn id="14" xr3:uid="{FA907992-7FCE-4CAD-8CF2-F5BEBC9B3756}" name="50m Retten - 17/18 - W" dataDxfId="215"/>
-    <tableColumn id="15" xr3:uid="{76B63DC0-CB67-48F4-9B5A-D22902F59334}" name="100m Retten - 17/18 - W" dataDxfId="214"/>
-    <tableColumn id="16" xr3:uid="{614A2419-51B1-44C0-8469-ADBFB078B81A}" name="100m Kombi -17/18 - W" dataDxfId="213"/>
-    <tableColumn id="17" xr3:uid="{2EC953EE-367D-4524-A25E-8DE3B8168E34}" name="100m Lifesaver - 17/18 - W" dataDxfId="212"/>
-    <tableColumn id="18" xr3:uid="{25711867-9BD7-4197-9094-A21392411249}" name="200m Superlifesaver - 17/18 - W" dataDxfId="211"/>
-    <tableColumn id="19" xr3:uid="{262DB142-CFB1-45C3-9332-7273CACD1B62}" name="200m Hindernis - 17/18 - W" dataDxfId="210"/>
-    <tableColumn id="20" xr3:uid="{938BA45A-8244-4637-8A14-DF49CD91A945}" name="50m Retten - 17/18 - M" dataDxfId="209"/>
-    <tableColumn id="21" xr3:uid="{737E28D8-900F-4A98-95FE-EE7B0AFDEE90}" name="100m Retten - 17/18 - M" dataDxfId="208"/>
-    <tableColumn id="22" xr3:uid="{330BD3A8-061C-45E2-ADDB-40C2F346772F}" name="100m Kombi - 17/18 - M" dataDxfId="207"/>
-    <tableColumn id="23" xr3:uid="{0CADDE90-A167-4E1D-8D33-8624E5E1A4E2}" name="100m Lifesaver - 17/18 - M" dataDxfId="206"/>
-    <tableColumn id="24" xr3:uid="{FCF9F42C-1291-4985-9D37-B9DE2DAA5DCB}" name="200m Superlifesaver - 17/18 - M" dataDxfId="205"/>
-    <tableColumn id="25" xr3:uid="{4E5397B2-F924-4F48-AE69-AF6D650AF88D}" name="200m Hindernis - 17/18 - M" dataDxfId="204"/>
-    <tableColumn id="26" xr3:uid="{0A78315A-BFDC-43EE-A66F-48B301F66508}" name="50m Retten - 15/16 - W" dataDxfId="203"/>
-    <tableColumn id="27" xr3:uid="{D3FCF8BD-6C76-450D-80C0-CC0519A79731}" name="100m Retten - 15/16 - W" dataDxfId="202"/>
-    <tableColumn id="28" xr3:uid="{6BE7937E-D62D-47CD-95DE-1730304B0DF3}" name="100m Kombi - 15/16 - W" dataDxfId="201"/>
-    <tableColumn id="29" xr3:uid="{098BA5BE-5AF6-4187-89B6-534498F24C51}" name="100m Lifesaver -  15/16 - W" dataDxfId="200"/>
-    <tableColumn id="30" xr3:uid="{2A6822CF-143C-4BF7-A440-5777527BE512}" name="200m Superlifesaver -  15/16 - W" dataDxfId="199"/>
-    <tableColumn id="31" xr3:uid="{541C7145-CDEA-4E4E-9E7A-A4F05BA6C3E5}" name="200m Hindernis -  15/16 - W" dataDxfId="198"/>
-    <tableColumn id="32" xr3:uid="{342C4488-8C61-42E6-87A9-C75BD8EB7452}" name="50m Retten - 15/16 - M" dataDxfId="197"/>
-    <tableColumn id="33" xr3:uid="{857B1D46-7D20-47F7-AB9B-732D50346E32}" name="100m Retten - 15/16 - M" dataDxfId="196"/>
-    <tableColumn id="34" xr3:uid="{4C8A2EB4-804B-45F1-A768-9A6958957F8B}" name="100m Kombi -15/16 - M" dataDxfId="195"/>
-    <tableColumn id="35" xr3:uid="{26C75B4F-21EC-4EB0-A9A9-54BC80140672}" name="100m Lifesaver - 15/16 - M" dataDxfId="194"/>
-    <tableColumn id="36" xr3:uid="{DBBB2A23-1A06-429A-A5D1-A547EF5EC16F}" name="200m Superlifesaver - 15/16 - M" dataDxfId="193"/>
-    <tableColumn id="37" xr3:uid="{84061231-CAE5-427A-87F5-6DDBA99F77D2}" name="200m Hindernis - 15/16 - M" dataDxfId="192"/>
-    <tableColumn id="38" xr3:uid="{878CCA80-A742-4B3C-90C9-E93BB814201B}" name="50m Retten - 13/14 - W" dataDxfId="191"/>
-    <tableColumn id="39" xr3:uid="{A1F57102-61CF-4784-8DE2-0B8F32D5D699}" name="50m Retten mit Flossen - 13/14 - W" dataDxfId="190"/>
-    <tableColumn id="40" xr3:uid="{0F6BAF78-3D79-42A9-9FED-E6D0E335A920}" name="100m Hindernis - 13/14 - W" dataDxfId="189"/>
-    <tableColumn id="41" xr3:uid="{EB748A68-E10D-4D76-B315-8FDB3AC33C8D}" name="50m Retten - 13/14 - M" dataDxfId="188"/>
-    <tableColumn id="42" xr3:uid="{C7B04167-6430-40F0-9A0F-D0D0BE2F9C77}" name="50m Retten mit Flossen - 13/14 - M" dataDxfId="187"/>
-    <tableColumn id="43" xr3:uid="{48704BB7-A853-445A-8CDC-8D8F86C2B66A}" name="100m Hindernis - 13/14 - M" dataDxfId="186"/>
-    <tableColumn id="44" xr3:uid="{9605FE9A-F41C-4A5F-A59C-B7A9D45C460F}" name="50m Flossen - 12 - W" dataDxfId="185"/>
-    <tableColumn id="45" xr3:uid="{4C9DBF61-35B1-4BC2-8272-526E0AFAAFFB}" name="50m komb. Schwimmen - 12 - W" dataDxfId="184"/>
-    <tableColumn id="46" xr3:uid="{CF433C95-C272-48F9-98CD-7E3C8DBB6F2C}" name="50m Hindernis - 12 - W" dataDxfId="183"/>
-    <tableColumn id="47" xr3:uid="{FADB7411-DB43-4B14-B9E8-D74CA1BA18B8}" name="50m Flossen - 12 - M" dataDxfId="182"/>
-    <tableColumn id="48" xr3:uid="{02936F84-1D82-48AC-8D7C-6D2954D68A06}" name="50m komb. Schwimmen - 12 - M" dataDxfId="181"/>
-    <tableColumn id="49" xr3:uid="{7FD9BD11-0597-4E07-8DA5-DB53384197F5}" name="50m Hindernis - 12 - M" dataDxfId="180"/>
+    <tableColumn id="13" xr3:uid="{5A5E9873-0C5F-4508-AF6B-4974E0526D84}" name="200m Hindernis - offen - M" dataDxfId="189"/>
+    <tableColumn id="14" xr3:uid="{FA907992-7FCE-4CAD-8CF2-F5BEBC9B3756}" name="50m Retten - 17/18 - W" dataDxfId="188"/>
+    <tableColumn id="15" xr3:uid="{76B63DC0-CB67-48F4-9B5A-D22902F59334}" name="100m Retten - 17/18 - W" dataDxfId="187"/>
+    <tableColumn id="16" xr3:uid="{614A2419-51B1-44C0-8469-ADBFB078B81A}" name="100m Kombi -17/18 - W" dataDxfId="186"/>
+    <tableColumn id="17" xr3:uid="{2EC953EE-367D-4524-A25E-8DE3B8168E34}" name="100m Lifesaver - 17/18 - W" dataDxfId="185"/>
+    <tableColumn id="18" xr3:uid="{25711867-9BD7-4197-9094-A21392411249}" name="200m Superlifesaver - 17/18 - W" dataDxfId="184"/>
+    <tableColumn id="19" xr3:uid="{262DB142-CFB1-45C3-9332-7273CACD1B62}" name="200m Hindernis - 17/18 - W" dataDxfId="183"/>
+    <tableColumn id="20" xr3:uid="{938BA45A-8244-4637-8A14-DF49CD91A945}" name="50m Retten - 17/18 - M" dataDxfId="182"/>
+    <tableColumn id="21" xr3:uid="{737E28D8-900F-4A98-95FE-EE7B0AFDEE90}" name="100m Retten - 17/18 - M" dataDxfId="181"/>
+    <tableColumn id="22" xr3:uid="{330BD3A8-061C-45E2-ADDB-40C2F346772F}" name="100m Kombi - 17/18 - M" dataDxfId="180"/>
+    <tableColumn id="23" xr3:uid="{0CADDE90-A167-4E1D-8D33-8624E5E1A4E2}" name="100m Lifesaver - 17/18 - M" dataDxfId="179"/>
+    <tableColumn id="24" xr3:uid="{FCF9F42C-1291-4985-9D37-B9DE2DAA5DCB}" name="200m Superlifesaver - 17/18 - M" dataDxfId="178"/>
+    <tableColumn id="25" xr3:uid="{4E5397B2-F924-4F48-AE69-AF6D650AF88D}" name="200m Hindernis - 17/18 - M" dataDxfId="177"/>
+    <tableColumn id="26" xr3:uid="{0A78315A-BFDC-43EE-A66F-48B301F66508}" name="50m Retten - 15/16 - W" dataDxfId="176"/>
+    <tableColumn id="27" xr3:uid="{D3FCF8BD-6C76-450D-80C0-CC0519A79731}" name="100m Retten - 15/16 - W" dataDxfId="175"/>
+    <tableColumn id="28" xr3:uid="{6BE7937E-D62D-47CD-95DE-1730304B0DF3}" name="100m Kombi - 15/16 - W" dataDxfId="174"/>
+    <tableColumn id="29" xr3:uid="{098BA5BE-5AF6-4187-89B6-534498F24C51}" name="100m Lifesaver -  15/16 - W" dataDxfId="173"/>
+    <tableColumn id="30" xr3:uid="{2A6822CF-143C-4BF7-A440-5777527BE512}" name="200m Superlifesaver -  15/16 - W" dataDxfId="172"/>
+    <tableColumn id="31" xr3:uid="{541C7145-CDEA-4E4E-9E7A-A4F05BA6C3E5}" name="200m Hindernis -  15/16 - W" dataDxfId="171"/>
+    <tableColumn id="32" xr3:uid="{342C4488-8C61-42E6-87A9-C75BD8EB7452}" name="50m Retten - 15/16 - M" dataDxfId="170"/>
+    <tableColumn id="33" xr3:uid="{857B1D46-7D20-47F7-AB9B-732D50346E32}" name="100m Retten - 15/16 - M" dataDxfId="169"/>
+    <tableColumn id="34" xr3:uid="{4C8A2EB4-804B-45F1-A768-9A6958957F8B}" name="100m Kombi -15/16 - M" dataDxfId="168"/>
+    <tableColumn id="35" xr3:uid="{26C75B4F-21EC-4EB0-A9A9-54BC80140672}" name="100m Lifesaver - 15/16 - M" dataDxfId="167"/>
+    <tableColumn id="36" xr3:uid="{DBBB2A23-1A06-429A-A5D1-A547EF5EC16F}" name="200m Superlifesaver - 15/16 - M" dataDxfId="166"/>
+    <tableColumn id="37" xr3:uid="{84061231-CAE5-427A-87F5-6DDBA99F77D2}" name="200m Hindernis - 15/16 - M" dataDxfId="165"/>
+    <tableColumn id="38" xr3:uid="{878CCA80-A742-4B3C-90C9-E93BB814201B}" name="50m Retten - 13/14 - W" dataDxfId="164"/>
+    <tableColumn id="39" xr3:uid="{A1F57102-61CF-4784-8DE2-0B8F32D5D699}" name="50m Retten mit Flossen - 13/14 - W" dataDxfId="163"/>
+    <tableColumn id="40" xr3:uid="{0F6BAF78-3D79-42A9-9FED-E6D0E335A920}" name="100m Hindernis - 13/14 - W" dataDxfId="162"/>
+    <tableColumn id="41" xr3:uid="{EB748A68-E10D-4D76-B315-8FDB3AC33C8D}" name="50m Retten - 13/14 - M" dataDxfId="161"/>
+    <tableColumn id="42" xr3:uid="{C7B04167-6430-40F0-9A0F-D0D0BE2F9C77}" name="50m Retten mit Flossen - 13/14 - M" dataDxfId="160"/>
+    <tableColumn id="43" xr3:uid="{48704BB7-A853-445A-8CDC-8D8F86C2B66A}" name="100m Hindernis - 13/14 - M" dataDxfId="159"/>
+    <tableColumn id="44" xr3:uid="{9605FE9A-F41C-4A5F-A59C-B7A9D45C460F}" name="50m Flossen - 12 - W" dataDxfId="158"/>
+    <tableColumn id="45" xr3:uid="{4C9DBF61-35B1-4BC2-8272-526E0AFAAFFB}" name="50m komb. Schwimmen - 12 - W" dataDxfId="157"/>
+    <tableColumn id="46" xr3:uid="{CF433C95-C272-48F9-98CD-7E3C8DBB6F2C}" name="50m Hindernis - 12 - W" dataDxfId="156"/>
+    <tableColumn id="47" xr3:uid="{FADB7411-DB43-4B14-B9E8-D74CA1BA18B8}" name="50m Flossen - 12 - M" dataDxfId="155"/>
+    <tableColumn id="48" xr3:uid="{02936F84-1D82-48AC-8D7C-6D2954D68A06}" name="50m komb. Schwimmen - 12 - M" dataDxfId="154"/>
+    <tableColumn id="49" xr3:uid="{7FD9BD11-0597-4E07-8DA5-DB53384197F5}" name="50m Hindernis - 12 - M" dataDxfId="153"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{4234D44E-A2BE-4790-B589-1A8CC19B714E}" name="WR_Youth" displayName="WR_Youth" ref="A4:M32" totalsRowShown="0" headerRowDxfId="179" dataDxfId="177" headerRowBorderDxfId="178" tableBorderDxfId="176">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{4234D44E-A2BE-4790-B589-1A8CC19B714E}" name="WR_Youth" displayName="WR_Youth" ref="A4:M32" totalsRowShown="0" headerRowDxfId="152" dataDxfId="150" headerRowBorderDxfId="151" tableBorderDxfId="149">
   <autoFilter ref="A4:M32" xr:uid="{4234D44E-A2BE-4790-B589-1A8CC19B714E}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{848E691A-41B0-42DD-B122-FB6DF43CB3EF}" name="WR-Youth" dataDxfId="175"/>
-    <tableColumn id="2" xr3:uid="{2FE43F18-485B-46A9-8946-FBC5FDAE5A8E}" name="50m Retten" dataDxfId="174"/>
-    <tableColumn id="3" xr3:uid="{CA5C3ABF-02E6-442B-868B-95B293B231D3}" name="100m Retten" dataDxfId="173"/>
-    <tableColumn id="4" xr3:uid="{7A6BBA52-2145-464D-8C04-B2CCFC1A90DC}" name="100m Kombi" dataDxfId="172"/>
-    <tableColumn id="5" xr3:uid="{21F420C9-E788-49EE-88F6-E37963ED31CF}" name="100m Lifesaver" dataDxfId="171"/>
-    <tableColumn id="6" xr3:uid="{CB87B7CD-8A9C-4775-A4D7-4D267F43FD1A}" name="200m Superlifesaver" dataDxfId="170"/>
-    <tableColumn id="7" xr3:uid="{2DC7F290-B564-4851-85AE-D211DA701B32}" name="200m Hindernis" dataDxfId="169"/>
-    <tableColumn id="8" xr3:uid="{8112783D-8796-4D6A-8414-AC675D745697}" name="50m Retten2" dataDxfId="168"/>
-    <tableColumn id="9" xr3:uid="{4E818CD4-8725-495D-9D1D-1AFCED9181F5}" name="100m Retten2" dataDxfId="167"/>
-    <tableColumn id="10" xr3:uid="{28C05A91-E302-40A9-B50A-ECF997F129FC}" name="100m Kombi2" dataDxfId="166"/>
-    <tableColumn id="11" xr3:uid="{D56FB9F2-45BF-4EC9-A84C-8A5FB59F2F05}" name="100m Lifesaver2" dataDxfId="165"/>
-    <tableColumn id="12" xr3:uid="{540169C0-2A40-4794-A872-F7DF8A887BF2}" name="200m Superlifesaver2" dataDxfId="164"/>
-    <tableColumn id="13" xr3:uid="{D104CB67-B55A-4C81-87E5-0AC758DD22A4}" name="200m Hindernis2" dataDxfId="163"/>
+    <tableColumn id="1" xr3:uid="{848E691A-41B0-42DD-B122-FB6DF43CB3EF}" name="WR-Youth" dataDxfId="148"/>
+    <tableColumn id="2" xr3:uid="{2FE43F18-485B-46A9-8946-FBC5FDAE5A8E}" name="50m Retten" dataDxfId="147"/>
+    <tableColumn id="3" xr3:uid="{CA5C3ABF-02E6-442B-868B-95B293B231D3}" name="100m Retten" dataDxfId="146"/>
+    <tableColumn id="4" xr3:uid="{7A6BBA52-2145-464D-8C04-B2CCFC1A90DC}" name="100m Kombi" dataDxfId="145"/>
+    <tableColumn id="5" xr3:uid="{21F420C9-E788-49EE-88F6-E37963ED31CF}" name="100m Lifesaver" dataDxfId="144"/>
+    <tableColumn id="6" xr3:uid="{CB87B7CD-8A9C-4775-A4D7-4D267F43FD1A}" name="200m Superlifesaver" dataDxfId="143"/>
+    <tableColumn id="7" xr3:uid="{2DC7F290-B564-4851-85AE-D211DA701B32}" name="200m Hindernis" dataDxfId="142"/>
+    <tableColumn id="8" xr3:uid="{8112783D-8796-4D6A-8414-AC675D745697}" name="50m Retten2" dataDxfId="141"/>
+    <tableColumn id="9" xr3:uid="{4E818CD4-8725-495D-9D1D-1AFCED9181F5}" name="100m Retten2" dataDxfId="140"/>
+    <tableColumn id="10" xr3:uid="{28C05A91-E302-40A9-B50A-ECF997F129FC}" name="100m Kombi2" dataDxfId="139"/>
+    <tableColumn id="11" xr3:uid="{D56FB9F2-45BF-4EC9-A84C-8A5FB59F2F05}" name="100m Lifesaver2" dataDxfId="138"/>
+    <tableColumn id="12" xr3:uid="{540169C0-2A40-4794-A872-F7DF8A887BF2}" name="200m Superlifesaver2" dataDxfId="137"/>
+    <tableColumn id="13" xr3:uid="{D104CB67-B55A-4C81-87E5-0AC758DD22A4}" name="200m Hindernis2" dataDxfId="136"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E2D2F97B-7645-4066-8AB3-F35CF6E035EB}" name="WR_Open" displayName="WR_Open" ref="A4:M32" totalsRowShown="0" headerRowDxfId="162" headerRowBorderDxfId="161" tableBorderDxfId="160">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E2D2F97B-7645-4066-8AB3-F35CF6E035EB}" name="WR_Open" displayName="WR_Open" ref="A4:M32" totalsRowShown="0" headerRowDxfId="135" headerRowBorderDxfId="134" tableBorderDxfId="133">
   <autoFilter ref="A4:M32" xr:uid="{E2D2F97B-7645-4066-8AB3-F35CF6E035EB}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{AE73402B-B27E-4B29-8DCF-30B7FC1855EF}" name="WR-Open" dataDxfId="159">
+    <tableColumn id="1" xr3:uid="{AE73402B-B27E-4B29-8DCF-30B7FC1855EF}" name="WR-Open" dataDxfId="132">
       <calculatedColumnFormula>A4+1</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{EA3EAC1F-184E-4A28-B3E3-08DE12F138EF}" name="50m Retten" dataDxfId="158"/>
-    <tableColumn id="3" xr3:uid="{E0305A3F-6087-4F8C-8B64-153E1ACAA32E}" name="100m Retten" dataDxfId="157"/>
-    <tableColumn id="4" xr3:uid="{F0B7AC37-315E-49AA-855C-7955D2B43A76}" name="100m Kombi" dataDxfId="156"/>
-    <tableColumn id="5" xr3:uid="{B5E690AB-DB7D-4864-8916-89D2A68C4128}" name="100m Lifesaver" dataDxfId="155"/>
-    <tableColumn id="6" xr3:uid="{D89BAF4D-36AE-4C73-9320-9C5736F02F8A}" name="200m Superlifesaver" dataDxfId="154"/>
-    <tableColumn id="7" xr3:uid="{58AE7517-1A90-459F-A7D2-B95265D217E7}" name="200m Hindernis" dataDxfId="153"/>
-    <tableColumn id="8" xr3:uid="{13A189FB-E897-4A1F-A001-525F61E9CFFF}" name="50m Retten2" dataDxfId="152"/>
-    <tableColumn id="9" xr3:uid="{36418AC5-46B8-400F-BD2E-D329CF4F92CD}" name="100m Retten2" dataDxfId="151"/>
+    <tableColumn id="2" xr3:uid="{EA3EAC1F-184E-4A28-B3E3-08DE12F138EF}" name="50m Retten" dataDxfId="131"/>
+    <tableColumn id="3" xr3:uid="{E0305A3F-6087-4F8C-8B64-153E1ACAA32E}" name="100m Retten" dataDxfId="130"/>
+    <tableColumn id="4" xr3:uid="{F0B7AC37-315E-49AA-855C-7955D2B43A76}" name="100m Kombi" dataDxfId="129"/>
+    <tableColumn id="5" xr3:uid="{B5E690AB-DB7D-4864-8916-89D2A68C4128}" name="100m Lifesaver" dataDxfId="128"/>
+    <tableColumn id="6" xr3:uid="{D89BAF4D-36AE-4C73-9320-9C5736F02F8A}" name="200m Superlifesaver" dataDxfId="127"/>
+    <tableColumn id="7" xr3:uid="{58AE7517-1A90-459F-A7D2-B95265D217E7}" name="200m Hindernis" dataDxfId="126"/>
+    <tableColumn id="8" xr3:uid="{13A189FB-E897-4A1F-A001-525F61E9CFFF}" name="50m Retten2" dataDxfId="125"/>
+    <tableColumn id="9" xr3:uid="{36418AC5-46B8-400F-BD2E-D329CF4F92CD}" name="100m Retten2" dataDxfId="124"/>
     <tableColumn id="10" xr3:uid="{06A35C2D-7313-472B-BC1F-4F2FB1D14782}" name="100m Kombi2"/>
     <tableColumn id="11" xr3:uid="{89966D0D-9131-4245-A7BE-1A7384D5ADA0}" name="100m Lifesaver2"/>
     <tableColumn id="12" xr3:uid="{D9D6CF56-869C-4DDE-9886-572D4E523A8F}" name="200m Superlifesaver2"/>
@@ -4360,7 +4360,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{CF3D303A-A04B-42DD-A44E-CEB6CECB77A4}" name="DP_konfig" displayName="DP_konfig" ref="A1:U3" totalsRowShown="0" headerRowDxfId="150" dataDxfId="149">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{CF3D303A-A04B-42DD-A44E-CEB6CECB77A4}" name="DP_konfig" displayName="DP_konfig" ref="A1:U3" totalsRowShown="0" headerRowDxfId="123" dataDxfId="122">
   <autoFilter ref="A1:U3" xr:uid="{CF3D303A-A04B-42DD-A44E-CEB6CECB77A4}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -4385,64 +4385,64 @@
     <filterColumn colId="20" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="21">
-    <tableColumn id="1" xr3:uid="{58D628F0-061E-4A82-8362-CDB37A2E7C60}" name="Tabellen Name" dataDxfId="148"/>
-    <tableColumn id="2" xr3:uid="{2F302F6C-F8AF-4FDE-AB08-6F30F9671015}" name="Geschlecht" dataDxfId="147"/>
-    <tableColumn id="3" xr3:uid="{4D91FBF9-386D-43DD-90D0-B49823FDB629}" name="Mindest alter" dataDxfId="146"/>
-    <tableColumn id="4" xr3:uid="{4126AAC6-AF2F-446C-B4EA-D86ACFD9FAC2}" name="Maximales Alter" dataDxfId="145"/>
-    <tableColumn id="5" xr3:uid="{8A10890A-A299-4B09-AC72-0E9AE9238AF3}" name="Qualizeitraum anfang" dataDxfId="144"/>
-    <tableColumn id="6" xr3:uid="{FBCD1C13-FC82-429B-8DE1-0C5A455FDAB8}" name="Qualizeitraum Ende" dataDxfId="143"/>
-    <tableColumn id="7" xr3:uid="{1DCCAC9B-BC46-468E-A3CE-57576C2FF11D}" name="Letzter Wettkampf am" dataDxfId="142"/>
-    <tableColumn id="8" xr3:uid="{9A6E47EE-ABD8-4A1E-87D3-9D286E4C124F}" name="Wertung" dataDxfId="141"/>
-    <tableColumn id="9" xr3:uid="{09E848D2-ED17-49C7-9775-CBF17D20DFC0}" name="Landesverband" dataDxfId="140"/>
-    <tableColumn id="10" xr3:uid="{70ABB713-23F6-4FCF-920E-3CB0CD451446}" name="OMS" dataDxfId="139"/>
-    <tableColumn id="11" xr3:uid="{9C108A1C-E6AB-4C13-9C1D-0FA8944A39A3}" name="Pool-Länge" dataDxfId="138"/>
-    <tableColumn id="12" xr3:uid="{087948DD-430D-48F1-906D-4F4EF4B46053}" name="Regelwerk" dataDxfId="137"/>
-    <tableColumn id="13" xr3:uid="{BF42D9C0-F77D-4971-A67E-32B0246C72C3}" name="Referenz" dataDxfId="136"/>
-    <tableColumn id="19" xr3:uid="{AFFB84E8-B398-4E99-805B-9A247071A040}" name="Referenz Jahr" dataDxfId="135"/>
-    <tableColumn id="20" xr3:uid="{0A59A474-DFBB-4437-8EFF-70284AFD9934}" name="Mindest Punktzahl" dataDxfId="134"/>
-    <tableColumn id="21" xr3:uid="{198BD231-EEF3-43C9-AD9B-39B4B7E9B337}" name="Mindest Disziplinen" dataDxfId="133"/>
-    <tableColumn id="14" xr3:uid="{443CD4F6-A2B2-480B-BB35-DCEEBC531727}" name="3-Kampf Regel" dataDxfId="132"/>
-    <tableColumn id="15" xr3:uid="{70116160-7666-42B1-92AC-FAC2620E6A60}" name="Anzahl Nominierte" dataDxfId="131"/>
-    <tableColumn id="16" xr3:uid="{0EFD0A46-D12B-4AB0-907C-08E5D9F282E0}" name="Anzahl Nachrücker" dataDxfId="130"/>
-    <tableColumn id="17" xr3:uid="{AA5430A0-8ED8-40E8-B7F8-DA25E4E8790F}" name="Seiten Anzahl" dataDxfId="129"/>
-    <tableColumn id="18" xr3:uid="{16F699D9-2741-43F3-AD5F-826A568EFEAC}" name="Absagen" dataDxfId="128"/>
+    <tableColumn id="1" xr3:uid="{58D628F0-061E-4A82-8362-CDB37A2E7C60}" name="Tabellen Name" dataDxfId="121"/>
+    <tableColumn id="2" xr3:uid="{2F302F6C-F8AF-4FDE-AB08-6F30F9671015}" name="Geschlecht" dataDxfId="120"/>
+    <tableColumn id="3" xr3:uid="{4D91FBF9-386D-43DD-90D0-B49823FDB629}" name="Mindest alter" dataDxfId="119"/>
+    <tableColumn id="4" xr3:uid="{4126AAC6-AF2F-446C-B4EA-D86ACFD9FAC2}" name="Maximales Alter" dataDxfId="118"/>
+    <tableColumn id="5" xr3:uid="{8A10890A-A299-4B09-AC72-0E9AE9238AF3}" name="Qualizeitraum anfang" dataDxfId="117"/>
+    <tableColumn id="6" xr3:uid="{FBCD1C13-FC82-429B-8DE1-0C5A455FDAB8}" name="Qualizeitraum Ende" dataDxfId="116"/>
+    <tableColumn id="7" xr3:uid="{1DCCAC9B-BC46-468E-A3CE-57576C2FF11D}" name="Letzter Wettkampf am" dataDxfId="115"/>
+    <tableColumn id="8" xr3:uid="{9A6E47EE-ABD8-4A1E-87D3-9D286E4C124F}" name="Wertung" dataDxfId="114"/>
+    <tableColumn id="9" xr3:uid="{09E848D2-ED17-49C7-9775-CBF17D20DFC0}" name="Landesverband" dataDxfId="113"/>
+    <tableColumn id="10" xr3:uid="{70ABB713-23F6-4FCF-920E-3CB0CD451446}" name="OMS" dataDxfId="112"/>
+    <tableColumn id="11" xr3:uid="{9C108A1C-E6AB-4C13-9C1D-0FA8944A39A3}" name="Pool-Länge" dataDxfId="111"/>
+    <tableColumn id="12" xr3:uid="{087948DD-430D-48F1-906D-4F4EF4B46053}" name="Regelwerk" dataDxfId="110"/>
+    <tableColumn id="13" xr3:uid="{BF42D9C0-F77D-4971-A67E-32B0246C72C3}" name="Referenz" dataDxfId="109"/>
+    <tableColumn id="19" xr3:uid="{AFFB84E8-B398-4E99-805B-9A247071A040}" name="Referenz Jahr" dataDxfId="108"/>
+    <tableColumn id="20" xr3:uid="{0A59A474-DFBB-4437-8EFF-70284AFD9934}" name="Mindest Punktzahl" dataDxfId="107"/>
+    <tableColumn id="21" xr3:uid="{198BD231-EEF3-43C9-AD9B-39B4B7E9B337}" name="Mindest Disziplinen" dataDxfId="106"/>
+    <tableColumn id="14" xr3:uid="{443CD4F6-A2B2-480B-BB35-DCEEBC531727}" name="3-Kampf Regel" dataDxfId="105"/>
+    <tableColumn id="15" xr3:uid="{70116160-7666-42B1-92AC-FAC2620E6A60}" name="Anzahl Nominierte" dataDxfId="104"/>
+    <tableColumn id="16" xr3:uid="{0EFD0A46-D12B-4AB0-907C-08E5D9F282E0}" name="Anzahl Nachrücker" dataDxfId="103"/>
+    <tableColumn id="17" xr3:uid="{AA5430A0-8ED8-40E8-B7F8-DA25E4E8790F}" name="Seiten Anzahl" dataDxfId="102"/>
+    <tableColumn id="18" xr3:uid="{16F699D9-2741-43F3-AD5F-826A568EFEAC}" name="Absagen" dataDxfId="101"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{CDBF6724-48A1-41AB-94B5-CC35C54BB15C}" name="BP_konfig" displayName="BP_konfig" ref="A1:U7" totalsRowShown="0" headerRowDxfId="127" dataDxfId="126">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{CDBF6724-48A1-41AB-94B5-CC35C54BB15C}" name="BP_konfig" displayName="BP_konfig" ref="A1:U7" totalsRowShown="0" headerRowDxfId="100" dataDxfId="99">
   <autoFilter ref="A1:U7" xr:uid="{CDBF6724-48A1-41AB-94B5-CC35C54BB15C}"/>
   <tableColumns count="21">
-    <tableColumn id="1" xr3:uid="{E1FB3D0C-B874-4874-BACC-6872CF171957}" name="Tabellen Name" dataDxfId="125"/>
-    <tableColumn id="2" xr3:uid="{FFDD2777-2097-450C-B020-F133CF643855}" name="Geschlecht" dataDxfId="124"/>
-    <tableColumn id="3" xr3:uid="{8CF52BE2-8020-48BD-A36D-63F13A1878DE}" name="Mindest alter" dataDxfId="123"/>
-    <tableColumn id="4" xr3:uid="{FD3A030F-CD97-4B6F-8E8C-BC2E67D79F1D}" name="Maximales Alter" dataDxfId="122"/>
-    <tableColumn id="5" xr3:uid="{3E22B645-D77C-4509-B031-9914FCB91599}" name="Qualizeitraum anfang" dataDxfId="121"/>
-    <tableColumn id="6" xr3:uid="{AE299324-3C1C-4063-ADF9-54555A161734}" name="Qualizeitraum Ende" dataDxfId="120"/>
-    <tableColumn id="7" xr3:uid="{DCC178B3-11FC-4C53-BBC6-C2FDA2C89857}" name="Letzter Wettkampf am" dataDxfId="119"/>
-    <tableColumn id="8" xr3:uid="{2811DB01-60A5-4BE4-B6F9-A806398A602A}" name="Wertung" dataDxfId="118"/>
-    <tableColumn id="9" xr3:uid="{0C16DAFE-847D-4E9E-9604-3A7D9FE924D0}" name="Landesverband" dataDxfId="117"/>
-    <tableColumn id="10" xr3:uid="{7A8A4101-A553-4BD5-9116-9AA5876B9401}" name="OMS" dataDxfId="116"/>
-    <tableColumn id="11" xr3:uid="{9807C9BD-6499-45F6-ACE0-4D13D64EF675}" name="Pool-Länge" dataDxfId="115"/>
-    <tableColumn id="12" xr3:uid="{13D336DD-650F-4F2C-836F-361CA1528F6D}" name="Regelwerk" dataDxfId="114"/>
-    <tableColumn id="13" xr3:uid="{66660E2D-ADF2-4FB5-8A13-004F826EE908}" name="Referenz" dataDxfId="113"/>
-    <tableColumn id="19" xr3:uid="{D72EDF8B-ECC3-4FF7-ABE6-B60BCE4A5E26}" name="Referenz Jahr" dataDxfId="112"/>
-    <tableColumn id="20" xr3:uid="{7B18E667-70F7-4BC1-AB1B-21C019F2AA89}" name="Mindest Punktzahl" dataDxfId="111"/>
-    <tableColumn id="21" xr3:uid="{FC185946-681B-42A6-AB1A-FC1EABB668C5}" name="Mindest Disziplinen" dataDxfId="110"/>
-    <tableColumn id="14" xr3:uid="{6A2676FD-2EC7-4C41-A35E-A1597A38F932}" name="3-Kampf Regel" dataDxfId="109"/>
-    <tableColumn id="15" xr3:uid="{718E0917-4F83-4A2B-832F-EBB16D5E21BF}" name="Anzahl Nominierte" dataDxfId="108"/>
-    <tableColumn id="16" xr3:uid="{5C66A461-D647-4E00-A81C-FD7AD44D7CC2}" name="Anzahl Nachrücker" dataDxfId="107"/>
-    <tableColumn id="17" xr3:uid="{D434BDEC-293B-4B4E-A5E9-479438960A03}" name="Seiten Anzahl" dataDxfId="106"/>
-    <tableColumn id="18" xr3:uid="{80908229-9247-473F-81C0-9C9D4C12FF06}" name="Absagen" dataDxfId="105"/>
+    <tableColumn id="1" xr3:uid="{E1FB3D0C-B874-4874-BACC-6872CF171957}" name="Tabellen Name" dataDxfId="98"/>
+    <tableColumn id="2" xr3:uid="{FFDD2777-2097-450C-B020-F133CF643855}" name="Geschlecht" dataDxfId="97"/>
+    <tableColumn id="3" xr3:uid="{8CF52BE2-8020-48BD-A36D-63F13A1878DE}" name="Mindest alter" dataDxfId="96"/>
+    <tableColumn id="4" xr3:uid="{FD3A030F-CD97-4B6F-8E8C-BC2E67D79F1D}" name="Maximales Alter" dataDxfId="95"/>
+    <tableColumn id="5" xr3:uid="{3E22B645-D77C-4509-B031-9914FCB91599}" name="Qualizeitraum anfang" dataDxfId="94"/>
+    <tableColumn id="6" xr3:uid="{AE299324-3C1C-4063-ADF9-54555A161734}" name="Qualizeitraum Ende" dataDxfId="93"/>
+    <tableColumn id="7" xr3:uid="{DCC178B3-11FC-4C53-BBC6-C2FDA2C89857}" name="Letzter Wettkampf am" dataDxfId="92"/>
+    <tableColumn id="8" xr3:uid="{2811DB01-60A5-4BE4-B6F9-A806398A602A}" name="Wertung" dataDxfId="91"/>
+    <tableColumn id="9" xr3:uid="{0C16DAFE-847D-4E9E-9604-3A7D9FE924D0}" name="Landesverband" dataDxfId="90"/>
+    <tableColumn id="10" xr3:uid="{7A8A4101-A553-4BD5-9116-9AA5876B9401}" name="OMS" dataDxfId="89"/>
+    <tableColumn id="11" xr3:uid="{9807C9BD-6499-45F6-ACE0-4D13D64EF675}" name="Pool-Länge" dataDxfId="88"/>
+    <tableColumn id="12" xr3:uid="{13D336DD-650F-4F2C-836F-361CA1528F6D}" name="Regelwerk" dataDxfId="87"/>
+    <tableColumn id="13" xr3:uid="{66660E2D-ADF2-4FB5-8A13-004F826EE908}" name="Referenz" dataDxfId="86"/>
+    <tableColumn id="19" xr3:uid="{D72EDF8B-ECC3-4FF7-ABE6-B60BCE4A5E26}" name="Referenz Jahr" dataDxfId="85"/>
+    <tableColumn id="20" xr3:uid="{7B18E667-70F7-4BC1-AB1B-21C019F2AA89}" name="Mindest Punktzahl" dataDxfId="84"/>
+    <tableColumn id="21" xr3:uid="{FC185946-681B-42A6-AB1A-FC1EABB668C5}" name="Mindest Disziplinen" dataDxfId="83"/>
+    <tableColumn id="14" xr3:uid="{6A2676FD-2EC7-4C41-A35E-A1597A38F932}" name="3-Kampf Regel" dataDxfId="82"/>
+    <tableColumn id="15" xr3:uid="{718E0917-4F83-4A2B-832F-EBB16D5E21BF}" name="Anzahl Nominierte" dataDxfId="81"/>
+    <tableColumn id="16" xr3:uid="{5C66A461-D647-4E00-A81C-FD7AD44D7CC2}" name="Anzahl Nachrücker" dataDxfId="80"/>
+    <tableColumn id="17" xr3:uid="{D434BDEC-293B-4B4E-A5E9-479438960A03}" name="Seiten Anzahl" dataDxfId="79"/>
+    <tableColumn id="18" xr3:uid="{80908229-9247-473F-81C0-9C9D4C12FF06}" name="Absagen" dataDxfId="78"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{16F87202-5A6A-4E2F-B973-3CE7EC2566C1}" name="DEM_konfig" displayName="DEM_konfig" ref="A1:X7" totalsRowShown="0" headerRowDxfId="104" dataDxfId="103">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{16F87202-5A6A-4E2F-B973-3CE7EC2566C1}" name="DEM_konfig" displayName="DEM_konfig" ref="A1:X7" totalsRowShown="0" headerRowDxfId="77" dataDxfId="76">
   <autoFilter ref="A1:X7" xr:uid="{16F87202-5A6A-4E2F-B973-3CE7EC2566C1}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -4470,37 +4470,37 @@
     <filterColumn colId="23" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="24">
-    <tableColumn id="1" xr3:uid="{4847B567-64E1-4AC3-8C4B-EFCF3F00CC6C}" name="Tabellen Name" dataDxfId="102"/>
-    <tableColumn id="2" xr3:uid="{6346FF3B-B334-4CD8-8B23-F2347E29C536}" name="Geschlecht" dataDxfId="101"/>
-    <tableColumn id="3" xr3:uid="{E793B48A-BC8A-439F-8AAF-6FD08104A619}" name="Mindest Alter" dataDxfId="100"/>
-    <tableColumn id="4" xr3:uid="{01A62C29-2F75-4107-A431-F69230BCCD0C}" name="Maximales Alter" dataDxfId="99"/>
-    <tableColumn id="5" xr3:uid="{B7E4DE90-7856-4A0C-9063-61414D7F227C}" name="Qualizeitraum anfang" dataDxfId="98"/>
-    <tableColumn id="6" xr3:uid="{B00F7CD1-82CB-42B9-A396-89F79EF419CA}" name="Qualizeitraum Ende" dataDxfId="97"/>
-    <tableColumn id="7" xr3:uid="{9E50DDE5-12E3-4BCB-801C-FBABCE309F0E}" name="Letzter Wettkampf am" dataDxfId="96"/>
-    <tableColumn id="8" xr3:uid="{57E68247-0FF2-48D8-8ACD-AB057E576A21}" name="Landesverband" dataDxfId="95"/>
-    <tableColumn id="9" xr3:uid="{EBAA439D-F69A-4C2A-8193-9AE08F1E57B8}" name="OMS" dataDxfId="94"/>
-    <tableColumn id="10" xr3:uid="{BBD11E7F-3DDF-428A-B005-4A40E6FA78DC}" name="Pool-Länge" dataDxfId="93"/>
-    <tableColumn id="11" xr3:uid="{6AE38DCA-A084-4F3D-A6A4-4E76E3E2CBC6}" name="Regelwerk" dataDxfId="92"/>
-    <tableColumn id="12" xr3:uid="{7F7470AD-5502-4CEE-BB4C-44BA308E61D7}" name="Seiten Anzahl" dataDxfId="91"/>
-    <tableColumn id="13" xr3:uid="{F416CBFA-4C9D-45CD-9BA7-E4BC57A08BC2}" name="PZ1 - 50m Retten" dataDxfId="90"/>
-    <tableColumn id="14" xr3:uid="{7117DBCA-0DA7-462C-84FE-0DC7E33B124C}" name="PZ1 - 100m Retten" dataDxfId="89"/>
-    <tableColumn id="15" xr3:uid="{E8630E91-DC30-4822-9E53-6D65487C3670}" name="PZ1 - 100m Kombi" dataDxfId="88"/>
-    <tableColumn id="16" xr3:uid="{4B3AA225-E042-430F-8259-D176887B4528}" name="PZ1 - 100m Lifesaver" dataDxfId="87"/>
-    <tableColumn id="17" xr3:uid="{798674BD-98CE-4531-BDFF-6AB06253AD7C}" name="PZ1 - 200m Super-Lifesaver" dataDxfId="86"/>
-    <tableColumn id="18" xr3:uid="{8809BB71-D58B-4E8B-A442-D0EB9A65A25D}" name="PZ1 - 200m Hindernis" dataDxfId="85"/>
-    <tableColumn id="19" xr3:uid="{93DCF463-806B-4117-B4E3-1FFAE976B37C}" name="PZ2 - 50m Retten" dataDxfId="84"/>
-    <tableColumn id="20" xr3:uid="{A514C961-559E-462F-B143-BA30974C0129}" name="PZ2 - 100m Retten" dataDxfId="83"/>
-    <tableColumn id="21" xr3:uid="{F1CF6143-45FE-498D-93D6-36F26D2F3C0B}" name="PZ2 - 100m Kombi" dataDxfId="82"/>
-    <tableColumn id="22" xr3:uid="{E90962FC-C214-467F-841F-40DF60E41456}" name="PZ2 - 100m Lifesaver" dataDxfId="81"/>
-    <tableColumn id="23" xr3:uid="{7FBC6334-C4C8-4B38-9F59-30ED95A44379}" name="PZ2 - 200m Super-Lifesaver" dataDxfId="80"/>
-    <tableColumn id="24" xr3:uid="{231BFF86-8F3A-4BA1-B25E-28175D9EDFA9}" name="PZ2 - 200m Hindernis" dataDxfId="79"/>
+    <tableColumn id="1" xr3:uid="{4847B567-64E1-4AC3-8C4B-EFCF3F00CC6C}" name="Tabellen Name" dataDxfId="75"/>
+    <tableColumn id="2" xr3:uid="{6346FF3B-B334-4CD8-8B23-F2347E29C536}" name="Geschlecht" dataDxfId="74"/>
+    <tableColumn id="3" xr3:uid="{E793B48A-BC8A-439F-8AAF-6FD08104A619}" name="Mindest Alter" dataDxfId="73"/>
+    <tableColumn id="4" xr3:uid="{01A62C29-2F75-4107-A431-F69230BCCD0C}" name="Maximales Alter" dataDxfId="72"/>
+    <tableColumn id="5" xr3:uid="{B7E4DE90-7856-4A0C-9063-61414D7F227C}" name="Qualizeitraum anfang" dataDxfId="71"/>
+    <tableColumn id="6" xr3:uid="{B00F7CD1-82CB-42B9-A396-89F79EF419CA}" name="Qualizeitraum Ende" dataDxfId="70"/>
+    <tableColumn id="7" xr3:uid="{9E50DDE5-12E3-4BCB-801C-FBABCE309F0E}" name="Letzter Wettkampf am" dataDxfId="69"/>
+    <tableColumn id="8" xr3:uid="{57E68247-0FF2-48D8-8ACD-AB057E576A21}" name="Landesverband" dataDxfId="68"/>
+    <tableColumn id="9" xr3:uid="{EBAA439D-F69A-4C2A-8193-9AE08F1E57B8}" name="OMS" dataDxfId="67"/>
+    <tableColumn id="10" xr3:uid="{BBD11E7F-3DDF-428A-B005-4A40E6FA78DC}" name="Pool-Länge" dataDxfId="66"/>
+    <tableColumn id="11" xr3:uid="{6AE38DCA-A084-4F3D-A6A4-4E76E3E2CBC6}" name="Regelwerk" dataDxfId="65"/>
+    <tableColumn id="12" xr3:uid="{7F7470AD-5502-4CEE-BB4C-44BA308E61D7}" name="Seiten Anzahl" dataDxfId="64"/>
+    <tableColumn id="13" xr3:uid="{F416CBFA-4C9D-45CD-9BA7-E4BC57A08BC2}" name="PZ1 - 50m Retten" dataDxfId="63"/>
+    <tableColumn id="14" xr3:uid="{7117DBCA-0DA7-462C-84FE-0DC7E33B124C}" name="PZ1 - 100m Retten" dataDxfId="62"/>
+    <tableColumn id="15" xr3:uid="{E8630E91-DC30-4822-9E53-6D65487C3670}" name="PZ1 - 100m Kombi" dataDxfId="61"/>
+    <tableColumn id="16" xr3:uid="{4B3AA225-E042-430F-8259-D176887B4528}" name="PZ1 - 100m Lifesaver" dataDxfId="60"/>
+    <tableColumn id="17" xr3:uid="{798674BD-98CE-4531-BDFF-6AB06253AD7C}" name="PZ1 - 200m Super-Lifesaver" dataDxfId="59"/>
+    <tableColumn id="18" xr3:uid="{8809BB71-D58B-4E8B-A442-D0EB9A65A25D}" name="PZ1 - 200m Hindernis" dataDxfId="58"/>
+    <tableColumn id="19" xr3:uid="{93DCF463-806B-4117-B4E3-1FFAE976B37C}" name="PZ2 - 50m Retten" dataDxfId="57"/>
+    <tableColumn id="20" xr3:uid="{A514C961-559E-462F-B143-BA30974C0129}" name="PZ2 - 100m Retten" dataDxfId="56"/>
+    <tableColumn id="21" xr3:uid="{F1CF6143-45FE-498D-93D6-36F26D2F3C0B}" name="PZ2 - 100m Kombi" dataDxfId="55"/>
+    <tableColumn id="22" xr3:uid="{E90962FC-C214-467F-841F-40DF60E41456}" name="PZ2 - 100m Lifesaver" dataDxfId="54"/>
+    <tableColumn id="23" xr3:uid="{7FBC6334-C4C8-4B38-9F59-30ED95A44379}" name="PZ2 - 200m Super-Lifesaver" dataDxfId="53"/>
+    <tableColumn id="24" xr3:uid="{231BFF86-8F3A-4BA1-B25E-28175D9EDFA9}" name="PZ2 - 200m Hindernis" dataDxfId="52"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D7CDEF11-F813-469D-9DE0-678961AB7005}" name="JRP_konfig" displayName="JRP_konfig" ref="A1:X3" totalsRowShown="0" headerRowDxfId="78" dataDxfId="77">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D7CDEF11-F813-469D-9DE0-678961AB7005}" name="JRP_konfig" displayName="JRP_konfig" ref="A1:X3" totalsRowShown="0" headerRowDxfId="51" dataDxfId="50">
   <autoFilter ref="A1:X3" xr:uid="{D7CDEF11-F813-469D-9DE0-678961AB7005}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -4528,64 +4528,64 @@
     <filterColumn colId="23" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="24">
-    <tableColumn id="1" xr3:uid="{021DA6E1-2C93-4474-9720-B6F016186D61}" name="Tabellen Name" dataDxfId="76"/>
-    <tableColumn id="2" xr3:uid="{733C1722-A9C9-4830-A9E2-FE62E96BCD98}" name="Geschlecht" dataDxfId="75"/>
-    <tableColumn id="3" xr3:uid="{80C0BF46-0E43-4947-BF86-B808C324772A}" name="Mindest Alter" dataDxfId="74"/>
-    <tableColumn id="4" xr3:uid="{DBA2A923-EEB7-43F9-A1A3-E78624448FB9}" name="Maximales Alter" dataDxfId="73"/>
-    <tableColumn id="5" xr3:uid="{3FDEE18A-328D-45AE-907D-69A916A93345}" name="Qualizeitraum anfang" dataDxfId="72"/>
-    <tableColumn id="6" xr3:uid="{BE002D7F-575F-4B60-9251-C71D93F59045}" name="Qualizeitraum Ende" dataDxfId="71"/>
-    <tableColumn id="7" xr3:uid="{208ABD57-DE4B-41D6-B9FC-93F2D8966E8D}" name="Letzter Wettkampf am" dataDxfId="70"/>
-    <tableColumn id="8" xr3:uid="{30C9697C-6550-4996-ADDB-7FEE5325B794}" name="Landesverband" dataDxfId="69"/>
-    <tableColumn id="9" xr3:uid="{ED2DAB77-EF46-4D8B-B8E4-90412E32E277}" name="OMS" dataDxfId="68"/>
-    <tableColumn id="10" xr3:uid="{AD534940-A91B-4A6E-9606-E3F3E517D401}" name="Pool-Länge" dataDxfId="67"/>
-    <tableColumn id="11" xr3:uid="{11F9D5D5-72FE-42CA-8624-01D513B4140F}" name="Regelwerk" dataDxfId="66"/>
-    <tableColumn id="12" xr3:uid="{3907872B-5438-4FBF-A045-3EF9EAACFC47}" name="Seiten Anzahl" dataDxfId="65"/>
-    <tableColumn id="13" xr3:uid="{FC821324-3638-40C0-BA1E-069B44E23C7A}" name="PZ1 - 50m Retten" dataDxfId="64"/>
-    <tableColumn id="14" xr3:uid="{70529619-443E-40D3-88C1-3E0F00BB2A50}" name="PZ1 - 100m Retten" dataDxfId="63"/>
-    <tableColumn id="15" xr3:uid="{EFA92FD2-C23F-42B3-83DC-5036513F19AF}" name="PZ1 - 100m Kombi" dataDxfId="62"/>
-    <tableColumn id="16" xr3:uid="{03309E52-8CF3-4E90-9EE6-A818901C3B32}" name="PZ1 - 100m Lifesaver" dataDxfId="61"/>
-    <tableColumn id="17" xr3:uid="{00B22013-AA11-4C17-9250-22060AE4B0A8}" name="PZ1 - 200m Super-Lifesaver" dataDxfId="60"/>
-    <tableColumn id="18" xr3:uid="{7E3508A9-0422-4561-A23E-53E613259B24}" name="PZ1 - 200m Hindernis" dataDxfId="59"/>
-    <tableColumn id="19" xr3:uid="{5CEA435F-F34B-4D8D-88D0-F5EBFF18B713}" name="PZ2 - 50m Retten" dataDxfId="58"/>
-    <tableColumn id="20" xr3:uid="{8585BE62-F7C4-4D5D-B287-052B43B08610}" name="PZ2 - 100m Retten" dataDxfId="57"/>
-    <tableColumn id="21" xr3:uid="{D981758B-ADAD-4E36-B787-0B0FDA808CA2}" name="PZ2 - 100m Kombi" dataDxfId="56"/>
-    <tableColumn id="22" xr3:uid="{1D4970A8-D22F-4962-934C-AEA295ED687A}" name="PZ2 - 100m Lifesaver" dataDxfId="55"/>
-    <tableColumn id="23" xr3:uid="{BE394430-C58F-4690-9615-44475E5AF9F8}" name="PZ2 - 200m Super-Lifesaver" dataDxfId="54"/>
-    <tableColumn id="24" xr3:uid="{A7036B1A-99CE-4F7C-AAB8-12E8B2696202}" name="PZ2 - 200m Hindernis" dataDxfId="53"/>
+    <tableColumn id="1" xr3:uid="{021DA6E1-2C93-4474-9720-B6F016186D61}" name="Tabellen Name" dataDxfId="49"/>
+    <tableColumn id="2" xr3:uid="{733C1722-A9C9-4830-A9E2-FE62E96BCD98}" name="Geschlecht" dataDxfId="48"/>
+    <tableColumn id="3" xr3:uid="{80C0BF46-0E43-4947-BF86-B808C324772A}" name="Mindest Alter" dataDxfId="47"/>
+    <tableColumn id="4" xr3:uid="{DBA2A923-EEB7-43F9-A1A3-E78624448FB9}" name="Maximales Alter" dataDxfId="46"/>
+    <tableColumn id="5" xr3:uid="{3FDEE18A-328D-45AE-907D-69A916A93345}" name="Qualizeitraum anfang" dataDxfId="45"/>
+    <tableColumn id="6" xr3:uid="{BE002D7F-575F-4B60-9251-C71D93F59045}" name="Qualizeitraum Ende" dataDxfId="44"/>
+    <tableColumn id="7" xr3:uid="{208ABD57-DE4B-41D6-B9FC-93F2D8966E8D}" name="Letzter Wettkampf am" dataDxfId="43"/>
+    <tableColumn id="8" xr3:uid="{30C9697C-6550-4996-ADDB-7FEE5325B794}" name="Landesverband" dataDxfId="42"/>
+    <tableColumn id="9" xr3:uid="{ED2DAB77-EF46-4D8B-B8E4-90412E32E277}" name="OMS" dataDxfId="41"/>
+    <tableColumn id="10" xr3:uid="{AD534940-A91B-4A6E-9606-E3F3E517D401}" name="Pool-Länge" dataDxfId="40"/>
+    <tableColumn id="11" xr3:uid="{11F9D5D5-72FE-42CA-8624-01D513B4140F}" name="Regelwerk" dataDxfId="39"/>
+    <tableColumn id="12" xr3:uid="{3907872B-5438-4FBF-A045-3EF9EAACFC47}" name="Seiten Anzahl" dataDxfId="38"/>
+    <tableColumn id="13" xr3:uid="{FC821324-3638-40C0-BA1E-069B44E23C7A}" name="PZ1 - 50m Retten" dataDxfId="37"/>
+    <tableColumn id="14" xr3:uid="{70529619-443E-40D3-88C1-3E0F00BB2A50}" name="PZ1 - 100m Retten" dataDxfId="36"/>
+    <tableColumn id="15" xr3:uid="{EFA92FD2-C23F-42B3-83DC-5036513F19AF}" name="PZ1 - 100m Kombi" dataDxfId="35"/>
+    <tableColumn id="16" xr3:uid="{03309E52-8CF3-4E90-9EE6-A818901C3B32}" name="PZ1 - 100m Lifesaver" dataDxfId="34"/>
+    <tableColumn id="17" xr3:uid="{00B22013-AA11-4C17-9250-22060AE4B0A8}" name="PZ1 - 200m Super-Lifesaver" dataDxfId="33"/>
+    <tableColumn id="18" xr3:uid="{7E3508A9-0422-4561-A23E-53E613259B24}" name="PZ1 - 200m Hindernis" dataDxfId="32"/>
+    <tableColumn id="19" xr3:uid="{5CEA435F-F34B-4D8D-88D0-F5EBFF18B713}" name="PZ2 - 50m Retten" dataDxfId="31"/>
+    <tableColumn id="20" xr3:uid="{8585BE62-F7C4-4D5D-B287-052B43B08610}" name="PZ2 - 100m Retten" dataDxfId="30"/>
+    <tableColumn id="21" xr3:uid="{D981758B-ADAD-4E36-B787-0B0FDA808CA2}" name="PZ2 - 100m Kombi" dataDxfId="29"/>
+    <tableColumn id="22" xr3:uid="{1D4970A8-D22F-4962-934C-AEA295ED687A}" name="PZ2 - 100m Lifesaver" dataDxfId="28"/>
+    <tableColumn id="23" xr3:uid="{BE394430-C58F-4690-9615-44475E5AF9F8}" name="PZ2 - 200m Super-Lifesaver" dataDxfId="27"/>
+    <tableColumn id="24" xr3:uid="{A7036B1A-99CE-4F7C-AAB8-12E8B2696202}" name="PZ2 - 200m Hindernis" dataDxfId="26"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{FED162EE-531E-453F-8C25-562B59ECE709}" name="LK_konfig" displayName="LK_konfig" ref="A1:Y37" totalsRowShown="0" headerRowDxfId="26" dataDxfId="25">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{FED162EE-531E-453F-8C25-562B59ECE709}" name="LK_konfig" displayName="LK_konfig" ref="A1:Y37" totalsRowShown="0" headerRowDxfId="228" dataDxfId="227">
   <autoFilter ref="A1:Y37" xr:uid="{FED162EE-531E-453F-8C25-562B59ECE709}"/>
   <tableColumns count="25">
-    <tableColumn id="1" xr3:uid="{F985A4F0-6B8C-47C6-816F-1A31A4973EB2}" name="Tabellen Name" dataDxfId="24"/>
-    <tableColumn id="2" xr3:uid="{5E5AD859-71A2-4E8E-B434-431A89C05C57}" name="Geschlecht" dataDxfId="23"/>
-    <tableColumn id="3" xr3:uid="{85BB892C-E151-404B-8974-FC5199E0909C}" name="Mindest Alter" dataDxfId="22"/>
-    <tableColumn id="4" xr3:uid="{790F6CF9-E475-4082-AE03-D30EDE22FB61}" name="Maximales Alter" dataDxfId="21"/>
-    <tableColumn id="5" xr3:uid="{FD4B0E6E-9B64-4731-A50F-D3CE3A4ED3FC}" name="Qualizeitraum anfang" dataDxfId="20"/>
-    <tableColumn id="6" xr3:uid="{5E84CAD2-C403-49B9-BB06-D56EC5784C8C}" name="Qualizeitraum Ende" dataDxfId="19"/>
-    <tableColumn id="7" xr3:uid="{6323F8E2-5DA4-4E5B-9C35-1E8C219ADECF}" name="Letzter Wettkampf am" dataDxfId="18"/>
-    <tableColumn id="8" xr3:uid="{D2845930-152E-432F-92A0-E7F7A3EE1FF0}" name="Landesverband" dataDxfId="17"/>
-    <tableColumn id="9" xr3:uid="{87046373-5CCD-41EC-B34C-C753E71FD26C}" name="OMS" dataDxfId="16"/>
-    <tableColumn id="10" xr3:uid="{A685FE01-F23C-4533-B399-857F5A1F6C37}" name="Pool-Länge" dataDxfId="15"/>
-    <tableColumn id="11" xr3:uid="{11E0A508-0C9D-4CB6-952E-7FAC5D05BDCD}" name="Regelwerk" dataDxfId="14"/>
-    <tableColumn id="12" xr3:uid="{F220BD5F-C3B5-4935-996A-BFCDF9F392D9}" name="Seiten Anzahl" dataDxfId="13"/>
-    <tableColumn id="25" xr3:uid="{7CDE58FE-A5B8-4329-9F48-3913AEBA21FC}" name="mind. erreichte Normen" dataDxfId="12"/>
-    <tableColumn id="13" xr3:uid="{A0A5E62D-9354-426D-9A08-13E43F36F55B}" name="PZ1 - 50m Retten" dataDxfId="11"/>
-    <tableColumn id="14" xr3:uid="{5D70F54C-57E9-45E2-BC99-0DBB0422383E}" name="PZ1 - 100m Retten" dataDxfId="10"/>
-    <tableColumn id="15" xr3:uid="{1C0CF5DB-156E-4813-A8BA-9EA29A40ABF3}" name="PZ1 - 100m Kombi" dataDxfId="9"/>
-    <tableColumn id="16" xr3:uid="{691CD4E1-13D9-4455-A2D1-14C9BC41A0EA}" name="PZ1 - 100m Lifesaver" dataDxfId="8"/>
-    <tableColumn id="17" xr3:uid="{CE1BA235-770B-4FA4-B327-187675DDA6B8}" name="PZ1 - 200m Super-Lifesaver" dataDxfId="7"/>
-    <tableColumn id="18" xr3:uid="{A326EF87-5FF5-4042-85D3-7806FEED4CFA}" name="PZ1 - 200m Hindernis" dataDxfId="6"/>
-    <tableColumn id="19" xr3:uid="{ABA5540C-4356-4D68-8579-E660F9FD6EA8}" name="PZ2 - 50m Retten" dataDxfId="5"/>
-    <tableColumn id="20" xr3:uid="{62E98437-16C9-4433-8683-E3C8A1B80E76}" name="PZ2 - 100m Retten" dataDxfId="4"/>
-    <tableColumn id="21" xr3:uid="{ED4E9448-4073-4B27-A491-5385DED08F83}" name="PZ2 - 100m Kombi" dataDxfId="3"/>
-    <tableColumn id="22" xr3:uid="{53F3DC0A-267B-434A-BD8A-320943916288}" name="PZ2 - 100m Lifesaver" dataDxfId="2"/>
-    <tableColumn id="23" xr3:uid="{1586F43C-8AD2-4942-A098-687AF0A028AC}" name="PZ2 - 200m Super-Lifesaver" dataDxfId="1"/>
-    <tableColumn id="24" xr3:uid="{98AA496B-EB58-437E-91F5-800894DDD85F}" name="PZ2 - 200m Hindernis" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{F985A4F0-6B8C-47C6-816F-1A31A4973EB2}" name="Tabellen Name" dataDxfId="226"/>
+    <tableColumn id="2" xr3:uid="{5E5AD859-71A2-4E8E-B434-431A89C05C57}" name="Geschlecht" dataDxfId="225"/>
+    <tableColumn id="3" xr3:uid="{85BB892C-E151-404B-8974-FC5199E0909C}" name="Mindest Alter" dataDxfId="224"/>
+    <tableColumn id="4" xr3:uid="{790F6CF9-E475-4082-AE03-D30EDE22FB61}" name="Maximales Alter" dataDxfId="223"/>
+    <tableColumn id="5" xr3:uid="{FD4B0E6E-9B64-4731-A50F-D3CE3A4ED3FC}" name="Qualizeitraum anfang" dataDxfId="222"/>
+    <tableColumn id="6" xr3:uid="{5E84CAD2-C403-49B9-BB06-D56EC5784C8C}" name="Qualizeitraum Ende" dataDxfId="221"/>
+    <tableColumn id="7" xr3:uid="{6323F8E2-5DA4-4E5B-9C35-1E8C219ADECF}" name="Letzter Wettkampf am" dataDxfId="220"/>
+    <tableColumn id="8" xr3:uid="{D2845930-152E-432F-92A0-E7F7A3EE1FF0}" name="Landesverband" dataDxfId="219"/>
+    <tableColumn id="9" xr3:uid="{87046373-5CCD-41EC-B34C-C753E71FD26C}" name="OMS" dataDxfId="218"/>
+    <tableColumn id="10" xr3:uid="{A685FE01-F23C-4533-B399-857F5A1F6C37}" name="Pool-Länge" dataDxfId="217"/>
+    <tableColumn id="11" xr3:uid="{11E0A508-0C9D-4CB6-952E-7FAC5D05BDCD}" name="Regelwerk" dataDxfId="216"/>
+    <tableColumn id="12" xr3:uid="{F220BD5F-C3B5-4935-996A-BFCDF9F392D9}" name="Seiten Anzahl" dataDxfId="215"/>
+    <tableColumn id="25" xr3:uid="{7CDE58FE-A5B8-4329-9F48-3913AEBA21FC}" name="mind. erreichte Normen" dataDxfId="214"/>
+    <tableColumn id="13" xr3:uid="{A0A5E62D-9354-426D-9A08-13E43F36F55B}" name="PZ1 - 50m Retten" dataDxfId="213"/>
+    <tableColumn id="14" xr3:uid="{5D70F54C-57E9-45E2-BC99-0DBB0422383E}" name="PZ1 - 100m Retten" dataDxfId="212"/>
+    <tableColumn id="15" xr3:uid="{1C0CF5DB-156E-4813-A8BA-9EA29A40ABF3}" name="PZ1 - 100m Kombi" dataDxfId="211"/>
+    <tableColumn id="16" xr3:uid="{691CD4E1-13D9-4455-A2D1-14C9BC41A0EA}" name="PZ1 - 100m Lifesaver" dataDxfId="210"/>
+    <tableColumn id="17" xr3:uid="{CE1BA235-770B-4FA4-B327-187675DDA6B8}" name="PZ1 - 200m Super-Lifesaver" dataDxfId="209"/>
+    <tableColumn id="18" xr3:uid="{A326EF87-5FF5-4042-85D3-7806FEED4CFA}" name="PZ1 - 200m Hindernis" dataDxfId="208"/>
+    <tableColumn id="19" xr3:uid="{ABA5540C-4356-4D68-8579-E660F9FD6EA8}" name="PZ2 - 50m Retten" dataDxfId="207"/>
+    <tableColumn id="20" xr3:uid="{62E98437-16C9-4433-8683-E3C8A1B80E76}" name="PZ2 - 100m Retten" dataDxfId="206"/>
+    <tableColumn id="21" xr3:uid="{ED4E9448-4073-4B27-A491-5385DED08F83}" name="PZ2 - 100m Kombi" dataDxfId="205"/>
+    <tableColumn id="22" xr3:uid="{53F3DC0A-267B-434A-BD8A-320943916288}" name="PZ2 - 100m Lifesaver" dataDxfId="204"/>
+    <tableColumn id="23" xr3:uid="{1586F43C-8AD2-4942-A098-687AF0A028AC}" name="PZ2 - 200m Super-Lifesaver" dataDxfId="203"/>
+    <tableColumn id="24" xr3:uid="{98AA496B-EB58-437E-91F5-800894DDD85F}" name="PZ2 - 200m Hindernis" dataDxfId="202"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4595,12 +4595,12 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{888CE7BE-8313-44C0-AE38-83992EABD44D}" name="LK_Kalender" displayName="LK_Kalender" ref="A1:H8" totalsRowShown="0">
   <autoFilter ref="A1:H8" xr:uid="{888CE7BE-8313-44C0-AE38-83992EABD44D}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{B26B9E90-F378-41EF-B35E-CE240017E4BE}" name="datum von" dataDxfId="52"/>
+    <tableColumn id="1" xr3:uid="{B26B9E90-F378-41EF-B35E-CE240017E4BE}" name="datum von" dataDxfId="25"/>
     <tableColumn id="2" xr3:uid="{38211212-0A92-428C-895C-E4CA68F52818}" name="datum bis"/>
-    <tableColumn id="3" xr3:uid="{66E541C6-0A5E-4B2D-9B89-5E52F449A4A6}" name="uhrzeit von" dataDxfId="51"/>
-    <tableColumn id="4" xr3:uid="{D93C06A2-29AD-4073-8E3C-A685B4474CC8}" name="uhrzeit bis" dataDxfId="50"/>
-    <tableColumn id="5" xr3:uid="{C5C3979C-B528-44E8-A5A6-36F020A6034F}" name="titel" dataDxfId="49"/>
-    <tableColumn id="6" xr3:uid="{9DC09E1D-44FD-40ED-9EBE-86A8E61C38B2}" name="meta" dataDxfId="48"/>
+    <tableColumn id="3" xr3:uid="{66E541C6-0A5E-4B2D-9B89-5E52F449A4A6}" name="uhrzeit von" dataDxfId="24"/>
+    <tableColumn id="4" xr3:uid="{D93C06A2-29AD-4073-8E3C-A685B4474CC8}" name="uhrzeit bis" dataDxfId="23"/>
+    <tableColumn id="5" xr3:uid="{C5C3979C-B528-44E8-A5A6-36F020A6034F}" name="titel" dataDxfId="22"/>
+    <tableColumn id="6" xr3:uid="{9DC09E1D-44FD-40ED-9EBE-86A8E61C38B2}" name="meta" dataDxfId="21"/>
     <tableColumn id="7" xr3:uid="{E7E62A34-7A76-4361-937D-F4DE76E6E7CC}" name="ort"/>
     <tableColumn id="8" xr3:uid="{84F02734-FC16-406B-ACCA-0CCDF547D94C}" name="kader"/>
   </tableColumns>
@@ -8542,52 +8542,52 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B5:G31">
-    <cfRule type="expression" dxfId="47" priority="15">
+    <cfRule type="expression" dxfId="20" priority="15">
       <formula>B5&lt;&gt;B4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H5:M31">
-    <cfRule type="expression" dxfId="46" priority="14">
+    <cfRule type="expression" dxfId="19" priority="14">
       <formula>H5&lt;&gt;H4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N5:S31">
-    <cfRule type="expression" dxfId="45" priority="13">
+    <cfRule type="expression" dxfId="18" priority="13">
       <formula>N5&lt;&gt;N4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="T5:Y31">
-    <cfRule type="expression" dxfId="44" priority="12">
+    <cfRule type="expression" dxfId="17" priority="12">
       <formula>T5&lt;&gt;T4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z5:AE31">
-    <cfRule type="expression" dxfId="43" priority="9">
+    <cfRule type="expression" dxfId="16" priority="9">
       <formula>Z5&lt;&gt;Z4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AF5:AK31">
-    <cfRule type="expression" dxfId="42" priority="8">
+    <cfRule type="expression" dxfId="15" priority="8">
       <formula>AF5&lt;&gt;AF4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AL5:AN31">
-    <cfRule type="expression" dxfId="41" priority="6">
+    <cfRule type="expression" dxfId="14" priority="6">
       <formula>AL5&lt;&gt;AL4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AO5:AQ31">
-    <cfRule type="expression" dxfId="40" priority="5">
+    <cfRule type="expression" dxfId="13" priority="5">
       <formula>AO5&lt;&gt;AO4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AR5:AT31">
-    <cfRule type="expression" dxfId="39" priority="2">
+    <cfRule type="expression" dxfId="12" priority="2">
       <formula>AR5&lt;&gt;AR4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AU5:AW31">
-    <cfRule type="expression" dxfId="38" priority="1">
+    <cfRule type="expression" dxfId="11" priority="1">
       <formula>AU5&lt;&gt;AU4</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8809,7 +8809,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:H8">
-    <cfRule type="expression" dxfId="27" priority="1">
+    <cfRule type="expression" dxfId="0" priority="1">
       <formula>$A2&lt;TODAY()</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9815,22 +9815,22 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B6:G6">
-    <cfRule type="expression" dxfId="37" priority="20">
+    <cfRule type="expression" dxfId="10" priority="20">
       <formula>B6&lt;&gt;B4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7:G32">
-    <cfRule type="expression" dxfId="36" priority="1">
+    <cfRule type="expression" dxfId="9" priority="1">
       <formula>B7&lt;&gt;B6</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H6:M6">
-    <cfRule type="expression" dxfId="35" priority="22">
+    <cfRule type="expression" dxfId="8" priority="22">
       <formula>H6&lt;&gt;H4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H7:M32">
-    <cfRule type="expression" dxfId="34" priority="2">
+    <cfRule type="expression" dxfId="7" priority="2">
       <formula>H7&lt;&gt;H6</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11161,22 +11161,22 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B6:G6">
-    <cfRule type="expression" dxfId="33" priority="19">
+    <cfRule type="expression" dxfId="6" priority="19">
       <formula>B6&lt;&gt;B4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7:G32">
-    <cfRule type="expression" dxfId="32" priority="2">
+    <cfRule type="expression" dxfId="5" priority="2">
       <formula>B7&lt;&gt;B6</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H6:M6">
-    <cfRule type="expression" dxfId="31" priority="20">
+    <cfRule type="expression" dxfId="4" priority="20">
       <formula>H6&lt;&gt;H4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H7:M32">
-    <cfRule type="expression" dxfId="30" priority="1">
+    <cfRule type="expression" dxfId="3" priority="1">
       <formula>H7&lt;&gt;H6</formula>
     </cfRule>
   </conditionalFormatting>
@@ -13610,7 +13610,9 @@
       <c r="I14" s="25" t="s">
         <v>146</v>
       </c>
-      <c r="J14" s="25"/>
+      <c r="J14" s="25">
+        <v>50</v>
+      </c>
       <c r="K14" s="25"/>
       <c r="L14" s="25">
         <v>10</v>
@@ -13677,7 +13679,9 @@
       <c r="I15" s="25" t="s">
         <v>146</v>
       </c>
-      <c r="J15" s="25"/>
+      <c r="J15" s="25">
+        <v>50</v>
+      </c>
       <c r="K15" s="25"/>
       <c r="L15" s="25">
         <v>10</v>
@@ -13744,7 +13748,9 @@
       <c r="I16" s="25" t="s">
         <v>146</v>
       </c>
-      <c r="J16" s="25"/>
+      <c r="J16" s="25">
+        <v>50</v>
+      </c>
       <c r="K16" s="25"/>
       <c r="L16" s="25">
         <v>10</v>
@@ -13811,7 +13817,9 @@
       <c r="I17" s="25" t="s">
         <v>146</v>
       </c>
-      <c r="J17" s="25"/>
+      <c r="J17" s="25">
+        <v>50</v>
+      </c>
       <c r="K17" s="25"/>
       <c r="L17" s="25">
         <v>10</v>
@@ -13878,7 +13886,9 @@
       <c r="I18" s="25" t="s">
         <v>146</v>
       </c>
-      <c r="J18" s="25"/>
+      <c r="J18" s="25">
+        <v>50</v>
+      </c>
       <c r="K18" s="25"/>
       <c r="L18" s="25">
         <v>10</v>
@@ -13945,7 +13955,9 @@
       <c r="I19" s="25" t="s">
         <v>146</v>
       </c>
-      <c r="J19" s="25"/>
+      <c r="J19" s="25">
+        <v>50</v>
+      </c>
       <c r="K19" s="25"/>
       <c r="L19" s="25">
         <v>10</v>
@@ -14012,7 +14024,9 @@
       <c r="I20" s="25" t="s">
         <v>146</v>
       </c>
-      <c r="J20" s="25"/>
+      <c r="J20" s="25">
+        <v>50</v>
+      </c>
       <c r="K20" s="25"/>
       <c r="L20" s="25">
         <v>10</v>
@@ -14079,7 +14093,9 @@
       <c r="I21" s="25" t="s">
         <v>146</v>
       </c>
-      <c r="J21" s="25"/>
+      <c r="J21" s="25">
+        <v>50</v>
+      </c>
       <c r="K21" s="25"/>
       <c r="L21" s="25">
         <v>10</v>
@@ -14146,7 +14162,9 @@
       <c r="I22" s="25" t="s">
         <v>146</v>
       </c>
-      <c r="J22" s="25"/>
+      <c r="J22" s="25">
+        <v>50</v>
+      </c>
       <c r="K22" s="25"/>
       <c r="L22" s="25">
         <v>10</v>
@@ -14213,7 +14231,9 @@
       <c r="I23" s="25" t="s">
         <v>146</v>
       </c>
-      <c r="J23" s="25"/>
+      <c r="J23" s="25">
+        <v>50</v>
+      </c>
       <c r="K23" s="25"/>
       <c r="L23" s="25">
         <v>10</v>
@@ -14280,7 +14300,9 @@
       <c r="I24" s="25" t="s">
         <v>146</v>
       </c>
-      <c r="J24" s="25"/>
+      <c r="J24" s="25">
+        <v>50</v>
+      </c>
       <c r="K24" s="25"/>
       <c r="L24" s="25">
         <v>10</v>
@@ -14347,7 +14369,9 @@
       <c r="I25" s="25" t="s">
         <v>146</v>
       </c>
-      <c r="J25" s="25"/>
+      <c r="J25" s="25">
+        <v>50</v>
+      </c>
       <c r="K25" s="25"/>
       <c r="L25" s="25">
         <v>10</v>
@@ -14414,7 +14438,9 @@
       <c r="I26" s="25" t="s">
         <v>146</v>
       </c>
-      <c r="J26" s="25"/>
+      <c r="J26" s="25">
+        <v>50</v>
+      </c>
       <c r="K26" s="25"/>
       <c r="L26" s="25">
         <v>10</v>
@@ -14481,7 +14507,9 @@
       <c r="I27" s="25" t="s">
         <v>146</v>
       </c>
-      <c r="J27" s="25"/>
+      <c r="J27" s="25">
+        <v>50</v>
+      </c>
       <c r="K27" s="25"/>
       <c r="L27" s="25">
         <v>10</v>
@@ -14548,7 +14576,9 @@
       <c r="I28" s="25" t="s">
         <v>146</v>
       </c>
-      <c r="J28" s="25"/>
+      <c r="J28" s="25">
+        <v>50</v>
+      </c>
       <c r="K28" s="25"/>
       <c r="L28" s="25">
         <v>10</v>
@@ -14615,7 +14645,9 @@
       <c r="I29" s="25" t="s">
         <v>146</v>
       </c>
-      <c r="J29" s="25"/>
+      <c r="J29" s="25">
+        <v>50</v>
+      </c>
       <c r="K29" s="25"/>
       <c r="L29" s="25">
         <v>10</v>
@@ -14682,7 +14714,9 @@
       <c r="I30" s="25" t="s">
         <v>146</v>
       </c>
-      <c r="J30" s="25"/>
+      <c r="J30" s="25">
+        <v>50</v>
+      </c>
       <c r="K30" s="25"/>
       <c r="L30" s="25">
         <v>10</v>
@@ -14749,7 +14783,9 @@
       <c r="I31" s="25" t="s">
         <v>146</v>
       </c>
-      <c r="J31" s="25"/>
+      <c r="J31" s="25">
+        <v>50</v>
+      </c>
       <c r="K31" s="25"/>
       <c r="L31" s="25">
         <v>10</v>
@@ -14816,7 +14852,9 @@
       <c r="I32" s="25" t="s">
         <v>146</v>
       </c>
-      <c r="J32" s="25"/>
+      <c r="J32" s="25">
+        <v>50</v>
+      </c>
       <c r="K32" s="25"/>
       <c r="L32" s="25">
         <v>10</v>
@@ -14883,7 +14921,9 @@
       <c r="I33" s="25" t="s">
         <v>146</v>
       </c>
-      <c r="J33" s="25"/>
+      <c r="J33" s="25">
+        <v>50</v>
+      </c>
       <c r="K33" s="25"/>
       <c r="L33" s="25">
         <v>10</v>
@@ -14950,7 +14990,9 @@
       <c r="I34" s="25" t="s">
         <v>146</v>
       </c>
-      <c r="J34" s="25"/>
+      <c r="J34" s="25">
+        <v>50</v>
+      </c>
       <c r="K34" s="25"/>
       <c r="L34" s="25">
         <v>10</v>
@@ -15017,7 +15059,9 @@
       <c r="I35" s="25" t="s">
         <v>146</v>
       </c>
-      <c r="J35" s="25"/>
+      <c r="J35" s="25">
+        <v>50</v>
+      </c>
       <c r="K35" s="25"/>
       <c r="L35" s="25">
         <v>10</v>
@@ -15084,7 +15128,9 @@
       <c r="I36" s="25" t="s">
         <v>146</v>
       </c>
-      <c r="J36" s="25"/>
+      <c r="J36" s="25">
+        <v>50</v>
+      </c>
       <c r="K36" s="25"/>
       <c r="L36" s="25">
         <v>10</v>
@@ -15151,7 +15197,9 @@
       <c r="I37" s="25" t="s">
         <v>146</v>
       </c>
-      <c r="J37" s="25"/>
+      <c r="J37" s="25">
+        <v>50</v>
+      </c>
       <c r="K37" s="25"/>
       <c r="L37" s="25">
         <v>10</v>
@@ -15215,133 +15263,133 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:78" s="40" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="125">
+      <c r="A1" s="106">
         <v>2025</v>
       </c>
       <c r="B1" s="45" t="str">
         <f ca="1">CONCATENATE("in: ",YEAR(TODAY())-1," für: ", YEAR(TODAY()))</f>
         <v>in: 2025 für: 2026</v>
       </c>
-      <c r="C1" s="106" t="s">
+      <c r="C1" s="107" t="s">
         <v>220</v>
       </c>
-      <c r="D1" s="106"/>
-      <c r="E1" s="107"/>
-      <c r="F1" s="110" t="s">
+      <c r="D1" s="107"/>
+      <c r="E1" s="108"/>
+      <c r="F1" s="109" t="s">
         <v>221</v>
       </c>
-      <c r="G1" s="111"/>
-      <c r="H1" s="111"/>
-      <c r="I1" s="111"/>
-      <c r="J1" s="112"/>
-      <c r="K1" s="116" t="s">
+      <c r="G1" s="110"/>
+      <c r="H1" s="110"/>
+      <c r="I1" s="110"/>
+      <c r="J1" s="111"/>
+      <c r="K1" s="112" t="s">
         <v>225</v>
       </c>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="118"/>
-      <c r="O1" s="108" t="s">
+      <c r="L1" s="113"/>
+      <c r="M1" s="113"/>
+      <c r="N1" s="114"/>
+      <c r="O1" s="132" t="s">
         <v>222</v>
       </c>
-      <c r="P1" s="108"/>
-      <c r="Q1" s="109"/>
-      <c r="R1" s="122" t="s">
+      <c r="P1" s="132"/>
+      <c r="Q1" s="133"/>
+      <c r="R1" s="134" t="s">
         <v>223</v>
       </c>
-      <c r="S1" s="123"/>
-      <c r="T1" s="123"/>
-      <c r="U1" s="123"/>
-      <c r="V1" s="124"/>
-      <c r="W1" s="119" t="s">
+      <c r="S1" s="135"/>
+      <c r="T1" s="135"/>
+      <c r="U1" s="135"/>
+      <c r="V1" s="136"/>
+      <c r="W1" s="137" t="s">
         <v>226</v>
       </c>
-      <c r="X1" s="120"/>
-      <c r="Y1" s="120"/>
-      <c r="Z1" s="121"/>
+      <c r="X1" s="138"/>
+      <c r="Y1" s="138"/>
+      <c r="Z1" s="139"/>
       <c r="AA1"/>
       <c r="AB1" s="45" t="str">
         <f ca="1">CONCATENATE("in: ",YEAR(TODAY())-1," für: ", YEAR(TODAY()))</f>
         <v>in: 2025 für: 2026</v>
       </c>
-      <c r="AC1" s="126" t="s">
+      <c r="AC1" s="115" t="s">
         <v>227</v>
       </c>
-      <c r="AD1" s="126"/>
-      <c r="AE1" s="127"/>
-      <c r="AF1" s="128" t="s">
+      <c r="AD1" s="115"/>
+      <c r="AE1" s="116"/>
+      <c r="AF1" s="117" t="s">
         <v>228</v>
       </c>
-      <c r="AG1" s="129"/>
-      <c r="AH1" s="129"/>
-      <c r="AI1" s="129"/>
-      <c r="AJ1" s="130"/>
-      <c r="AK1" s="131" t="s">
+      <c r="AG1" s="118"/>
+      <c r="AH1" s="118"/>
+      <c r="AI1" s="118"/>
+      <c r="AJ1" s="119"/>
+      <c r="AK1" s="120" t="s">
         <v>229</v>
       </c>
-      <c r="AL1" s="132"/>
-      <c r="AM1" s="132"/>
-      <c r="AN1" s="133"/>
-      <c r="AO1" s="134" t="s">
+      <c r="AL1" s="121"/>
+      <c r="AM1" s="121"/>
+      <c r="AN1" s="122"/>
+      <c r="AO1" s="123" t="s">
         <v>230</v>
       </c>
-      <c r="AP1" s="135"/>
-      <c r="AQ1" s="136"/>
-      <c r="AR1" s="137" t="s">
+      <c r="AP1" s="124"/>
+      <c r="AQ1" s="125"/>
+      <c r="AR1" s="126" t="s">
         <v>231</v>
       </c>
-      <c r="AS1" s="138"/>
-      <c r="AT1" s="138"/>
-      <c r="AU1" s="138"/>
-      <c r="AV1" s="139"/>
-      <c r="AW1" s="113" t="s">
+      <c r="AS1" s="127"/>
+      <c r="AT1" s="127"/>
+      <c r="AU1" s="127"/>
+      <c r="AV1" s="128"/>
+      <c r="AW1" s="129" t="s">
         <v>232</v>
       </c>
-      <c r="AX1" s="114"/>
-      <c r="AY1" s="114"/>
-      <c r="AZ1" s="115"/>
+      <c r="AX1" s="130"/>
+      <c r="AY1" s="130"/>
+      <c r="AZ1" s="131"/>
       <c r="BB1" s="45" t="str">
         <f ca="1">CONCATENATE("in: ",YEAR(TODAY())-1," für: ", YEAR(TODAY()))</f>
         <v>in: 2025 für: 2026</v>
       </c>
-      <c r="BC1" s="106" t="s">
+      <c r="BC1" s="107" t="s">
         <v>233</v>
       </c>
-      <c r="BD1" s="106"/>
-      <c r="BE1" s="107"/>
-      <c r="BF1" s="110" t="s">
+      <c r="BD1" s="107"/>
+      <c r="BE1" s="108"/>
+      <c r="BF1" s="109" t="s">
         <v>234</v>
       </c>
-      <c r="BG1" s="111"/>
-      <c r="BH1" s="111"/>
-      <c r="BI1" s="111"/>
-      <c r="BJ1" s="112"/>
-      <c r="BK1" s="116" t="s">
+      <c r="BG1" s="110"/>
+      <c r="BH1" s="110"/>
+      <c r="BI1" s="110"/>
+      <c r="BJ1" s="111"/>
+      <c r="BK1" s="112" t="s">
         <v>235</v>
       </c>
-      <c r="BL1" s="117"/>
-      <c r="BM1" s="117"/>
-      <c r="BN1" s="118"/>
-      <c r="BO1" s="108" t="s">
+      <c r="BL1" s="113"/>
+      <c r="BM1" s="113"/>
+      <c r="BN1" s="114"/>
+      <c r="BO1" s="132" t="s">
         <v>241</v>
       </c>
-      <c r="BP1" s="108"/>
-      <c r="BQ1" s="109"/>
-      <c r="BR1" s="122" t="s">
+      <c r="BP1" s="132"/>
+      <c r="BQ1" s="133"/>
+      <c r="BR1" s="134" t="s">
         <v>242</v>
       </c>
-      <c r="BS1" s="123"/>
-      <c r="BT1" s="123"/>
-      <c r="BU1" s="123"/>
-      <c r="BV1" s="124"/>
-      <c r="BW1" s="119" t="s">
+      <c r="BS1" s="135"/>
+      <c r="BT1" s="135"/>
+      <c r="BU1" s="135"/>
+      <c r="BV1" s="136"/>
+      <c r="BW1" s="137" t="s">
         <v>236</v>
       </c>
-      <c r="BX1" s="120"/>
-      <c r="BY1" s="120"/>
-      <c r="BZ1" s="121"/>
+      <c r="BX1" s="138"/>
+      <c r="BY1" s="138"/>
+      <c r="BZ1" s="139"/>
     </row>
     <row r="2" spans="1:78" s="94" customFormat="1" ht="21.4" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="125"/>
+      <c r="A2" s="106"/>
       <c r="B2" s="46" t="s">
         <v>224</v>
       </c>
@@ -15642,7 +15690,7 @@
       </c>
     </row>
     <row r="3" spans="1:78" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A3" s="125"/>
+      <c r="A3" s="106"/>
       <c r="B3" s="47" t="s">
         <v>0</v>
       </c>
@@ -15895,7 +15943,7 @@
       </c>
     </row>
     <row r="4" spans="1:78" x14ac:dyDescent="0.45">
-      <c r="A4" s="125"/>
+      <c r="A4" s="106"/>
       <c r="B4" s="47" t="s">
         <v>185</v>
       </c>
@@ -16147,7 +16195,7 @@
       </c>
     </row>
     <row r="5" spans="1:78" x14ac:dyDescent="0.45">
-      <c r="A5" s="125"/>
+      <c r="A5" s="106"/>
       <c r="B5" s="47" t="s">
         <v>186</v>
       </c>
@@ -16399,7 +16447,7 @@
       </c>
     </row>
     <row r="6" spans="1:78" x14ac:dyDescent="0.45">
-      <c r="A6" s="125"/>
+      <c r="A6" s="106"/>
       <c r="B6" s="47" t="s">
         <v>187</v>
       </c>
@@ -16651,7 +16699,7 @@
       </c>
     </row>
     <row r="7" spans="1:78" x14ac:dyDescent="0.45">
-      <c r="A7" s="125"/>
+      <c r="A7" s="106"/>
       <c r="B7" s="47" t="s">
         <v>188</v>
       </c>
@@ -16903,7 +16951,7 @@
       </c>
     </row>
     <row r="8" spans="1:78" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A8" s="125"/>
+      <c r="A8" s="106"/>
       <c r="B8" s="50" t="s">
         <v>4</v>
       </c>
@@ -17156,132 +17204,132 @@
     </row>
     <row r="9" spans="1:78" ht="14.65" thickTop="1" x14ac:dyDescent="0.45"/>
     <row r="10" spans="1:78" ht="18" x14ac:dyDescent="0.45">
-      <c r="A10" s="125">
+      <c r="A10" s="106">
         <v>2026</v>
       </c>
       <c r="B10" s="45" t="str">
         <f ca="1">CONCATENATE("in: ",YEAR(TODAY())," für: ", YEAR(TODAY())+1)</f>
         <v>in: 2026 für: 2027</v>
       </c>
-      <c r="C10" s="106" t="s">
+      <c r="C10" s="107" t="s">
         <v>220</v>
       </c>
-      <c r="D10" s="106"/>
-      <c r="E10" s="107"/>
-      <c r="F10" s="110" t="s">
+      <c r="D10" s="107"/>
+      <c r="E10" s="108"/>
+      <c r="F10" s="109" t="s">
         <v>221</v>
       </c>
-      <c r="G10" s="111"/>
-      <c r="H10" s="111"/>
-      <c r="I10" s="111"/>
-      <c r="J10" s="112"/>
-      <c r="K10" s="116" t="s">
+      <c r="G10" s="110"/>
+      <c r="H10" s="110"/>
+      <c r="I10" s="110"/>
+      <c r="J10" s="111"/>
+      <c r="K10" s="112" t="s">
         <v>225</v>
       </c>
-      <c r="L10" s="117"/>
-      <c r="M10" s="117"/>
-      <c r="N10" s="118"/>
-      <c r="O10" s="108" t="s">
+      <c r="L10" s="113"/>
+      <c r="M10" s="113"/>
+      <c r="N10" s="114"/>
+      <c r="O10" s="132" t="s">
         <v>222</v>
       </c>
-      <c r="P10" s="108"/>
-      <c r="Q10" s="109"/>
-      <c r="R10" s="122" t="s">
+      <c r="P10" s="132"/>
+      <c r="Q10" s="133"/>
+      <c r="R10" s="134" t="s">
         <v>223</v>
       </c>
-      <c r="S10" s="123"/>
-      <c r="T10" s="123"/>
-      <c r="U10" s="123"/>
-      <c r="V10" s="124"/>
-      <c r="W10" s="119" t="s">
+      <c r="S10" s="135"/>
+      <c r="T10" s="135"/>
+      <c r="U10" s="135"/>
+      <c r="V10" s="136"/>
+      <c r="W10" s="137" t="s">
         <v>226</v>
       </c>
-      <c r="X10" s="120"/>
-      <c r="Y10" s="120"/>
-      <c r="Z10" s="121"/>
+      <c r="X10" s="138"/>
+      <c r="Y10" s="138"/>
+      <c r="Z10" s="139"/>
       <c r="AB10" s="45" t="str">
         <f ca="1">CONCATENATE("in: ",YEAR(TODAY())," für: ", YEAR(TODAY())+1)</f>
         <v>in: 2026 für: 2027</v>
       </c>
-      <c r="AC10" s="126" t="s">
+      <c r="AC10" s="115" t="s">
         <v>227</v>
       </c>
-      <c r="AD10" s="126"/>
-      <c r="AE10" s="127"/>
-      <c r="AF10" s="128" t="s">
+      <c r="AD10" s="115"/>
+      <c r="AE10" s="116"/>
+      <c r="AF10" s="117" t="s">
         <v>228</v>
       </c>
-      <c r="AG10" s="129"/>
-      <c r="AH10" s="129"/>
-      <c r="AI10" s="129"/>
-      <c r="AJ10" s="130"/>
-      <c r="AK10" s="131" t="s">
+      <c r="AG10" s="118"/>
+      <c r="AH10" s="118"/>
+      <c r="AI10" s="118"/>
+      <c r="AJ10" s="119"/>
+      <c r="AK10" s="120" t="s">
         <v>229</v>
       </c>
-      <c r="AL10" s="132"/>
-      <c r="AM10" s="132"/>
-      <c r="AN10" s="133"/>
-      <c r="AO10" s="134" t="s">
+      <c r="AL10" s="121"/>
+      <c r="AM10" s="121"/>
+      <c r="AN10" s="122"/>
+      <c r="AO10" s="123" t="s">
         <v>230</v>
       </c>
-      <c r="AP10" s="135"/>
-      <c r="AQ10" s="136"/>
-      <c r="AR10" s="137" t="s">
+      <c r="AP10" s="124"/>
+      <c r="AQ10" s="125"/>
+      <c r="AR10" s="126" t="s">
         <v>231</v>
       </c>
-      <c r="AS10" s="138"/>
-      <c r="AT10" s="138"/>
-      <c r="AU10" s="138"/>
-      <c r="AV10" s="139"/>
-      <c r="AW10" s="113" t="s">
+      <c r="AS10" s="127"/>
+      <c r="AT10" s="127"/>
+      <c r="AU10" s="127"/>
+      <c r="AV10" s="128"/>
+      <c r="AW10" s="129" t="s">
         <v>232</v>
       </c>
-      <c r="AX10" s="114"/>
-      <c r="AY10" s="114"/>
-      <c r="AZ10" s="115"/>
+      <c r="AX10" s="130"/>
+      <c r="AY10" s="130"/>
+      <c r="AZ10" s="131"/>
       <c r="BB10" s="45" t="str">
         <f ca="1">CONCATENATE("in: ",YEAR(TODAY())," für: ", YEAR(TODAY())+1)</f>
         <v>in: 2026 für: 2027</v>
       </c>
-      <c r="BC10" s="106" t="s">
+      <c r="BC10" s="107" t="s">
         <v>233</v>
       </c>
-      <c r="BD10" s="106"/>
-      <c r="BE10" s="107"/>
-      <c r="BF10" s="110" t="s">
+      <c r="BD10" s="107"/>
+      <c r="BE10" s="108"/>
+      <c r="BF10" s="109" t="s">
         <v>234</v>
       </c>
-      <c r="BG10" s="111"/>
-      <c r="BH10" s="111"/>
-      <c r="BI10" s="111"/>
-      <c r="BJ10" s="112"/>
-      <c r="BK10" s="116" t="s">
+      <c r="BG10" s="110"/>
+      <c r="BH10" s="110"/>
+      <c r="BI10" s="110"/>
+      <c r="BJ10" s="111"/>
+      <c r="BK10" s="112" t="s">
         <v>235</v>
       </c>
-      <c r="BL10" s="117"/>
-      <c r="BM10" s="117"/>
-      <c r="BN10" s="118"/>
-      <c r="BO10" s="108" t="s">
+      <c r="BL10" s="113"/>
+      <c r="BM10" s="113"/>
+      <c r="BN10" s="114"/>
+      <c r="BO10" s="132" t="s">
         <v>241</v>
       </c>
-      <c r="BP10" s="108"/>
-      <c r="BQ10" s="109"/>
-      <c r="BR10" s="122" t="s">
+      <c r="BP10" s="132"/>
+      <c r="BQ10" s="133"/>
+      <c r="BR10" s="134" t="s">
         <v>242</v>
       </c>
-      <c r="BS10" s="123"/>
-      <c r="BT10" s="123"/>
-      <c r="BU10" s="123"/>
-      <c r="BV10" s="124"/>
-      <c r="BW10" s="119" t="s">
+      <c r="BS10" s="135"/>
+      <c r="BT10" s="135"/>
+      <c r="BU10" s="135"/>
+      <c r="BV10" s="136"/>
+      <c r="BW10" s="137" t="s">
         <v>236</v>
       </c>
-      <c r="BX10" s="120"/>
-      <c r="BY10" s="120"/>
-      <c r="BZ10" s="121"/>
+      <c r="BX10" s="138"/>
+      <c r="BY10" s="138"/>
+      <c r="BZ10" s="139"/>
     </row>
     <row r="11" spans="1:78" ht="21.4" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A11" s="125"/>
+      <c r="A11" s="106"/>
       <c r="B11" s="46" t="s">
         <v>224</v>
       </c>
@@ -17582,7 +17630,7 @@
       </c>
     </row>
     <row r="12" spans="1:78" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A12" s="125"/>
+      <c r="A12" s="106"/>
       <c r="B12" s="47" t="s">
         <v>0</v>
       </c>
@@ -17834,7 +17882,7 @@
       </c>
     </row>
     <row r="13" spans="1:78" x14ac:dyDescent="0.45">
-      <c r="A13" s="125"/>
+      <c r="A13" s="106"/>
       <c r="B13" s="47" t="s">
         <v>185</v>
       </c>
@@ -18086,7 +18134,7 @@
       </c>
     </row>
     <row r="14" spans="1:78" x14ac:dyDescent="0.45">
-      <c r="A14" s="125"/>
+      <c r="A14" s="106"/>
       <c r="B14" s="47" t="s">
         <v>186</v>
       </c>
@@ -18338,7 +18386,7 @@
       </c>
     </row>
     <row r="15" spans="1:78" x14ac:dyDescent="0.45">
-      <c r="A15" s="125"/>
+      <c r="A15" s="106"/>
       <c r="B15" s="47" t="s">
         <v>187</v>
       </c>
@@ -18590,7 +18638,7 @@
       </c>
     </row>
     <row r="16" spans="1:78" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A16" s="125"/>
+      <c r="A16" s="106"/>
       <c r="B16" s="47" t="s">
         <v>188</v>
       </c>
@@ -18842,7 +18890,7 @@
       </c>
     </row>
     <row r="17" spans="1:78" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A17" s="125"/>
+      <c r="A17" s="106"/>
       <c r="B17" s="50" t="s">
         <v>4</v>
       </c>
@@ -19309,6 +19357,28 @@
     </row>
   </sheetData>
   <mergeCells count="38">
+    <mergeCell ref="C10:E10"/>
+    <mergeCell ref="O10:Q10"/>
+    <mergeCell ref="C1:E1"/>
+    <mergeCell ref="O1:Q1"/>
+    <mergeCell ref="F10:J10"/>
+    <mergeCell ref="AW10:AZ10"/>
+    <mergeCell ref="K10:N10"/>
+    <mergeCell ref="W10:Z10"/>
+    <mergeCell ref="F1:J1"/>
+    <mergeCell ref="K1:N1"/>
+    <mergeCell ref="R1:V1"/>
+    <mergeCell ref="W1:Z1"/>
+    <mergeCell ref="R10:V10"/>
+    <mergeCell ref="BO10:BQ10"/>
+    <mergeCell ref="BR10:BV10"/>
+    <mergeCell ref="BW10:BZ10"/>
+    <mergeCell ref="BC1:BE1"/>
+    <mergeCell ref="BF1:BJ1"/>
+    <mergeCell ref="BK1:BN1"/>
+    <mergeCell ref="BO1:BQ1"/>
+    <mergeCell ref="BR1:BV1"/>
+    <mergeCell ref="BW1:BZ1"/>
     <mergeCell ref="A1:A8"/>
     <mergeCell ref="A10:A17"/>
     <mergeCell ref="BC10:BE10"/>
@@ -19325,36 +19395,14 @@
     <mergeCell ref="AK10:AN10"/>
     <mergeCell ref="AO10:AQ10"/>
     <mergeCell ref="AR10:AV10"/>
-    <mergeCell ref="BO10:BQ10"/>
-    <mergeCell ref="BR10:BV10"/>
-    <mergeCell ref="BW10:BZ10"/>
-    <mergeCell ref="BC1:BE1"/>
-    <mergeCell ref="BF1:BJ1"/>
-    <mergeCell ref="BK1:BN1"/>
-    <mergeCell ref="BO1:BQ1"/>
-    <mergeCell ref="BR1:BV1"/>
-    <mergeCell ref="BW1:BZ1"/>
-    <mergeCell ref="AW10:AZ10"/>
-    <mergeCell ref="K10:N10"/>
-    <mergeCell ref="W10:Z10"/>
-    <mergeCell ref="F1:J1"/>
-    <mergeCell ref="K1:N1"/>
-    <mergeCell ref="R1:V1"/>
-    <mergeCell ref="W1:Z1"/>
-    <mergeCell ref="R10:V10"/>
-    <mergeCell ref="C10:E10"/>
-    <mergeCell ref="O10:Q10"/>
-    <mergeCell ref="C1:E1"/>
-    <mergeCell ref="O1:Q1"/>
-    <mergeCell ref="F10:J10"/>
   </mergeCells>
   <conditionalFormatting sqref="AC3:AZ8">
-    <cfRule type="cellIs" dxfId="29" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AC12:AZ17">
-    <cfRule type="cellIs" dxfId="28" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Pz2 aus Quali Tabellen raus
</commit_message>
<xml_diff>
--- a/web/utilities/records_kriterien.xlsx
+++ b/web/utilities/records_kriterien.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jpgna\Documents\GitHub\Lifesaving_Baden\web\utilities\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3EF3FC4-98F1-4B17-964A-463DF977B517}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBE8BAB8-837C-4BDA-86D3-795FBF6081E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="687" firstSheet="1" activeTab="7" xr2:uid="{E1AB626B-3773-4829-92A5-28DD4DB7C8F8}"/>
   </bookViews>
@@ -185,7 +185,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="673" uniqueCount="248">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="667" uniqueCount="254">
   <si>
     <t>50m Retten</t>
   </si>
@@ -929,6 +929,24 @@
   </si>
   <si>
     <t>mind. erreichte Normen</t>
+  </si>
+  <si>
+    <t>PZ - 50m Retten</t>
+  </si>
+  <si>
+    <t>PZ - 100m Retten</t>
+  </si>
+  <si>
+    <t>PZ - 100m Kombi</t>
+  </si>
+  <si>
+    <t>PZ - 100m Lifesaver</t>
+  </si>
+  <si>
+    <t>PZ - 200m Super-Lifesaver</t>
+  </si>
+  <si>
+    <t>PZ - 200m Hindernis</t>
   </si>
 </sst>
 </file>
@@ -1614,13 +1632,16 @@
     <xf numFmtId="0" fontId="14" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1632,6 +1653,15 @@
     <xf numFmtId="0" fontId="14" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="10" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1640,6 +1670,27 @@
     </xf>
     <xf numFmtId="0" fontId="14" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1683,45 +1734,12 @@
     <xf numFmtId="0" fontId="17" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Prozent" xfId="1" builtinId="5"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="229">
+  <dxfs count="223">
     <dxf>
       <font>
         <color theme="4"/>
@@ -4143,30 +4161,6 @@
         </patternFill>
       </fill>
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="m:ss.00"/>
@@ -4558,34 +4552,28 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{FED162EE-531E-453F-8C25-562B59ECE709}" name="LK_konfig" displayName="LK_konfig" ref="A1:Y37" totalsRowShown="0" headerRowDxfId="228" dataDxfId="227">
-  <autoFilter ref="A1:Y37" xr:uid="{FED162EE-531E-453F-8C25-562B59ECE709}"/>
-  <tableColumns count="25">
-    <tableColumn id="1" xr3:uid="{F985A4F0-6B8C-47C6-816F-1A31A4973EB2}" name="Tabellen Name" dataDxfId="226"/>
-    <tableColumn id="2" xr3:uid="{5E5AD859-71A2-4E8E-B434-431A89C05C57}" name="Geschlecht" dataDxfId="225"/>
-    <tableColumn id="3" xr3:uid="{85BB892C-E151-404B-8974-FC5199E0909C}" name="Mindest Alter" dataDxfId="224"/>
-    <tableColumn id="4" xr3:uid="{790F6CF9-E475-4082-AE03-D30EDE22FB61}" name="Maximales Alter" dataDxfId="223"/>
-    <tableColumn id="5" xr3:uid="{FD4B0E6E-9B64-4731-A50F-D3CE3A4ED3FC}" name="Qualizeitraum anfang" dataDxfId="222"/>
-    <tableColumn id="6" xr3:uid="{5E84CAD2-C403-49B9-BB06-D56EC5784C8C}" name="Qualizeitraum Ende" dataDxfId="221"/>
-    <tableColumn id="7" xr3:uid="{6323F8E2-5DA4-4E5B-9C35-1E8C219ADECF}" name="Letzter Wettkampf am" dataDxfId="220"/>
-    <tableColumn id="8" xr3:uid="{D2845930-152E-432F-92A0-E7F7A3EE1FF0}" name="Landesverband" dataDxfId="219"/>
-    <tableColumn id="9" xr3:uid="{87046373-5CCD-41EC-B34C-C753E71FD26C}" name="OMS" dataDxfId="218"/>
-    <tableColumn id="10" xr3:uid="{A685FE01-F23C-4533-B399-857F5A1F6C37}" name="Pool-Länge" dataDxfId="217"/>
-    <tableColumn id="11" xr3:uid="{11E0A508-0C9D-4CB6-952E-7FAC5D05BDCD}" name="Regelwerk" dataDxfId="216"/>
-    <tableColumn id="12" xr3:uid="{F220BD5F-C3B5-4935-996A-BFCDF9F392D9}" name="Seiten Anzahl" dataDxfId="215"/>
-    <tableColumn id="25" xr3:uid="{7CDE58FE-A5B8-4329-9F48-3913AEBA21FC}" name="mind. erreichte Normen" dataDxfId="214"/>
-    <tableColumn id="13" xr3:uid="{A0A5E62D-9354-426D-9A08-13E43F36F55B}" name="PZ1 - 50m Retten" dataDxfId="213"/>
-    <tableColumn id="14" xr3:uid="{5D70F54C-57E9-45E2-BC99-0DBB0422383E}" name="PZ1 - 100m Retten" dataDxfId="212"/>
-    <tableColumn id="15" xr3:uid="{1C0CF5DB-156E-4813-A8BA-9EA29A40ABF3}" name="PZ1 - 100m Kombi" dataDxfId="211"/>
-    <tableColumn id="16" xr3:uid="{691CD4E1-13D9-4455-A2D1-14C9BC41A0EA}" name="PZ1 - 100m Lifesaver" dataDxfId="210"/>
-    <tableColumn id="17" xr3:uid="{CE1BA235-770B-4FA4-B327-187675DDA6B8}" name="PZ1 - 200m Super-Lifesaver" dataDxfId="209"/>
-    <tableColumn id="18" xr3:uid="{A326EF87-5FF5-4042-85D3-7806FEED4CFA}" name="PZ1 - 200m Hindernis" dataDxfId="208"/>
-    <tableColumn id="19" xr3:uid="{ABA5540C-4356-4D68-8579-E660F9FD6EA8}" name="PZ2 - 50m Retten" dataDxfId="207"/>
-    <tableColumn id="20" xr3:uid="{62E98437-16C9-4433-8683-E3C8A1B80E76}" name="PZ2 - 100m Retten" dataDxfId="206"/>
-    <tableColumn id="21" xr3:uid="{ED4E9448-4073-4B27-A491-5385DED08F83}" name="PZ2 - 100m Kombi" dataDxfId="205"/>
-    <tableColumn id="22" xr3:uid="{53F3DC0A-267B-434A-BD8A-320943916288}" name="PZ2 - 100m Lifesaver" dataDxfId="204"/>
-    <tableColumn id="23" xr3:uid="{1586F43C-8AD2-4942-A098-687AF0A028AC}" name="PZ2 - 200m Super-Lifesaver" dataDxfId="203"/>
-    <tableColumn id="24" xr3:uid="{98AA496B-EB58-437E-91F5-800894DDD85F}" name="PZ2 - 200m Hindernis" dataDxfId="202"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{FED162EE-531E-453F-8C25-562B59ECE709}" name="LK_konfig" displayName="LK_konfig" ref="A1:S37" totalsRowShown="0" headerRowDxfId="222" dataDxfId="221">
+  <autoFilter ref="A1:S37" xr:uid="{FED162EE-531E-453F-8C25-562B59ECE709}"/>
+  <tableColumns count="19">
+    <tableColumn id="1" xr3:uid="{F985A4F0-6B8C-47C6-816F-1A31A4973EB2}" name="Tabellen Name" dataDxfId="220"/>
+    <tableColumn id="2" xr3:uid="{5E5AD859-71A2-4E8E-B434-431A89C05C57}" name="Geschlecht" dataDxfId="219"/>
+    <tableColumn id="3" xr3:uid="{85BB892C-E151-404B-8974-FC5199E0909C}" name="Mindest Alter" dataDxfId="218"/>
+    <tableColumn id="4" xr3:uid="{790F6CF9-E475-4082-AE03-D30EDE22FB61}" name="Maximales Alter" dataDxfId="217"/>
+    <tableColumn id="5" xr3:uid="{FD4B0E6E-9B64-4731-A50F-D3CE3A4ED3FC}" name="Qualizeitraum anfang" dataDxfId="216"/>
+    <tableColumn id="6" xr3:uid="{5E84CAD2-C403-49B9-BB06-D56EC5784C8C}" name="Qualizeitraum Ende" dataDxfId="215"/>
+    <tableColumn id="7" xr3:uid="{6323F8E2-5DA4-4E5B-9C35-1E8C219ADECF}" name="Letzter Wettkampf am" dataDxfId="214"/>
+    <tableColumn id="8" xr3:uid="{D2845930-152E-432F-92A0-E7F7A3EE1FF0}" name="Landesverband" dataDxfId="213"/>
+    <tableColumn id="9" xr3:uid="{87046373-5CCD-41EC-B34C-C753E71FD26C}" name="OMS" dataDxfId="212"/>
+    <tableColumn id="10" xr3:uid="{A685FE01-F23C-4533-B399-857F5A1F6C37}" name="Pool-Länge" dataDxfId="211"/>
+    <tableColumn id="11" xr3:uid="{11E0A508-0C9D-4CB6-952E-7FAC5D05BDCD}" name="Regelwerk" dataDxfId="210"/>
+    <tableColumn id="12" xr3:uid="{F220BD5F-C3B5-4935-996A-BFCDF9F392D9}" name="Seiten Anzahl" dataDxfId="209"/>
+    <tableColumn id="25" xr3:uid="{7CDE58FE-A5B8-4329-9F48-3913AEBA21FC}" name="mind. erreichte Normen" dataDxfId="208"/>
+    <tableColumn id="13" xr3:uid="{A0A5E62D-9354-426D-9A08-13E43F36F55B}" name="PZ - 50m Retten" dataDxfId="207"/>
+    <tableColumn id="14" xr3:uid="{5D70F54C-57E9-45E2-BC99-0DBB0422383E}" name="PZ - 100m Retten" dataDxfId="206"/>
+    <tableColumn id="15" xr3:uid="{1C0CF5DB-156E-4813-A8BA-9EA29A40ABF3}" name="PZ - 100m Kombi" dataDxfId="205"/>
+    <tableColumn id="16" xr3:uid="{691CD4E1-13D9-4455-A2D1-14C9BC41A0EA}" name="PZ - 100m Lifesaver" dataDxfId="204"/>
+    <tableColumn id="17" xr3:uid="{CE1BA235-770B-4FA4-B327-187675DDA6B8}" name="PZ - 200m Super-Lifesaver" dataDxfId="203"/>
+    <tableColumn id="18" xr3:uid="{A326EF87-5FF5-4042-85D3-7806FEED4CFA}" name="PZ - 200m Hindernis" dataDxfId="202"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -12671,7 +12659,7 @@
   <sheetPr>
     <tabColor theme="5" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="A1:Y37"/>
+  <dimension ref="A1:S37"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="17.3984375" bestFit="1" customWidth="1"/>
@@ -12693,15 +12681,9 @@
     <col min="17" max="17" width="19.3984375" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="24.86328125" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="19.86328125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="16.3984375" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="17.3984375" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="17.1328125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="19.3984375" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="24.86328125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="19.86328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.45">
       <c r="A1" s="25" t="s">
         <v>127</v>
       </c>
@@ -12742,43 +12724,25 @@
         <v>247</v>
       </c>
       <c r="N1" s="25" t="s">
-        <v>166</v>
+        <v>248</v>
       </c>
       <c r="O1" s="25" t="s">
-        <v>167</v>
+        <v>249</v>
       </c>
       <c r="P1" s="25" t="s">
-        <v>168</v>
+        <v>250</v>
       </c>
       <c r="Q1" s="25" t="s">
-        <v>171</v>
+        <v>251</v>
       </c>
       <c r="R1" s="25" t="s">
-        <v>170</v>
+        <v>252</v>
       </c>
       <c r="S1" s="25" t="s">
-        <v>169</v>
-      </c>
-      <c r="T1" s="25" t="s">
-        <v>172</v>
-      </c>
-      <c r="U1" s="25" t="s">
-        <v>173</v>
-      </c>
-      <c r="V1" s="25" t="s">
-        <v>174</v>
-      </c>
-      <c r="W1" s="25" t="s">
-        <v>175</v>
-      </c>
-      <c r="X1" s="25" t="s">
-        <v>176</v>
-      </c>
-      <c r="Y1" s="25" t="s">
-        <v>177</v>
+        <v>253</v>
       </c>
     </row>
-    <row r="2" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.45">
       <c r="A2" s="25" t="s">
         <v>241</v>
       </c>
@@ -12838,14 +12802,8 @@
         <f>'NK-LK Transf.'!BQ16</f>
         <v>1.9327962962962964E-3</v>
       </c>
-      <c r="T2" s="28"/>
-      <c r="U2" s="28"/>
-      <c r="V2" s="28"/>
-      <c r="W2" s="28"/>
-      <c r="X2" s="28"/>
-      <c r="Y2" s="28"/>
     </row>
-    <row r="3" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.45">
       <c r="A3" s="25" t="s">
         <v>241</v>
       </c>
@@ -12905,14 +12863,8 @@
         <f>'NK-LK Transf.'!BP16</f>
         <v>1.9621597222222223E-3</v>
       </c>
-      <c r="T3" s="28"/>
-      <c r="U3" s="28"/>
-      <c r="V3" s="28"/>
-      <c r="W3" s="28"/>
-      <c r="X3" s="28"/>
-      <c r="Y3" s="28"/>
     </row>
-    <row r="4" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.45">
       <c r="A4" s="25" t="s">
         <v>241</v>
       </c>
@@ -12972,14 +12924,8 @@
         <f>'NK-LK Transf.'!BO16</f>
         <v>1.9916597222222219E-3</v>
       </c>
-      <c r="T4" s="28"/>
-      <c r="U4" s="28"/>
-      <c r="V4" s="28"/>
-      <c r="W4" s="28"/>
-      <c r="X4" s="28"/>
-      <c r="Y4" s="28"/>
     </row>
-    <row r="5" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.45">
       <c r="A5" s="25" t="s">
         <v>233</v>
       </c>
@@ -13039,14 +12985,8 @@
         <f>'NK-LK Transf.'!BE16</f>
         <v>1.8218055555555552E-3</v>
       </c>
-      <c r="T5" s="28"/>
-      <c r="U5" s="28"/>
-      <c r="V5" s="28"/>
-      <c r="W5" s="28"/>
-      <c r="X5" s="28"/>
-      <c r="Y5" s="28"/>
     </row>
-    <row r="6" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.45">
       <c r="A6" s="25" t="s">
         <v>233</v>
       </c>
@@ -13106,14 +13046,8 @@
         <f>'NK-LK Transf.'!BD16</f>
         <v>1.8773611111111109E-3</v>
       </c>
-      <c r="T6" s="28"/>
-      <c r="U6" s="28"/>
-      <c r="V6" s="28"/>
-      <c r="W6" s="28"/>
-      <c r="X6" s="28"/>
-      <c r="Y6" s="28"/>
     </row>
-    <row r="7" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.45">
       <c r="A7" s="25" t="s">
         <v>233</v>
       </c>
@@ -13173,14 +13107,8 @@
         <f>'NK-LK Transf.'!BC16</f>
         <v>1.9152777777777779E-3</v>
       </c>
-      <c r="T7" s="28"/>
-      <c r="U7" s="28"/>
-      <c r="V7" s="28"/>
-      <c r="W7" s="28"/>
-      <c r="X7" s="28"/>
-      <c r="Y7" s="28"/>
     </row>
-    <row r="8" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:19" x14ac:dyDescent="0.45">
       <c r="A8" s="25" t="s">
         <v>240</v>
       </c>
@@ -13240,14 +13168,8 @@
         <f>'NK-LK Transf.'!BV16</f>
         <v>1.8239270833333334E-3</v>
       </c>
-      <c r="T8" s="28"/>
-      <c r="U8" s="28"/>
-      <c r="V8" s="28"/>
-      <c r="W8" s="28"/>
-      <c r="X8" s="28"/>
-      <c r="Y8" s="28"/>
     </row>
-    <row r="9" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:19" x14ac:dyDescent="0.45">
       <c r="A9" s="25" t="s">
         <v>240</v>
       </c>
@@ -13307,14 +13229,8 @@
         <f>'NK-LK Transf.'!BU16</f>
         <v>1.8506041666666666E-3</v>
       </c>
-      <c r="T9" s="28"/>
-      <c r="U9" s="28"/>
-      <c r="V9" s="28"/>
-      <c r="W9" s="28"/>
-      <c r="X9" s="28"/>
-      <c r="Y9" s="28"/>
     </row>
-    <row r="10" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:19" x14ac:dyDescent="0.45">
       <c r="A10" s="25" t="s">
         <v>240</v>
       </c>
@@ -13374,14 +13290,8 @@
         <f>'NK-LK Transf.'!BT16</f>
         <v>1.887166666666667E-3</v>
       </c>
-      <c r="T10" s="28"/>
-      <c r="U10" s="28"/>
-      <c r="V10" s="28"/>
-      <c r="W10" s="28"/>
-      <c r="X10" s="28"/>
-      <c r="Y10" s="28"/>
     </row>
-    <row r="11" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:19" x14ac:dyDescent="0.45">
       <c r="A11" s="25" t="s">
         <v>239</v>
       </c>
@@ -13441,14 +13351,8 @@
         <f>'NK-LK Transf.'!BJ16</f>
         <v>1.6026527777777777E-3</v>
       </c>
-      <c r="T11" s="28"/>
-      <c r="U11" s="28"/>
-      <c r="V11" s="28"/>
-      <c r="W11" s="28"/>
-      <c r="X11" s="28"/>
-      <c r="Y11" s="28"/>
     </row>
-    <row r="12" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:19" x14ac:dyDescent="0.45">
       <c r="A12" s="25" t="s">
         <v>239</v>
       </c>
@@ -13508,14 +13412,8 @@
         <f>'NK-LK Transf.'!BI16</f>
         <v>1.6571620370370373E-3</v>
       </c>
-      <c r="T12" s="28"/>
-      <c r="U12" s="28"/>
-      <c r="V12" s="28"/>
-      <c r="W12" s="28"/>
-      <c r="X12" s="28"/>
-      <c r="Y12" s="28"/>
     </row>
-    <row r="13" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:19" x14ac:dyDescent="0.45">
       <c r="A13" s="25" t="s">
         <v>239</v>
       </c>
@@ -13575,14 +13473,8 @@
         <f>'NK-LK Transf.'!BH16</f>
         <v>1.7049583333333333E-3</v>
       </c>
-      <c r="T13" s="28"/>
-      <c r="U13" s="28"/>
-      <c r="V13" s="28"/>
-      <c r="W13" s="28"/>
-      <c r="X13" s="28"/>
-      <c r="Y13" s="28"/>
     </row>
-    <row r="14" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:19" x14ac:dyDescent="0.45">
       <c r="A14" s="25" t="s">
         <v>222</v>
       </c>
@@ -13644,14 +13536,8 @@
         <f>'NK-LK Transf.'!Q16</f>
         <v>1.637962962962963E-3</v>
       </c>
-      <c r="T14" s="28"/>
-      <c r="U14" s="28"/>
-      <c r="V14" s="28"/>
-      <c r="W14" s="28"/>
-      <c r="X14" s="28"/>
-      <c r="Y14" s="28"/>
     </row>
-    <row r="15" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:19" x14ac:dyDescent="0.45">
       <c r="A15" s="25" t="s">
         <v>222</v>
       </c>
@@ -13713,14 +13599,8 @@
         <f>'NK-LK Transf.'!P16</f>
         <v>1.6628472222222225E-3</v>
       </c>
-      <c r="T15" s="28"/>
-      <c r="U15" s="28"/>
-      <c r="V15" s="28"/>
-      <c r="W15" s="28"/>
-      <c r="X15" s="28"/>
-      <c r="Y15" s="28"/>
     </row>
-    <row r="16" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:19" x14ac:dyDescent="0.45">
       <c r="A16" s="25" t="s">
         <v>222</v>
       </c>
@@ -13782,14 +13662,8 @@
         <f>'NK-LK Transf.'!O16</f>
         <v>1.6878472222222221E-3</v>
       </c>
-      <c r="T16" s="28"/>
-      <c r="U16" s="28"/>
-      <c r="V16" s="28"/>
-      <c r="W16" s="28"/>
-      <c r="X16" s="28"/>
-      <c r="Y16" s="28"/>
     </row>
-    <row r="17" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:19" x14ac:dyDescent="0.45">
       <c r="A17" s="25" t="s">
         <v>220</v>
       </c>
@@ -13851,14 +13725,8 @@
         <f>'NK-LK Transf.'!E16</f>
         <v>1.5181712962962961E-3</v>
       </c>
-      <c r="T17" s="28"/>
-      <c r="U17" s="28"/>
-      <c r="V17" s="28"/>
-      <c r="W17" s="28"/>
-      <c r="X17" s="28"/>
-      <c r="Y17" s="28"/>
     </row>
-    <row r="18" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:19" x14ac:dyDescent="0.45">
       <c r="A18" s="25" t="s">
         <v>220</v>
       </c>
@@ -13920,14 +13788,8 @@
         <f>'NK-LK Transf.'!D16</f>
         <v>1.5644675925925923E-3</v>
       </c>
-      <c r="T18" s="28"/>
-      <c r="U18" s="28"/>
-      <c r="V18" s="28"/>
-      <c r="W18" s="28"/>
-      <c r="X18" s="28"/>
-      <c r="Y18" s="28"/>
     </row>
-    <row r="19" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:19" x14ac:dyDescent="0.45">
       <c r="A19" s="25" t="s">
         <v>220</v>
       </c>
@@ -13989,14 +13851,8 @@
         <f>'NK-LK Transf.'!C16</f>
         <v>1.5960648148148149E-3</v>
       </c>
-      <c r="T19" s="28"/>
-      <c r="U19" s="28"/>
-      <c r="V19" s="28"/>
-      <c r="W19" s="28"/>
-      <c r="X19" s="28"/>
-      <c r="Y19" s="28"/>
     </row>
-    <row r="20" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:19" x14ac:dyDescent="0.45">
       <c r="A20" s="25" t="s">
         <v>243</v>
       </c>
@@ -14058,14 +13914,8 @@
         <f>'NK-LK Transf.'!V16</f>
         <v>1.558912037037037E-3</v>
       </c>
-      <c r="T20" s="28"/>
-      <c r="U20" s="28"/>
-      <c r="V20" s="28"/>
-      <c r="W20" s="28"/>
-      <c r="X20" s="28"/>
-      <c r="Y20" s="28"/>
     </row>
-    <row r="21" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:19" x14ac:dyDescent="0.45">
       <c r="A21" s="25" t="s">
         <v>243</v>
       </c>
@@ -14127,14 +13977,8 @@
         <f>'NK-LK Transf.'!U16</f>
         <v>1.5817129629629629E-3</v>
       </c>
-      <c r="T21" s="28"/>
-      <c r="U21" s="28"/>
-      <c r="V21" s="28"/>
-      <c r="W21" s="28"/>
-      <c r="X21" s="28"/>
-      <c r="Y21" s="28"/>
     </row>
-    <row r="22" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:19" x14ac:dyDescent="0.45">
       <c r="A22" s="25" t="s">
         <v>243</v>
       </c>
@@ -14196,14 +14040,8 @@
         <f>'NK-LK Transf.'!T16</f>
         <v>1.6129629629629632E-3</v>
       </c>
-      <c r="T22" s="28"/>
-      <c r="U22" s="28"/>
-      <c r="V22" s="28"/>
-      <c r="W22" s="28"/>
-      <c r="X22" s="28"/>
-      <c r="Y22" s="28"/>
     </row>
-    <row r="23" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:19" x14ac:dyDescent="0.45">
       <c r="A23" s="25" t="s">
         <v>243</v>
       </c>
@@ -14265,14 +14103,8 @@
         <f>'NK-LK Transf.'!S16</f>
         <v>1.6278935185185185E-3</v>
       </c>
-      <c r="T23" s="28"/>
-      <c r="U23" s="28"/>
-      <c r="V23" s="28"/>
-      <c r="W23" s="28"/>
-      <c r="X23" s="28"/>
-      <c r="Y23" s="28"/>
     </row>
-    <row r="24" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:19" x14ac:dyDescent="0.45">
       <c r="A24" s="25" t="s">
         <v>243</v>
       </c>
@@ -14334,14 +14166,8 @@
         <f>'NK-LK Transf.'!R16</f>
         <v>1.644212962962963E-3</v>
       </c>
-      <c r="T24" s="28"/>
-      <c r="U24" s="28"/>
-      <c r="V24" s="28"/>
-      <c r="W24" s="28"/>
-      <c r="X24" s="28"/>
-      <c r="Y24" s="28"/>
     </row>
-    <row r="25" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:19" x14ac:dyDescent="0.45">
       <c r="A25" s="25" t="s">
         <v>244</v>
       </c>
@@ -14403,14 +14229,8 @@
         <f>'NK-LK Transf.'!J16</f>
         <v>1.3815972222222222E-3</v>
       </c>
-      <c r="T25" s="28"/>
-      <c r="U25" s="28"/>
-      <c r="V25" s="28"/>
-      <c r="W25" s="28"/>
-      <c r="X25" s="28"/>
-      <c r="Y25" s="28"/>
     </row>
-    <row r="26" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:19" x14ac:dyDescent="0.45">
       <c r="A26" s="25" t="s">
         <v>244</v>
       </c>
@@ -14472,14 +14292,8 @@
         <f>'NK-LK Transf.'!I16</f>
         <v>1.4285879629629631E-3</v>
       </c>
-      <c r="T26" s="28"/>
-      <c r="U26" s="28"/>
-      <c r="V26" s="28"/>
-      <c r="W26" s="28"/>
-      <c r="X26" s="28"/>
-      <c r="Y26" s="28"/>
     </row>
-    <row r="27" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:19" x14ac:dyDescent="0.45">
       <c r="A27" s="25" t="s">
         <v>244</v>
       </c>
@@ -14541,14 +14355,8 @@
         <f>'NK-LK Transf.'!H16</f>
         <v>1.4697916666666666E-3</v>
       </c>
-      <c r="T27" s="28"/>
-      <c r="U27" s="28"/>
-      <c r="V27" s="28"/>
-      <c r="W27" s="28"/>
-      <c r="X27" s="28"/>
-      <c r="Y27" s="28"/>
     </row>
-    <row r="28" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:19" x14ac:dyDescent="0.45">
       <c r="A28" s="25" t="s">
         <v>244</v>
       </c>
@@ -14610,14 +14418,8 @@
         <f>'NK-LK Transf.'!G16</f>
         <v>1.4950231481481481E-3</v>
       </c>
-      <c r="T28" s="28"/>
-      <c r="U28" s="28"/>
-      <c r="V28" s="28"/>
-      <c r="W28" s="28"/>
-      <c r="X28" s="28"/>
-      <c r="Y28" s="28"/>
     </row>
-    <row r="29" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:19" x14ac:dyDescent="0.45">
       <c r="A29" s="25" t="s">
         <v>244</v>
       </c>
@@ -14679,14 +14481,8 @@
         <f>'NK-LK Transf.'!F16</f>
         <v>1.522337962962963E-3</v>
       </c>
-      <c r="T29" s="28"/>
-      <c r="U29" s="28"/>
-      <c r="V29" s="28"/>
-      <c r="W29" s="28"/>
-      <c r="X29" s="28"/>
-      <c r="Y29" s="28"/>
     </row>
-    <row r="30" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:19" x14ac:dyDescent="0.45">
       <c r="A30" s="25" t="s">
         <v>245</v>
       </c>
@@ -14748,14 +14544,8 @@
         <f>'NK-LK Transf.'!Z16</f>
         <v>1.5517361111111109E-3</v>
       </c>
-      <c r="T30" s="28"/>
-      <c r="U30" s="28"/>
-      <c r="V30" s="28"/>
-      <c r="W30" s="28"/>
-      <c r="X30" s="28"/>
-      <c r="Y30" s="28"/>
     </row>
-    <row r="31" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:19" x14ac:dyDescent="0.45">
       <c r="A31" s="25" t="s">
         <v>245</v>
       </c>
@@ -14817,14 +14607,8 @@
         <f>'NK-LK Transf.'!Y16</f>
         <v>1.5564814814814814E-3</v>
       </c>
-      <c r="T31" s="28"/>
-      <c r="U31" s="28"/>
-      <c r="V31" s="28"/>
-      <c r="W31" s="28"/>
-      <c r="X31" s="28"/>
-      <c r="Y31" s="28"/>
     </row>
-    <row r="32" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:19" x14ac:dyDescent="0.45">
       <c r="A32" s="25" t="s">
         <v>245</v>
       </c>
@@ -14886,14 +14670,8 @@
         <f>'NK-LK Transf.'!X16</f>
         <v>1.570949074074074E-3</v>
       </c>
-      <c r="T32" s="28"/>
-      <c r="U32" s="28"/>
-      <c r="V32" s="28"/>
-      <c r="W32" s="28"/>
-      <c r="X32" s="28"/>
-      <c r="Y32" s="28"/>
     </row>
-    <row r="33" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:19" x14ac:dyDescent="0.45">
       <c r="A33" s="25" t="s">
         <v>245</v>
       </c>
@@ -14955,14 +14733,8 @@
         <f>'NK-LK Transf.'!W16</f>
         <v>1.5829861111111112E-3</v>
       </c>
-      <c r="T33" s="28"/>
-      <c r="U33" s="28"/>
-      <c r="V33" s="28"/>
-      <c r="W33" s="28"/>
-      <c r="X33" s="28"/>
-      <c r="Y33" s="28"/>
     </row>
-    <row r="34" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:19" x14ac:dyDescent="0.45">
       <c r="A34" s="25" t="s">
         <v>246</v>
       </c>
@@ -15024,14 +14796,8 @@
         <f>'NK-LK Transf.'!N16</f>
         <v>1.3697916666666665E-3</v>
       </c>
-      <c r="T34" s="28"/>
-      <c r="U34" s="28"/>
-      <c r="V34" s="28"/>
-      <c r="W34" s="28"/>
-      <c r="X34" s="28"/>
-      <c r="Y34" s="28"/>
     </row>
-    <row r="35" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:19" x14ac:dyDescent="0.45">
       <c r="A35" s="25" t="s">
         <v>246</v>
       </c>
@@ -15093,14 +14859,8 @@
         <f>'NK-LK Transf.'!M16</f>
         <v>1.377662037037037E-3</v>
       </c>
-      <c r="T35" s="28"/>
-      <c r="U35" s="28"/>
-      <c r="V35" s="28"/>
-      <c r="W35" s="28"/>
-      <c r="X35" s="28"/>
-      <c r="Y35" s="28"/>
     </row>
-    <row r="36" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:19" x14ac:dyDescent="0.45">
       <c r="A36" s="25" t="s">
         <v>246</v>
       </c>
@@ -15162,14 +14922,8 @@
         <f>'NK-LK Transf.'!L16</f>
         <v>1.4011574074074074E-3</v>
       </c>
-      <c r="T36" s="28"/>
-      <c r="U36" s="28"/>
-      <c r="V36" s="28"/>
-      <c r="W36" s="28"/>
-      <c r="X36" s="28"/>
-      <c r="Y36" s="28"/>
     </row>
-    <row r="37" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:19" x14ac:dyDescent="0.45">
       <c r="A37" s="25" t="s">
         <v>246</v>
       </c>
@@ -15231,12 +14985,6 @@
         <f>'NK-LK Transf.'!K16</f>
         <v>1.4207175925925926E-3</v>
       </c>
-      <c r="T37" s="28"/>
-      <c r="U37" s="28"/>
-      <c r="V37" s="28"/>
-      <c r="W37" s="28"/>
-      <c r="X37" s="28"/>
-      <c r="Y37" s="28"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
@@ -15263,133 +15011,133 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:78" s="40" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="106">
+      <c r="A1" s="125">
         <v>2025</v>
       </c>
       <c r="B1" s="45" t="str">
         <f ca="1">CONCATENATE("in: ",YEAR(TODAY())-1," für: ", YEAR(TODAY()))</f>
         <v>in: 2025 für: 2026</v>
       </c>
-      <c r="C1" s="107" t="s">
+      <c r="C1" s="106" t="s">
         <v>220</v>
       </c>
-      <c r="D1" s="107"/>
-      <c r="E1" s="108"/>
-      <c r="F1" s="109" t="s">
+      <c r="D1" s="106"/>
+      <c r="E1" s="107"/>
+      <c r="F1" s="110" t="s">
         <v>221</v>
       </c>
-      <c r="G1" s="110"/>
-      <c r="H1" s="110"/>
-      <c r="I1" s="110"/>
-      <c r="J1" s="111"/>
-      <c r="K1" s="112" t="s">
+      <c r="G1" s="111"/>
+      <c r="H1" s="111"/>
+      <c r="I1" s="111"/>
+      <c r="J1" s="112"/>
+      <c r="K1" s="116" t="s">
         <v>225</v>
       </c>
-      <c r="L1" s="113"/>
-      <c r="M1" s="113"/>
-      <c r="N1" s="114"/>
-      <c r="O1" s="132" t="s">
+      <c r="L1" s="117"/>
+      <c r="M1" s="117"/>
+      <c r="N1" s="118"/>
+      <c r="O1" s="108" t="s">
         <v>222</v>
       </c>
-      <c r="P1" s="132"/>
-      <c r="Q1" s="133"/>
-      <c r="R1" s="134" t="s">
+      <c r="P1" s="108"/>
+      <c r="Q1" s="109"/>
+      <c r="R1" s="122" t="s">
         <v>223</v>
       </c>
-      <c r="S1" s="135"/>
-      <c r="T1" s="135"/>
-      <c r="U1" s="135"/>
-      <c r="V1" s="136"/>
-      <c r="W1" s="137" t="s">
+      <c r="S1" s="123"/>
+      <c r="T1" s="123"/>
+      <c r="U1" s="123"/>
+      <c r="V1" s="124"/>
+      <c r="W1" s="119" t="s">
         <v>226</v>
       </c>
-      <c r="X1" s="138"/>
-      <c r="Y1" s="138"/>
-      <c r="Z1" s="139"/>
+      <c r="X1" s="120"/>
+      <c r="Y1" s="120"/>
+      <c r="Z1" s="121"/>
       <c r="AA1"/>
       <c r="AB1" s="45" t="str">
         <f ca="1">CONCATENATE("in: ",YEAR(TODAY())-1," für: ", YEAR(TODAY()))</f>
         <v>in: 2025 für: 2026</v>
       </c>
-      <c r="AC1" s="115" t="s">
+      <c r="AC1" s="126" t="s">
         <v>227</v>
       </c>
-      <c r="AD1" s="115"/>
-      <c r="AE1" s="116"/>
-      <c r="AF1" s="117" t="s">
+      <c r="AD1" s="126"/>
+      <c r="AE1" s="127"/>
+      <c r="AF1" s="128" t="s">
         <v>228</v>
       </c>
-      <c r="AG1" s="118"/>
-      <c r="AH1" s="118"/>
-      <c r="AI1" s="118"/>
-      <c r="AJ1" s="119"/>
-      <c r="AK1" s="120" t="s">
+      <c r="AG1" s="129"/>
+      <c r="AH1" s="129"/>
+      <c r="AI1" s="129"/>
+      <c r="AJ1" s="130"/>
+      <c r="AK1" s="131" t="s">
         <v>229</v>
       </c>
-      <c r="AL1" s="121"/>
-      <c r="AM1" s="121"/>
-      <c r="AN1" s="122"/>
-      <c r="AO1" s="123" t="s">
+      <c r="AL1" s="132"/>
+      <c r="AM1" s="132"/>
+      <c r="AN1" s="133"/>
+      <c r="AO1" s="134" t="s">
         <v>230</v>
       </c>
-      <c r="AP1" s="124"/>
-      <c r="AQ1" s="125"/>
-      <c r="AR1" s="126" t="s">
+      <c r="AP1" s="135"/>
+      <c r="AQ1" s="136"/>
+      <c r="AR1" s="137" t="s">
         <v>231</v>
       </c>
-      <c r="AS1" s="127"/>
-      <c r="AT1" s="127"/>
-      <c r="AU1" s="127"/>
-      <c r="AV1" s="128"/>
-      <c r="AW1" s="129" t="s">
+      <c r="AS1" s="138"/>
+      <c r="AT1" s="138"/>
+      <c r="AU1" s="138"/>
+      <c r="AV1" s="139"/>
+      <c r="AW1" s="113" t="s">
         <v>232</v>
       </c>
-      <c r="AX1" s="130"/>
-      <c r="AY1" s="130"/>
-      <c r="AZ1" s="131"/>
+      <c r="AX1" s="114"/>
+      <c r="AY1" s="114"/>
+      <c r="AZ1" s="115"/>
       <c r="BB1" s="45" t="str">
         <f ca="1">CONCATENATE("in: ",YEAR(TODAY())-1," für: ", YEAR(TODAY()))</f>
         <v>in: 2025 für: 2026</v>
       </c>
-      <c r="BC1" s="107" t="s">
+      <c r="BC1" s="106" t="s">
         <v>233</v>
       </c>
-      <c r="BD1" s="107"/>
-      <c r="BE1" s="108"/>
-      <c r="BF1" s="109" t="s">
+      <c r="BD1" s="106"/>
+      <c r="BE1" s="107"/>
+      <c r="BF1" s="110" t="s">
         <v>234</v>
       </c>
-      <c r="BG1" s="110"/>
-      <c r="BH1" s="110"/>
-      <c r="BI1" s="110"/>
-      <c r="BJ1" s="111"/>
-      <c r="BK1" s="112" t="s">
+      <c r="BG1" s="111"/>
+      <c r="BH1" s="111"/>
+      <c r="BI1" s="111"/>
+      <c r="BJ1" s="112"/>
+      <c r="BK1" s="116" t="s">
         <v>235</v>
       </c>
-      <c r="BL1" s="113"/>
-      <c r="BM1" s="113"/>
-      <c r="BN1" s="114"/>
-      <c r="BO1" s="132" t="s">
+      <c r="BL1" s="117"/>
+      <c r="BM1" s="117"/>
+      <c r="BN1" s="118"/>
+      <c r="BO1" s="108" t="s">
         <v>241</v>
       </c>
-      <c r="BP1" s="132"/>
-      <c r="BQ1" s="133"/>
-      <c r="BR1" s="134" t="s">
+      <c r="BP1" s="108"/>
+      <c r="BQ1" s="109"/>
+      <c r="BR1" s="122" t="s">
         <v>242</v>
       </c>
-      <c r="BS1" s="135"/>
-      <c r="BT1" s="135"/>
-      <c r="BU1" s="135"/>
-      <c r="BV1" s="136"/>
-      <c r="BW1" s="137" t="s">
+      <c r="BS1" s="123"/>
+      <c r="BT1" s="123"/>
+      <c r="BU1" s="123"/>
+      <c r="BV1" s="124"/>
+      <c r="BW1" s="119" t="s">
         <v>236</v>
       </c>
-      <c r="BX1" s="138"/>
-      <c r="BY1" s="138"/>
-      <c r="BZ1" s="139"/>
+      <c r="BX1" s="120"/>
+      <c r="BY1" s="120"/>
+      <c r="BZ1" s="121"/>
     </row>
     <row r="2" spans="1:78" s="94" customFormat="1" ht="21.4" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="106"/>
+      <c r="A2" s="125"/>
       <c r="B2" s="46" t="s">
         <v>224</v>
       </c>
@@ -15690,7 +15438,7 @@
       </c>
     </row>
     <row r="3" spans="1:78" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A3" s="106"/>
+      <c r="A3" s="125"/>
       <c r="B3" s="47" t="s">
         <v>0</v>
       </c>
@@ -15943,7 +15691,7 @@
       </c>
     </row>
     <row r="4" spans="1:78" x14ac:dyDescent="0.45">
-      <c r="A4" s="106"/>
+      <c r="A4" s="125"/>
       <c r="B4" s="47" t="s">
         <v>185</v>
       </c>
@@ -16195,7 +15943,7 @@
       </c>
     </row>
     <row r="5" spans="1:78" x14ac:dyDescent="0.45">
-      <c r="A5" s="106"/>
+      <c r="A5" s="125"/>
       <c r="B5" s="47" t="s">
         <v>186</v>
       </c>
@@ -16447,7 +16195,7 @@
       </c>
     </row>
     <row r="6" spans="1:78" x14ac:dyDescent="0.45">
-      <c r="A6" s="106"/>
+      <c r="A6" s="125"/>
       <c r="B6" s="47" t="s">
         <v>187</v>
       </c>
@@ -16699,7 +16447,7 @@
       </c>
     </row>
     <row r="7" spans="1:78" x14ac:dyDescent="0.45">
-      <c r="A7" s="106"/>
+      <c r="A7" s="125"/>
       <c r="B7" s="47" t="s">
         <v>188</v>
       </c>
@@ -16951,7 +16699,7 @@
       </c>
     </row>
     <row r="8" spans="1:78" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A8" s="106"/>
+      <c r="A8" s="125"/>
       <c r="B8" s="50" t="s">
         <v>4</v>
       </c>
@@ -17204,132 +16952,132 @@
     </row>
     <row r="9" spans="1:78" ht="14.65" thickTop="1" x14ac:dyDescent="0.45"/>
     <row r="10" spans="1:78" ht="18" x14ac:dyDescent="0.45">
-      <c r="A10" s="106">
+      <c r="A10" s="125">
         <v>2026</v>
       </c>
       <c r="B10" s="45" t="str">
         <f ca="1">CONCATENATE("in: ",YEAR(TODAY())," für: ", YEAR(TODAY())+1)</f>
         <v>in: 2026 für: 2027</v>
       </c>
-      <c r="C10" s="107" t="s">
+      <c r="C10" s="106" t="s">
         <v>220</v>
       </c>
-      <c r="D10" s="107"/>
-      <c r="E10" s="108"/>
-      <c r="F10" s="109" t="s">
+      <c r="D10" s="106"/>
+      <c r="E10" s="107"/>
+      <c r="F10" s="110" t="s">
         <v>221</v>
       </c>
-      <c r="G10" s="110"/>
-      <c r="H10" s="110"/>
-      <c r="I10" s="110"/>
-      <c r="J10" s="111"/>
-      <c r="K10" s="112" t="s">
+      <c r="G10" s="111"/>
+      <c r="H10" s="111"/>
+      <c r="I10" s="111"/>
+      <c r="J10" s="112"/>
+      <c r="K10" s="116" t="s">
         <v>225</v>
       </c>
-      <c r="L10" s="113"/>
-      <c r="M10" s="113"/>
-      <c r="N10" s="114"/>
-      <c r="O10" s="132" t="s">
+      <c r="L10" s="117"/>
+      <c r="M10" s="117"/>
+      <c r="N10" s="118"/>
+      <c r="O10" s="108" t="s">
         <v>222</v>
       </c>
-      <c r="P10" s="132"/>
-      <c r="Q10" s="133"/>
-      <c r="R10" s="134" t="s">
+      <c r="P10" s="108"/>
+      <c r="Q10" s="109"/>
+      <c r="R10" s="122" t="s">
         <v>223</v>
       </c>
-      <c r="S10" s="135"/>
-      <c r="T10" s="135"/>
-      <c r="U10" s="135"/>
-      <c r="V10" s="136"/>
-      <c r="W10" s="137" t="s">
+      <c r="S10" s="123"/>
+      <c r="T10" s="123"/>
+      <c r="U10" s="123"/>
+      <c r="V10" s="124"/>
+      <c r="W10" s="119" t="s">
         <v>226</v>
       </c>
-      <c r="X10" s="138"/>
-      <c r="Y10" s="138"/>
-      <c r="Z10" s="139"/>
+      <c r="X10" s="120"/>
+      <c r="Y10" s="120"/>
+      <c r="Z10" s="121"/>
       <c r="AB10" s="45" t="str">
         <f ca="1">CONCATENATE("in: ",YEAR(TODAY())," für: ", YEAR(TODAY())+1)</f>
         <v>in: 2026 für: 2027</v>
       </c>
-      <c r="AC10" s="115" t="s">
+      <c r="AC10" s="126" t="s">
         <v>227</v>
       </c>
-      <c r="AD10" s="115"/>
-      <c r="AE10" s="116"/>
-      <c r="AF10" s="117" t="s">
+      <c r="AD10" s="126"/>
+      <c r="AE10" s="127"/>
+      <c r="AF10" s="128" t="s">
         <v>228</v>
       </c>
-      <c r="AG10" s="118"/>
-      <c r="AH10" s="118"/>
-      <c r="AI10" s="118"/>
-      <c r="AJ10" s="119"/>
-      <c r="AK10" s="120" t="s">
+      <c r="AG10" s="129"/>
+      <c r="AH10" s="129"/>
+      <c r="AI10" s="129"/>
+      <c r="AJ10" s="130"/>
+      <c r="AK10" s="131" t="s">
         <v>229</v>
       </c>
-      <c r="AL10" s="121"/>
-      <c r="AM10" s="121"/>
-      <c r="AN10" s="122"/>
-      <c r="AO10" s="123" t="s">
+      <c r="AL10" s="132"/>
+      <c r="AM10" s="132"/>
+      <c r="AN10" s="133"/>
+      <c r="AO10" s="134" t="s">
         <v>230</v>
       </c>
-      <c r="AP10" s="124"/>
-      <c r="AQ10" s="125"/>
-      <c r="AR10" s="126" t="s">
+      <c r="AP10" s="135"/>
+      <c r="AQ10" s="136"/>
+      <c r="AR10" s="137" t="s">
         <v>231</v>
       </c>
-      <c r="AS10" s="127"/>
-      <c r="AT10" s="127"/>
-      <c r="AU10" s="127"/>
-      <c r="AV10" s="128"/>
-      <c r="AW10" s="129" t="s">
+      <c r="AS10" s="138"/>
+      <c r="AT10" s="138"/>
+      <c r="AU10" s="138"/>
+      <c r="AV10" s="139"/>
+      <c r="AW10" s="113" t="s">
         <v>232</v>
       </c>
-      <c r="AX10" s="130"/>
-      <c r="AY10" s="130"/>
-      <c r="AZ10" s="131"/>
+      <c r="AX10" s="114"/>
+      <c r="AY10" s="114"/>
+      <c r="AZ10" s="115"/>
       <c r="BB10" s="45" t="str">
         <f ca="1">CONCATENATE("in: ",YEAR(TODAY())," für: ", YEAR(TODAY())+1)</f>
         <v>in: 2026 für: 2027</v>
       </c>
-      <c r="BC10" s="107" t="s">
+      <c r="BC10" s="106" t="s">
         <v>233</v>
       </c>
-      <c r="BD10" s="107"/>
-      <c r="BE10" s="108"/>
-      <c r="BF10" s="109" t="s">
+      <c r="BD10" s="106"/>
+      <c r="BE10" s="107"/>
+      <c r="BF10" s="110" t="s">
         <v>234</v>
       </c>
-      <c r="BG10" s="110"/>
-      <c r="BH10" s="110"/>
-      <c r="BI10" s="110"/>
-      <c r="BJ10" s="111"/>
-      <c r="BK10" s="112" t="s">
+      <c r="BG10" s="111"/>
+      <c r="BH10" s="111"/>
+      <c r="BI10" s="111"/>
+      <c r="BJ10" s="112"/>
+      <c r="BK10" s="116" t="s">
         <v>235</v>
       </c>
-      <c r="BL10" s="113"/>
-      <c r="BM10" s="113"/>
-      <c r="BN10" s="114"/>
-      <c r="BO10" s="132" t="s">
+      <c r="BL10" s="117"/>
+      <c r="BM10" s="117"/>
+      <c r="BN10" s="118"/>
+      <c r="BO10" s="108" t="s">
         <v>241</v>
       </c>
-      <c r="BP10" s="132"/>
-      <c r="BQ10" s="133"/>
-      <c r="BR10" s="134" t="s">
+      <c r="BP10" s="108"/>
+      <c r="BQ10" s="109"/>
+      <c r="BR10" s="122" t="s">
         <v>242</v>
       </c>
-      <c r="BS10" s="135"/>
-      <c r="BT10" s="135"/>
-      <c r="BU10" s="135"/>
-      <c r="BV10" s="136"/>
-      <c r="BW10" s="137" t="s">
+      <c r="BS10" s="123"/>
+      <c r="BT10" s="123"/>
+      <c r="BU10" s="123"/>
+      <c r="BV10" s="124"/>
+      <c r="BW10" s="119" t="s">
         <v>236</v>
       </c>
-      <c r="BX10" s="138"/>
-      <c r="BY10" s="138"/>
-      <c r="BZ10" s="139"/>
+      <c r="BX10" s="120"/>
+      <c r="BY10" s="120"/>
+      <c r="BZ10" s="121"/>
     </row>
     <row r="11" spans="1:78" ht="21.4" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A11" s="106"/>
+      <c r="A11" s="125"/>
       <c r="B11" s="46" t="s">
         <v>224</v>
       </c>
@@ -17630,7 +17378,7 @@
       </c>
     </row>
     <row r="12" spans="1:78" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A12" s="106"/>
+      <c r="A12" s="125"/>
       <c r="B12" s="47" t="s">
         <v>0</v>
       </c>
@@ -17882,7 +17630,7 @@
       </c>
     </row>
     <row r="13" spans="1:78" x14ac:dyDescent="0.45">
-      <c r="A13" s="106"/>
+      <c r="A13" s="125"/>
       <c r="B13" s="47" t="s">
         <v>185</v>
       </c>
@@ -18134,7 +17882,7 @@
       </c>
     </row>
     <row r="14" spans="1:78" x14ac:dyDescent="0.45">
-      <c r="A14" s="106"/>
+      <c r="A14" s="125"/>
       <c r="B14" s="47" t="s">
         <v>186</v>
       </c>
@@ -18386,7 +18134,7 @@
       </c>
     </row>
     <row r="15" spans="1:78" x14ac:dyDescent="0.45">
-      <c r="A15" s="106"/>
+      <c r="A15" s="125"/>
       <c r="B15" s="47" t="s">
         <v>187</v>
       </c>
@@ -18638,7 +18386,7 @@
       </c>
     </row>
     <row r="16" spans="1:78" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A16" s="106"/>
+      <c r="A16" s="125"/>
       <c r="B16" s="47" t="s">
         <v>188</v>
       </c>
@@ -18890,7 +18638,7 @@
       </c>
     </row>
     <row r="17" spans="1:78" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A17" s="106"/>
+      <c r="A17" s="125"/>
       <c r="B17" s="50" t="s">
         <v>4</v>
       </c>
@@ -19357,28 +19105,6 @@
     </row>
   </sheetData>
   <mergeCells count="38">
-    <mergeCell ref="C10:E10"/>
-    <mergeCell ref="O10:Q10"/>
-    <mergeCell ref="C1:E1"/>
-    <mergeCell ref="O1:Q1"/>
-    <mergeCell ref="F10:J10"/>
-    <mergeCell ref="AW10:AZ10"/>
-    <mergeCell ref="K10:N10"/>
-    <mergeCell ref="W10:Z10"/>
-    <mergeCell ref="F1:J1"/>
-    <mergeCell ref="K1:N1"/>
-    <mergeCell ref="R1:V1"/>
-    <mergeCell ref="W1:Z1"/>
-    <mergeCell ref="R10:V10"/>
-    <mergeCell ref="BO10:BQ10"/>
-    <mergeCell ref="BR10:BV10"/>
-    <mergeCell ref="BW10:BZ10"/>
-    <mergeCell ref="BC1:BE1"/>
-    <mergeCell ref="BF1:BJ1"/>
-    <mergeCell ref="BK1:BN1"/>
-    <mergeCell ref="BO1:BQ1"/>
-    <mergeCell ref="BR1:BV1"/>
-    <mergeCell ref="BW1:BZ1"/>
     <mergeCell ref="A1:A8"/>
     <mergeCell ref="A10:A17"/>
     <mergeCell ref="BC10:BE10"/>
@@ -19395,6 +19121,28 @@
     <mergeCell ref="AK10:AN10"/>
     <mergeCell ref="AO10:AQ10"/>
     <mergeCell ref="AR10:AV10"/>
+    <mergeCell ref="BO10:BQ10"/>
+    <mergeCell ref="BR10:BV10"/>
+    <mergeCell ref="BW10:BZ10"/>
+    <mergeCell ref="BC1:BE1"/>
+    <mergeCell ref="BF1:BJ1"/>
+    <mergeCell ref="BK1:BN1"/>
+    <mergeCell ref="BO1:BQ1"/>
+    <mergeCell ref="BR1:BV1"/>
+    <mergeCell ref="BW1:BZ1"/>
+    <mergeCell ref="AW10:AZ10"/>
+    <mergeCell ref="K10:N10"/>
+    <mergeCell ref="W10:Z10"/>
+    <mergeCell ref="F1:J1"/>
+    <mergeCell ref="K1:N1"/>
+    <mergeCell ref="R1:V1"/>
+    <mergeCell ref="W1:Z1"/>
+    <mergeCell ref="R10:V10"/>
+    <mergeCell ref="C10:E10"/>
+    <mergeCell ref="O10:Q10"/>
+    <mergeCell ref="C1:E1"/>
+    <mergeCell ref="O1:Q1"/>
+    <mergeCell ref="F10:J10"/>
   </mergeCells>
   <conditionalFormatting sqref="AC3:AZ8">
     <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">

</xml_diff>

<commit_message>
profil anpassung für search Funktion
</commit_message>
<xml_diff>
--- a/web/utilities/records_kriterien.xlsx
+++ b/web/utilities/records_kriterien.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jpgna\Documents\GitHub\Lifesaving_Baden\web\utilities\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBE8BAB8-837C-4BDA-86D3-795FBF6081E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E78AB87A-A4E0-4AC8-BD5A-1F316EAB842B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="687" firstSheet="1" activeTab="7" xr2:uid="{E1AB626B-3773-4829-92A5-28DD4DB7C8F8}"/>
   </bookViews>
@@ -185,7 +185,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="667" uniqueCount="254">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="814" uniqueCount="276">
   <si>
     <t>50m Retten</t>
   </si>
@@ -947,6 +947,72 @@
   </si>
   <si>
     <t>PZ - 200m Hindernis</t>
+  </si>
+  <si>
+    <t>LMS</t>
+  </si>
+  <si>
+    <t>DMM</t>
+  </si>
+  <si>
+    <t>DEM</t>
+  </si>
+  <si>
+    <t>Trophy</t>
+  </si>
+  <si>
+    <t>JRP</t>
+  </si>
+  <si>
+    <t>WM</t>
+  </si>
+  <si>
+    <t>EM</t>
+  </si>
+  <si>
+    <t>JWM</t>
+  </si>
+  <si>
+    <t>JEM</t>
+  </si>
+  <si>
+    <t>DMO</t>
+  </si>
+  <si>
+    <t>DMO Ocean</t>
+  </si>
+  <si>
+    <t>Ocean Perf</t>
+  </si>
+  <si>
+    <t>Filcow</t>
+  </si>
+  <si>
+    <t>9-16</t>
+  </si>
+  <si>
+    <t>4-8</t>
+  </si>
+  <si>
+    <t>1-5</t>
+  </si>
+  <si>
+    <t>1-3</t>
+  </si>
+  <si>
+    <t>6-9</t>
+  </si>
+  <si>
+    <t>4-6</t>
+  </si>
+  <si>
+    <t>6-10</t>
+  </si>
+  <si>
+    <t>1-8</t>
+  </si>
+  <si>
+    <t>1000</t>
   </si>
 </sst>
 </file>
@@ -1331,7 +1397,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="140">
+  <cellXfs count="141">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1632,16 +1698,13 @@
     <xf numFmtId="0" fontId="14" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1653,15 +1716,6 @@
     <xf numFmtId="0" fontId="14" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="10" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1670,27 +1724,6 @@
     </xf>
     <xf numFmtId="0" fontId="14" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1734,12 +1767,104 @@
     <xf numFmtId="0" fontId="17" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Prozent" xfId="1" builtinId="5"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="223">
+  <dxfs count="236">
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <font>
         <color theme="4"/>
@@ -4183,10 +4308,6 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -4248,102 +4369,102 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{2C5E83EE-6B6F-478A-9C90-A846A1A76536}" name="WR_Open4" displayName="WR_Open4" ref="A4:AW31" totalsRowShown="0" headerRowDxfId="201" headerRowBorderDxfId="200" tableBorderDxfId="199">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{2C5E83EE-6B6F-478A-9C90-A846A1A76536}" name="WR_Open4" displayName="WR_Open4" ref="A4:AW31" totalsRowShown="0" headerRowDxfId="215" headerRowBorderDxfId="214" tableBorderDxfId="213">
   <autoFilter ref="A4:AW31" xr:uid="{2C5E83EE-6B6F-478A-9C90-A846A1A76536}"/>
   <tableColumns count="49">
-    <tableColumn id="1" xr3:uid="{7C0C4105-A61A-4B8D-9129-EDC4F18765AF}" name="WR-Open" dataDxfId="198">
+    <tableColumn id="1" xr3:uid="{7C0C4105-A61A-4B8D-9129-EDC4F18765AF}" name="WR-Open" dataDxfId="212">
       <calculatedColumnFormula>A4+1</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{516F5612-F85F-413F-9012-E235F415E34B}" name="50m Retten - offen - W" dataDxfId="197"/>
-    <tableColumn id="3" xr3:uid="{BC9ACAC9-0D45-42FD-B596-D19FBE3A4D83}" name="100m Retten - offen - W" dataDxfId="196"/>
-    <tableColumn id="4" xr3:uid="{CB6DBE59-EB65-43F0-93E7-0BDC3F82832B}" name="100m Kombi - offen - W" dataDxfId="195"/>
-    <tableColumn id="5" xr3:uid="{AA603C60-6831-4C14-A8CD-0AA050DA7551}" name="100m Lifesaver - offen - W" dataDxfId="194"/>
-    <tableColumn id="6" xr3:uid="{7920F147-7717-4582-940A-2610F7D310CA}" name="200m Superlifesaver - offen - W" dataDxfId="193"/>
-    <tableColumn id="7" xr3:uid="{04E21F1D-AC8D-4A1B-9B43-59B8F7901673}" name="200m Hindernis - offen - W" dataDxfId="192"/>
-    <tableColumn id="8" xr3:uid="{40E8A083-653A-48A8-9B37-0A2D850B7829}" name="50m Retten - offen - M" dataDxfId="191"/>
-    <tableColumn id="9" xr3:uid="{863824A9-134F-4189-BB14-225AE224FC44}" name="100m Retten - offen - M" dataDxfId="190"/>
+    <tableColumn id="2" xr3:uid="{516F5612-F85F-413F-9012-E235F415E34B}" name="50m Retten - offen - W" dataDxfId="211"/>
+    <tableColumn id="3" xr3:uid="{BC9ACAC9-0D45-42FD-B596-D19FBE3A4D83}" name="100m Retten - offen - W" dataDxfId="210"/>
+    <tableColumn id="4" xr3:uid="{CB6DBE59-EB65-43F0-93E7-0BDC3F82832B}" name="100m Kombi - offen - W" dataDxfId="209"/>
+    <tableColumn id="5" xr3:uid="{AA603C60-6831-4C14-A8CD-0AA050DA7551}" name="100m Lifesaver - offen - W" dataDxfId="208"/>
+    <tableColumn id="6" xr3:uid="{7920F147-7717-4582-940A-2610F7D310CA}" name="200m Superlifesaver - offen - W" dataDxfId="207"/>
+    <tableColumn id="7" xr3:uid="{04E21F1D-AC8D-4A1B-9B43-59B8F7901673}" name="200m Hindernis - offen - W" dataDxfId="206"/>
+    <tableColumn id="8" xr3:uid="{40E8A083-653A-48A8-9B37-0A2D850B7829}" name="50m Retten - offen - M" dataDxfId="205"/>
+    <tableColumn id="9" xr3:uid="{863824A9-134F-4189-BB14-225AE224FC44}" name="100m Retten - offen - M" dataDxfId="204"/>
     <tableColumn id="10" xr3:uid="{598FC6AE-DEA2-4475-9A35-CDCB8C81496A}" name="100m Kombi - offen - M"/>
     <tableColumn id="11" xr3:uid="{9FC50B37-0D51-422E-A268-A6506D4F3854}" name="100m Lifesaver - offen - M"/>
     <tableColumn id="12" xr3:uid="{B8D2552B-5D82-442A-98F0-E47D5C5F6728}" name="200m Superlifesaver - offen - M"/>
-    <tableColumn id="13" xr3:uid="{5A5E9873-0C5F-4508-AF6B-4974E0526D84}" name="200m Hindernis - offen - M" dataDxfId="189"/>
-    <tableColumn id="14" xr3:uid="{FA907992-7FCE-4CAD-8CF2-F5BEBC9B3756}" name="50m Retten - 17/18 - W" dataDxfId="188"/>
-    <tableColumn id="15" xr3:uid="{76B63DC0-CB67-48F4-9B5A-D22902F59334}" name="100m Retten - 17/18 - W" dataDxfId="187"/>
-    <tableColumn id="16" xr3:uid="{614A2419-51B1-44C0-8469-ADBFB078B81A}" name="100m Kombi -17/18 - W" dataDxfId="186"/>
-    <tableColumn id="17" xr3:uid="{2EC953EE-367D-4524-A25E-8DE3B8168E34}" name="100m Lifesaver - 17/18 - W" dataDxfId="185"/>
-    <tableColumn id="18" xr3:uid="{25711867-9BD7-4197-9094-A21392411249}" name="200m Superlifesaver - 17/18 - W" dataDxfId="184"/>
-    <tableColumn id="19" xr3:uid="{262DB142-CFB1-45C3-9332-7273CACD1B62}" name="200m Hindernis - 17/18 - W" dataDxfId="183"/>
-    <tableColumn id="20" xr3:uid="{938BA45A-8244-4637-8A14-DF49CD91A945}" name="50m Retten - 17/18 - M" dataDxfId="182"/>
-    <tableColumn id="21" xr3:uid="{737E28D8-900F-4A98-95FE-EE7B0AFDEE90}" name="100m Retten - 17/18 - M" dataDxfId="181"/>
-    <tableColumn id="22" xr3:uid="{330BD3A8-061C-45E2-ADDB-40C2F346772F}" name="100m Kombi - 17/18 - M" dataDxfId="180"/>
-    <tableColumn id="23" xr3:uid="{0CADDE90-A167-4E1D-8D33-8624E5E1A4E2}" name="100m Lifesaver - 17/18 - M" dataDxfId="179"/>
-    <tableColumn id="24" xr3:uid="{FCF9F42C-1291-4985-9D37-B9DE2DAA5DCB}" name="200m Superlifesaver - 17/18 - M" dataDxfId="178"/>
-    <tableColumn id="25" xr3:uid="{4E5397B2-F924-4F48-AE69-AF6D650AF88D}" name="200m Hindernis - 17/18 - M" dataDxfId="177"/>
-    <tableColumn id="26" xr3:uid="{0A78315A-BFDC-43EE-A66F-48B301F66508}" name="50m Retten - 15/16 - W" dataDxfId="176"/>
-    <tableColumn id="27" xr3:uid="{D3FCF8BD-6C76-450D-80C0-CC0519A79731}" name="100m Retten - 15/16 - W" dataDxfId="175"/>
-    <tableColumn id="28" xr3:uid="{6BE7937E-D62D-47CD-95DE-1730304B0DF3}" name="100m Kombi - 15/16 - W" dataDxfId="174"/>
-    <tableColumn id="29" xr3:uid="{098BA5BE-5AF6-4187-89B6-534498F24C51}" name="100m Lifesaver -  15/16 - W" dataDxfId="173"/>
-    <tableColumn id="30" xr3:uid="{2A6822CF-143C-4BF7-A440-5777527BE512}" name="200m Superlifesaver -  15/16 - W" dataDxfId="172"/>
-    <tableColumn id="31" xr3:uid="{541C7145-CDEA-4E4E-9E7A-A4F05BA6C3E5}" name="200m Hindernis -  15/16 - W" dataDxfId="171"/>
-    <tableColumn id="32" xr3:uid="{342C4488-8C61-42E6-87A9-C75BD8EB7452}" name="50m Retten - 15/16 - M" dataDxfId="170"/>
-    <tableColumn id="33" xr3:uid="{857B1D46-7D20-47F7-AB9B-732D50346E32}" name="100m Retten - 15/16 - M" dataDxfId="169"/>
-    <tableColumn id="34" xr3:uid="{4C8A2EB4-804B-45F1-A768-9A6958957F8B}" name="100m Kombi -15/16 - M" dataDxfId="168"/>
-    <tableColumn id="35" xr3:uid="{26C75B4F-21EC-4EB0-A9A9-54BC80140672}" name="100m Lifesaver - 15/16 - M" dataDxfId="167"/>
-    <tableColumn id="36" xr3:uid="{DBBB2A23-1A06-429A-A5D1-A547EF5EC16F}" name="200m Superlifesaver - 15/16 - M" dataDxfId="166"/>
-    <tableColumn id="37" xr3:uid="{84061231-CAE5-427A-87F5-6DDBA99F77D2}" name="200m Hindernis - 15/16 - M" dataDxfId="165"/>
-    <tableColumn id="38" xr3:uid="{878CCA80-A742-4B3C-90C9-E93BB814201B}" name="50m Retten - 13/14 - W" dataDxfId="164"/>
-    <tableColumn id="39" xr3:uid="{A1F57102-61CF-4784-8DE2-0B8F32D5D699}" name="50m Retten mit Flossen - 13/14 - W" dataDxfId="163"/>
-    <tableColumn id="40" xr3:uid="{0F6BAF78-3D79-42A9-9FED-E6D0E335A920}" name="100m Hindernis - 13/14 - W" dataDxfId="162"/>
-    <tableColumn id="41" xr3:uid="{EB748A68-E10D-4D76-B315-8FDB3AC33C8D}" name="50m Retten - 13/14 - M" dataDxfId="161"/>
-    <tableColumn id="42" xr3:uid="{C7B04167-6430-40F0-9A0F-D0D0BE2F9C77}" name="50m Retten mit Flossen - 13/14 - M" dataDxfId="160"/>
-    <tableColumn id="43" xr3:uid="{48704BB7-A853-445A-8CDC-8D8F86C2B66A}" name="100m Hindernis - 13/14 - M" dataDxfId="159"/>
-    <tableColumn id="44" xr3:uid="{9605FE9A-F41C-4A5F-A59C-B7A9D45C460F}" name="50m Flossen - 12 - W" dataDxfId="158"/>
-    <tableColumn id="45" xr3:uid="{4C9DBF61-35B1-4BC2-8272-526E0AFAAFFB}" name="50m komb. Schwimmen - 12 - W" dataDxfId="157"/>
-    <tableColumn id="46" xr3:uid="{CF433C95-C272-48F9-98CD-7E3C8DBB6F2C}" name="50m Hindernis - 12 - W" dataDxfId="156"/>
-    <tableColumn id="47" xr3:uid="{FADB7411-DB43-4B14-B9E8-D74CA1BA18B8}" name="50m Flossen - 12 - M" dataDxfId="155"/>
-    <tableColumn id="48" xr3:uid="{02936F84-1D82-48AC-8D7C-6D2954D68A06}" name="50m komb. Schwimmen - 12 - M" dataDxfId="154"/>
-    <tableColumn id="49" xr3:uid="{7FD9BD11-0597-4E07-8DA5-DB53384197F5}" name="50m Hindernis - 12 - M" dataDxfId="153"/>
+    <tableColumn id="13" xr3:uid="{5A5E9873-0C5F-4508-AF6B-4974E0526D84}" name="200m Hindernis - offen - M" dataDxfId="203"/>
+    <tableColumn id="14" xr3:uid="{FA907992-7FCE-4CAD-8CF2-F5BEBC9B3756}" name="50m Retten - 17/18 - W" dataDxfId="202"/>
+    <tableColumn id="15" xr3:uid="{76B63DC0-CB67-48F4-9B5A-D22902F59334}" name="100m Retten - 17/18 - W" dataDxfId="201"/>
+    <tableColumn id="16" xr3:uid="{614A2419-51B1-44C0-8469-ADBFB078B81A}" name="100m Kombi -17/18 - W" dataDxfId="200"/>
+    <tableColumn id="17" xr3:uid="{2EC953EE-367D-4524-A25E-8DE3B8168E34}" name="100m Lifesaver - 17/18 - W" dataDxfId="199"/>
+    <tableColumn id="18" xr3:uid="{25711867-9BD7-4197-9094-A21392411249}" name="200m Superlifesaver - 17/18 - W" dataDxfId="198"/>
+    <tableColumn id="19" xr3:uid="{262DB142-CFB1-45C3-9332-7273CACD1B62}" name="200m Hindernis - 17/18 - W" dataDxfId="197"/>
+    <tableColumn id="20" xr3:uid="{938BA45A-8244-4637-8A14-DF49CD91A945}" name="50m Retten - 17/18 - M" dataDxfId="196"/>
+    <tableColumn id="21" xr3:uid="{737E28D8-900F-4A98-95FE-EE7B0AFDEE90}" name="100m Retten - 17/18 - M" dataDxfId="195"/>
+    <tableColumn id="22" xr3:uid="{330BD3A8-061C-45E2-ADDB-40C2F346772F}" name="100m Kombi - 17/18 - M" dataDxfId="194"/>
+    <tableColumn id="23" xr3:uid="{0CADDE90-A167-4E1D-8D33-8624E5E1A4E2}" name="100m Lifesaver - 17/18 - M" dataDxfId="193"/>
+    <tableColumn id="24" xr3:uid="{FCF9F42C-1291-4985-9D37-B9DE2DAA5DCB}" name="200m Superlifesaver - 17/18 - M" dataDxfId="192"/>
+    <tableColumn id="25" xr3:uid="{4E5397B2-F924-4F48-AE69-AF6D650AF88D}" name="200m Hindernis - 17/18 - M" dataDxfId="191"/>
+    <tableColumn id="26" xr3:uid="{0A78315A-BFDC-43EE-A66F-48B301F66508}" name="50m Retten - 15/16 - W" dataDxfId="190"/>
+    <tableColumn id="27" xr3:uid="{D3FCF8BD-6C76-450D-80C0-CC0519A79731}" name="100m Retten - 15/16 - W" dataDxfId="189"/>
+    <tableColumn id="28" xr3:uid="{6BE7937E-D62D-47CD-95DE-1730304B0DF3}" name="100m Kombi - 15/16 - W" dataDxfId="188"/>
+    <tableColumn id="29" xr3:uid="{098BA5BE-5AF6-4187-89B6-534498F24C51}" name="100m Lifesaver -  15/16 - W" dataDxfId="187"/>
+    <tableColumn id="30" xr3:uid="{2A6822CF-143C-4BF7-A440-5777527BE512}" name="200m Superlifesaver -  15/16 - W" dataDxfId="186"/>
+    <tableColumn id="31" xr3:uid="{541C7145-CDEA-4E4E-9E7A-A4F05BA6C3E5}" name="200m Hindernis -  15/16 - W" dataDxfId="185"/>
+    <tableColumn id="32" xr3:uid="{342C4488-8C61-42E6-87A9-C75BD8EB7452}" name="50m Retten - 15/16 - M" dataDxfId="184"/>
+    <tableColumn id="33" xr3:uid="{857B1D46-7D20-47F7-AB9B-732D50346E32}" name="100m Retten - 15/16 - M" dataDxfId="183"/>
+    <tableColumn id="34" xr3:uid="{4C8A2EB4-804B-45F1-A768-9A6958957F8B}" name="100m Kombi -15/16 - M" dataDxfId="182"/>
+    <tableColumn id="35" xr3:uid="{26C75B4F-21EC-4EB0-A9A9-54BC80140672}" name="100m Lifesaver - 15/16 - M" dataDxfId="181"/>
+    <tableColumn id="36" xr3:uid="{DBBB2A23-1A06-429A-A5D1-A547EF5EC16F}" name="200m Superlifesaver - 15/16 - M" dataDxfId="180"/>
+    <tableColumn id="37" xr3:uid="{84061231-CAE5-427A-87F5-6DDBA99F77D2}" name="200m Hindernis - 15/16 - M" dataDxfId="179"/>
+    <tableColumn id="38" xr3:uid="{878CCA80-A742-4B3C-90C9-E93BB814201B}" name="50m Retten - 13/14 - W" dataDxfId="178"/>
+    <tableColumn id="39" xr3:uid="{A1F57102-61CF-4784-8DE2-0B8F32D5D699}" name="50m Retten mit Flossen - 13/14 - W" dataDxfId="177"/>
+    <tableColumn id="40" xr3:uid="{0F6BAF78-3D79-42A9-9FED-E6D0E335A920}" name="100m Hindernis - 13/14 - W" dataDxfId="176"/>
+    <tableColumn id="41" xr3:uid="{EB748A68-E10D-4D76-B315-8FDB3AC33C8D}" name="50m Retten - 13/14 - M" dataDxfId="175"/>
+    <tableColumn id="42" xr3:uid="{C7B04167-6430-40F0-9A0F-D0D0BE2F9C77}" name="50m Retten mit Flossen - 13/14 - M" dataDxfId="174"/>
+    <tableColumn id="43" xr3:uid="{48704BB7-A853-445A-8CDC-8D8F86C2B66A}" name="100m Hindernis - 13/14 - M" dataDxfId="173"/>
+    <tableColumn id="44" xr3:uid="{9605FE9A-F41C-4A5F-A59C-B7A9D45C460F}" name="50m Flossen - 12 - W" dataDxfId="172"/>
+    <tableColumn id="45" xr3:uid="{4C9DBF61-35B1-4BC2-8272-526E0AFAAFFB}" name="50m komb. Schwimmen - 12 - W" dataDxfId="171"/>
+    <tableColumn id="46" xr3:uid="{CF433C95-C272-48F9-98CD-7E3C8DBB6F2C}" name="50m Hindernis - 12 - W" dataDxfId="170"/>
+    <tableColumn id="47" xr3:uid="{FADB7411-DB43-4B14-B9E8-D74CA1BA18B8}" name="50m Flossen - 12 - M" dataDxfId="169"/>
+    <tableColumn id="48" xr3:uid="{02936F84-1D82-48AC-8D7C-6D2954D68A06}" name="50m komb. Schwimmen - 12 - M" dataDxfId="168"/>
+    <tableColumn id="49" xr3:uid="{7FD9BD11-0597-4E07-8DA5-DB53384197F5}" name="50m Hindernis - 12 - M" dataDxfId="167"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{4234D44E-A2BE-4790-B589-1A8CC19B714E}" name="WR_Youth" displayName="WR_Youth" ref="A4:M32" totalsRowShown="0" headerRowDxfId="152" dataDxfId="150" headerRowBorderDxfId="151" tableBorderDxfId="149">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{4234D44E-A2BE-4790-B589-1A8CC19B714E}" name="WR_Youth" displayName="WR_Youth" ref="A4:M32" totalsRowShown="0" headerRowDxfId="166" dataDxfId="164" headerRowBorderDxfId="165" tableBorderDxfId="163">
   <autoFilter ref="A4:M32" xr:uid="{4234D44E-A2BE-4790-B589-1A8CC19B714E}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{848E691A-41B0-42DD-B122-FB6DF43CB3EF}" name="WR-Youth" dataDxfId="148"/>
-    <tableColumn id="2" xr3:uid="{2FE43F18-485B-46A9-8946-FBC5FDAE5A8E}" name="50m Retten" dataDxfId="147"/>
-    <tableColumn id="3" xr3:uid="{CA5C3ABF-02E6-442B-868B-95B293B231D3}" name="100m Retten" dataDxfId="146"/>
-    <tableColumn id="4" xr3:uid="{7A6BBA52-2145-464D-8C04-B2CCFC1A90DC}" name="100m Kombi" dataDxfId="145"/>
-    <tableColumn id="5" xr3:uid="{21F420C9-E788-49EE-88F6-E37963ED31CF}" name="100m Lifesaver" dataDxfId="144"/>
-    <tableColumn id="6" xr3:uid="{CB87B7CD-8A9C-4775-A4D7-4D267F43FD1A}" name="200m Superlifesaver" dataDxfId="143"/>
-    <tableColumn id="7" xr3:uid="{2DC7F290-B564-4851-85AE-D211DA701B32}" name="200m Hindernis" dataDxfId="142"/>
-    <tableColumn id="8" xr3:uid="{8112783D-8796-4D6A-8414-AC675D745697}" name="50m Retten2" dataDxfId="141"/>
-    <tableColumn id="9" xr3:uid="{4E818CD4-8725-495D-9D1D-1AFCED9181F5}" name="100m Retten2" dataDxfId="140"/>
-    <tableColumn id="10" xr3:uid="{28C05A91-E302-40A9-B50A-ECF997F129FC}" name="100m Kombi2" dataDxfId="139"/>
-    <tableColumn id="11" xr3:uid="{D56FB9F2-45BF-4EC9-A84C-8A5FB59F2F05}" name="100m Lifesaver2" dataDxfId="138"/>
-    <tableColumn id="12" xr3:uid="{540169C0-2A40-4794-A872-F7DF8A887BF2}" name="200m Superlifesaver2" dataDxfId="137"/>
-    <tableColumn id="13" xr3:uid="{D104CB67-B55A-4C81-87E5-0AC758DD22A4}" name="200m Hindernis2" dataDxfId="136"/>
+    <tableColumn id="1" xr3:uid="{848E691A-41B0-42DD-B122-FB6DF43CB3EF}" name="WR-Youth" dataDxfId="162"/>
+    <tableColumn id="2" xr3:uid="{2FE43F18-485B-46A9-8946-FBC5FDAE5A8E}" name="50m Retten" dataDxfId="161"/>
+    <tableColumn id="3" xr3:uid="{CA5C3ABF-02E6-442B-868B-95B293B231D3}" name="100m Retten" dataDxfId="160"/>
+    <tableColumn id="4" xr3:uid="{7A6BBA52-2145-464D-8C04-B2CCFC1A90DC}" name="100m Kombi" dataDxfId="159"/>
+    <tableColumn id="5" xr3:uid="{21F420C9-E788-49EE-88F6-E37963ED31CF}" name="100m Lifesaver" dataDxfId="158"/>
+    <tableColumn id="6" xr3:uid="{CB87B7CD-8A9C-4775-A4D7-4D267F43FD1A}" name="200m Superlifesaver" dataDxfId="157"/>
+    <tableColumn id="7" xr3:uid="{2DC7F290-B564-4851-85AE-D211DA701B32}" name="200m Hindernis" dataDxfId="156"/>
+    <tableColumn id="8" xr3:uid="{8112783D-8796-4D6A-8414-AC675D745697}" name="50m Retten2" dataDxfId="155"/>
+    <tableColumn id="9" xr3:uid="{4E818CD4-8725-495D-9D1D-1AFCED9181F5}" name="100m Retten2" dataDxfId="154"/>
+    <tableColumn id="10" xr3:uid="{28C05A91-E302-40A9-B50A-ECF997F129FC}" name="100m Kombi2" dataDxfId="153"/>
+    <tableColumn id="11" xr3:uid="{D56FB9F2-45BF-4EC9-A84C-8A5FB59F2F05}" name="100m Lifesaver2" dataDxfId="152"/>
+    <tableColumn id="12" xr3:uid="{540169C0-2A40-4794-A872-F7DF8A887BF2}" name="200m Superlifesaver2" dataDxfId="151"/>
+    <tableColumn id="13" xr3:uid="{D104CB67-B55A-4C81-87E5-0AC758DD22A4}" name="200m Hindernis2" dataDxfId="150"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E2D2F97B-7645-4066-8AB3-F35CF6E035EB}" name="WR_Open" displayName="WR_Open" ref="A4:M32" totalsRowShown="0" headerRowDxfId="135" headerRowBorderDxfId="134" tableBorderDxfId="133">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E2D2F97B-7645-4066-8AB3-F35CF6E035EB}" name="WR_Open" displayName="WR_Open" ref="A4:M32" totalsRowShown="0" headerRowDxfId="149" headerRowBorderDxfId="148" tableBorderDxfId="147">
   <autoFilter ref="A4:M32" xr:uid="{E2D2F97B-7645-4066-8AB3-F35CF6E035EB}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{AE73402B-B27E-4B29-8DCF-30B7FC1855EF}" name="WR-Open" dataDxfId="132">
+    <tableColumn id="1" xr3:uid="{AE73402B-B27E-4B29-8DCF-30B7FC1855EF}" name="WR-Open" dataDxfId="146">
       <calculatedColumnFormula>A4+1</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{EA3EAC1F-184E-4A28-B3E3-08DE12F138EF}" name="50m Retten" dataDxfId="131"/>
-    <tableColumn id="3" xr3:uid="{E0305A3F-6087-4F8C-8B64-153E1ACAA32E}" name="100m Retten" dataDxfId="130"/>
-    <tableColumn id="4" xr3:uid="{F0B7AC37-315E-49AA-855C-7955D2B43A76}" name="100m Kombi" dataDxfId="129"/>
-    <tableColumn id="5" xr3:uid="{B5E690AB-DB7D-4864-8916-89D2A68C4128}" name="100m Lifesaver" dataDxfId="128"/>
-    <tableColumn id="6" xr3:uid="{D89BAF4D-36AE-4C73-9320-9C5736F02F8A}" name="200m Superlifesaver" dataDxfId="127"/>
-    <tableColumn id="7" xr3:uid="{58AE7517-1A90-459F-A7D2-B95265D217E7}" name="200m Hindernis" dataDxfId="126"/>
-    <tableColumn id="8" xr3:uid="{13A189FB-E897-4A1F-A001-525F61E9CFFF}" name="50m Retten2" dataDxfId="125"/>
-    <tableColumn id="9" xr3:uid="{36418AC5-46B8-400F-BD2E-D329CF4F92CD}" name="100m Retten2" dataDxfId="124"/>
+    <tableColumn id="2" xr3:uid="{EA3EAC1F-184E-4A28-B3E3-08DE12F138EF}" name="50m Retten" dataDxfId="145"/>
+    <tableColumn id="3" xr3:uid="{E0305A3F-6087-4F8C-8B64-153E1ACAA32E}" name="100m Retten" dataDxfId="144"/>
+    <tableColumn id="4" xr3:uid="{F0B7AC37-315E-49AA-855C-7955D2B43A76}" name="100m Kombi" dataDxfId="143"/>
+    <tableColumn id="5" xr3:uid="{B5E690AB-DB7D-4864-8916-89D2A68C4128}" name="100m Lifesaver" dataDxfId="142"/>
+    <tableColumn id="6" xr3:uid="{D89BAF4D-36AE-4C73-9320-9C5736F02F8A}" name="200m Superlifesaver" dataDxfId="141"/>
+    <tableColumn id="7" xr3:uid="{58AE7517-1A90-459F-A7D2-B95265D217E7}" name="200m Hindernis" dataDxfId="140"/>
+    <tableColumn id="8" xr3:uid="{13A189FB-E897-4A1F-A001-525F61E9CFFF}" name="50m Retten2" dataDxfId="139"/>
+    <tableColumn id="9" xr3:uid="{36418AC5-46B8-400F-BD2E-D329CF4F92CD}" name="100m Retten2" dataDxfId="138"/>
     <tableColumn id="10" xr3:uid="{06A35C2D-7313-472B-BC1F-4F2FB1D14782}" name="100m Kombi2"/>
     <tableColumn id="11" xr3:uid="{89966D0D-9131-4245-A7BE-1A7384D5ADA0}" name="100m Lifesaver2"/>
     <tableColumn id="12" xr3:uid="{D9D6CF56-869C-4DDE-9886-572D4E523A8F}" name="200m Superlifesaver2"/>
@@ -4354,7 +4475,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{CF3D303A-A04B-42DD-A44E-CEB6CECB77A4}" name="DP_konfig" displayName="DP_konfig" ref="A1:U3" totalsRowShown="0" headerRowDxfId="123" dataDxfId="122">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{CF3D303A-A04B-42DD-A44E-CEB6CECB77A4}" name="DP_konfig" displayName="DP_konfig" ref="A1:U3" totalsRowShown="0" headerRowDxfId="137" dataDxfId="136">
   <autoFilter ref="A1:U3" xr:uid="{CF3D303A-A04B-42DD-A44E-CEB6CECB77A4}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -4379,64 +4500,64 @@
     <filterColumn colId="20" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="21">
-    <tableColumn id="1" xr3:uid="{58D628F0-061E-4A82-8362-CDB37A2E7C60}" name="Tabellen Name" dataDxfId="121"/>
-    <tableColumn id="2" xr3:uid="{2F302F6C-F8AF-4FDE-AB08-6F30F9671015}" name="Geschlecht" dataDxfId="120"/>
-    <tableColumn id="3" xr3:uid="{4D91FBF9-386D-43DD-90D0-B49823FDB629}" name="Mindest alter" dataDxfId="119"/>
-    <tableColumn id="4" xr3:uid="{4126AAC6-AF2F-446C-B4EA-D86ACFD9FAC2}" name="Maximales Alter" dataDxfId="118"/>
-    <tableColumn id="5" xr3:uid="{8A10890A-A299-4B09-AC72-0E9AE9238AF3}" name="Qualizeitraum anfang" dataDxfId="117"/>
-    <tableColumn id="6" xr3:uid="{FBCD1C13-FC82-429B-8DE1-0C5A455FDAB8}" name="Qualizeitraum Ende" dataDxfId="116"/>
-    <tableColumn id="7" xr3:uid="{1DCCAC9B-BC46-468E-A3CE-57576C2FF11D}" name="Letzter Wettkampf am" dataDxfId="115"/>
-    <tableColumn id="8" xr3:uid="{9A6E47EE-ABD8-4A1E-87D3-9D286E4C124F}" name="Wertung" dataDxfId="114"/>
-    <tableColumn id="9" xr3:uid="{09E848D2-ED17-49C7-9775-CBF17D20DFC0}" name="Landesverband" dataDxfId="113"/>
-    <tableColumn id="10" xr3:uid="{70ABB713-23F6-4FCF-920E-3CB0CD451446}" name="OMS" dataDxfId="112"/>
-    <tableColumn id="11" xr3:uid="{9C108A1C-E6AB-4C13-9C1D-0FA8944A39A3}" name="Pool-Länge" dataDxfId="111"/>
-    <tableColumn id="12" xr3:uid="{087948DD-430D-48F1-906D-4F4EF4B46053}" name="Regelwerk" dataDxfId="110"/>
-    <tableColumn id="13" xr3:uid="{BF42D9C0-F77D-4971-A67E-32B0246C72C3}" name="Referenz" dataDxfId="109"/>
-    <tableColumn id="19" xr3:uid="{AFFB84E8-B398-4E99-805B-9A247071A040}" name="Referenz Jahr" dataDxfId="108"/>
-    <tableColumn id="20" xr3:uid="{0A59A474-DFBB-4437-8EFF-70284AFD9934}" name="Mindest Punktzahl" dataDxfId="107"/>
-    <tableColumn id="21" xr3:uid="{198BD231-EEF3-43C9-AD9B-39B4B7E9B337}" name="Mindest Disziplinen" dataDxfId="106"/>
-    <tableColumn id="14" xr3:uid="{443CD4F6-A2B2-480B-BB35-DCEEBC531727}" name="3-Kampf Regel" dataDxfId="105"/>
-    <tableColumn id="15" xr3:uid="{70116160-7666-42B1-92AC-FAC2620E6A60}" name="Anzahl Nominierte" dataDxfId="104"/>
-    <tableColumn id="16" xr3:uid="{0EFD0A46-D12B-4AB0-907C-08E5D9F282E0}" name="Anzahl Nachrücker" dataDxfId="103"/>
-    <tableColumn id="17" xr3:uid="{AA5430A0-8ED8-40E8-B7F8-DA25E4E8790F}" name="Seiten Anzahl" dataDxfId="102"/>
-    <tableColumn id="18" xr3:uid="{16F699D9-2741-43F3-AD5F-826A568EFEAC}" name="Absagen" dataDxfId="101"/>
+    <tableColumn id="1" xr3:uid="{58D628F0-061E-4A82-8362-CDB37A2E7C60}" name="Tabellen Name" dataDxfId="135"/>
+    <tableColumn id="2" xr3:uid="{2F302F6C-F8AF-4FDE-AB08-6F30F9671015}" name="Geschlecht" dataDxfId="134"/>
+    <tableColumn id="3" xr3:uid="{4D91FBF9-386D-43DD-90D0-B49823FDB629}" name="Mindest alter" dataDxfId="133"/>
+    <tableColumn id="4" xr3:uid="{4126AAC6-AF2F-446C-B4EA-D86ACFD9FAC2}" name="Maximales Alter" dataDxfId="132"/>
+    <tableColumn id="5" xr3:uid="{8A10890A-A299-4B09-AC72-0E9AE9238AF3}" name="Qualizeitraum anfang" dataDxfId="131"/>
+    <tableColumn id="6" xr3:uid="{FBCD1C13-FC82-429B-8DE1-0C5A455FDAB8}" name="Qualizeitraum Ende" dataDxfId="130"/>
+    <tableColumn id="7" xr3:uid="{1DCCAC9B-BC46-468E-A3CE-57576C2FF11D}" name="Letzter Wettkampf am" dataDxfId="129"/>
+    <tableColumn id="8" xr3:uid="{9A6E47EE-ABD8-4A1E-87D3-9D286E4C124F}" name="Wertung" dataDxfId="128"/>
+    <tableColumn id="9" xr3:uid="{09E848D2-ED17-49C7-9775-CBF17D20DFC0}" name="Landesverband" dataDxfId="127"/>
+    <tableColumn id="10" xr3:uid="{70ABB713-23F6-4FCF-920E-3CB0CD451446}" name="OMS" dataDxfId="126"/>
+    <tableColumn id="11" xr3:uid="{9C108A1C-E6AB-4C13-9C1D-0FA8944A39A3}" name="Pool-Länge" dataDxfId="125"/>
+    <tableColumn id="12" xr3:uid="{087948DD-430D-48F1-906D-4F4EF4B46053}" name="Regelwerk" dataDxfId="124"/>
+    <tableColumn id="13" xr3:uid="{BF42D9C0-F77D-4971-A67E-32B0246C72C3}" name="Referenz" dataDxfId="123"/>
+    <tableColumn id="19" xr3:uid="{AFFB84E8-B398-4E99-805B-9A247071A040}" name="Referenz Jahr" dataDxfId="122"/>
+    <tableColumn id="20" xr3:uid="{0A59A474-DFBB-4437-8EFF-70284AFD9934}" name="Mindest Punktzahl" dataDxfId="121"/>
+    <tableColumn id="21" xr3:uid="{198BD231-EEF3-43C9-AD9B-39B4B7E9B337}" name="Mindest Disziplinen" dataDxfId="120"/>
+    <tableColumn id="14" xr3:uid="{443CD4F6-A2B2-480B-BB35-DCEEBC531727}" name="3-Kampf Regel" dataDxfId="119"/>
+    <tableColumn id="15" xr3:uid="{70116160-7666-42B1-92AC-FAC2620E6A60}" name="Anzahl Nominierte" dataDxfId="118"/>
+    <tableColumn id="16" xr3:uid="{0EFD0A46-D12B-4AB0-907C-08E5D9F282E0}" name="Anzahl Nachrücker" dataDxfId="117"/>
+    <tableColumn id="17" xr3:uid="{AA5430A0-8ED8-40E8-B7F8-DA25E4E8790F}" name="Seiten Anzahl" dataDxfId="116"/>
+    <tableColumn id="18" xr3:uid="{16F699D9-2741-43F3-AD5F-826A568EFEAC}" name="Absagen" dataDxfId="115"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{CDBF6724-48A1-41AB-94B5-CC35C54BB15C}" name="BP_konfig" displayName="BP_konfig" ref="A1:U7" totalsRowShown="0" headerRowDxfId="100" dataDxfId="99">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{CDBF6724-48A1-41AB-94B5-CC35C54BB15C}" name="BP_konfig" displayName="BP_konfig" ref="A1:U7" totalsRowShown="0" headerRowDxfId="114" dataDxfId="113">
   <autoFilter ref="A1:U7" xr:uid="{CDBF6724-48A1-41AB-94B5-CC35C54BB15C}"/>
   <tableColumns count="21">
-    <tableColumn id="1" xr3:uid="{E1FB3D0C-B874-4874-BACC-6872CF171957}" name="Tabellen Name" dataDxfId="98"/>
-    <tableColumn id="2" xr3:uid="{FFDD2777-2097-450C-B020-F133CF643855}" name="Geschlecht" dataDxfId="97"/>
-    <tableColumn id="3" xr3:uid="{8CF52BE2-8020-48BD-A36D-63F13A1878DE}" name="Mindest alter" dataDxfId="96"/>
-    <tableColumn id="4" xr3:uid="{FD3A030F-CD97-4B6F-8E8C-BC2E67D79F1D}" name="Maximales Alter" dataDxfId="95"/>
-    <tableColumn id="5" xr3:uid="{3E22B645-D77C-4509-B031-9914FCB91599}" name="Qualizeitraum anfang" dataDxfId="94"/>
-    <tableColumn id="6" xr3:uid="{AE299324-3C1C-4063-ADF9-54555A161734}" name="Qualizeitraum Ende" dataDxfId="93"/>
-    <tableColumn id="7" xr3:uid="{DCC178B3-11FC-4C53-BBC6-C2FDA2C89857}" name="Letzter Wettkampf am" dataDxfId="92"/>
-    <tableColumn id="8" xr3:uid="{2811DB01-60A5-4BE4-B6F9-A806398A602A}" name="Wertung" dataDxfId="91"/>
-    <tableColumn id="9" xr3:uid="{0C16DAFE-847D-4E9E-9604-3A7D9FE924D0}" name="Landesverband" dataDxfId="90"/>
-    <tableColumn id="10" xr3:uid="{7A8A4101-A553-4BD5-9116-9AA5876B9401}" name="OMS" dataDxfId="89"/>
-    <tableColumn id="11" xr3:uid="{9807C9BD-6499-45F6-ACE0-4D13D64EF675}" name="Pool-Länge" dataDxfId="88"/>
-    <tableColumn id="12" xr3:uid="{13D336DD-650F-4F2C-836F-361CA1528F6D}" name="Regelwerk" dataDxfId="87"/>
-    <tableColumn id="13" xr3:uid="{66660E2D-ADF2-4FB5-8A13-004F826EE908}" name="Referenz" dataDxfId="86"/>
-    <tableColumn id="19" xr3:uid="{D72EDF8B-ECC3-4FF7-ABE6-B60BCE4A5E26}" name="Referenz Jahr" dataDxfId="85"/>
-    <tableColumn id="20" xr3:uid="{7B18E667-70F7-4BC1-AB1B-21C019F2AA89}" name="Mindest Punktzahl" dataDxfId="84"/>
-    <tableColumn id="21" xr3:uid="{FC185946-681B-42A6-AB1A-FC1EABB668C5}" name="Mindest Disziplinen" dataDxfId="83"/>
-    <tableColumn id="14" xr3:uid="{6A2676FD-2EC7-4C41-A35E-A1597A38F932}" name="3-Kampf Regel" dataDxfId="82"/>
-    <tableColumn id="15" xr3:uid="{718E0917-4F83-4A2B-832F-EBB16D5E21BF}" name="Anzahl Nominierte" dataDxfId="81"/>
-    <tableColumn id="16" xr3:uid="{5C66A461-D647-4E00-A81C-FD7AD44D7CC2}" name="Anzahl Nachrücker" dataDxfId="80"/>
-    <tableColumn id="17" xr3:uid="{D434BDEC-293B-4B4E-A5E9-479438960A03}" name="Seiten Anzahl" dataDxfId="79"/>
-    <tableColumn id="18" xr3:uid="{80908229-9247-473F-81C0-9C9D4C12FF06}" name="Absagen" dataDxfId="78"/>
+    <tableColumn id="1" xr3:uid="{E1FB3D0C-B874-4874-BACC-6872CF171957}" name="Tabellen Name" dataDxfId="112"/>
+    <tableColumn id="2" xr3:uid="{FFDD2777-2097-450C-B020-F133CF643855}" name="Geschlecht" dataDxfId="111"/>
+    <tableColumn id="3" xr3:uid="{8CF52BE2-8020-48BD-A36D-63F13A1878DE}" name="Mindest alter" dataDxfId="110"/>
+    <tableColumn id="4" xr3:uid="{FD3A030F-CD97-4B6F-8E8C-BC2E67D79F1D}" name="Maximales Alter" dataDxfId="109"/>
+    <tableColumn id="5" xr3:uid="{3E22B645-D77C-4509-B031-9914FCB91599}" name="Qualizeitraum anfang" dataDxfId="108"/>
+    <tableColumn id="6" xr3:uid="{AE299324-3C1C-4063-ADF9-54555A161734}" name="Qualizeitraum Ende" dataDxfId="107"/>
+    <tableColumn id="7" xr3:uid="{DCC178B3-11FC-4C53-BBC6-C2FDA2C89857}" name="Letzter Wettkampf am" dataDxfId="106"/>
+    <tableColumn id="8" xr3:uid="{2811DB01-60A5-4BE4-B6F9-A806398A602A}" name="Wertung" dataDxfId="105"/>
+    <tableColumn id="9" xr3:uid="{0C16DAFE-847D-4E9E-9604-3A7D9FE924D0}" name="Landesverband" dataDxfId="104"/>
+    <tableColumn id="10" xr3:uid="{7A8A4101-A553-4BD5-9116-9AA5876B9401}" name="OMS" dataDxfId="103"/>
+    <tableColumn id="11" xr3:uid="{9807C9BD-6499-45F6-ACE0-4D13D64EF675}" name="Pool-Länge" dataDxfId="102"/>
+    <tableColumn id="12" xr3:uid="{13D336DD-650F-4F2C-836F-361CA1528F6D}" name="Regelwerk" dataDxfId="101"/>
+    <tableColumn id="13" xr3:uid="{66660E2D-ADF2-4FB5-8A13-004F826EE908}" name="Referenz" dataDxfId="100"/>
+    <tableColumn id="19" xr3:uid="{D72EDF8B-ECC3-4FF7-ABE6-B60BCE4A5E26}" name="Referenz Jahr" dataDxfId="99"/>
+    <tableColumn id="20" xr3:uid="{7B18E667-70F7-4BC1-AB1B-21C019F2AA89}" name="Mindest Punktzahl" dataDxfId="98"/>
+    <tableColumn id="21" xr3:uid="{FC185946-681B-42A6-AB1A-FC1EABB668C5}" name="Mindest Disziplinen" dataDxfId="97"/>
+    <tableColumn id="14" xr3:uid="{6A2676FD-2EC7-4C41-A35E-A1597A38F932}" name="3-Kampf Regel" dataDxfId="96"/>
+    <tableColumn id="15" xr3:uid="{718E0917-4F83-4A2B-832F-EBB16D5E21BF}" name="Anzahl Nominierte" dataDxfId="95"/>
+    <tableColumn id="16" xr3:uid="{5C66A461-D647-4E00-A81C-FD7AD44D7CC2}" name="Anzahl Nachrücker" dataDxfId="94"/>
+    <tableColumn id="17" xr3:uid="{D434BDEC-293B-4B4E-A5E9-479438960A03}" name="Seiten Anzahl" dataDxfId="93"/>
+    <tableColumn id="18" xr3:uid="{80908229-9247-473F-81C0-9C9D4C12FF06}" name="Absagen" dataDxfId="92"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{16F87202-5A6A-4E2F-B973-3CE7EC2566C1}" name="DEM_konfig" displayName="DEM_konfig" ref="A1:X7" totalsRowShown="0" headerRowDxfId="77" dataDxfId="76">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{16F87202-5A6A-4E2F-B973-3CE7EC2566C1}" name="DEM_konfig" displayName="DEM_konfig" ref="A1:X7" totalsRowShown="0" headerRowDxfId="91" dataDxfId="90">
   <autoFilter ref="A1:X7" xr:uid="{16F87202-5A6A-4E2F-B973-3CE7EC2566C1}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -4464,37 +4585,37 @@
     <filterColumn colId="23" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="24">
-    <tableColumn id="1" xr3:uid="{4847B567-64E1-4AC3-8C4B-EFCF3F00CC6C}" name="Tabellen Name" dataDxfId="75"/>
-    <tableColumn id="2" xr3:uid="{6346FF3B-B334-4CD8-8B23-F2347E29C536}" name="Geschlecht" dataDxfId="74"/>
-    <tableColumn id="3" xr3:uid="{E793B48A-BC8A-439F-8AAF-6FD08104A619}" name="Mindest Alter" dataDxfId="73"/>
-    <tableColumn id="4" xr3:uid="{01A62C29-2F75-4107-A431-F69230BCCD0C}" name="Maximales Alter" dataDxfId="72"/>
-    <tableColumn id="5" xr3:uid="{B7E4DE90-7856-4A0C-9063-61414D7F227C}" name="Qualizeitraum anfang" dataDxfId="71"/>
-    <tableColumn id="6" xr3:uid="{B00F7CD1-82CB-42B9-A396-89F79EF419CA}" name="Qualizeitraum Ende" dataDxfId="70"/>
-    <tableColumn id="7" xr3:uid="{9E50DDE5-12E3-4BCB-801C-FBABCE309F0E}" name="Letzter Wettkampf am" dataDxfId="69"/>
-    <tableColumn id="8" xr3:uid="{57E68247-0FF2-48D8-8ACD-AB057E576A21}" name="Landesverband" dataDxfId="68"/>
-    <tableColumn id="9" xr3:uid="{EBAA439D-F69A-4C2A-8193-9AE08F1E57B8}" name="OMS" dataDxfId="67"/>
-    <tableColumn id="10" xr3:uid="{BBD11E7F-3DDF-428A-B005-4A40E6FA78DC}" name="Pool-Länge" dataDxfId="66"/>
-    <tableColumn id="11" xr3:uid="{6AE38DCA-A084-4F3D-A6A4-4E76E3E2CBC6}" name="Regelwerk" dataDxfId="65"/>
-    <tableColumn id="12" xr3:uid="{7F7470AD-5502-4CEE-BB4C-44BA308E61D7}" name="Seiten Anzahl" dataDxfId="64"/>
-    <tableColumn id="13" xr3:uid="{F416CBFA-4C9D-45CD-9BA7-E4BC57A08BC2}" name="PZ1 - 50m Retten" dataDxfId="63"/>
-    <tableColumn id="14" xr3:uid="{7117DBCA-0DA7-462C-84FE-0DC7E33B124C}" name="PZ1 - 100m Retten" dataDxfId="62"/>
-    <tableColumn id="15" xr3:uid="{E8630E91-DC30-4822-9E53-6D65487C3670}" name="PZ1 - 100m Kombi" dataDxfId="61"/>
-    <tableColumn id="16" xr3:uid="{4B3AA225-E042-430F-8259-D176887B4528}" name="PZ1 - 100m Lifesaver" dataDxfId="60"/>
-    <tableColumn id="17" xr3:uid="{798674BD-98CE-4531-BDFF-6AB06253AD7C}" name="PZ1 - 200m Super-Lifesaver" dataDxfId="59"/>
-    <tableColumn id="18" xr3:uid="{8809BB71-D58B-4E8B-A442-D0EB9A65A25D}" name="PZ1 - 200m Hindernis" dataDxfId="58"/>
-    <tableColumn id="19" xr3:uid="{93DCF463-806B-4117-B4E3-1FFAE976B37C}" name="PZ2 - 50m Retten" dataDxfId="57"/>
-    <tableColumn id="20" xr3:uid="{A514C961-559E-462F-B143-BA30974C0129}" name="PZ2 - 100m Retten" dataDxfId="56"/>
-    <tableColumn id="21" xr3:uid="{F1CF6143-45FE-498D-93D6-36F26D2F3C0B}" name="PZ2 - 100m Kombi" dataDxfId="55"/>
-    <tableColumn id="22" xr3:uid="{E90962FC-C214-467F-841F-40DF60E41456}" name="PZ2 - 100m Lifesaver" dataDxfId="54"/>
-    <tableColumn id="23" xr3:uid="{7FBC6334-C4C8-4B38-9F59-30ED95A44379}" name="PZ2 - 200m Super-Lifesaver" dataDxfId="53"/>
-    <tableColumn id="24" xr3:uid="{231BFF86-8F3A-4BA1-B25E-28175D9EDFA9}" name="PZ2 - 200m Hindernis" dataDxfId="52"/>
+    <tableColumn id="1" xr3:uid="{4847B567-64E1-4AC3-8C4B-EFCF3F00CC6C}" name="Tabellen Name" dataDxfId="89"/>
+    <tableColumn id="2" xr3:uid="{6346FF3B-B334-4CD8-8B23-F2347E29C536}" name="Geschlecht" dataDxfId="88"/>
+    <tableColumn id="3" xr3:uid="{E793B48A-BC8A-439F-8AAF-6FD08104A619}" name="Mindest Alter" dataDxfId="87"/>
+    <tableColumn id="4" xr3:uid="{01A62C29-2F75-4107-A431-F69230BCCD0C}" name="Maximales Alter" dataDxfId="86"/>
+    <tableColumn id="5" xr3:uid="{B7E4DE90-7856-4A0C-9063-61414D7F227C}" name="Qualizeitraum anfang" dataDxfId="85"/>
+    <tableColumn id="6" xr3:uid="{B00F7CD1-82CB-42B9-A396-89F79EF419CA}" name="Qualizeitraum Ende" dataDxfId="84"/>
+    <tableColumn id="7" xr3:uid="{9E50DDE5-12E3-4BCB-801C-FBABCE309F0E}" name="Letzter Wettkampf am" dataDxfId="83"/>
+    <tableColumn id="8" xr3:uid="{57E68247-0FF2-48D8-8ACD-AB057E576A21}" name="Landesverband" dataDxfId="82"/>
+    <tableColumn id="9" xr3:uid="{EBAA439D-F69A-4C2A-8193-9AE08F1E57B8}" name="OMS" dataDxfId="81"/>
+    <tableColumn id="10" xr3:uid="{BBD11E7F-3DDF-428A-B005-4A40E6FA78DC}" name="Pool-Länge" dataDxfId="80"/>
+    <tableColumn id="11" xr3:uid="{6AE38DCA-A084-4F3D-A6A4-4E76E3E2CBC6}" name="Regelwerk" dataDxfId="79"/>
+    <tableColumn id="12" xr3:uid="{7F7470AD-5502-4CEE-BB4C-44BA308E61D7}" name="Seiten Anzahl" dataDxfId="78"/>
+    <tableColumn id="13" xr3:uid="{F416CBFA-4C9D-45CD-9BA7-E4BC57A08BC2}" name="PZ1 - 50m Retten" dataDxfId="77"/>
+    <tableColumn id="14" xr3:uid="{7117DBCA-0DA7-462C-84FE-0DC7E33B124C}" name="PZ1 - 100m Retten" dataDxfId="76"/>
+    <tableColumn id="15" xr3:uid="{E8630E91-DC30-4822-9E53-6D65487C3670}" name="PZ1 - 100m Kombi" dataDxfId="75"/>
+    <tableColumn id="16" xr3:uid="{4B3AA225-E042-430F-8259-D176887B4528}" name="PZ1 - 100m Lifesaver" dataDxfId="74"/>
+    <tableColumn id="17" xr3:uid="{798674BD-98CE-4531-BDFF-6AB06253AD7C}" name="PZ1 - 200m Super-Lifesaver" dataDxfId="73"/>
+    <tableColumn id="18" xr3:uid="{8809BB71-D58B-4E8B-A442-D0EB9A65A25D}" name="PZ1 - 200m Hindernis" dataDxfId="72"/>
+    <tableColumn id="19" xr3:uid="{93DCF463-806B-4117-B4E3-1FFAE976B37C}" name="PZ2 - 50m Retten" dataDxfId="71"/>
+    <tableColumn id="20" xr3:uid="{A514C961-559E-462F-B143-BA30974C0129}" name="PZ2 - 100m Retten" dataDxfId="70"/>
+    <tableColumn id="21" xr3:uid="{F1CF6143-45FE-498D-93D6-36F26D2F3C0B}" name="PZ2 - 100m Kombi" dataDxfId="69"/>
+    <tableColumn id="22" xr3:uid="{E90962FC-C214-467F-841F-40DF60E41456}" name="PZ2 - 100m Lifesaver" dataDxfId="68"/>
+    <tableColumn id="23" xr3:uid="{7FBC6334-C4C8-4B38-9F59-30ED95A44379}" name="PZ2 - 200m Super-Lifesaver" dataDxfId="67"/>
+    <tableColumn id="24" xr3:uid="{231BFF86-8F3A-4BA1-B25E-28175D9EDFA9}" name="PZ2 - 200m Hindernis" dataDxfId="66"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D7CDEF11-F813-469D-9DE0-678961AB7005}" name="JRP_konfig" displayName="JRP_konfig" ref="A1:X3" totalsRowShown="0" headerRowDxfId="51" dataDxfId="50">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D7CDEF11-F813-469D-9DE0-678961AB7005}" name="JRP_konfig" displayName="JRP_konfig" ref="A1:X3" totalsRowShown="0" headerRowDxfId="65" dataDxfId="64">
   <autoFilter ref="A1:X3" xr:uid="{D7CDEF11-F813-469D-9DE0-678961AB7005}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -4522,58 +4643,71 @@
     <filterColumn colId="23" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="24">
-    <tableColumn id="1" xr3:uid="{021DA6E1-2C93-4474-9720-B6F016186D61}" name="Tabellen Name" dataDxfId="49"/>
-    <tableColumn id="2" xr3:uid="{733C1722-A9C9-4830-A9E2-FE62E96BCD98}" name="Geschlecht" dataDxfId="48"/>
-    <tableColumn id="3" xr3:uid="{80C0BF46-0E43-4947-BF86-B808C324772A}" name="Mindest Alter" dataDxfId="47"/>
-    <tableColumn id="4" xr3:uid="{DBA2A923-EEB7-43F9-A1A3-E78624448FB9}" name="Maximales Alter" dataDxfId="46"/>
-    <tableColumn id="5" xr3:uid="{3FDEE18A-328D-45AE-907D-69A916A93345}" name="Qualizeitraum anfang" dataDxfId="45"/>
-    <tableColumn id="6" xr3:uid="{BE002D7F-575F-4B60-9251-C71D93F59045}" name="Qualizeitraum Ende" dataDxfId="44"/>
-    <tableColumn id="7" xr3:uid="{208ABD57-DE4B-41D6-B9FC-93F2D8966E8D}" name="Letzter Wettkampf am" dataDxfId="43"/>
-    <tableColumn id="8" xr3:uid="{30C9697C-6550-4996-ADDB-7FEE5325B794}" name="Landesverband" dataDxfId="42"/>
-    <tableColumn id="9" xr3:uid="{ED2DAB77-EF46-4D8B-B8E4-90412E32E277}" name="OMS" dataDxfId="41"/>
-    <tableColumn id="10" xr3:uid="{AD534940-A91B-4A6E-9606-E3F3E517D401}" name="Pool-Länge" dataDxfId="40"/>
-    <tableColumn id="11" xr3:uid="{11F9D5D5-72FE-42CA-8624-01D513B4140F}" name="Regelwerk" dataDxfId="39"/>
-    <tableColumn id="12" xr3:uid="{3907872B-5438-4FBF-A045-3EF9EAACFC47}" name="Seiten Anzahl" dataDxfId="38"/>
-    <tableColumn id="13" xr3:uid="{FC821324-3638-40C0-BA1E-069B44E23C7A}" name="PZ1 - 50m Retten" dataDxfId="37"/>
-    <tableColumn id="14" xr3:uid="{70529619-443E-40D3-88C1-3E0F00BB2A50}" name="PZ1 - 100m Retten" dataDxfId="36"/>
-    <tableColumn id="15" xr3:uid="{EFA92FD2-C23F-42B3-83DC-5036513F19AF}" name="PZ1 - 100m Kombi" dataDxfId="35"/>
-    <tableColumn id="16" xr3:uid="{03309E52-8CF3-4E90-9EE6-A818901C3B32}" name="PZ1 - 100m Lifesaver" dataDxfId="34"/>
-    <tableColumn id="17" xr3:uid="{00B22013-AA11-4C17-9250-22060AE4B0A8}" name="PZ1 - 200m Super-Lifesaver" dataDxfId="33"/>
-    <tableColumn id="18" xr3:uid="{7E3508A9-0422-4561-A23E-53E613259B24}" name="PZ1 - 200m Hindernis" dataDxfId="32"/>
-    <tableColumn id="19" xr3:uid="{5CEA435F-F34B-4D8D-88D0-F5EBFF18B713}" name="PZ2 - 50m Retten" dataDxfId="31"/>
-    <tableColumn id="20" xr3:uid="{8585BE62-F7C4-4D5D-B287-052B43B08610}" name="PZ2 - 100m Retten" dataDxfId="30"/>
-    <tableColumn id="21" xr3:uid="{D981758B-ADAD-4E36-B787-0B0FDA808CA2}" name="PZ2 - 100m Kombi" dataDxfId="29"/>
-    <tableColumn id="22" xr3:uid="{1D4970A8-D22F-4962-934C-AEA295ED687A}" name="PZ2 - 100m Lifesaver" dataDxfId="28"/>
-    <tableColumn id="23" xr3:uid="{BE394430-C58F-4690-9615-44475E5AF9F8}" name="PZ2 - 200m Super-Lifesaver" dataDxfId="27"/>
-    <tableColumn id="24" xr3:uid="{A7036B1A-99CE-4F7C-AAB8-12E8B2696202}" name="PZ2 - 200m Hindernis" dataDxfId="26"/>
+    <tableColumn id="1" xr3:uid="{021DA6E1-2C93-4474-9720-B6F016186D61}" name="Tabellen Name" dataDxfId="63"/>
+    <tableColumn id="2" xr3:uid="{733C1722-A9C9-4830-A9E2-FE62E96BCD98}" name="Geschlecht" dataDxfId="62"/>
+    <tableColumn id="3" xr3:uid="{80C0BF46-0E43-4947-BF86-B808C324772A}" name="Mindest Alter" dataDxfId="61"/>
+    <tableColumn id="4" xr3:uid="{DBA2A923-EEB7-43F9-A1A3-E78624448FB9}" name="Maximales Alter" dataDxfId="60"/>
+    <tableColumn id="5" xr3:uid="{3FDEE18A-328D-45AE-907D-69A916A93345}" name="Qualizeitraum anfang" dataDxfId="59"/>
+    <tableColumn id="6" xr3:uid="{BE002D7F-575F-4B60-9251-C71D93F59045}" name="Qualizeitraum Ende" dataDxfId="58"/>
+    <tableColumn id="7" xr3:uid="{208ABD57-DE4B-41D6-B9FC-93F2D8966E8D}" name="Letzter Wettkampf am" dataDxfId="57"/>
+    <tableColumn id="8" xr3:uid="{30C9697C-6550-4996-ADDB-7FEE5325B794}" name="Landesverband" dataDxfId="56"/>
+    <tableColumn id="9" xr3:uid="{ED2DAB77-EF46-4D8B-B8E4-90412E32E277}" name="OMS" dataDxfId="55"/>
+    <tableColumn id="10" xr3:uid="{AD534940-A91B-4A6E-9606-E3F3E517D401}" name="Pool-Länge" dataDxfId="54"/>
+    <tableColumn id="11" xr3:uid="{11F9D5D5-72FE-42CA-8624-01D513B4140F}" name="Regelwerk" dataDxfId="53"/>
+    <tableColumn id="12" xr3:uid="{3907872B-5438-4FBF-A045-3EF9EAACFC47}" name="Seiten Anzahl" dataDxfId="52"/>
+    <tableColumn id="13" xr3:uid="{FC821324-3638-40C0-BA1E-069B44E23C7A}" name="PZ1 - 50m Retten" dataDxfId="51"/>
+    <tableColumn id="14" xr3:uid="{70529619-443E-40D3-88C1-3E0F00BB2A50}" name="PZ1 - 100m Retten" dataDxfId="50"/>
+    <tableColumn id="15" xr3:uid="{EFA92FD2-C23F-42B3-83DC-5036513F19AF}" name="PZ1 - 100m Kombi" dataDxfId="49"/>
+    <tableColumn id="16" xr3:uid="{03309E52-8CF3-4E90-9EE6-A818901C3B32}" name="PZ1 - 100m Lifesaver" dataDxfId="48"/>
+    <tableColumn id="17" xr3:uid="{00B22013-AA11-4C17-9250-22060AE4B0A8}" name="PZ1 - 200m Super-Lifesaver" dataDxfId="47"/>
+    <tableColumn id="18" xr3:uid="{7E3508A9-0422-4561-A23E-53E613259B24}" name="PZ1 - 200m Hindernis" dataDxfId="46"/>
+    <tableColumn id="19" xr3:uid="{5CEA435F-F34B-4D8D-88D0-F5EBFF18B713}" name="PZ2 - 50m Retten" dataDxfId="45"/>
+    <tableColumn id="20" xr3:uid="{8585BE62-F7C4-4D5D-B287-052B43B08610}" name="PZ2 - 100m Retten" dataDxfId="44"/>
+    <tableColumn id="21" xr3:uid="{D981758B-ADAD-4E36-B787-0B0FDA808CA2}" name="PZ2 - 100m Kombi" dataDxfId="43"/>
+    <tableColumn id="22" xr3:uid="{1D4970A8-D22F-4962-934C-AEA295ED687A}" name="PZ2 - 100m Lifesaver" dataDxfId="42"/>
+    <tableColumn id="23" xr3:uid="{BE394430-C58F-4690-9615-44475E5AF9F8}" name="PZ2 - 200m Super-Lifesaver" dataDxfId="41"/>
+    <tableColumn id="24" xr3:uid="{A7036B1A-99CE-4F7C-AAB8-12E8B2696202}" name="PZ2 - 200m Hindernis" dataDxfId="40"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{FED162EE-531E-453F-8C25-562B59ECE709}" name="LK_konfig" displayName="LK_konfig" ref="A1:S37" totalsRowShown="0" headerRowDxfId="222" dataDxfId="221">
-  <autoFilter ref="A1:S37" xr:uid="{FED162EE-531E-453F-8C25-562B59ECE709}"/>
-  <tableColumns count="19">
-    <tableColumn id="1" xr3:uid="{F985A4F0-6B8C-47C6-816F-1A31A4973EB2}" name="Tabellen Name" dataDxfId="220"/>
-    <tableColumn id="2" xr3:uid="{5E5AD859-71A2-4E8E-B434-431A89C05C57}" name="Geschlecht" dataDxfId="219"/>
-    <tableColumn id="3" xr3:uid="{85BB892C-E151-404B-8974-FC5199E0909C}" name="Mindest Alter" dataDxfId="218"/>
-    <tableColumn id="4" xr3:uid="{790F6CF9-E475-4082-AE03-D30EDE22FB61}" name="Maximales Alter" dataDxfId="217"/>
-    <tableColumn id="5" xr3:uid="{FD4B0E6E-9B64-4731-A50F-D3CE3A4ED3FC}" name="Qualizeitraum anfang" dataDxfId="216"/>
-    <tableColumn id="6" xr3:uid="{5E84CAD2-C403-49B9-BB06-D56EC5784C8C}" name="Qualizeitraum Ende" dataDxfId="215"/>
-    <tableColumn id="7" xr3:uid="{6323F8E2-5DA4-4E5B-9C35-1E8C219ADECF}" name="Letzter Wettkampf am" dataDxfId="214"/>
-    <tableColumn id="8" xr3:uid="{D2845930-152E-432F-92A0-E7F7A3EE1FF0}" name="Landesverband" dataDxfId="213"/>
-    <tableColumn id="9" xr3:uid="{87046373-5CCD-41EC-B34C-C753E71FD26C}" name="OMS" dataDxfId="212"/>
-    <tableColumn id="10" xr3:uid="{A685FE01-F23C-4533-B399-857F5A1F6C37}" name="Pool-Länge" dataDxfId="211"/>
-    <tableColumn id="11" xr3:uid="{11E0A508-0C9D-4CB6-952E-7FAC5D05BDCD}" name="Regelwerk" dataDxfId="210"/>
-    <tableColumn id="12" xr3:uid="{F220BD5F-C3B5-4935-996A-BFCDF9F392D9}" name="Seiten Anzahl" dataDxfId="209"/>
-    <tableColumn id="25" xr3:uid="{7CDE58FE-A5B8-4329-9F48-3913AEBA21FC}" name="mind. erreichte Normen" dataDxfId="208"/>
-    <tableColumn id="13" xr3:uid="{A0A5E62D-9354-426D-9A08-13E43F36F55B}" name="PZ - 50m Retten" dataDxfId="207"/>
-    <tableColumn id="14" xr3:uid="{5D70F54C-57E9-45E2-BC99-0DBB0422383E}" name="PZ - 100m Retten" dataDxfId="206"/>
-    <tableColumn id="15" xr3:uid="{1C0CF5DB-156E-4813-A8BA-9EA29A40ABF3}" name="PZ - 100m Kombi" dataDxfId="205"/>
-    <tableColumn id="16" xr3:uid="{691CD4E1-13D9-4455-A2D1-14C9BC41A0EA}" name="PZ - 100m Lifesaver" dataDxfId="204"/>
-    <tableColumn id="17" xr3:uid="{CE1BA235-770B-4FA4-B327-187675DDA6B8}" name="PZ - 200m Super-Lifesaver" dataDxfId="203"/>
-    <tableColumn id="18" xr3:uid="{A326EF87-5FF5-4042-85D3-7806FEED4CFA}" name="PZ - 200m Hindernis" dataDxfId="202"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{FED162EE-531E-453F-8C25-562B59ECE709}" name="LK_konfig" displayName="LK_konfig" ref="A1:AF37" totalsRowShown="0" headerRowDxfId="235" dataDxfId="234">
+  <autoFilter ref="A1:AF37" xr:uid="{FED162EE-531E-453F-8C25-562B59ECE709}"/>
+  <tableColumns count="32">
+    <tableColumn id="1" xr3:uid="{F985A4F0-6B8C-47C6-816F-1A31A4973EB2}" name="Tabellen Name" dataDxfId="233"/>
+    <tableColumn id="2" xr3:uid="{5E5AD859-71A2-4E8E-B434-431A89C05C57}" name="Geschlecht" dataDxfId="232"/>
+    <tableColumn id="3" xr3:uid="{85BB892C-E151-404B-8974-FC5199E0909C}" name="Mindest Alter" dataDxfId="231"/>
+    <tableColumn id="4" xr3:uid="{790F6CF9-E475-4082-AE03-D30EDE22FB61}" name="Maximales Alter" dataDxfId="230"/>
+    <tableColumn id="5" xr3:uid="{FD4B0E6E-9B64-4731-A50F-D3CE3A4ED3FC}" name="Qualizeitraum anfang" dataDxfId="229"/>
+    <tableColumn id="6" xr3:uid="{5E84CAD2-C403-49B9-BB06-D56EC5784C8C}" name="Qualizeitraum Ende" dataDxfId="228"/>
+    <tableColumn id="7" xr3:uid="{6323F8E2-5DA4-4E5B-9C35-1E8C219ADECF}" name="Letzter Wettkampf am" dataDxfId="227"/>
+    <tableColumn id="8" xr3:uid="{D2845930-152E-432F-92A0-E7F7A3EE1FF0}" name="Landesverband" dataDxfId="226"/>
+    <tableColumn id="9" xr3:uid="{87046373-5CCD-41EC-B34C-C753E71FD26C}" name="OMS" dataDxfId="225"/>
+    <tableColumn id="10" xr3:uid="{A685FE01-F23C-4533-B399-857F5A1F6C37}" name="Pool-Länge" dataDxfId="224"/>
+    <tableColumn id="11" xr3:uid="{11E0A508-0C9D-4CB6-952E-7FAC5D05BDCD}" name="Regelwerk" dataDxfId="223"/>
+    <tableColumn id="12" xr3:uid="{F220BD5F-C3B5-4935-996A-BFCDF9F392D9}" name="Seiten Anzahl" dataDxfId="222"/>
+    <tableColumn id="25" xr3:uid="{7CDE58FE-A5B8-4329-9F48-3913AEBA21FC}" name="mind. erreichte Normen" dataDxfId="221"/>
+    <tableColumn id="13" xr3:uid="{A0A5E62D-9354-426D-9A08-13E43F36F55B}" name="PZ - 50m Retten" dataDxfId="220"/>
+    <tableColumn id="14" xr3:uid="{5D70F54C-57E9-45E2-BC99-0DBB0422383E}" name="PZ - 100m Retten" dataDxfId="219"/>
+    <tableColumn id="15" xr3:uid="{1C0CF5DB-156E-4813-A8BA-9EA29A40ABF3}" name="PZ - 100m Kombi" dataDxfId="218"/>
+    <tableColumn id="16" xr3:uid="{691CD4E1-13D9-4455-A2D1-14C9BC41A0EA}" name="PZ - 100m Lifesaver" dataDxfId="217"/>
+    <tableColumn id="17" xr3:uid="{CE1BA235-770B-4FA4-B327-187675DDA6B8}" name="PZ - 200m Super-Lifesaver" dataDxfId="216"/>
+    <tableColumn id="18" xr3:uid="{A326EF87-5FF5-4042-85D3-7806FEED4CFA}" name="PZ - 200m Hindernis" dataDxfId="13"/>
+    <tableColumn id="19" xr3:uid="{3F3DF994-C8AE-408C-BCA1-99A143BA81D4}" name="LMS" dataDxfId="12"/>
+    <tableColumn id="20" xr3:uid="{7461FBF0-E903-4B09-9C11-C9C1047FA39D}" name="DMM" dataDxfId="11"/>
+    <tableColumn id="21" xr3:uid="{675AEE5F-BEC3-499A-A337-72DD69B663E7}" name="DEM" dataDxfId="10"/>
+    <tableColumn id="24" xr3:uid="{17E128CD-0800-40BC-B850-0CE3966127B2}" name="JRP" dataDxfId="9"/>
+    <tableColumn id="22" xr3:uid="{A92C8C64-1269-48FF-8F43-8EF273E7864F}" name="DMO" dataDxfId="8"/>
+    <tableColumn id="30" xr3:uid="{84286FAC-A077-44AC-889C-09543C869BF4}" name="DMO Ocean" dataDxfId="7"/>
+    <tableColumn id="23" xr3:uid="{40EF7D68-4E22-4866-ADAA-28DC8A82A09C}" name="Trophy" dataDxfId="6"/>
+    <tableColumn id="31" xr3:uid="{33F8EB16-27F6-453C-81FD-376213F45978}" name="Ocean Perf" dataDxfId="5"/>
+    <tableColumn id="32" xr3:uid="{5B81C846-FAFA-4E74-8678-47219E5942AF}" name="Filcow" dataDxfId="4"/>
+    <tableColumn id="26" xr3:uid="{C7421A01-D221-4C7A-9F0B-8BD025E0F1CF}" name="WM" dataDxfId="3"/>
+    <tableColumn id="27" xr3:uid="{4050AB9D-D7D4-4B88-8218-9206C91AD9A0}" name="EM" dataDxfId="2"/>
+    <tableColumn id="28" xr3:uid="{6FC272EA-276B-4249-818D-C220B87D52A6}" name="JWM" dataDxfId="1"/>
+    <tableColumn id="29" xr3:uid="{51F99A1A-8D2C-444F-9E7C-AA537C8FFA08}" name="JEM" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4583,12 +4717,12 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{888CE7BE-8313-44C0-AE38-83992EABD44D}" name="LK_Kalender" displayName="LK_Kalender" ref="A1:H8" totalsRowShown="0">
   <autoFilter ref="A1:H8" xr:uid="{888CE7BE-8313-44C0-AE38-83992EABD44D}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{B26B9E90-F378-41EF-B35E-CE240017E4BE}" name="datum von" dataDxfId="25"/>
+    <tableColumn id="1" xr3:uid="{B26B9E90-F378-41EF-B35E-CE240017E4BE}" name="datum von" dataDxfId="39"/>
     <tableColumn id="2" xr3:uid="{38211212-0A92-428C-895C-E4CA68F52818}" name="datum bis"/>
-    <tableColumn id="3" xr3:uid="{66E541C6-0A5E-4B2D-9B89-5E52F449A4A6}" name="uhrzeit von" dataDxfId="24"/>
-    <tableColumn id="4" xr3:uid="{D93C06A2-29AD-4073-8E3C-A685B4474CC8}" name="uhrzeit bis" dataDxfId="23"/>
-    <tableColumn id="5" xr3:uid="{C5C3979C-B528-44E8-A5A6-36F020A6034F}" name="titel" dataDxfId="22"/>
-    <tableColumn id="6" xr3:uid="{9DC09E1D-44FD-40ED-9EBE-86A8E61C38B2}" name="meta" dataDxfId="21"/>
+    <tableColumn id="3" xr3:uid="{66E541C6-0A5E-4B2D-9B89-5E52F449A4A6}" name="uhrzeit von" dataDxfId="38"/>
+    <tableColumn id="4" xr3:uid="{D93C06A2-29AD-4073-8E3C-A685B4474CC8}" name="uhrzeit bis" dataDxfId="37"/>
+    <tableColumn id="5" xr3:uid="{C5C3979C-B528-44E8-A5A6-36F020A6034F}" name="titel" dataDxfId="36"/>
+    <tableColumn id="6" xr3:uid="{9DC09E1D-44FD-40ED-9EBE-86A8E61C38B2}" name="meta" dataDxfId="35"/>
     <tableColumn id="7" xr3:uid="{E7E62A34-7A76-4361-937D-F4DE76E6E7CC}" name="ort"/>
     <tableColumn id="8" xr3:uid="{84F02734-FC16-406B-ACCA-0CCDF547D94C}" name="kader"/>
   </tableColumns>
@@ -8530,52 +8664,52 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B5:G31">
-    <cfRule type="expression" dxfId="20" priority="15">
+    <cfRule type="expression" dxfId="34" priority="15">
       <formula>B5&lt;&gt;B4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H5:M31">
-    <cfRule type="expression" dxfId="19" priority="14">
+    <cfRule type="expression" dxfId="33" priority="14">
       <formula>H5&lt;&gt;H4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N5:S31">
-    <cfRule type="expression" dxfId="18" priority="13">
+    <cfRule type="expression" dxfId="32" priority="13">
       <formula>N5&lt;&gt;N4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="T5:Y31">
-    <cfRule type="expression" dxfId="17" priority="12">
+    <cfRule type="expression" dxfId="31" priority="12">
       <formula>T5&lt;&gt;T4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z5:AE31">
-    <cfRule type="expression" dxfId="16" priority="9">
+    <cfRule type="expression" dxfId="30" priority="9">
       <formula>Z5&lt;&gt;Z4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AF5:AK31">
-    <cfRule type="expression" dxfId="15" priority="8">
+    <cfRule type="expression" dxfId="29" priority="8">
       <formula>AF5&lt;&gt;AF4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AL5:AN31">
-    <cfRule type="expression" dxfId="14" priority="6">
+    <cfRule type="expression" dxfId="28" priority="6">
       <formula>AL5&lt;&gt;AL4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AO5:AQ31">
-    <cfRule type="expression" dxfId="13" priority="5">
+    <cfRule type="expression" dxfId="27" priority="5">
       <formula>AO5&lt;&gt;AO4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AR5:AT31">
-    <cfRule type="expression" dxfId="12" priority="2">
+    <cfRule type="expression" dxfId="26" priority="2">
       <formula>AR5&lt;&gt;AR4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AU5:AW31">
-    <cfRule type="expression" dxfId="11" priority="1">
+    <cfRule type="expression" dxfId="25" priority="1">
       <formula>AU5&lt;&gt;AU4</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8797,7 +8931,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:H8">
-    <cfRule type="expression" dxfId="0" priority="1">
+    <cfRule type="expression" dxfId="14" priority="1">
       <formula>$A2&lt;TODAY()</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9803,22 +9937,22 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B6:G6">
-    <cfRule type="expression" dxfId="10" priority="20">
+    <cfRule type="expression" dxfId="24" priority="20">
       <formula>B6&lt;&gt;B4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7:G32">
-    <cfRule type="expression" dxfId="9" priority="1">
+    <cfRule type="expression" dxfId="23" priority="1">
       <formula>B7&lt;&gt;B6</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H6:M6">
-    <cfRule type="expression" dxfId="8" priority="22">
+    <cfRule type="expression" dxfId="22" priority="22">
       <formula>H6&lt;&gt;H4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H7:M32">
-    <cfRule type="expression" dxfId="7" priority="2">
+    <cfRule type="expression" dxfId="21" priority="2">
       <formula>H7&lt;&gt;H6</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11149,22 +11283,22 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B6:G6">
-    <cfRule type="expression" dxfId="6" priority="19">
+    <cfRule type="expression" dxfId="20" priority="19">
       <formula>B6&lt;&gt;B4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7:G32">
-    <cfRule type="expression" dxfId="5" priority="2">
+    <cfRule type="expression" dxfId="19" priority="2">
       <formula>B7&lt;&gt;B6</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H6:M6">
-    <cfRule type="expression" dxfId="4" priority="20">
+    <cfRule type="expression" dxfId="18" priority="20">
       <formula>H6&lt;&gt;H4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H7:M32">
-    <cfRule type="expression" dxfId="3" priority="1">
+    <cfRule type="expression" dxfId="17" priority="1">
       <formula>H7&lt;&gt;H6</formula>
     </cfRule>
   </conditionalFormatting>
@@ -12659,7 +12793,7 @@
   <sheetPr>
     <tabColor theme="5" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="A1:S37"/>
+  <dimension ref="A1:AF37"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="17.3984375" bestFit="1" customWidth="1"/>
@@ -12683,7 +12817,7 @@
     <col min="19" max="19" width="19.86328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A1" s="25" t="s">
         <v>127</v>
       </c>
@@ -12741,8 +12875,47 @@
       <c r="S1" s="25" t="s">
         <v>253</v>
       </c>
+      <c r="T1" s="25" t="s">
+        <v>254</v>
+      </c>
+      <c r="U1" s="25" t="s">
+        <v>255</v>
+      </c>
+      <c r="V1" s="25" t="s">
+        <v>256</v>
+      </c>
+      <c r="W1" s="25" t="s">
+        <v>258</v>
+      </c>
+      <c r="X1" s="25" t="s">
+        <v>263</v>
+      </c>
+      <c r="Y1" s="25" t="s">
+        <v>264</v>
+      </c>
+      <c r="Z1" s="25" t="s">
+        <v>257</v>
+      </c>
+      <c r="AA1" s="25" t="s">
+        <v>265</v>
+      </c>
+      <c r="AB1" s="25" t="s">
+        <v>266</v>
+      </c>
+      <c r="AC1" s="25" t="s">
+        <v>259</v>
+      </c>
+      <c r="AD1" s="25" t="s">
+        <v>260</v>
+      </c>
+      <c r="AE1" s="25" t="s">
+        <v>261</v>
+      </c>
+      <c r="AF1" s="25" t="s">
+        <v>262</v>
+      </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A2" s="25" t="s">
         <v>241</v>
       </c>
@@ -12802,8 +12975,21 @@
         <f>'NK-LK Transf.'!BQ16</f>
         <v>1.9327962962962964E-3</v>
       </c>
+      <c r="T2" s="140"/>
+      <c r="U2" s="140"/>
+      <c r="V2" s="140"/>
+      <c r="W2" s="140"/>
+      <c r="X2" s="140"/>
+      <c r="Y2" s="140"/>
+      <c r="Z2" s="140"/>
+      <c r="AA2" s="140"/>
+      <c r="AB2" s="140"/>
+      <c r="AC2" s="140"/>
+      <c r="AD2" s="140"/>
+      <c r="AE2" s="140"/>
+      <c r="AF2" s="140"/>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A3" s="25" t="s">
         <v>241</v>
       </c>
@@ -12863,8 +13049,21 @@
         <f>'NK-LK Transf.'!BP16</f>
         <v>1.9621597222222223E-3</v>
       </c>
+      <c r="T3" s="140"/>
+      <c r="U3" s="140"/>
+      <c r="V3" s="140"/>
+      <c r="W3" s="140"/>
+      <c r="X3" s="140"/>
+      <c r="Y3" s="140"/>
+      <c r="Z3" s="140"/>
+      <c r="AA3" s="140"/>
+      <c r="AB3" s="140"/>
+      <c r="AC3" s="140"/>
+      <c r="AD3" s="140"/>
+      <c r="AE3" s="140"/>
+      <c r="AF3" s="140"/>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A4" s="25" t="s">
         <v>241</v>
       </c>
@@ -12924,8 +13123,21 @@
         <f>'NK-LK Transf.'!BO16</f>
         <v>1.9916597222222219E-3</v>
       </c>
+      <c r="T4" s="140"/>
+      <c r="U4" s="140"/>
+      <c r="V4" s="140"/>
+      <c r="W4" s="140"/>
+      <c r="X4" s="140"/>
+      <c r="Y4" s="140"/>
+      <c r="Z4" s="140"/>
+      <c r="AA4" s="140"/>
+      <c r="AB4" s="140"/>
+      <c r="AC4" s="140"/>
+      <c r="AD4" s="140"/>
+      <c r="AE4" s="140"/>
+      <c r="AF4" s="140"/>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A5" s="25" t="s">
         <v>233</v>
       </c>
@@ -12985,8 +13197,21 @@
         <f>'NK-LK Transf.'!BE16</f>
         <v>1.8218055555555552E-3</v>
       </c>
+      <c r="T5" s="140"/>
+      <c r="U5" s="140"/>
+      <c r="V5" s="140"/>
+      <c r="W5" s="140"/>
+      <c r="X5" s="140"/>
+      <c r="Y5" s="140"/>
+      <c r="Z5" s="140"/>
+      <c r="AA5" s="140"/>
+      <c r="AB5" s="140"/>
+      <c r="AC5" s="140"/>
+      <c r="AD5" s="140"/>
+      <c r="AE5" s="140"/>
+      <c r="AF5" s="140"/>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A6" s="25" t="s">
         <v>233</v>
       </c>
@@ -13046,8 +13271,21 @@
         <f>'NK-LK Transf.'!BD16</f>
         <v>1.8773611111111109E-3</v>
       </c>
+      <c r="T6" s="140"/>
+      <c r="U6" s="140"/>
+      <c r="V6" s="140"/>
+      <c r="W6" s="140"/>
+      <c r="X6" s="140"/>
+      <c r="Y6" s="140"/>
+      <c r="Z6" s="140"/>
+      <c r="AA6" s="140"/>
+      <c r="AB6" s="140"/>
+      <c r="AC6" s="140"/>
+      <c r="AD6" s="140"/>
+      <c r="AE6" s="140"/>
+      <c r="AF6" s="140"/>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A7" s="25" t="s">
         <v>233</v>
       </c>
@@ -13107,8 +13345,21 @@
         <f>'NK-LK Transf.'!BC16</f>
         <v>1.9152777777777779E-3</v>
       </c>
+      <c r="T7" s="140"/>
+      <c r="U7" s="140"/>
+      <c r="V7" s="140"/>
+      <c r="W7" s="140"/>
+      <c r="X7" s="140"/>
+      <c r="Y7" s="140"/>
+      <c r="Z7" s="140"/>
+      <c r="AA7" s="140"/>
+      <c r="AB7" s="140"/>
+      <c r="AC7" s="140"/>
+      <c r="AD7" s="140"/>
+      <c r="AE7" s="140"/>
+      <c r="AF7" s="140"/>
     </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A8" s="25" t="s">
         <v>240</v>
       </c>
@@ -13168,8 +13419,21 @@
         <f>'NK-LK Transf.'!BV16</f>
         <v>1.8239270833333334E-3</v>
       </c>
+      <c r="T8" s="140"/>
+      <c r="U8" s="140"/>
+      <c r="V8" s="140"/>
+      <c r="W8" s="140"/>
+      <c r="X8" s="140"/>
+      <c r="Y8" s="140"/>
+      <c r="Z8" s="140"/>
+      <c r="AA8" s="140"/>
+      <c r="AB8" s="140"/>
+      <c r="AC8" s="140"/>
+      <c r="AD8" s="140"/>
+      <c r="AE8" s="140"/>
+      <c r="AF8" s="140"/>
     </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A9" s="25" t="s">
         <v>240</v>
       </c>
@@ -13229,8 +13493,21 @@
         <f>'NK-LK Transf.'!BU16</f>
         <v>1.8506041666666666E-3</v>
       </c>
+      <c r="T9" s="140"/>
+      <c r="U9" s="140"/>
+      <c r="V9" s="140"/>
+      <c r="W9" s="140"/>
+      <c r="X9" s="140"/>
+      <c r="Y9" s="140"/>
+      <c r="Z9" s="140"/>
+      <c r="AA9" s="140"/>
+      <c r="AB9" s="140"/>
+      <c r="AC9" s="140"/>
+      <c r="AD9" s="140"/>
+      <c r="AE9" s="140"/>
+      <c r="AF9" s="140"/>
     </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A10" s="25" t="s">
         <v>240</v>
       </c>
@@ -13290,8 +13567,21 @@
         <f>'NK-LK Transf.'!BT16</f>
         <v>1.887166666666667E-3</v>
       </c>
+      <c r="T10" s="140"/>
+      <c r="U10" s="140"/>
+      <c r="V10" s="140"/>
+      <c r="W10" s="140"/>
+      <c r="X10" s="140"/>
+      <c r="Y10" s="140"/>
+      <c r="Z10" s="140"/>
+      <c r="AA10" s="140"/>
+      <c r="AB10" s="140"/>
+      <c r="AC10" s="140"/>
+      <c r="AD10" s="140"/>
+      <c r="AE10" s="140"/>
+      <c r="AF10" s="140"/>
     </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A11" s="25" t="s">
         <v>239</v>
       </c>
@@ -13351,8 +13641,21 @@
         <f>'NK-LK Transf.'!BJ16</f>
         <v>1.6026527777777777E-3</v>
       </c>
+      <c r="T11" s="140"/>
+      <c r="U11" s="140"/>
+      <c r="V11" s="140"/>
+      <c r="W11" s="140"/>
+      <c r="X11" s="140"/>
+      <c r="Y11" s="140"/>
+      <c r="Z11" s="140"/>
+      <c r="AA11" s="140"/>
+      <c r="AB11" s="140"/>
+      <c r="AC11" s="140"/>
+      <c r="AD11" s="140"/>
+      <c r="AE11" s="140"/>
+      <c r="AF11" s="140"/>
     </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A12" s="25" t="s">
         <v>239</v>
       </c>
@@ -13412,8 +13715,21 @@
         <f>'NK-LK Transf.'!BI16</f>
         <v>1.6571620370370373E-3</v>
       </c>
+      <c r="T12" s="140"/>
+      <c r="U12" s="140"/>
+      <c r="V12" s="140"/>
+      <c r="W12" s="140"/>
+      <c r="X12" s="140"/>
+      <c r="Y12" s="140"/>
+      <c r="Z12" s="140"/>
+      <c r="AA12" s="140"/>
+      <c r="AB12" s="140"/>
+      <c r="AC12" s="140"/>
+      <c r="AD12" s="140"/>
+      <c r="AE12" s="140"/>
+      <c r="AF12" s="140"/>
     </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A13" s="25" t="s">
         <v>239</v>
       </c>
@@ -13473,8 +13789,21 @@
         <f>'NK-LK Transf.'!BH16</f>
         <v>1.7049583333333333E-3</v>
       </c>
+      <c r="T13" s="140"/>
+      <c r="U13" s="140"/>
+      <c r="V13" s="140"/>
+      <c r="W13" s="140"/>
+      <c r="X13" s="140"/>
+      <c r="Y13" s="140"/>
+      <c r="Z13" s="140"/>
+      <c r="AA13" s="140"/>
+      <c r="AB13" s="140"/>
+      <c r="AC13" s="140"/>
+      <c r="AD13" s="140"/>
+      <c r="AE13" s="140"/>
+      <c r="AF13" s="140"/>
     </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A14" s="25" t="s">
         <v>222</v>
       </c>
@@ -13536,8 +13865,31 @@
         <f>'NK-LK Transf.'!Q16</f>
         <v>1.637962962962963E-3</v>
       </c>
+      <c r="T14" s="140"/>
+      <c r="U14" s="140"/>
+      <c r="V14" s="140"/>
+      <c r="W14" s="140"/>
+      <c r="X14" s="140" t="s">
+        <v>272</v>
+      </c>
+      <c r="Y14" s="140" t="s">
+        <v>271</v>
+      </c>
+      <c r="Z14" s="140" t="s">
+        <v>274</v>
+      </c>
+      <c r="AA14" s="140"/>
+      <c r="AB14" s="140"/>
+      <c r="AC14" s="140"/>
+      <c r="AD14" s="140"/>
+      <c r="AE14" s="140" t="s">
+        <v>275</v>
+      </c>
+      <c r="AF14" s="140" t="s">
+        <v>275</v>
+      </c>
     </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A15" s="25" t="s">
         <v>222</v>
       </c>
@@ -13599,8 +13951,33 @@
         <f>'NK-LK Transf.'!P16</f>
         <v>1.6628472222222225E-3</v>
       </c>
+      <c r="T15" s="140"/>
+      <c r="U15" s="140" t="s">
+        <v>270</v>
+      </c>
+      <c r="V15" s="140"/>
+      <c r="W15" s="140"/>
+      <c r="X15" s="140" t="s">
+        <v>272</v>
+      </c>
+      <c r="Y15" s="140" t="s">
+        <v>271</v>
+      </c>
+      <c r="Z15" s="140" t="s">
+        <v>274</v>
+      </c>
+      <c r="AA15" s="140"/>
+      <c r="AB15" s="140"/>
+      <c r="AC15" s="140"/>
+      <c r="AD15" s="140"/>
+      <c r="AE15" s="140" t="s">
+        <v>275</v>
+      </c>
+      <c r="AF15" s="140" t="s">
+        <v>275</v>
+      </c>
     </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A16" s="25" t="s">
         <v>222</v>
       </c>
@@ -13662,8 +14039,33 @@
         <f>'NK-LK Transf.'!O16</f>
         <v>1.6878472222222221E-3</v>
       </c>
+      <c r="T16" s="140"/>
+      <c r="U16" s="140" t="s">
+        <v>270</v>
+      </c>
+      <c r="V16" s="140"/>
+      <c r="W16" s="140"/>
+      <c r="X16" s="140" t="s">
+        <v>272</v>
+      </c>
+      <c r="Y16" s="140" t="s">
+        <v>271</v>
+      </c>
+      <c r="Z16" s="140" t="s">
+        <v>274</v>
+      </c>
+      <c r="AA16" s="140"/>
+      <c r="AB16" s="140"/>
+      <c r="AC16" s="140"/>
+      <c r="AD16" s="140"/>
+      <c r="AE16" s="140" t="s">
+        <v>275</v>
+      </c>
+      <c r="AF16" s="140" t="s">
+        <v>275</v>
+      </c>
     </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A17" s="25" t="s">
         <v>220</v>
       </c>
@@ -13725,8 +14127,31 @@
         <f>'NK-LK Transf.'!E16</f>
         <v>1.5181712962962961E-3</v>
       </c>
+      <c r="T17" s="140"/>
+      <c r="U17" s="140"/>
+      <c r="V17" s="140"/>
+      <c r="W17" s="140"/>
+      <c r="X17" s="140" t="s">
+        <v>272</v>
+      </c>
+      <c r="Y17" s="140" t="s">
+        <v>271</v>
+      </c>
+      <c r="Z17" s="140" t="s">
+        <v>274</v>
+      </c>
+      <c r="AA17" s="140"/>
+      <c r="AB17" s="140"/>
+      <c r="AC17" s="140"/>
+      <c r="AD17" s="140"/>
+      <c r="AE17" s="140" t="s">
+        <v>275</v>
+      </c>
+      <c r="AF17" s="140" t="s">
+        <v>275</v>
+      </c>
     </row>
-    <row r="18" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A18" s="25" t="s">
         <v>220</v>
       </c>
@@ -13788,8 +14213,33 @@
         <f>'NK-LK Transf.'!D16</f>
         <v>1.5644675925925923E-3</v>
       </c>
+      <c r="T18" s="140"/>
+      <c r="U18" s="140" t="s">
+        <v>270</v>
+      </c>
+      <c r="V18" s="140"/>
+      <c r="W18" s="140"/>
+      <c r="X18" s="140" t="s">
+        <v>272</v>
+      </c>
+      <c r="Y18" s="140" t="s">
+        <v>271</v>
+      </c>
+      <c r="Z18" s="140" t="s">
+        <v>274</v>
+      </c>
+      <c r="AA18" s="140"/>
+      <c r="AB18" s="140"/>
+      <c r="AC18" s="140"/>
+      <c r="AD18" s="140"/>
+      <c r="AE18" s="140" t="s">
+        <v>275</v>
+      </c>
+      <c r="AF18" s="140" t="s">
+        <v>275</v>
+      </c>
     </row>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A19" s="25" t="s">
         <v>220</v>
       </c>
@@ -13851,8 +14301,33 @@
         <f>'NK-LK Transf.'!C16</f>
         <v>1.5960648148148149E-3</v>
       </c>
+      <c r="T19" s="140"/>
+      <c r="U19" s="140" t="s">
+        <v>270</v>
+      </c>
+      <c r="V19" s="140"/>
+      <c r="W19" s="140"/>
+      <c r="X19" s="140" t="s">
+        <v>272</v>
+      </c>
+      <c r="Y19" s="140" t="s">
+        <v>271</v>
+      </c>
+      <c r="Z19" s="140" t="s">
+        <v>274</v>
+      </c>
+      <c r="AA19" s="140"/>
+      <c r="AB19" s="140"/>
+      <c r="AC19" s="140"/>
+      <c r="AD19" s="140"/>
+      <c r="AE19" s="140" t="s">
+        <v>275</v>
+      </c>
+      <c r="AF19" s="140" t="s">
+        <v>275</v>
+      </c>
     </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A20" s="25" t="s">
         <v>243</v>
       </c>
@@ -13914,8 +14389,31 @@
         <f>'NK-LK Transf.'!V16</f>
         <v>1.558912037037037E-3</v>
       </c>
+      <c r="T20" s="140"/>
+      <c r="U20" s="140"/>
+      <c r="V20" s="140"/>
+      <c r="W20" s="140"/>
+      <c r="X20" s="140" t="s">
+        <v>272</v>
+      </c>
+      <c r="Y20" s="140" t="s">
+        <v>271</v>
+      </c>
+      <c r="Z20" s="140"/>
+      <c r="AA20" s="140" t="s">
+        <v>273</v>
+      </c>
+      <c r="AB20" s="140" t="s">
+        <v>270</v>
+      </c>
+      <c r="AC20" s="140"/>
+      <c r="AD20" s="140" t="s">
+        <v>267</v>
+      </c>
+      <c r="AE20" s="140"/>
+      <c r="AF20" s="140"/>
     </row>
-    <row r="21" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A21" s="25" t="s">
         <v>243</v>
       </c>
@@ -13977,8 +14475,31 @@
         <f>'NK-LK Transf.'!U16</f>
         <v>1.5817129629629629E-3</v>
       </c>
+      <c r="T21" s="140"/>
+      <c r="U21" s="140"/>
+      <c r="V21" s="140"/>
+      <c r="W21" s="140"/>
+      <c r="X21" s="140" t="s">
+        <v>272</v>
+      </c>
+      <c r="Y21" s="140" t="s">
+        <v>271</v>
+      </c>
+      <c r="Z21" s="140"/>
+      <c r="AA21" s="140" t="s">
+        <v>273</v>
+      </c>
+      <c r="AB21" s="140" t="s">
+        <v>270</v>
+      </c>
+      <c r="AC21" s="140"/>
+      <c r="AD21" s="140" t="s">
+        <v>267</v>
+      </c>
+      <c r="AE21" s="140"/>
+      <c r="AF21" s="140"/>
     </row>
-    <row r="22" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A22" s="25" t="s">
         <v>243</v>
       </c>
@@ -14040,8 +14561,35 @@
         <f>'NK-LK Transf.'!T16</f>
         <v>1.6129629629629632E-3</v>
       </c>
+      <c r="T22" s="140"/>
+      <c r="U22" s="140" t="s">
+        <v>270</v>
+      </c>
+      <c r="V22" s="140"/>
+      <c r="W22" s="140"/>
+      <c r="X22" s="140" t="s">
+        <v>270</v>
+      </c>
+      <c r="Y22" s="140" t="s">
+        <v>269</v>
+      </c>
+      <c r="Z22" s="140"/>
+      <c r="AA22" s="140" t="s">
+        <v>273</v>
+      </c>
+      <c r="AB22" s="140" t="s">
+        <v>274</v>
+      </c>
+      <c r="AC22" s="140"/>
+      <c r="AD22" s="140"/>
+      <c r="AE22" s="140" t="s">
+        <v>274</v>
+      </c>
+      <c r="AF22" s="140" t="s">
+        <v>274</v>
+      </c>
     </row>
-    <row r="23" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A23" s="25" t="s">
         <v>243</v>
       </c>
@@ -14103,8 +14651,35 @@
         <f>'NK-LK Transf.'!S16</f>
         <v>1.6278935185185185E-3</v>
       </c>
+      <c r="T23" s="140"/>
+      <c r="U23" s="140" t="s">
+        <v>270</v>
+      </c>
+      <c r="V23" s="140"/>
+      <c r="W23" s="140"/>
+      <c r="X23" s="140" t="s">
+        <v>270</v>
+      </c>
+      <c r="Y23" s="140" t="s">
+        <v>269</v>
+      </c>
+      <c r="Z23" s="140"/>
+      <c r="AA23" s="140" t="s">
+        <v>273</v>
+      </c>
+      <c r="AB23" s="140" t="s">
+        <v>274</v>
+      </c>
+      <c r="AC23" s="140"/>
+      <c r="AD23" s="140"/>
+      <c r="AE23" s="140" t="s">
+        <v>274</v>
+      </c>
+      <c r="AF23" s="140" t="s">
+        <v>274</v>
+      </c>
     </row>
-    <row r="24" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A24" s="25" t="s">
         <v>243</v>
       </c>
@@ -14166,8 +14741,33 @@
         <f>'NK-LK Transf.'!R16</f>
         <v>1.644212962962963E-3</v>
       </c>
+      <c r="T24" s="140"/>
+      <c r="U24" s="140"/>
+      <c r="V24" s="140"/>
+      <c r="W24" s="140"/>
+      <c r="X24" s="140" t="s">
+        <v>270</v>
+      </c>
+      <c r="Y24" s="140" t="s">
+        <v>269</v>
+      </c>
+      <c r="Z24" s="140"/>
+      <c r="AA24" s="140" t="s">
+        <v>273</v>
+      </c>
+      <c r="AB24" s="140" t="s">
+        <v>274</v>
+      </c>
+      <c r="AC24" s="140"/>
+      <c r="AD24" s="140"/>
+      <c r="AE24" s="140" t="s">
+        <v>274</v>
+      </c>
+      <c r="AF24" s="140" t="s">
+        <v>274</v>
+      </c>
     </row>
-    <row r="25" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A25" s="25" t="s">
         <v>244</v>
       </c>
@@ -14229,8 +14829,31 @@
         <f>'NK-LK Transf.'!J16</f>
         <v>1.3815972222222222E-3</v>
       </c>
+      <c r="T25" s="140"/>
+      <c r="U25" s="140"/>
+      <c r="V25" s="140"/>
+      <c r="W25" s="140"/>
+      <c r="X25" s="140" t="s">
+        <v>272</v>
+      </c>
+      <c r="Y25" s="140" t="s">
+        <v>271</v>
+      </c>
+      <c r="Z25" s="140"/>
+      <c r="AA25" s="140" t="s">
+        <v>273</v>
+      </c>
+      <c r="AB25" s="140" t="s">
+        <v>270</v>
+      </c>
+      <c r="AC25" s="140"/>
+      <c r="AD25" s="140" t="s">
+        <v>267</v>
+      </c>
+      <c r="AE25" s="140"/>
+      <c r="AF25" s="140"/>
     </row>
-    <row r="26" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A26" s="25" t="s">
         <v>244</v>
       </c>
@@ -14292,8 +14915,31 @@
         <f>'NK-LK Transf.'!I16</f>
         <v>1.4285879629629631E-3</v>
       </c>
+      <c r="T26" s="140"/>
+      <c r="U26" s="140"/>
+      <c r="V26" s="140"/>
+      <c r="W26" s="140"/>
+      <c r="X26" s="140" t="s">
+        <v>272</v>
+      </c>
+      <c r="Y26" s="140" t="s">
+        <v>271</v>
+      </c>
+      <c r="Z26" s="140"/>
+      <c r="AA26" s="140" t="s">
+        <v>273</v>
+      </c>
+      <c r="AB26" s="140" t="s">
+        <v>270</v>
+      </c>
+      <c r="AC26" s="140"/>
+      <c r="AD26" s="140" t="s">
+        <v>267</v>
+      </c>
+      <c r="AE26" s="140"/>
+      <c r="AF26" s="140"/>
     </row>
-    <row r="27" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A27" s="25" t="s">
         <v>244</v>
       </c>
@@ -14355,8 +15001,35 @@
         <f>'NK-LK Transf.'!H16</f>
         <v>1.4697916666666666E-3</v>
       </c>
+      <c r="T27" s="140"/>
+      <c r="U27" s="140" t="s">
+        <v>270</v>
+      </c>
+      <c r="V27" s="140"/>
+      <c r="W27" s="140"/>
+      <c r="X27" s="140" t="s">
+        <v>270</v>
+      </c>
+      <c r="Y27" s="140" t="s">
+        <v>269</v>
+      </c>
+      <c r="Z27" s="140"/>
+      <c r="AA27" s="140" t="s">
+        <v>273</v>
+      </c>
+      <c r="AB27" s="140" t="s">
+        <v>274</v>
+      </c>
+      <c r="AC27" s="140"/>
+      <c r="AD27" s="140"/>
+      <c r="AE27" s="140" t="s">
+        <v>274</v>
+      </c>
+      <c r="AF27" s="140" t="s">
+        <v>274</v>
+      </c>
     </row>
-    <row r="28" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A28" s="25" t="s">
         <v>244</v>
       </c>
@@ -14418,8 +15091,35 @@
         <f>'NK-LK Transf.'!G16</f>
         <v>1.4950231481481481E-3</v>
       </c>
+      <c r="T28" s="140"/>
+      <c r="U28" s="140" t="s">
+        <v>270</v>
+      </c>
+      <c r="V28" s="140"/>
+      <c r="W28" s="140"/>
+      <c r="X28" s="140" t="s">
+        <v>270</v>
+      </c>
+      <c r="Y28" s="140" t="s">
+        <v>269</v>
+      </c>
+      <c r="Z28" s="140"/>
+      <c r="AA28" s="140" t="s">
+        <v>273</v>
+      </c>
+      <c r="AB28" s="140" t="s">
+        <v>274</v>
+      </c>
+      <c r="AC28" s="140"/>
+      <c r="AD28" s="140"/>
+      <c r="AE28" s="140" t="s">
+        <v>274</v>
+      </c>
+      <c r="AF28" s="140" t="s">
+        <v>274</v>
+      </c>
     </row>
-    <row r="29" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A29" s="25" t="s">
         <v>244</v>
       </c>
@@ -14481,8 +15181,33 @@
         <f>'NK-LK Transf.'!F16</f>
         <v>1.522337962962963E-3</v>
       </c>
+      <c r="T29" s="140"/>
+      <c r="U29" s="140"/>
+      <c r="V29" s="140"/>
+      <c r="W29" s="140"/>
+      <c r="X29" s="140" t="s">
+        <v>270</v>
+      </c>
+      <c r="Y29" s="140" t="s">
+        <v>269</v>
+      </c>
+      <c r="Z29" s="140"/>
+      <c r="AA29" s="140" t="s">
+        <v>273</v>
+      </c>
+      <c r="AB29" s="140" t="s">
+        <v>274</v>
+      </c>
+      <c r="AC29" s="140"/>
+      <c r="AD29" s="140"/>
+      <c r="AE29" s="140" t="s">
+        <v>274</v>
+      </c>
+      <c r="AF29" s="140" t="s">
+        <v>274</v>
+      </c>
     </row>
-    <row r="30" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A30" s="25" t="s">
         <v>245</v>
       </c>
@@ -14544,8 +15269,31 @@
         <f>'NK-LK Transf.'!Z16</f>
         <v>1.5517361111111109E-3</v>
       </c>
+      <c r="T30" s="140"/>
+      <c r="U30" s="140"/>
+      <c r="V30" s="140"/>
+      <c r="W30" s="140"/>
+      <c r="X30" s="140" t="s">
+        <v>270</v>
+      </c>
+      <c r="Y30" s="140" t="s">
+        <v>269</v>
+      </c>
+      <c r="Z30" s="140"/>
+      <c r="AA30" s="140" t="s">
+        <v>269</v>
+      </c>
+      <c r="AB30" s="140"/>
+      <c r="AC30" s="140" t="s">
+        <v>267</v>
+      </c>
+      <c r="AD30" s="140" t="s">
+        <v>268</v>
+      </c>
+      <c r="AE30" s="140"/>
+      <c r="AF30" s="140"/>
     </row>
-    <row r="31" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A31" s="25" t="s">
         <v>245</v>
       </c>
@@ -14607,8 +15355,31 @@
         <f>'NK-LK Transf.'!Y16</f>
         <v>1.5564814814814814E-3</v>
       </c>
+      <c r="T31" s="140"/>
+      <c r="U31" s="140"/>
+      <c r="V31" s="140"/>
+      <c r="W31" s="140"/>
+      <c r="X31" s="140" t="s">
+        <v>270</v>
+      </c>
+      <c r="Y31" s="140" t="s">
+        <v>269</v>
+      </c>
+      <c r="Z31" s="140"/>
+      <c r="AA31" s="140" t="s">
+        <v>269</v>
+      </c>
+      <c r="AB31" s="140"/>
+      <c r="AC31" s="140" t="s">
+        <v>267</v>
+      </c>
+      <c r="AD31" s="140" t="s">
+        <v>268</v>
+      </c>
+      <c r="AE31" s="140"/>
+      <c r="AF31" s="140"/>
     </row>
-    <row r="32" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A32" s="25" t="s">
         <v>245</v>
       </c>
@@ -14670,8 +15441,31 @@
         <f>'NK-LK Transf.'!X16</f>
         <v>1.570949074074074E-3</v>
       </c>
+      <c r="T32" s="140"/>
+      <c r="U32" s="140"/>
+      <c r="V32" s="140"/>
+      <c r="W32" s="140"/>
+      <c r="X32" s="140" t="s">
+        <v>270</v>
+      </c>
+      <c r="Y32" s="140" t="s">
+        <v>269</v>
+      </c>
+      <c r="Z32" s="140"/>
+      <c r="AA32" s="140" t="s">
+        <v>269</v>
+      </c>
+      <c r="AB32" s="140"/>
+      <c r="AC32" s="140" t="s">
+        <v>267</v>
+      </c>
+      <c r="AD32" s="140" t="s">
+        <v>268</v>
+      </c>
+      <c r="AE32" s="140"/>
+      <c r="AF32" s="140"/>
     </row>
-    <row r="33" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A33" s="25" t="s">
         <v>245</v>
       </c>
@@ -14733,8 +15527,31 @@
         <f>'NK-LK Transf.'!W16</f>
         <v>1.5829861111111112E-3</v>
       </c>
+      <c r="T33" s="140"/>
+      <c r="U33" s="140"/>
+      <c r="V33" s="140"/>
+      <c r="W33" s="140"/>
+      <c r="X33" s="140" t="s">
+        <v>270</v>
+      </c>
+      <c r="Y33" s="140" t="s">
+        <v>269</v>
+      </c>
+      <c r="Z33" s="140"/>
+      <c r="AA33" s="140" t="s">
+        <v>269</v>
+      </c>
+      <c r="AB33" s="140"/>
+      <c r="AC33" s="140" t="s">
+        <v>267</v>
+      </c>
+      <c r="AD33" s="140" t="s">
+        <v>268</v>
+      </c>
+      <c r="AE33" s="140"/>
+      <c r="AF33" s="140"/>
     </row>
-    <row r="34" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A34" s="25" t="s">
         <v>246</v>
       </c>
@@ -14796,8 +15613,31 @@
         <f>'NK-LK Transf.'!N16</f>
         <v>1.3697916666666665E-3</v>
       </c>
+      <c r="T34" s="140"/>
+      <c r="U34" s="140"/>
+      <c r="V34" s="140"/>
+      <c r="W34" s="140"/>
+      <c r="X34" s="140" t="s">
+        <v>270</v>
+      </c>
+      <c r="Y34" s="140" t="s">
+        <v>269</v>
+      </c>
+      <c r="Z34" s="140"/>
+      <c r="AA34" s="140" t="s">
+        <v>269</v>
+      </c>
+      <c r="AB34" s="140"/>
+      <c r="AC34" s="140" t="s">
+        <v>267</v>
+      </c>
+      <c r="AD34" s="140" t="s">
+        <v>268</v>
+      </c>
+      <c r="AE34" s="140"/>
+      <c r="AF34" s="140"/>
     </row>
-    <row r="35" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A35" s="25" t="s">
         <v>246</v>
       </c>
@@ -14859,8 +15699,31 @@
         <f>'NK-LK Transf.'!M16</f>
         <v>1.377662037037037E-3</v>
       </c>
+      <c r="T35" s="140"/>
+      <c r="U35" s="140"/>
+      <c r="V35" s="140"/>
+      <c r="W35" s="140"/>
+      <c r="X35" s="140" t="s">
+        <v>270</v>
+      </c>
+      <c r="Y35" s="140" t="s">
+        <v>269</v>
+      </c>
+      <c r="Z35" s="140"/>
+      <c r="AA35" s="140" t="s">
+        <v>269</v>
+      </c>
+      <c r="AB35" s="140"/>
+      <c r="AC35" s="140" t="s">
+        <v>267</v>
+      </c>
+      <c r="AD35" s="140" t="s">
+        <v>268</v>
+      </c>
+      <c r="AE35" s="140"/>
+      <c r="AF35" s="140"/>
     </row>
-    <row r="36" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A36" s="25" t="s">
         <v>246</v>
       </c>
@@ -14922,8 +15785,31 @@
         <f>'NK-LK Transf.'!L16</f>
         <v>1.4011574074074074E-3</v>
       </c>
+      <c r="T36" s="140"/>
+      <c r="U36" s="140"/>
+      <c r="V36" s="140"/>
+      <c r="W36" s="140"/>
+      <c r="X36" s="140" t="s">
+        <v>270</v>
+      </c>
+      <c r="Y36" s="140" t="s">
+        <v>269</v>
+      </c>
+      <c r="Z36" s="140"/>
+      <c r="AA36" s="140" t="s">
+        <v>269</v>
+      </c>
+      <c r="AB36" s="140"/>
+      <c r="AC36" s="140" t="s">
+        <v>267</v>
+      </c>
+      <c r="AD36" s="140" t="s">
+        <v>268</v>
+      </c>
+      <c r="AE36" s="140"/>
+      <c r="AF36" s="140"/>
     </row>
-    <row r="37" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A37" s="25" t="s">
         <v>246</v>
       </c>
@@ -14985,6 +15871,29 @@
         <f>'NK-LK Transf.'!K16</f>
         <v>1.4207175925925926E-3</v>
       </c>
+      <c r="T37" s="140"/>
+      <c r="U37" s="140"/>
+      <c r="V37" s="140"/>
+      <c r="W37" s="140"/>
+      <c r="X37" s="140" t="s">
+        <v>270</v>
+      </c>
+      <c r="Y37" s="140" t="s">
+        <v>269</v>
+      </c>
+      <c r="Z37" s="140"/>
+      <c r="AA37" s="140" t="s">
+        <v>269</v>
+      </c>
+      <c r="AB37" s="140"/>
+      <c r="AC37" s="140" t="s">
+        <v>267</v>
+      </c>
+      <c r="AD37" s="140" t="s">
+        <v>268</v>
+      </c>
+      <c r="AE37" s="140"/>
+      <c r="AF37" s="140"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
@@ -15011,133 +15920,133 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:78" s="40" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="125">
+      <c r="A1" s="106">
         <v>2025</v>
       </c>
       <c r="B1" s="45" t="str">
         <f ca="1">CONCATENATE("in: ",YEAR(TODAY())-1," für: ", YEAR(TODAY()))</f>
         <v>in: 2025 für: 2026</v>
       </c>
-      <c r="C1" s="106" t="s">
+      <c r="C1" s="107" t="s">
         <v>220</v>
       </c>
-      <c r="D1" s="106"/>
-      <c r="E1" s="107"/>
-      <c r="F1" s="110" t="s">
+      <c r="D1" s="107"/>
+      <c r="E1" s="108"/>
+      <c r="F1" s="109" t="s">
         <v>221</v>
       </c>
-      <c r="G1" s="111"/>
-      <c r="H1" s="111"/>
-      <c r="I1" s="111"/>
-      <c r="J1" s="112"/>
-      <c r="K1" s="116" t="s">
+      <c r="G1" s="110"/>
+      <c r="H1" s="110"/>
+      <c r="I1" s="110"/>
+      <c r="J1" s="111"/>
+      <c r="K1" s="112" t="s">
         <v>225</v>
       </c>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="118"/>
-      <c r="O1" s="108" t="s">
+      <c r="L1" s="113"/>
+      <c r="M1" s="113"/>
+      <c r="N1" s="114"/>
+      <c r="O1" s="132" t="s">
         <v>222</v>
       </c>
-      <c r="P1" s="108"/>
-      <c r="Q1" s="109"/>
-      <c r="R1" s="122" t="s">
+      <c r="P1" s="132"/>
+      <c r="Q1" s="133"/>
+      <c r="R1" s="134" t="s">
         <v>223</v>
       </c>
-      <c r="S1" s="123"/>
-      <c r="T1" s="123"/>
-      <c r="U1" s="123"/>
-      <c r="V1" s="124"/>
-      <c r="W1" s="119" t="s">
+      <c r="S1" s="135"/>
+      <c r="T1" s="135"/>
+      <c r="U1" s="135"/>
+      <c r="V1" s="136"/>
+      <c r="W1" s="137" t="s">
         <v>226</v>
       </c>
-      <c r="X1" s="120"/>
-      <c r="Y1" s="120"/>
-      <c r="Z1" s="121"/>
+      <c r="X1" s="138"/>
+      <c r="Y1" s="138"/>
+      <c r="Z1" s="139"/>
       <c r="AA1"/>
       <c r="AB1" s="45" t="str">
         <f ca="1">CONCATENATE("in: ",YEAR(TODAY())-1," für: ", YEAR(TODAY()))</f>
         <v>in: 2025 für: 2026</v>
       </c>
-      <c r="AC1" s="126" t="s">
+      <c r="AC1" s="115" t="s">
         <v>227</v>
       </c>
-      <c r="AD1" s="126"/>
-      <c r="AE1" s="127"/>
-      <c r="AF1" s="128" t="s">
+      <c r="AD1" s="115"/>
+      <c r="AE1" s="116"/>
+      <c r="AF1" s="117" t="s">
         <v>228</v>
       </c>
-      <c r="AG1" s="129"/>
-      <c r="AH1" s="129"/>
-      <c r="AI1" s="129"/>
-      <c r="AJ1" s="130"/>
-      <c r="AK1" s="131" t="s">
+      <c r="AG1" s="118"/>
+      <c r="AH1" s="118"/>
+      <c r="AI1" s="118"/>
+      <c r="AJ1" s="119"/>
+      <c r="AK1" s="120" t="s">
         <v>229</v>
       </c>
-      <c r="AL1" s="132"/>
-      <c r="AM1" s="132"/>
-      <c r="AN1" s="133"/>
-      <c r="AO1" s="134" t="s">
+      <c r="AL1" s="121"/>
+      <c r="AM1" s="121"/>
+      <c r="AN1" s="122"/>
+      <c r="AO1" s="123" t="s">
         <v>230</v>
       </c>
-      <c r="AP1" s="135"/>
-      <c r="AQ1" s="136"/>
-      <c r="AR1" s="137" t="s">
+      <c r="AP1" s="124"/>
+      <c r="AQ1" s="125"/>
+      <c r="AR1" s="126" t="s">
         <v>231</v>
       </c>
-      <c r="AS1" s="138"/>
-      <c r="AT1" s="138"/>
-      <c r="AU1" s="138"/>
-      <c r="AV1" s="139"/>
-      <c r="AW1" s="113" t="s">
+      <c r="AS1" s="127"/>
+      <c r="AT1" s="127"/>
+      <c r="AU1" s="127"/>
+      <c r="AV1" s="128"/>
+      <c r="AW1" s="129" t="s">
         <v>232</v>
       </c>
-      <c r="AX1" s="114"/>
-      <c r="AY1" s="114"/>
-      <c r="AZ1" s="115"/>
+      <c r="AX1" s="130"/>
+      <c r="AY1" s="130"/>
+      <c r="AZ1" s="131"/>
       <c r="BB1" s="45" t="str">
         <f ca="1">CONCATENATE("in: ",YEAR(TODAY())-1," für: ", YEAR(TODAY()))</f>
         <v>in: 2025 für: 2026</v>
       </c>
-      <c r="BC1" s="106" t="s">
+      <c r="BC1" s="107" t="s">
         <v>233</v>
       </c>
-      <c r="BD1" s="106"/>
-      <c r="BE1" s="107"/>
-      <c r="BF1" s="110" t="s">
+      <c r="BD1" s="107"/>
+      <c r="BE1" s="108"/>
+      <c r="BF1" s="109" t="s">
         <v>234</v>
       </c>
-      <c r="BG1" s="111"/>
-      <c r="BH1" s="111"/>
-      <c r="BI1" s="111"/>
-      <c r="BJ1" s="112"/>
-      <c r="BK1" s="116" t="s">
+      <c r="BG1" s="110"/>
+      <c r="BH1" s="110"/>
+      <c r="BI1" s="110"/>
+      <c r="BJ1" s="111"/>
+      <c r="BK1" s="112" t="s">
         <v>235</v>
       </c>
-      <c r="BL1" s="117"/>
-      <c r="BM1" s="117"/>
-      <c r="BN1" s="118"/>
-      <c r="BO1" s="108" t="s">
+      <c r="BL1" s="113"/>
+      <c r="BM1" s="113"/>
+      <c r="BN1" s="114"/>
+      <c r="BO1" s="132" t="s">
         <v>241</v>
       </c>
-      <c r="BP1" s="108"/>
-      <c r="BQ1" s="109"/>
-      <c r="BR1" s="122" t="s">
+      <c r="BP1" s="132"/>
+      <c r="BQ1" s="133"/>
+      <c r="BR1" s="134" t="s">
         <v>242</v>
       </c>
-      <c r="BS1" s="123"/>
-      <c r="BT1" s="123"/>
-      <c r="BU1" s="123"/>
-      <c r="BV1" s="124"/>
-      <c r="BW1" s="119" t="s">
+      <c r="BS1" s="135"/>
+      <c r="BT1" s="135"/>
+      <c r="BU1" s="135"/>
+      <c r="BV1" s="136"/>
+      <c r="BW1" s="137" t="s">
         <v>236</v>
       </c>
-      <c r="BX1" s="120"/>
-      <c r="BY1" s="120"/>
-      <c r="BZ1" s="121"/>
+      <c r="BX1" s="138"/>
+      <c r="BY1" s="138"/>
+      <c r="BZ1" s="139"/>
     </row>
     <row r="2" spans="1:78" s="94" customFormat="1" ht="21.4" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="125"/>
+      <c r="A2" s="106"/>
       <c r="B2" s="46" t="s">
         <v>224</v>
       </c>
@@ -15438,7 +16347,7 @@
       </c>
     </row>
     <row r="3" spans="1:78" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A3" s="125"/>
+      <c r="A3" s="106"/>
       <c r="B3" s="47" t="s">
         <v>0</v>
       </c>
@@ -15691,7 +16600,7 @@
       </c>
     </row>
     <row r="4" spans="1:78" x14ac:dyDescent="0.45">
-      <c r="A4" s="125"/>
+      <c r="A4" s="106"/>
       <c r="B4" s="47" t="s">
         <v>185</v>
       </c>
@@ -15943,7 +16852,7 @@
       </c>
     </row>
     <row r="5" spans="1:78" x14ac:dyDescent="0.45">
-      <c r="A5" s="125"/>
+      <c r="A5" s="106"/>
       <c r="B5" s="47" t="s">
         <v>186</v>
       </c>
@@ -16195,7 +17104,7 @@
       </c>
     </row>
     <row r="6" spans="1:78" x14ac:dyDescent="0.45">
-      <c r="A6" s="125"/>
+      <c r="A6" s="106"/>
       <c r="B6" s="47" t="s">
         <v>187</v>
       </c>
@@ -16447,7 +17356,7 @@
       </c>
     </row>
     <row r="7" spans="1:78" x14ac:dyDescent="0.45">
-      <c r="A7" s="125"/>
+      <c r="A7" s="106"/>
       <c r="B7" s="47" t="s">
         <v>188</v>
       </c>
@@ -16699,7 +17608,7 @@
       </c>
     </row>
     <row r="8" spans="1:78" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A8" s="125"/>
+      <c r="A8" s="106"/>
       <c r="B8" s="50" t="s">
         <v>4</v>
       </c>
@@ -16952,132 +17861,132 @@
     </row>
     <row r="9" spans="1:78" ht="14.65" thickTop="1" x14ac:dyDescent="0.45"/>
     <row r="10" spans="1:78" ht="18" x14ac:dyDescent="0.45">
-      <c r="A10" s="125">
+      <c r="A10" s="106">
         <v>2026</v>
       </c>
       <c r="B10" s="45" t="str">
         <f ca="1">CONCATENATE("in: ",YEAR(TODAY())," für: ", YEAR(TODAY())+1)</f>
         <v>in: 2026 für: 2027</v>
       </c>
-      <c r="C10" s="106" t="s">
+      <c r="C10" s="107" t="s">
         <v>220</v>
       </c>
-      <c r="D10" s="106"/>
-      <c r="E10" s="107"/>
-      <c r="F10" s="110" t="s">
+      <c r="D10" s="107"/>
+      <c r="E10" s="108"/>
+      <c r="F10" s="109" t="s">
         <v>221</v>
       </c>
-      <c r="G10" s="111"/>
-      <c r="H10" s="111"/>
-      <c r="I10" s="111"/>
-      <c r="J10" s="112"/>
-      <c r="K10" s="116" t="s">
+      <c r="G10" s="110"/>
+      <c r="H10" s="110"/>
+      <c r="I10" s="110"/>
+      <c r="J10" s="111"/>
+      <c r="K10" s="112" t="s">
         <v>225</v>
       </c>
-      <c r="L10" s="117"/>
-      <c r="M10" s="117"/>
-      <c r="N10" s="118"/>
-      <c r="O10" s="108" t="s">
+      <c r="L10" s="113"/>
+      <c r="M10" s="113"/>
+      <c r="N10" s="114"/>
+      <c r="O10" s="132" t="s">
         <v>222</v>
       </c>
-      <c r="P10" s="108"/>
-      <c r="Q10" s="109"/>
-      <c r="R10" s="122" t="s">
+      <c r="P10" s="132"/>
+      <c r="Q10" s="133"/>
+      <c r="R10" s="134" t="s">
         <v>223</v>
       </c>
-      <c r="S10" s="123"/>
-      <c r="T10" s="123"/>
-      <c r="U10" s="123"/>
-      <c r="V10" s="124"/>
-      <c r="W10" s="119" t="s">
+      <c r="S10" s="135"/>
+      <c r="T10" s="135"/>
+      <c r="U10" s="135"/>
+      <c r="V10" s="136"/>
+      <c r="W10" s="137" t="s">
         <v>226</v>
       </c>
-      <c r="X10" s="120"/>
-      <c r="Y10" s="120"/>
-      <c r="Z10" s="121"/>
+      <c r="X10" s="138"/>
+      <c r="Y10" s="138"/>
+      <c r="Z10" s="139"/>
       <c r="AB10" s="45" t="str">
         <f ca="1">CONCATENATE("in: ",YEAR(TODAY())," für: ", YEAR(TODAY())+1)</f>
         <v>in: 2026 für: 2027</v>
       </c>
-      <c r="AC10" s="126" t="s">
+      <c r="AC10" s="115" t="s">
         <v>227</v>
       </c>
-      <c r="AD10" s="126"/>
-      <c r="AE10" s="127"/>
-      <c r="AF10" s="128" t="s">
+      <c r="AD10" s="115"/>
+      <c r="AE10" s="116"/>
+      <c r="AF10" s="117" t="s">
         <v>228</v>
       </c>
-      <c r="AG10" s="129"/>
-      <c r="AH10" s="129"/>
-      <c r="AI10" s="129"/>
-      <c r="AJ10" s="130"/>
-      <c r="AK10" s="131" t="s">
+      <c r="AG10" s="118"/>
+      <c r="AH10" s="118"/>
+      <c r="AI10" s="118"/>
+      <c r="AJ10" s="119"/>
+      <c r="AK10" s="120" t="s">
         <v>229</v>
       </c>
-      <c r="AL10" s="132"/>
-      <c r="AM10" s="132"/>
-      <c r="AN10" s="133"/>
-      <c r="AO10" s="134" t="s">
+      <c r="AL10" s="121"/>
+      <c r="AM10" s="121"/>
+      <c r="AN10" s="122"/>
+      <c r="AO10" s="123" t="s">
         <v>230</v>
       </c>
-      <c r="AP10" s="135"/>
-      <c r="AQ10" s="136"/>
-      <c r="AR10" s="137" t="s">
+      <c r="AP10" s="124"/>
+      <c r="AQ10" s="125"/>
+      <c r="AR10" s="126" t="s">
         <v>231</v>
       </c>
-      <c r="AS10" s="138"/>
-      <c r="AT10" s="138"/>
-      <c r="AU10" s="138"/>
-      <c r="AV10" s="139"/>
-      <c r="AW10" s="113" t="s">
+      <c r="AS10" s="127"/>
+      <c r="AT10" s="127"/>
+      <c r="AU10" s="127"/>
+      <c r="AV10" s="128"/>
+      <c r="AW10" s="129" t="s">
         <v>232</v>
       </c>
-      <c r="AX10" s="114"/>
-      <c r="AY10" s="114"/>
-      <c r="AZ10" s="115"/>
+      <c r="AX10" s="130"/>
+      <c r="AY10" s="130"/>
+      <c r="AZ10" s="131"/>
       <c r="BB10" s="45" t="str">
         <f ca="1">CONCATENATE("in: ",YEAR(TODAY())," für: ", YEAR(TODAY())+1)</f>
         <v>in: 2026 für: 2027</v>
       </c>
-      <c r="BC10" s="106" t="s">
+      <c r="BC10" s="107" t="s">
         <v>233</v>
       </c>
-      <c r="BD10" s="106"/>
-      <c r="BE10" s="107"/>
-      <c r="BF10" s="110" t="s">
+      <c r="BD10" s="107"/>
+      <c r="BE10" s="108"/>
+      <c r="BF10" s="109" t="s">
         <v>234</v>
       </c>
-      <c r="BG10" s="111"/>
-      <c r="BH10" s="111"/>
-      <c r="BI10" s="111"/>
-      <c r="BJ10" s="112"/>
-      <c r="BK10" s="116" t="s">
+      <c r="BG10" s="110"/>
+      <c r="BH10" s="110"/>
+      <c r="BI10" s="110"/>
+      <c r="BJ10" s="111"/>
+      <c r="BK10" s="112" t="s">
         <v>235</v>
       </c>
-      <c r="BL10" s="117"/>
-      <c r="BM10" s="117"/>
-      <c r="BN10" s="118"/>
-      <c r="BO10" s="108" t="s">
+      <c r="BL10" s="113"/>
+      <c r="BM10" s="113"/>
+      <c r="BN10" s="114"/>
+      <c r="BO10" s="132" t="s">
         <v>241</v>
       </c>
-      <c r="BP10" s="108"/>
-      <c r="BQ10" s="109"/>
-      <c r="BR10" s="122" t="s">
+      <c r="BP10" s="132"/>
+      <c r="BQ10" s="133"/>
+      <c r="BR10" s="134" t="s">
         <v>242</v>
       </c>
-      <c r="BS10" s="123"/>
-      <c r="BT10" s="123"/>
-      <c r="BU10" s="123"/>
-      <c r="BV10" s="124"/>
-      <c r="BW10" s="119" t="s">
+      <c r="BS10" s="135"/>
+      <c r="BT10" s="135"/>
+      <c r="BU10" s="135"/>
+      <c r="BV10" s="136"/>
+      <c r="BW10" s="137" t="s">
         <v>236</v>
       </c>
-      <c r="BX10" s="120"/>
-      <c r="BY10" s="120"/>
-      <c r="BZ10" s="121"/>
+      <c r="BX10" s="138"/>
+      <c r="BY10" s="138"/>
+      <c r="BZ10" s="139"/>
     </row>
     <row r="11" spans="1:78" ht="21.4" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A11" s="125"/>
+      <c r="A11" s="106"/>
       <c r="B11" s="46" t="s">
         <v>224</v>
       </c>
@@ -17378,7 +18287,7 @@
       </c>
     </row>
     <row r="12" spans="1:78" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A12" s="125"/>
+      <c r="A12" s="106"/>
       <c r="B12" s="47" t="s">
         <v>0</v>
       </c>
@@ -17630,7 +18539,7 @@
       </c>
     </row>
     <row r="13" spans="1:78" x14ac:dyDescent="0.45">
-      <c r="A13" s="125"/>
+      <c r="A13" s="106"/>
       <c r="B13" s="47" t="s">
         <v>185</v>
       </c>
@@ -17882,7 +18791,7 @@
       </c>
     </row>
     <row r="14" spans="1:78" x14ac:dyDescent="0.45">
-      <c r="A14" s="125"/>
+      <c r="A14" s="106"/>
       <c r="B14" s="47" t="s">
         <v>186</v>
       </c>
@@ -18134,7 +19043,7 @@
       </c>
     </row>
     <row r="15" spans="1:78" x14ac:dyDescent="0.45">
-      <c r="A15" s="125"/>
+      <c r="A15" s="106"/>
       <c r="B15" s="47" t="s">
         <v>187</v>
       </c>
@@ -18386,7 +19295,7 @@
       </c>
     </row>
     <row r="16" spans="1:78" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A16" s="125"/>
+      <c r="A16" s="106"/>
       <c r="B16" s="47" t="s">
         <v>188</v>
       </c>
@@ -18638,7 +19547,7 @@
       </c>
     </row>
     <row r="17" spans="1:78" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A17" s="125"/>
+      <c r="A17" s="106"/>
       <c r="B17" s="50" t="s">
         <v>4</v>
       </c>
@@ -19105,6 +20014,28 @@
     </row>
   </sheetData>
   <mergeCells count="38">
+    <mergeCell ref="C10:E10"/>
+    <mergeCell ref="O10:Q10"/>
+    <mergeCell ref="C1:E1"/>
+    <mergeCell ref="O1:Q1"/>
+    <mergeCell ref="F10:J10"/>
+    <mergeCell ref="AW10:AZ10"/>
+    <mergeCell ref="K10:N10"/>
+    <mergeCell ref="W10:Z10"/>
+    <mergeCell ref="F1:J1"/>
+    <mergeCell ref="K1:N1"/>
+    <mergeCell ref="R1:V1"/>
+    <mergeCell ref="W1:Z1"/>
+    <mergeCell ref="R10:V10"/>
+    <mergeCell ref="BO10:BQ10"/>
+    <mergeCell ref="BR10:BV10"/>
+    <mergeCell ref="BW10:BZ10"/>
+    <mergeCell ref="BC1:BE1"/>
+    <mergeCell ref="BF1:BJ1"/>
+    <mergeCell ref="BK1:BN1"/>
+    <mergeCell ref="BO1:BQ1"/>
+    <mergeCell ref="BR1:BV1"/>
+    <mergeCell ref="BW1:BZ1"/>
     <mergeCell ref="A1:A8"/>
     <mergeCell ref="A10:A17"/>
     <mergeCell ref="BC10:BE10"/>
@@ -19121,36 +20052,14 @@
     <mergeCell ref="AK10:AN10"/>
     <mergeCell ref="AO10:AQ10"/>
     <mergeCell ref="AR10:AV10"/>
-    <mergeCell ref="BO10:BQ10"/>
-    <mergeCell ref="BR10:BV10"/>
-    <mergeCell ref="BW10:BZ10"/>
-    <mergeCell ref="BC1:BE1"/>
-    <mergeCell ref="BF1:BJ1"/>
-    <mergeCell ref="BK1:BN1"/>
-    <mergeCell ref="BO1:BQ1"/>
-    <mergeCell ref="BR1:BV1"/>
-    <mergeCell ref="BW1:BZ1"/>
-    <mergeCell ref="AW10:AZ10"/>
-    <mergeCell ref="K10:N10"/>
-    <mergeCell ref="W10:Z10"/>
-    <mergeCell ref="F1:J1"/>
-    <mergeCell ref="K1:N1"/>
-    <mergeCell ref="R1:V1"/>
-    <mergeCell ref="W1:Z1"/>
-    <mergeCell ref="R10:V10"/>
-    <mergeCell ref="C10:E10"/>
-    <mergeCell ref="O10:Q10"/>
-    <mergeCell ref="C1:E1"/>
-    <mergeCell ref="O1:Q1"/>
-    <mergeCell ref="F10:J10"/>
   </mergeCells>
   <conditionalFormatting sqref="AC3:AZ8">
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="16" priority="1" operator="equal">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AC12:AZ17">
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="15" priority="2" operator="equal">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>